<commit_message>
update generated data Triggered by 23f32ff031dbc709cb301e62b2fa3072a881d709
</commit_message>
<xml_diff>
--- a/DC-Colos.xlsx
+++ b/DC-Colos.xlsx
@@ -6219,12 +6219,12 @@
     <row r="183">
       <c r="A183" s="1" t="inlineStr">
         <is>
-          <t>LLW</t>
+          <t>CZL</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>Lilongwe, Malawi</t>
+          <t>Constantine, Algeria</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
@@ -6234,29 +6234,29 @@
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>Lilongwe</t>
+          <t>Constantine</t>
         </is>
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>Malawi</t>
+          <t>Algeria</t>
         </is>
       </c>
       <c r="F183" t="inlineStr">
         <is>
-          <t>MW</t>
+          <t>DZ</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="1" t="inlineStr">
         <is>
-          <t>CZL</t>
+          <t>DLA</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>Constantine, Algeria</t>
+          <t>Douala, Cameroon</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
@@ -6266,61 +6266,61 @@
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>Constantine</t>
+          <t>Douala</t>
         </is>
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>Algeria</t>
+          <t>Cameroon</t>
         </is>
       </c>
       <c r="F184" t="inlineStr">
         <is>
-          <t>DZ</t>
+          <t>CM</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="1" t="inlineStr">
         <is>
-          <t>DLA</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>Douala, Cameroon</t>
+          <t>Ahmedabad, India</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>Africa</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>Douala</t>
+          <t>Ahmedabad</t>
         </is>
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>Cameroon</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F185" t="inlineStr">
         <is>
-          <t>CM</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="1" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>ALA</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>Ahmedabad, India</t>
+          <t>Almaty, Kazakhstan</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
@@ -6330,29 +6330,29 @@
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>Ahmedabad</t>
+          <t>Almaty</t>
         </is>
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Kazakhstan</t>
         </is>
       </c>
       <c r="F186" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>KZ</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="1" t="inlineStr">
         <is>
-          <t>ALA</t>
+          <t>BLR</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>Almaty, Kazakhstan</t>
+          <t>Bangalore, India</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
@@ -6362,29 +6362,29 @@
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>Almaty</t>
+          <t>Bangalore</t>
         </is>
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>Kazakhstan</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F187" t="inlineStr">
         <is>
-          <t>KZ</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="1" t="inlineStr">
         <is>
-          <t>BLR</t>
+          <t>BKK</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>Bangalore, India</t>
+          <t>Bangkok, Thailand</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
@@ -6394,29 +6394,29 @@
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bangkok</t>
         </is>
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Thailand</t>
         </is>
       </c>
       <c r="F188" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>TH</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="1" t="inlineStr">
         <is>
-          <t>BKK</t>
+          <t>BWN</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>Bangkok, Thailand</t>
+          <t>Bandar Seri Begawan, Brunei</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
@@ -6426,29 +6426,29 @@
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>Bangkok</t>
+          <t>Bandar Seri Begawan</t>
         </is>
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>Brunei</t>
         </is>
       </c>
       <c r="F189" t="inlineStr">
         <is>
-          <t>TH</t>
+          <t>BN</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" s="1" t="inlineStr">
         <is>
-          <t>BWN</t>
+          <t>CEB</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>Bandar Seri Begawan, Brunei</t>
+          <t>Cebu, Philippines</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
@@ -6458,29 +6458,29 @@
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>Bandar Seri Begawan</t>
+          <t>Cebu</t>
         </is>
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>Brunei</t>
+          <t>Philippines</t>
         </is>
       </c>
       <c r="F190" t="inlineStr">
         <is>
-          <t>BN</t>
+          <t>PH</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="1" t="inlineStr">
         <is>
-          <t>CEB</t>
+          <t>IXC</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>Cebu, Philippines</t>
+          <t>Chandigarh, India</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
@@ -6490,29 +6490,29 @@
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>Cebu</t>
+          <t>Chandigarh</t>
         </is>
       </c>
       <c r="E191" t="inlineStr">
         <is>
-          <t>Philippines</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F191" t="inlineStr">
         <is>
-          <t>PH</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="1" t="inlineStr">
         <is>
-          <t>IXC</t>
+          <t>CGD</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>Chandigarh, India</t>
+          <t>Changde, China</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
@@ -6522,29 +6522,29 @@
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>Chandigarh</t>
+          <t>Changde</t>
         </is>
       </c>
       <c r="E192" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F192" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="1" t="inlineStr">
         <is>
-          <t>CGD</t>
+          <t>MAA</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>Changde, China</t>
+          <t>Chennai, India</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
@@ -6554,29 +6554,29 @@
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>Changde</t>
+          <t>Chennai</t>
         </is>
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F193" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="1" t="inlineStr">
         <is>
-          <t>MAA</t>
+          <t>CGP</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>Chennai, India</t>
+          <t>Chittagong, Bangladesh</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
@@ -6586,29 +6586,29 @@
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>Chennai</t>
+          <t>Chittagong</t>
         </is>
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Bangladesh</t>
         </is>
       </c>
       <c r="F194" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>BD</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" s="1" t="inlineStr">
         <is>
-          <t>CGP</t>
+          <t>CMB</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>Chittagong, Bangladesh</t>
+          <t>Colombo, Sri Lanka</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
@@ -6618,29 +6618,29 @@
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>Chittagong</t>
+          <t>Colombo</t>
         </is>
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>Bangladesh</t>
+          <t>Sri Lanka</t>
         </is>
       </c>
       <c r="F195" t="inlineStr">
         <is>
-          <t>BD</t>
+          <t>LK</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="1" t="inlineStr">
         <is>
-          <t>CMB</t>
+          <t>DAC</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>Colombo, Sri Lanka</t>
+          <t>Dhaka, Bangladesh</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
@@ -6650,29 +6650,29 @@
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>Colombo</t>
+          <t>Dhaka</t>
         </is>
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t>Sri Lanka</t>
+          <t>Bangladesh</t>
         </is>
       </c>
       <c r="F196" t="inlineStr">
         <is>
-          <t>LK</t>
+          <t>BD</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="1" t="inlineStr">
         <is>
-          <t>DAC</t>
+          <t>FUO</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>Dhaka, Bangladesh</t>
+          <t>Foshan, China</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
@@ -6682,29 +6682,29 @@
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>Dhaka</t>
+          <t>Foshan</t>
         </is>
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t>Bangladesh</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F197" t="inlineStr">
         <is>
-          <t>BD</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="1" t="inlineStr">
         <is>
-          <t>FUO</t>
+          <t>FUK</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>Foshan, China</t>
+          <t>Fukuoka, Japan</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
@@ -6714,29 +6714,29 @@
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>Foshan</t>
+          <t>Fukuoka</t>
         </is>
       </c>
       <c r="E198" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="F198" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>JP</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="1" t="inlineStr">
         <is>
-          <t>FUK</t>
+          <t>FOC</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>Fukuoka, Japan</t>
+          <t>Fuzhou, China</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
@@ -6746,29 +6746,29 @@
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>Fukuoka</t>
+          <t>Fuzhou</t>
         </is>
       </c>
       <c r="E199" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F199" t="inlineStr">
         <is>
-          <t>JP</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="1" t="inlineStr">
         <is>
-          <t>FOC</t>
+          <t>CAN</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>Fuzhou, China</t>
+          <t>Guangzhou, China</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
@@ -6778,7 +6778,7 @@
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>Fuzhou</t>
+          <t>Guangzhou</t>
         </is>
       </c>
       <c r="E200" t="inlineStr">
@@ -6795,12 +6795,12 @@
     <row r="201">
       <c r="A201" s="1" t="inlineStr">
         <is>
-          <t>CAN</t>
+          <t>HAK</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>Guangzhou, China</t>
+          <t>Haikou, China</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
@@ -6810,7 +6810,7 @@
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>Guangzhou</t>
+          <t>Haikou</t>
         </is>
       </c>
       <c r="E201" t="inlineStr">
@@ -6827,12 +6827,12 @@
     <row r="202">
       <c r="A202" s="1" t="inlineStr">
         <is>
-          <t>HAK</t>
+          <t>HAN</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>Haikou, China</t>
+          <t>Hanoi, Vietnam</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
@@ -6842,29 +6842,29 @@
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t>Haikou</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="E202" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Vietnam</t>
         </is>
       </c>
       <c r="F202" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>VN</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="1" t="inlineStr">
         <is>
-          <t>HAN</t>
+          <t>SJW</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>Hanoi, Vietnam</t>
+          <t>Hengshui, China</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
@@ -6874,29 +6874,29 @@
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Hengshui</t>
         </is>
       </c>
       <c r="E203" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F203" t="inlineStr">
         <is>
-          <t>VN</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="1" t="inlineStr">
         <is>
-          <t>SJW</t>
+          <t>SGN</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>Hengshui, China</t>
+          <t>Ho Chi Minh City, Vietnam</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
@@ -6906,29 +6906,29 @@
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>Hengshui</t>
+          <t>Ho Chi Minh City</t>
         </is>
       </c>
       <c r="E204" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Vietnam</t>
         </is>
       </c>
       <c r="F204" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>VN</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="1" t="inlineStr">
         <is>
-          <t>SGN</t>
+          <t>HKG</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City, Vietnam</t>
+          <t>Hong Kong</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
@@ -6936,31 +6936,19 @@
           <t>Asia</t>
         </is>
       </c>
-      <c r="D205" t="inlineStr">
-        <is>
-          <t>Ho Chi Minh City</t>
-        </is>
-      </c>
-      <c r="E205" t="inlineStr">
-        <is>
-          <t>Vietnam</t>
-        </is>
-      </c>
-      <c r="F205" t="inlineStr">
-        <is>
-          <t>VN</t>
-        </is>
-      </c>
+      <c r="D205" t="inlineStr"/>
+      <c r="E205" t="inlineStr"/>
+      <c r="F205" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" s="1" t="inlineStr">
         <is>
-          <t>HKG</t>
+          <t>HYD</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>Hong Kong</t>
+          <t>Hyderabad, India</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
@@ -6968,19 +6956,31 @@
           <t>Asia</t>
         </is>
       </c>
-      <c r="D206" t="inlineStr"/>
-      <c r="E206" t="inlineStr"/>
-      <c r="F206" t="inlineStr"/>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>Hyderabad</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" s="1" t="inlineStr">
         <is>
-          <t>HYD</t>
+          <t>ISB</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>Hyderabad, India</t>
+          <t>Islamabad, Pakistan</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
@@ -6990,29 +6990,29 @@
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>Hyderabad</t>
+          <t>Islamabad</t>
         </is>
       </c>
       <c r="E207" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Pakistan</t>
         </is>
       </c>
       <c r="F207" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>PK</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="1" t="inlineStr">
         <is>
-          <t>ISB</t>
+          <t>CGK</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>Islamabad, Pakistan</t>
+          <t>Jakarta, Indonesia</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
@@ -7022,29 +7022,29 @@
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t>Islamabad</t>
+          <t>Jakarta</t>
         </is>
       </c>
       <c r="E208" t="inlineStr">
         <is>
-          <t>Pakistan</t>
+          <t>Indonesia</t>
         </is>
       </c>
       <c r="F208" t="inlineStr">
         <is>
-          <t>PK</t>
+          <t>ID</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="1" t="inlineStr">
         <is>
-          <t>CGK</t>
+          <t>TNA</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>Jakarta, Indonesia</t>
+          <t>Jinan, China</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
@@ -7054,29 +7054,29 @@
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t>Jakarta</t>
+          <t>Jinan</t>
         </is>
       </c>
       <c r="E209" t="inlineStr">
         <is>
-          <t>Indonesia</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F209" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" s="1" t="inlineStr">
         <is>
-          <t>TNA</t>
+          <t>JHB</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>Jinan, China</t>
+          <t>Johor Bahru, Malaysia</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
@@ -7086,29 +7086,29 @@
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>Jinan</t>
+          <t>Johor Bahru</t>
         </is>
       </c>
       <c r="E210" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Malaysia</t>
         </is>
       </c>
       <c r="F210" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>MY</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" s="1" t="inlineStr">
         <is>
-          <t>JHB</t>
+          <t>KNU</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>Johor Bahru, Malaysia</t>
+          <t>Kanpur, India</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
@@ -7118,29 +7118,29 @@
       </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t>Johor Bahru</t>
+          <t>Kanpur</t>
         </is>
       </c>
       <c r="E211" t="inlineStr">
         <is>
-          <t>Malaysia</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F211" t="inlineStr">
         <is>
-          <t>MY</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" s="1" t="inlineStr">
         <is>
-          <t>KNU</t>
+          <t>KHH</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>Kanpur, India</t>
+          <t>Kaohsiung City</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
@@ -7148,31 +7148,19 @@
           <t>Asia</t>
         </is>
       </c>
-      <c r="D212" t="inlineStr">
-        <is>
-          <t>Kanpur</t>
-        </is>
-      </c>
-      <c r="E212" t="inlineStr">
-        <is>
-          <t>India</t>
-        </is>
-      </c>
-      <c r="F212" t="inlineStr">
-        <is>
-          <t>IN</t>
-        </is>
-      </c>
+      <c r="D212" t="inlineStr"/>
+      <c r="E212" t="inlineStr"/>
+      <c r="F212" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" s="1" t="inlineStr">
         <is>
-          <t>KHH</t>
+          <t>KHI</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>Kaohsiung City</t>
+          <t>Karachi, Pakistan</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
@@ -7180,19 +7168,31 @@
           <t>Asia</t>
         </is>
       </c>
-      <c r="D213" t="inlineStr"/>
-      <c r="E213" t="inlineStr"/>
-      <c r="F213" t="inlineStr"/>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>Karachi</t>
+        </is>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>Pakistan</t>
+        </is>
+      </c>
+      <c r="F213" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
     </row>
     <row r="214">
       <c r="A214" s="1" t="inlineStr">
         <is>
-          <t>KHI</t>
+          <t>KTM</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>Karachi, Pakistan</t>
+          <t>Kathmandu, Nepal</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
@@ -7202,29 +7202,29 @@
       </c>
       <c r="D214" t="inlineStr">
         <is>
-          <t>Karachi</t>
+          <t>Kathmandu</t>
         </is>
       </c>
       <c r="E214" t="inlineStr">
         <is>
-          <t>Pakistan</t>
+          <t>Nepal</t>
         </is>
       </c>
       <c r="F214" t="inlineStr">
         <is>
-          <t>PK</t>
+          <t>NP</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" s="1" t="inlineStr">
         <is>
-          <t>KTM</t>
+          <t>CCU</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>Kathmandu, Nepal</t>
+          <t>Kolkata, India</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
@@ -7234,29 +7234,29 @@
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>Kathmandu</t>
+          <t>Kolkata</t>
         </is>
       </c>
       <c r="E215" t="inlineStr">
         <is>
-          <t>Nepal</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F215" t="inlineStr">
         <is>
-          <t>NP</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="1" t="inlineStr">
         <is>
-          <t>CCU</t>
+          <t>KJA</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>Kolkata, India</t>
+          <t>Krasnoyarsk, Russia</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
@@ -7266,29 +7266,29 @@
       </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t>Kolkata</t>
+          <t>Krasnoyarsk</t>
         </is>
       </c>
       <c r="E216" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Russia</t>
         </is>
       </c>
       <c r="F216" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>RU</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="1" t="inlineStr">
         <is>
-          <t>KJA</t>
+          <t>KUL</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>Krasnoyarsk, Russia</t>
+          <t>Kuala Lumpur, Malaysia</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
@@ -7298,29 +7298,29 @@
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>Krasnoyarsk</t>
+          <t>Kuala Lumpur</t>
         </is>
       </c>
       <c r="E217" t="inlineStr">
         <is>
-          <t>Russia</t>
+          <t>Malaysia</t>
         </is>
       </c>
       <c r="F217" t="inlineStr">
         <is>
-          <t>RU</t>
+          <t>MY</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="1" t="inlineStr">
         <is>
-          <t>KUL</t>
+          <t>PKX</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>Kuala Lumpur, Malaysia</t>
+          <t>Langfang, China</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
@@ -7330,29 +7330,29 @@
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>Kuala Lumpur</t>
+          <t>Langfang</t>
         </is>
       </c>
       <c r="E218" t="inlineStr">
         <is>
-          <t>Malaysia</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F218" t="inlineStr">
         <is>
-          <t>MY</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="1" t="inlineStr">
         <is>
-          <t>PKX</t>
+          <t>MFM</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>Langfang, China</t>
+          <t>Macau</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
@@ -7360,31 +7360,19 @@
           <t>Asia</t>
         </is>
       </c>
-      <c r="D219" t="inlineStr">
-        <is>
-          <t>Langfang</t>
-        </is>
-      </c>
-      <c r="E219" t="inlineStr">
-        <is>
-          <t>China</t>
-        </is>
-      </c>
-      <c r="F219" t="inlineStr">
-        <is>
-          <t>CN</t>
-        </is>
-      </c>
+      <c r="D219" t="inlineStr"/>
+      <c r="E219" t="inlineStr"/>
+      <c r="F219" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" s="1" t="inlineStr">
         <is>
-          <t>MFM</t>
+          <t>MLE</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>Macau</t>
+          <t>Malé, Maldives</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
@@ -7392,19 +7380,31 @@
           <t>Asia</t>
         </is>
       </c>
-      <c r="D220" t="inlineStr"/>
-      <c r="E220" t="inlineStr"/>
-      <c r="F220" t="inlineStr"/>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>Malé</t>
+        </is>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>Maldives</t>
+        </is>
+      </c>
+      <c r="F220" t="inlineStr">
+        <is>
+          <t>MV</t>
+        </is>
+      </c>
     </row>
     <row r="221">
       <c r="A221" s="1" t="inlineStr">
         <is>
-          <t>MLE</t>
+          <t>MNL</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>Malé, Maldives</t>
+          <t>Manila, Philippines</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
@@ -7414,29 +7414,29 @@
       </c>
       <c r="D221" t="inlineStr">
         <is>
-          <t>Malé</t>
+          <t>Manila</t>
         </is>
       </c>
       <c r="E221" t="inlineStr">
         <is>
-          <t>Maldives</t>
+          <t>Philippines</t>
         </is>
       </c>
       <c r="F221" t="inlineStr">
         <is>
-          <t>MV</t>
+          <t>PH</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="1" t="inlineStr">
         <is>
-          <t>MNL</t>
+          <t>BOM</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>Manila, Philippines</t>
+          <t>Mumbai, India</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
@@ -7446,29 +7446,29 @@
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t>Manila</t>
+          <t>Mumbai</t>
         </is>
       </c>
       <c r="E222" t="inlineStr">
         <is>
-          <t>Philippines</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F222" t="inlineStr">
         <is>
-          <t>PH</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="1" t="inlineStr">
         <is>
-          <t>BOM</t>
+          <t>NAG</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>Mumbai, India</t>
+          <t>Nagpur, India</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
@@ -7478,7 +7478,7 @@
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>Mumbai</t>
+          <t>Nagpur</t>
         </is>
       </c>
       <c r="E223" t="inlineStr">
@@ -7495,12 +7495,12 @@
     <row r="224">
       <c r="A224" s="1" t="inlineStr">
         <is>
-          <t>NAG</t>
+          <t>OKA</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>Nagpur, India</t>
+          <t>Naha, Japan</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
@@ -7510,29 +7510,29 @@
       </c>
       <c r="D224" t="inlineStr">
         <is>
-          <t>Nagpur</t>
+          <t>Naha</t>
         </is>
       </c>
       <c r="E224" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="F224" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>JP</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" s="1" t="inlineStr">
         <is>
-          <t>OKA</t>
+          <t>DEL</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>Naha, Japan</t>
+          <t>New Delhi, India</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
@@ -7542,29 +7542,29 @@
       </c>
       <c r="D225" t="inlineStr">
         <is>
-          <t>Naha</t>
+          <t>New Delhi</t>
         </is>
       </c>
       <c r="E225" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F225" t="inlineStr">
         <is>
-          <t>JP</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" s="1" t="inlineStr">
         <is>
-          <t>DEL</t>
+          <t>KIX</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>New Delhi, India</t>
+          <t>Osaka, Japan</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
@@ -7574,29 +7574,29 @@
       </c>
       <c r="D226" t="inlineStr">
         <is>
-          <t>New Delhi</t>
+          <t>Osaka</t>
         </is>
       </c>
       <c r="E226" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="F226" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>JP</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" s="1" t="inlineStr">
         <is>
-          <t>KIX</t>
+          <t>PAT</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>Osaka, Japan</t>
+          <t>Patna, India</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
@@ -7606,29 +7606,29 @@
       </c>
       <c r="D227" t="inlineStr">
         <is>
-          <t>Osaka</t>
+          <t>Patna</t>
         </is>
       </c>
       <c r="E227" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F227" t="inlineStr">
         <is>
-          <t>JP</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" s="1" t="inlineStr">
         <is>
-          <t>PAT</t>
+          <t>PNH</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>Patna, India</t>
+          <t>Phnom Penh, Cambodia</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
@@ -7638,29 +7638,29 @@
       </c>
       <c r="D228" t="inlineStr">
         <is>
-          <t>Patna</t>
+          <t>Phnom Penh</t>
         </is>
       </c>
       <c r="E228" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Cambodia</t>
         </is>
       </c>
       <c r="F228" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>KH</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" s="1" t="inlineStr">
         <is>
-          <t>PNH</t>
+          <t>TAO</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>Phnom Penh, Cambodia</t>
+          <t>Qingdao, China</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
@@ -7670,29 +7670,29 @@
       </c>
       <c r="D229" t="inlineStr">
         <is>
-          <t>Phnom Penh</t>
+          <t>Qingdao</t>
         </is>
       </c>
       <c r="E229" t="inlineStr">
         <is>
-          <t>Cambodia</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F229" t="inlineStr">
         <is>
-          <t>KH</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" s="1" t="inlineStr">
         <is>
-          <t>TAO</t>
+          <t>ICN</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>Qingdao, China</t>
+          <t>Seoul, South Korea</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
@@ -7702,29 +7702,29 @@
       </c>
       <c r="D230" t="inlineStr">
         <is>
-          <t>Qingdao</t>
+          <t>Seoul</t>
         </is>
       </c>
       <c r="E230" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>South Korea</t>
         </is>
       </c>
       <c r="F230" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>KR</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" s="1" t="inlineStr">
         <is>
-          <t>ICN</t>
+          <t>SHA</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>Seoul, South Korea</t>
+          <t>Shanghai, China</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
@@ -7734,29 +7734,29 @@
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>Seoul</t>
+          <t>Shanghai</t>
         </is>
       </c>
       <c r="E231" t="inlineStr">
         <is>
-          <t>South Korea</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F231" t="inlineStr">
         <is>
-          <t>KR</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" s="1" t="inlineStr">
         <is>
-          <t>SHA</t>
+          <t>SIN</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>Shanghai, China</t>
+          <t>Singapore, Singapore</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
@@ -7766,29 +7766,29 @@
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>Shanghai</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="E232" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="F232" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>SG</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" s="1" t="inlineStr">
         <is>
-          <t>SIN</t>
+          <t>URT</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>Singapore, Singapore</t>
+          <t>Surat Thani, Thailand</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
@@ -7798,29 +7798,29 @@
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Surat Thani</t>
         </is>
       </c>
       <c r="E233" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Thailand</t>
         </is>
       </c>
       <c r="F233" t="inlineStr">
         <is>
-          <t>SG</t>
+          <t>TH</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" s="1" t="inlineStr">
         <is>
-          <t>URT</t>
+          <t>TPE</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>Surat Thani, Thailand</t>
+          <t>Taipei</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
@@ -7828,31 +7828,19 @@
           <t>Asia</t>
         </is>
       </c>
-      <c r="D234" t="inlineStr">
-        <is>
-          <t>Surat Thani</t>
-        </is>
-      </c>
-      <c r="E234" t="inlineStr">
-        <is>
-          <t>Thailand</t>
-        </is>
-      </c>
-      <c r="F234" t="inlineStr">
-        <is>
-          <t>TH</t>
-        </is>
-      </c>
+      <c r="D234" t="inlineStr"/>
+      <c r="E234" t="inlineStr"/>
+      <c r="F234" t="inlineStr"/>
     </row>
     <row r="235">
       <c r="A235" s="1" t="inlineStr">
         <is>
-          <t>TPE</t>
+          <t>NRT</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>Taipei</t>
+          <t>Tokyo, Japan</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
@@ -7860,19 +7848,31 @@
           <t>Asia</t>
         </is>
       </c>
-      <c r="D235" t="inlineStr"/>
-      <c r="E235" t="inlineStr"/>
-      <c r="F235" t="inlineStr"/>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>Tokyo</t>
+        </is>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="F235" t="inlineStr">
+        <is>
+          <t>JP</t>
+        </is>
+      </c>
     </row>
     <row r="236">
       <c r="A236" s="1" t="inlineStr">
         <is>
-          <t>NRT</t>
+          <t>ULN</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>Tokyo, Japan</t>
+          <t>Ulaanbaatar, Mongolia</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
@@ -7882,29 +7882,29 @@
       </c>
       <c r="D236" t="inlineStr">
         <is>
-          <t>Tokyo</t>
+          <t>Ulaanbaatar</t>
         </is>
       </c>
       <c r="E236" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Mongolia</t>
         </is>
       </c>
       <c r="F236" t="inlineStr">
         <is>
-          <t>JP</t>
+          <t>MN</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" s="1" t="inlineStr">
         <is>
-          <t>ULN</t>
+          <t>VTE</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>Ulaanbaatar, Mongolia</t>
+          <t>Vientiane, Laos</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
@@ -7914,29 +7914,29 @@
       </c>
       <c r="D237" t="inlineStr">
         <is>
-          <t>Ulaanbaatar</t>
+          <t>Vientiane</t>
         </is>
       </c>
       <c r="E237" t="inlineStr">
         <is>
-          <t>Mongolia</t>
+          <t>Laos</t>
         </is>
       </c>
       <c r="F237" t="inlineStr">
         <is>
-          <t>MN</t>
+          <t>LA</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" s="1" t="inlineStr">
         <is>
-          <t>VTE</t>
+          <t>KHN</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>Vientiane, Laos</t>
+          <t>Xinyu, China</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
@@ -7946,29 +7946,29 @@
       </c>
       <c r="D238" t="inlineStr">
         <is>
-          <t>Vientiane</t>
+          <t>Xinyu</t>
         </is>
       </c>
       <c r="E238" t="inlineStr">
         <is>
-          <t>Laos</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F238" t="inlineStr">
         <is>
-          <t>LA</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" s="1" t="inlineStr">
         <is>
-          <t>KHN</t>
+          <t>EVN</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>Xinyu, China</t>
+          <t>Yerevan, Armenia</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
@@ -7978,29 +7978,29 @@
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>Xinyu</t>
+          <t>Yerevan</t>
         </is>
       </c>
       <c r="E239" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Armenia</t>
         </is>
       </c>
       <c r="F239" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>AM</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" s="1" t="inlineStr">
         <is>
-          <t>EVN</t>
+          <t>JOG</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>Yerevan, Armenia</t>
+          <t>Yogyakarta, Indonesia</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
@@ -8010,29 +8010,29 @@
       </c>
       <c r="D240" t="inlineStr">
         <is>
-          <t>Yerevan</t>
+          <t>Yogyakarta</t>
         </is>
       </c>
       <c r="E240" t="inlineStr">
         <is>
-          <t>Armenia</t>
+          <t>Indonesia</t>
         </is>
       </c>
       <c r="F240" t="inlineStr">
         <is>
-          <t>AM</t>
+          <t>ID</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" s="1" t="inlineStr">
         <is>
-          <t>JOG</t>
+          <t>CGY</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>Yogyakarta, Indonesia</t>
+          <t>Cagayan de Oro, Philippines</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
@@ -8042,29 +8042,29 @@
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t>Yogyakarta</t>
+          <t>Cagayan de Oro</t>
         </is>
       </c>
       <c r="E241" t="inlineStr">
         <is>
-          <t>Indonesia</t>
+          <t>Philippines</t>
         </is>
       </c>
       <c r="F241" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>PH</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" s="1" t="inlineStr">
         <is>
-          <t>CGY</t>
+          <t>COK</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>Cagayan de Oro, Philippines</t>
+          <t>Kochi, India</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
@@ -8074,29 +8074,29 @@
       </c>
       <c r="D242" t="inlineStr">
         <is>
-          <t>Cagayan de Oro</t>
+          <t>Kochi</t>
         </is>
       </c>
       <c r="E242" t="inlineStr">
         <is>
-          <t>Philippines</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F242" t="inlineStr">
         <is>
-          <t>PH</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" s="1" t="inlineStr">
         <is>
-          <t>COK</t>
+          <t>DPS</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>Kochi, India</t>
+          <t>Denpasar, Indonesia</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
@@ -8106,29 +8106,29 @@
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>Kochi</t>
+          <t>Denpasar</t>
         </is>
       </c>
       <c r="E243" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Indonesia</t>
         </is>
       </c>
       <c r="F243" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>ID</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" s="1" t="inlineStr">
         <is>
-          <t>DPS</t>
+          <t>CNN</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>Denpasar, Indonesia</t>
+          <t>Kannur, India</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
@@ -8138,29 +8138,29 @@
       </c>
       <c r="D244" t="inlineStr">
         <is>
-          <t>Denpasar</t>
+          <t>Kannur</t>
         </is>
       </c>
       <c r="E244" t="inlineStr">
         <is>
-          <t>Indonesia</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F244" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" s="1" t="inlineStr">
         <is>
-          <t>CNN</t>
+          <t>SZX</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>Kannur, India</t>
+          <t>Shenzhen, China</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
@@ -8170,29 +8170,29 @@
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>Kannur</t>
+          <t>Shenzhen</t>
         </is>
       </c>
       <c r="E245" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F245" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" s="1" t="inlineStr">
         <is>
-          <t>SZX</t>
+          <t>KWE</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>Shenzhen, China</t>
+          <t>Guiyang, China</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
@@ -8202,7 +8202,7 @@
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>Shenzhen</t>
+          <t>Guiyang</t>
         </is>
       </c>
       <c r="E246" t="inlineStr">
@@ -8219,12 +8219,12 @@
     <row r="247">
       <c r="A247" s="1" t="inlineStr">
         <is>
-          <t>KWE</t>
+          <t>HGH</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>Guiyang, China</t>
+          <t>Shaoxing, China</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
@@ -8234,7 +8234,7 @@
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>Guiyang</t>
+          <t>Shaoxing</t>
         </is>
       </c>
       <c r="E247" t="inlineStr">
@@ -8251,12 +8251,12 @@
     <row r="248">
       <c r="A248" s="1" t="inlineStr">
         <is>
-          <t>HGH</t>
+          <t>CZX</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>Shaoxing, China</t>
+          <t>Changzhou, China</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
@@ -8266,7 +8266,7 @@
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>Shaoxing</t>
+          <t>Changzhou</t>
         </is>
       </c>
       <c r="E248" t="inlineStr">
@@ -8283,12 +8283,12 @@
     <row r="249">
       <c r="A249" s="1" t="inlineStr">
         <is>
-          <t>CZX</t>
+          <t>KMG</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>Changzhou, China</t>
+          <t>Kunming, China</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
@@ -8298,7 +8298,7 @@
       </c>
       <c r="D249" t="inlineStr">
         <is>
-          <t>Changzhou</t>
+          <t>Kunming</t>
         </is>
       </c>
       <c r="E249" t="inlineStr">
@@ -8315,12 +8315,12 @@
     <row r="250">
       <c r="A250" s="1" t="inlineStr">
         <is>
-          <t>KMG</t>
+          <t>CNX</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>Kunming, China</t>
+          <t>Chiang Mai, Thailand</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
@@ -8330,29 +8330,29 @@
       </c>
       <c r="D250" t="inlineStr">
         <is>
-          <t>Kunming</t>
+          <t>Chiang Mai</t>
         </is>
       </c>
       <c r="E250" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Thailand</t>
         </is>
       </c>
       <c r="F250" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>TH</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" s="1" t="inlineStr">
         <is>
-          <t>CNX</t>
+          <t>CGO</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>Chiang Mai, Thailand</t>
+          <t>Zhengzhou, China</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
@@ -8362,29 +8362,29 @@
       </c>
       <c r="D251" t="inlineStr">
         <is>
-          <t>Chiang Mai</t>
+          <t>Zhengzhou</t>
         </is>
       </c>
       <c r="E251" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F251" t="inlineStr">
         <is>
-          <t>TH</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" s="1" t="inlineStr">
         <is>
-          <t>CGO</t>
+          <t>TYN</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>Zhengzhou, China</t>
+          <t>Yangquan, China</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
@@ -8394,7 +8394,7 @@
       </c>
       <c r="D252" t="inlineStr">
         <is>
-          <t>Zhengzhou</t>
+          <t>Yangquan</t>
         </is>
       </c>
       <c r="E252" t="inlineStr">
@@ -8411,12 +8411,12 @@
     <row r="253">
       <c r="A253" s="1" t="inlineStr">
         <is>
-          <t>TYN</t>
+          <t>CSX</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>Yangquan, China</t>
+          <t>Changsha, China</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
@@ -8426,7 +8426,7 @@
       </c>
       <c r="D253" t="inlineStr">
         <is>
-          <t>Yangquan</t>
+          <t>Changsha</t>
         </is>
       </c>
       <c r="E253" t="inlineStr">
@@ -8443,12 +8443,12 @@
     <row r="254">
       <c r="A254" s="1" t="inlineStr">
         <is>
-          <t>CSX</t>
+          <t>DLC</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>Changsha, China</t>
+          <t>Dalian, China</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
@@ -8458,7 +8458,7 @@
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t>Changsha</t>
+          <t>Dalian</t>
         </is>
       </c>
       <c r="E254" t="inlineStr">
@@ -8475,12 +8475,12 @@
     <row r="255">
       <c r="A255" s="1" t="inlineStr">
         <is>
-          <t>DLC</t>
+          <t>BHY</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>Dalian, China</t>
+          <t>Beihai, China</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
@@ -8490,7 +8490,7 @@
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>Dalian</t>
+          <t>Beihai</t>
         </is>
       </c>
       <c r="E255" t="inlineStr">
@@ -8507,12 +8507,12 @@
     <row r="256">
       <c r="A256" s="1" t="inlineStr">
         <is>
-          <t>BHY</t>
+          <t>CKG</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>Beihai, China</t>
+          <t>Chongqing, China</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
@@ -8522,7 +8522,7 @@
       </c>
       <c r="D256" t="inlineStr">
         <is>
-          <t>Beihai</t>
+          <t>Chongqing</t>
         </is>
       </c>
       <c r="E256" t="inlineStr">
@@ -8539,12 +8539,12 @@
     <row r="257">
       <c r="A257" s="1" t="inlineStr">
         <is>
-          <t>CKG</t>
+          <t>XFN</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>Chongqing, China</t>
+          <t>Xiangyang, China</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
@@ -8554,7 +8554,7 @@
       </c>
       <c r="D257" t="inlineStr">
         <is>
-          <t>Chongqing</t>
+          <t>Xiangyang</t>
         </is>
       </c>
       <c r="E257" t="inlineStr">
@@ -8571,12 +8571,12 @@
     <row r="258">
       <c r="A258" s="1" t="inlineStr">
         <is>
-          <t>XFN</t>
+          <t>DAD</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>Xiangyang, China</t>
+          <t>Da Nang, Vietnam</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
@@ -8586,29 +8586,29 @@
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>Xiangyang</t>
+          <t>Da Nang</t>
         </is>
       </c>
       <c r="E258" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Vietnam</t>
         </is>
       </c>
       <c r="F258" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>VN</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" s="1" t="inlineStr">
         <is>
-          <t>DAD</t>
+          <t>JXG</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>Da Nang, Vietnam</t>
+          <t>Jiaxing, China</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
@@ -8618,29 +8618,29 @@
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>Da Nang</t>
+          <t>Jiaxing</t>
         </is>
       </c>
       <c r="E259" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F259" t="inlineStr">
         <is>
-          <t>VN</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" s="1" t="inlineStr">
         <is>
-          <t>JXG</t>
+          <t>CRK</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>Jiaxing, China</t>
+          <t>Tarlac City, Philippines</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
@@ -8650,29 +8650,29 @@
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>Jiaxing</t>
+          <t>Tarlac City</t>
         </is>
       </c>
       <c r="E260" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Philippines</t>
         </is>
       </c>
       <c r="F260" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>PH</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" s="1" t="inlineStr">
         <is>
-          <t>CRK</t>
+          <t>PBH</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>Tarlac City, Philippines</t>
+          <t>Thimphu, Bhutan</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
@@ -8682,29 +8682,29 @@
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>Tarlac City</t>
+          <t>Thimphu</t>
         </is>
       </c>
       <c r="E261" t="inlineStr">
         <is>
-          <t>Philippines</t>
+          <t>Bhutan</t>
         </is>
       </c>
       <c r="F261" t="inlineStr">
         <is>
-          <t>PH</t>
+          <t>BT</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" s="1" t="inlineStr">
         <is>
-          <t>PBH</t>
+          <t>XIY</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>Thimphu, Bhutan</t>
+          <t>Baoji, China</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
@@ -8714,29 +8714,29 @@
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t>Thimphu</t>
+          <t>Baoji</t>
         </is>
       </c>
       <c r="E262" t="inlineStr">
         <is>
-          <t>Bhutan</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F262" t="inlineStr">
         <is>
-          <t>BT</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" s="1" t="inlineStr">
         <is>
-          <t>XIY</t>
+          <t>KCH</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>Baoji, China</t>
+          <t>Kuching, Malaysia</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
@@ -8746,29 +8746,29 @@
       </c>
       <c r="D263" t="inlineStr">
         <is>
-          <t>Baoji</t>
+          <t>Kuching</t>
         </is>
       </c>
       <c r="E263" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Malaysia</t>
         </is>
       </c>
       <c r="F263" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>MY</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" s="1" t="inlineStr">
         <is>
-          <t>KCH</t>
+          <t>AKX</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>Kuching, Malaysia</t>
+          <t>Aktobe, Kazakhstan</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
@@ -8778,29 +8778,29 @@
       </c>
       <c r="D264" t="inlineStr">
         <is>
-          <t>Kuching</t>
+          <t>Aktobe</t>
         </is>
       </c>
       <c r="E264" t="inlineStr">
         <is>
-          <t>Malaysia</t>
+          <t>Kazakhstan</t>
         </is>
       </c>
       <c r="F264" t="inlineStr">
         <is>
-          <t>MY</t>
+          <t>KZ</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" s="1" t="inlineStr">
         <is>
-          <t>AKX</t>
+          <t>TEN</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>Aktobe, Kazakhstan</t>
+          <t>Tongren, China</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
@@ -8810,29 +8810,29 @@
       </c>
       <c r="D265" t="inlineStr">
         <is>
-          <t>Aktobe</t>
+          <t>Tongren</t>
         </is>
       </c>
       <c r="E265" t="inlineStr">
         <is>
-          <t>Kazakhstan</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F265" t="inlineStr">
         <is>
-          <t>KZ</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" s="1" t="inlineStr">
         <is>
-          <t>TEN</t>
+          <t>HYN</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>Tongren, China</t>
+          <t>Taizhou, China</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
@@ -8842,7 +8842,7 @@
       </c>
       <c r="D266" t="inlineStr">
         <is>
-          <t>Tongren</t>
+          <t>Taizhou</t>
         </is>
       </c>
       <c r="E266" t="inlineStr">
@@ -8859,12 +8859,12 @@
     <row r="267">
       <c r="A267" s="1" t="inlineStr">
         <is>
-          <t>HYN</t>
+          <t>FRU</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>Taizhou, China</t>
+          <t>Bishkek, Kyrgyzstan</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
@@ -8874,29 +8874,29 @@
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>Taizhou</t>
+          <t>Bishkek</t>
         </is>
       </c>
       <c r="E267" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Kyrgyzstan</t>
         </is>
       </c>
       <c r="F267" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>KG</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" s="1" t="inlineStr">
         <is>
-          <t>FRU</t>
+          <t>MLG</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>Bishkek, Kyrgyzstan</t>
+          <t>Malang, Indonesia</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
@@ -8906,29 +8906,29 @@
       </c>
       <c r="D268" t="inlineStr">
         <is>
-          <t>Bishkek</t>
+          <t>Malang</t>
         </is>
       </c>
       <c r="E268" t="inlineStr">
         <is>
-          <t>Kyrgyzstan</t>
+          <t>Indonesia</t>
         </is>
       </c>
       <c r="F268" t="inlineStr">
         <is>
-          <t>KG</t>
+          <t>ID</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" s="1" t="inlineStr">
         <is>
-          <t>MLG</t>
+          <t>LHE</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>Malang, Indonesia</t>
+          <t>Lahore, Pakistan</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
@@ -8938,29 +8938,29 @@
       </c>
       <c r="D269" t="inlineStr">
         <is>
-          <t>Malang</t>
+          <t>Lahore</t>
         </is>
       </c>
       <c r="E269" t="inlineStr">
         <is>
-          <t>Indonesia</t>
+          <t>Pakistan</t>
         </is>
       </c>
       <c r="F269" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>PK</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" s="1" t="inlineStr">
         <is>
-          <t>LHE</t>
+          <t>CTU</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>Lahore, Pakistan</t>
+          <t>Chengdu, China</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
@@ -8970,29 +8970,29 @@
       </c>
       <c r="D270" t="inlineStr">
         <is>
-          <t>Lahore</t>
+          <t>Chengdu</t>
         </is>
       </c>
       <c r="E270" t="inlineStr">
         <is>
-          <t>Pakistan</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F270" t="inlineStr">
         <is>
-          <t>PK</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" s="1" t="inlineStr">
         <is>
-          <t>CTU</t>
+          <t>AGR</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>Chengdu, China</t>
+          <t>Agra, India</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
@@ -9002,29 +9002,29 @@
       </c>
       <c r="D271" t="inlineStr">
         <is>
-          <t>Chengdu</t>
+          <t>Agra</t>
         </is>
       </c>
       <c r="E271" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F271" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" s="1" t="inlineStr">
         <is>
-          <t>AGR</t>
+          <t>CJB</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>Agra, India</t>
+          <t>Coimbatore, India</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
@@ -9034,7 +9034,7 @@
       </c>
       <c r="D272" t="inlineStr">
         <is>
-          <t>Agra</t>
+          <t>Coimbatore</t>
         </is>
       </c>
       <c r="E272" t="inlineStr">
@@ -9051,12 +9051,12 @@
     <row r="273">
       <c r="A273" s="1" t="inlineStr">
         <is>
-          <t>CJB</t>
+          <t>ACX</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>Coimbatore, India</t>
+          <t>Xingyi, China</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
@@ -9066,29 +9066,29 @@
       </c>
       <c r="D273" t="inlineStr">
         <is>
-          <t>Coimbatore</t>
+          <t>Xingyi</t>
         </is>
       </c>
       <c r="E273" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F273" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="274">
       <c r="A274" s="1" t="inlineStr">
         <is>
-          <t>ACX</t>
+          <t>BBI</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>Xingyi, China</t>
+          <t>Bhubaneswar, India</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
@@ -9098,29 +9098,29 @@
       </c>
       <c r="D274" t="inlineStr">
         <is>
-          <t>Xingyi</t>
+          <t>Bhubaneswar</t>
         </is>
       </c>
       <c r="E274" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F274" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="275">
       <c r="A275" s="1" t="inlineStr">
         <is>
-          <t>BBI</t>
+          <t>LYA</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>Bhubaneswar, India</t>
+          <t>Luoyang, China</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
@@ -9130,29 +9130,29 @@
       </c>
       <c r="D275" t="inlineStr">
         <is>
-          <t>Bhubaneswar</t>
+          <t>Luoyang</t>
         </is>
       </c>
       <c r="E275" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F275" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="276">
       <c r="A276" s="1" t="inlineStr">
         <is>
-          <t>LYA</t>
+          <t>PNQ</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>Luoyang, China</t>
+          <t>Pune, India</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
@@ -9162,29 +9162,29 @@
       </c>
       <c r="D276" t="inlineStr">
         <is>
-          <t>Luoyang</t>
+          <t>Pune</t>
         </is>
       </c>
       <c r="E276" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F276" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="277">
       <c r="A277" s="1" t="inlineStr">
         <is>
-          <t>PNQ</t>
+          <t>JRG</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>Pune, India</t>
+          <t>Sambalpur, India</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
@@ -9194,7 +9194,7 @@
       </c>
       <c r="D277" t="inlineStr">
         <is>
-          <t>Pune</t>
+          <t>Sambalpur</t>
         </is>
       </c>
       <c r="E277" t="inlineStr">
@@ -9211,12 +9211,12 @@
     <row r="278">
       <c r="A278" s="1" t="inlineStr">
         <is>
-          <t>JRG</t>
+          <t>AVA</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>Sambalpur, India</t>
+          <t>Anshun, China</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
@@ -9226,17 +9226,17 @@
       </c>
       <c r="D278" t="inlineStr">
         <is>
-          <t>Sambalpur</t>
+          <t>Anshun</t>
         </is>
       </c>
       <c r="E278" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F278" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>CN</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
update generated data Triggered by 6541fec92185113ca5ce721901e42ccd033320b4
</commit_message>
<xml_diff>
--- a/DC-Colos.xlsx
+++ b/DC-Colos.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F337"/>
+  <dimension ref="A1:F338"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9243,44 +9243,44 @@
     <row r="279">
       <c r="A279" s="1" t="inlineStr">
         <is>
-          <t>ABQ</t>
+          <t>NQZ</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>Albuquerque, NM, United States</t>
+          <t>Astana, Kazakhstan</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>North America</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>Albuquerque, NM</t>
+          <t>Astana</t>
         </is>
       </c>
       <c r="E279" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Kazakhstan</t>
         </is>
       </c>
       <c r="F279" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>KZ</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" s="1" t="inlineStr">
         <is>
-          <t>ANC</t>
+          <t>ABQ</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>Anchorage, AK, United States</t>
+          <t>Albuquerque, NM, United States</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
@@ -9290,7 +9290,7 @@
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>Anchorage, AK</t>
+          <t>Albuquerque, NM</t>
         </is>
       </c>
       <c r="E280" t="inlineStr">
@@ -9307,12 +9307,12 @@
     <row r="281">
       <c r="A281" s="1" t="inlineStr">
         <is>
-          <t>IAD</t>
+          <t>ANC</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>Ashburn, VA, United States</t>
+          <t>Anchorage, AK, United States</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
@@ -9322,7 +9322,7 @@
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>Ashburn, VA</t>
+          <t>Anchorage, AK</t>
         </is>
       </c>
       <c r="E281" t="inlineStr">
@@ -9339,12 +9339,12 @@
     <row r="282">
       <c r="A282" s="1" t="inlineStr">
         <is>
-          <t>ATL</t>
+          <t>IAD</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>Atlanta, GA, United States</t>
+          <t>Ashburn, VA, United States</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
@@ -9354,7 +9354,7 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>Atlanta, GA</t>
+          <t>Ashburn, VA</t>
         </is>
       </c>
       <c r="E282" t="inlineStr">
@@ -9371,12 +9371,12 @@
     <row r="283">
       <c r="A283" s="1" t="inlineStr">
         <is>
-          <t>AUS</t>
+          <t>ATL</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>Austin, TX, United States</t>
+          <t>Atlanta, GA, United States</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
@@ -9386,7 +9386,7 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>Austin, TX</t>
+          <t>Atlanta, GA</t>
         </is>
       </c>
       <c r="E283" t="inlineStr">
@@ -9403,12 +9403,12 @@
     <row r="284">
       <c r="A284" s="1" t="inlineStr">
         <is>
-          <t>BGR</t>
+          <t>AUS</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>Bangor, ME, United States</t>
+          <t>Austin, TX, United States</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
@@ -9418,7 +9418,7 @@
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>Bangor, ME</t>
+          <t>Austin, TX</t>
         </is>
       </c>
       <c r="E284" t="inlineStr">
@@ -9435,12 +9435,12 @@
     <row r="285">
       <c r="A285" s="1" t="inlineStr">
         <is>
-          <t>BOS</t>
+          <t>BGR</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>Boston, MA, United States</t>
+          <t>Bangor, ME, United States</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
@@ -9450,7 +9450,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>Boston, MA</t>
+          <t>Bangor, ME</t>
         </is>
       </c>
       <c r="E285" t="inlineStr">
@@ -9467,12 +9467,12 @@
     <row r="286">
       <c r="A286" s="1" t="inlineStr">
         <is>
-          <t>BUF</t>
+          <t>BOS</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>Buffalo, NY, United States</t>
+          <t>Boston, MA, United States</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
@@ -9482,7 +9482,7 @@
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>Buffalo, NY</t>
+          <t>Boston, MA</t>
         </is>
       </c>
       <c r="E286" t="inlineStr">
@@ -9499,12 +9499,12 @@
     <row r="287">
       <c r="A287" s="1" t="inlineStr">
         <is>
-          <t>YYC</t>
+          <t>BUF</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>Calgary, AB, Canada</t>
+          <t>Buffalo, NY, United States</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
@@ -9514,29 +9514,29 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Buffalo, NY</t>
         </is>
       </c>
       <c r="E287" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F287" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="288">
       <c r="A288" s="1" t="inlineStr">
         <is>
-          <t>CLT</t>
+          <t>YYC</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>Charlotte, NC, United States</t>
+          <t>Calgary, AB, Canada</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
@@ -9546,29 +9546,29 @@
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>Charlotte, NC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="E288" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F288" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="289">
       <c r="A289" s="1" t="inlineStr">
         <is>
-          <t>ORD</t>
+          <t>CLT</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>Chicago, IL, United States</t>
+          <t>Charlotte, NC, United States</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
@@ -9578,7 +9578,7 @@
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>Chicago, IL</t>
+          <t>Charlotte, NC</t>
         </is>
       </c>
       <c r="E289" t="inlineStr">
@@ -9595,12 +9595,12 @@
     <row r="290">
       <c r="A290" s="1" t="inlineStr">
         <is>
-          <t>CLE</t>
+          <t>ORD</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>Cleveland, OH, United States</t>
+          <t>Chicago, IL, United States</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
@@ -9610,7 +9610,7 @@
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>Cleveland, OH</t>
+          <t>Chicago, IL</t>
         </is>
       </c>
       <c r="E290" t="inlineStr">
@@ -9627,12 +9627,12 @@
     <row r="291">
       <c r="A291" s="1" t="inlineStr">
         <is>
-          <t>CMH</t>
+          <t>CLE</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>Columbus, OH, United States</t>
+          <t>Cleveland, OH, United States</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
@@ -9642,7 +9642,7 @@
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>Columbus, OH</t>
+          <t>Cleveland, OH</t>
         </is>
       </c>
       <c r="E291" t="inlineStr">
@@ -9659,12 +9659,12 @@
     <row r="292">
       <c r="A292" s="1" t="inlineStr">
         <is>
-          <t>DFW</t>
+          <t>CMH</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>Dallas, TX, United States</t>
+          <t>Columbus, OH, United States</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
@@ -9674,7 +9674,7 @@
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>Dallas, TX</t>
+          <t>Columbus, OH</t>
         </is>
       </c>
       <c r="E292" t="inlineStr">
@@ -9691,12 +9691,12 @@
     <row r="293">
       <c r="A293" s="1" t="inlineStr">
         <is>
-          <t>DEN</t>
+          <t>DFW</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>Denver, CO, United States</t>
+          <t>Dallas, TX, United States</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
@@ -9706,7 +9706,7 @@
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>Denver, CO</t>
+          <t>Dallas, TX</t>
         </is>
       </c>
       <c r="E293" t="inlineStr">
@@ -9723,12 +9723,12 @@
     <row r="294">
       <c r="A294" s="1" t="inlineStr">
         <is>
-          <t>DTW</t>
+          <t>DEN</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>Detroit, MI, United States</t>
+          <t>Denver, CO, United States</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
@@ -9738,7 +9738,7 @@
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>Detroit, MI</t>
+          <t>Denver, CO</t>
         </is>
       </c>
       <c r="E294" t="inlineStr">
@@ -9755,12 +9755,12 @@
     <row r="295">
       <c r="A295" s="1" t="inlineStr">
         <is>
-          <t>RDU</t>
+          <t>DTW</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>Durham, NC, United States</t>
+          <t>Detroit, MI, United States</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -9770,7 +9770,7 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>Durham, NC</t>
+          <t>Detroit, MI</t>
         </is>
       </c>
       <c r="E295" t="inlineStr">
@@ -9787,12 +9787,12 @@
     <row r="296">
       <c r="A296" s="1" t="inlineStr">
         <is>
-          <t>GDL</t>
+          <t>RDU</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>Guadalajara, Mexico</t>
+          <t>Durham, NC, United States</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -9802,29 +9802,29 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>Guadalajara</t>
+          <t>Durham, NC</t>
         </is>
       </c>
       <c r="E296" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F296" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="297">
       <c r="A297" s="1" t="inlineStr">
         <is>
-          <t>YHZ</t>
+          <t>GDL</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>Halifax, Canada</t>
+          <t>Guadalajara, Mexico</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
@@ -9834,29 +9834,29 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>Halifax</t>
+          <t>Guadalajara</t>
         </is>
       </c>
       <c r="E297" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F297" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>MX</t>
         </is>
       </c>
     </row>
     <row r="298">
       <c r="A298" s="1" t="inlineStr">
         <is>
-          <t>HNL</t>
+          <t>YHZ</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>Honolulu, HI, United States</t>
+          <t>Halifax, Canada</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
@@ -9866,29 +9866,29 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>Honolulu, HI</t>
+          <t>Halifax</t>
         </is>
       </c>
       <c r="E298" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F298" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="299">
       <c r="A299" s="1" t="inlineStr">
         <is>
-          <t>IAH</t>
+          <t>HNL</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>Houston, TX, United States</t>
+          <t>Honolulu, HI, United States</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
@@ -9898,7 +9898,7 @@
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>Houston, TX</t>
+          <t>Honolulu, HI</t>
         </is>
       </c>
       <c r="E299" t="inlineStr">
@@ -9915,12 +9915,12 @@
     <row r="300">
       <c r="A300" s="1" t="inlineStr">
         <is>
-          <t>IND</t>
+          <t>IAH</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>Indianapolis, IN, United States</t>
+          <t>Houston, TX, United States</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
@@ -9930,7 +9930,7 @@
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>Indianapolis, IN</t>
+          <t>Houston, TX</t>
         </is>
       </c>
       <c r="E300" t="inlineStr">
@@ -9947,12 +9947,12 @@
     <row r="301">
       <c r="A301" s="1" t="inlineStr">
         <is>
-          <t>JAX</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>Jacksonville, FL, United States</t>
+          <t>Indianapolis, IN, United States</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
@@ -9962,7 +9962,7 @@
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>Jacksonville, FL</t>
+          <t>Indianapolis, IN</t>
         </is>
       </c>
       <c r="E301" t="inlineStr">
@@ -9979,12 +9979,12 @@
     <row r="302">
       <c r="A302" s="1" t="inlineStr">
         <is>
-          <t>MCI</t>
+          <t>JAX</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>Kansas City, MO, United States</t>
+          <t>Jacksonville, FL, United States</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
@@ -9994,7 +9994,7 @@
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>Kansas City, MO</t>
+          <t>Jacksonville, FL</t>
         </is>
       </c>
       <c r="E302" t="inlineStr">
@@ -10011,12 +10011,12 @@
     <row r="303">
       <c r="A303" s="1" t="inlineStr">
         <is>
-          <t>KIN</t>
+          <t>MCI</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>Kingston, Jamaica</t>
+          <t>Kansas City, MO, United States</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
@@ -10026,29 +10026,29 @@
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>Kingston</t>
+          <t>Kansas City, MO</t>
         </is>
       </c>
       <c r="E303" t="inlineStr">
         <is>
-          <t>Jamaica</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F303" t="inlineStr">
         <is>
-          <t>JM</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="304">
       <c r="A304" s="1" t="inlineStr">
         <is>
-          <t>LAS</t>
+          <t>KIN</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>Las Vegas, NV, United States</t>
+          <t>Kingston, Jamaica</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
@@ -10058,29 +10058,29 @@
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>Las Vegas, NV</t>
+          <t>Kingston</t>
         </is>
       </c>
       <c r="E304" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Jamaica</t>
         </is>
       </c>
       <c r="F304" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>JM</t>
         </is>
       </c>
     </row>
     <row r="305">
       <c r="A305" s="1" t="inlineStr">
         <is>
-          <t>LAX</t>
+          <t>LAS</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>Los Angeles, CA, United States</t>
+          <t>Las Vegas, NV, United States</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
@@ -10090,7 +10090,7 @@
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>Los Angeles, CA</t>
+          <t>Las Vegas, NV</t>
         </is>
       </c>
       <c r="E305" t="inlineStr">
@@ -10107,12 +10107,12 @@
     <row r="306">
       <c r="A306" s="1" t="inlineStr">
         <is>
-          <t>MEM</t>
+          <t>LAX</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>Memphis, TN, United States</t>
+          <t>Los Angeles, CA, United States</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
@@ -10122,7 +10122,7 @@
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t>Memphis, TN</t>
+          <t>Los Angeles, CA</t>
         </is>
       </c>
       <c r="E306" t="inlineStr">
@@ -10139,12 +10139,12 @@
     <row r="307">
       <c r="A307" s="1" t="inlineStr">
         <is>
-          <t>MEX</t>
+          <t>MEM</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>Mexico City, Mexico</t>
+          <t>Memphis, TN, United States</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
@@ -10154,29 +10154,29 @@
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>Mexico City</t>
+          <t>Memphis, TN</t>
         </is>
       </c>
       <c r="E307" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F307" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="308">
       <c r="A308" s="1" t="inlineStr">
         <is>
-          <t>MIA</t>
+          <t>MEX</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>Miami, FL, United States</t>
+          <t>Mexico City, Mexico</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
@@ -10186,29 +10186,29 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>Miami, FL</t>
+          <t>Mexico City</t>
         </is>
       </c>
       <c r="E308" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F308" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
     </row>
     <row r="309">
       <c r="A309" s="1" t="inlineStr">
         <is>
-          <t>MSP</t>
+          <t>MIA</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>Minneapolis, MN, United States</t>
+          <t>Miami, FL, United States</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
@@ -10218,7 +10218,7 @@
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>Minneapolis, MN</t>
+          <t>Miami, FL</t>
         </is>
       </c>
       <c r="E309" t="inlineStr">
@@ -10235,12 +10235,12 @@
     <row r="310">
       <c r="A310" s="1" t="inlineStr">
         <is>
-          <t>YUL</t>
+          <t>MSP</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>Montréal, QC, Canada</t>
+          <t>Minneapolis, MN, United States</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
@@ -10250,29 +10250,29 @@
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>Montréal, QC</t>
+          <t>Minneapolis, MN</t>
         </is>
       </c>
       <c r="E310" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F310" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="311">
       <c r="A311" s="1" t="inlineStr">
         <is>
-          <t>BNA</t>
+          <t>YUL</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Nashville, United States</t>
+          <t>Montréal, QC, Canada</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
@@ -10282,29 +10282,29 @@
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>Nashville</t>
+          <t>Montréal, QC</t>
         </is>
       </c>
       <c r="E311" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F311" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="312">
       <c r="A312" s="1" t="inlineStr">
         <is>
-          <t>EWR</t>
+          <t>BNA</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>Newark, NJ, United States</t>
+          <t>Nashville, United States</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
@@ -10314,7 +10314,7 @@
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>Newark, NJ</t>
+          <t>Nashville</t>
         </is>
       </c>
       <c r="E312" t="inlineStr">
@@ -10331,12 +10331,12 @@
     <row r="313">
       <c r="A313" s="1" t="inlineStr">
         <is>
-          <t>ORF</t>
+          <t>EWR</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Norfolk, VA, United States</t>
+          <t>Newark, NJ, United States</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
@@ -10346,7 +10346,7 @@
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>Norfolk, VA</t>
+          <t>Newark, NJ</t>
         </is>
       </c>
       <c r="E313" t="inlineStr">
@@ -10363,12 +10363,12 @@
     <row r="314">
       <c r="A314" s="1" t="inlineStr">
         <is>
-          <t>OKC</t>
+          <t>ORF</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Oklahoma City, OK, United States</t>
+          <t>Norfolk, VA, United States</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -10378,7 +10378,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>Oklahoma City, OK</t>
+          <t>Norfolk, VA</t>
         </is>
       </c>
       <c r="E314" t="inlineStr">
@@ -10395,12 +10395,12 @@
     <row r="315">
       <c r="A315" s="1" t="inlineStr">
         <is>
-          <t>OMA</t>
+          <t>OKC</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>Omaha, NE, United States</t>
+          <t>Oklahoma City, OK, United States</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
@@ -10410,7 +10410,7 @@
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>Omaha, NE</t>
+          <t>Oklahoma City, OK</t>
         </is>
       </c>
       <c r="E315" t="inlineStr">
@@ -10427,12 +10427,12 @@
     <row r="316">
       <c r="A316" s="1" t="inlineStr">
         <is>
-          <t>PHL</t>
+          <t>OMA</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Philadelphia, United States</t>
+          <t>Omaha, NE, United States</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
@@ -10442,7 +10442,7 @@
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>Philadelphia</t>
+          <t>Omaha, NE</t>
         </is>
       </c>
       <c r="E316" t="inlineStr">
@@ -10459,12 +10459,12 @@
     <row r="317">
       <c r="A317" s="1" t="inlineStr">
         <is>
-          <t>PHX</t>
+          <t>PHL</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Phoenix, AZ, United States</t>
+          <t>Philadelphia, United States</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -10474,7 +10474,7 @@
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t>Phoenix, AZ</t>
+          <t>Philadelphia</t>
         </is>
       </c>
       <c r="E317" t="inlineStr">
@@ -10491,12 +10491,12 @@
     <row r="318">
       <c r="A318" s="1" t="inlineStr">
         <is>
-          <t>PIT</t>
+          <t>PHX</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>Pittsburgh, PA, United States</t>
+          <t>Phoenix, AZ, United States</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
@@ -10506,7 +10506,7 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>Pittsburgh, PA</t>
+          <t>Phoenix, AZ</t>
         </is>
       </c>
       <c r="E318" t="inlineStr">
@@ -10523,12 +10523,12 @@
     <row r="319">
       <c r="A319" s="1" t="inlineStr">
         <is>
-          <t>PDX</t>
+          <t>PIT</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Portland, OR, United States</t>
+          <t>Pittsburgh, PA, United States</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
@@ -10538,7 +10538,7 @@
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>Portland, OR</t>
+          <t>Pittsburgh, PA</t>
         </is>
       </c>
       <c r="E319" t="inlineStr">
@@ -10555,12 +10555,12 @@
     <row r="320">
       <c r="A320" s="1" t="inlineStr">
         <is>
-          <t>QRO</t>
+          <t>PDX</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Queretaro, MX, Mexico</t>
+          <t>Portland, OR, United States</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -10570,29 +10570,29 @@
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t>Queretaro, MX</t>
+          <t>Portland, OR</t>
         </is>
       </c>
       <c r="E320" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F320" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="321">
       <c r="A321" s="1" t="inlineStr">
         <is>
-          <t>RIC</t>
+          <t>QRO</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>Richmond, VA, United States</t>
+          <t>Queretaro, MX, Mexico</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
@@ -10602,29 +10602,29 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>Richmond, VA</t>
+          <t>Queretaro, MX</t>
         </is>
       </c>
       <c r="E321" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F321" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
     </row>
     <row r="322">
       <c r="A322" s="1" t="inlineStr">
         <is>
-          <t>SMF</t>
+          <t>RIC</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>Sacramento, CA, United States</t>
+          <t>Richmond, VA, United States</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
@@ -10634,7 +10634,7 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>Sacramento, CA</t>
+          <t>Richmond, VA</t>
         </is>
       </c>
       <c r="E322" t="inlineStr">
@@ -10651,12 +10651,12 @@
     <row r="323">
       <c r="A323" s="1" t="inlineStr">
         <is>
-          <t>SLC</t>
+          <t>SMF</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>Salt Lake City, UT, United States</t>
+          <t>Sacramento, CA, United States</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -10666,7 +10666,7 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>Salt Lake City, UT</t>
+          <t>Sacramento, CA</t>
         </is>
       </c>
       <c r="E323" t="inlineStr">
@@ -10683,12 +10683,12 @@
     <row r="324">
       <c r="A324" s="1" t="inlineStr">
         <is>
-          <t>SAT</t>
+          <t>SLC</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>San Antonio, TX, United States</t>
+          <t>Salt Lake City, UT, United States</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -10698,7 +10698,7 @@
       </c>
       <c r="D324" t="inlineStr">
         <is>
-          <t>San Antonio, TX</t>
+          <t>Salt Lake City, UT</t>
         </is>
       </c>
       <c r="E324" t="inlineStr">
@@ -10715,12 +10715,12 @@
     <row r="325">
       <c r="A325" s="1" t="inlineStr">
         <is>
-          <t>SAN</t>
+          <t>SAT</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>San Diego, CA, United States</t>
+          <t>San Antonio, TX, United States</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -10730,7 +10730,7 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>San Diego, CA</t>
+          <t>San Antonio, TX</t>
         </is>
       </c>
       <c r="E325" t="inlineStr">
@@ -10747,12 +10747,12 @@
     <row r="326">
       <c r="A326" s="1" t="inlineStr">
         <is>
-          <t>SFO</t>
+          <t>SAN</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>San Francisco, CA, United States</t>
+          <t>San Diego, CA, United States</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
@@ -10762,7 +10762,7 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>San Francisco, CA</t>
+          <t>San Diego, CA</t>
         </is>
       </c>
       <c r="E326" t="inlineStr">
@@ -10779,12 +10779,12 @@
     <row r="327">
       <c r="A327" s="1" t="inlineStr">
         <is>
-          <t>SJC</t>
+          <t>SFO</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>San Jose, CA, United States</t>
+          <t>San Francisco, CA, United States</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
@@ -10794,7 +10794,7 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>San Jose, CA</t>
+          <t>San Francisco, CA</t>
         </is>
       </c>
       <c r="E327" t="inlineStr">
@@ -10811,12 +10811,12 @@
     <row r="328">
       <c r="A328" s="1" t="inlineStr">
         <is>
-          <t>YXE</t>
+          <t>SJC</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>Saskatoon, SK, Canada</t>
+          <t>San Jose, CA, United States</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
@@ -10826,29 +10826,29 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>Saskatoon, SK</t>
+          <t>San Jose, CA</t>
         </is>
       </c>
       <c r="E328" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F328" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="329">
       <c r="A329" s="1" t="inlineStr">
         <is>
-          <t>SEA</t>
+          <t>YXE</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>Seattle, WA, United States</t>
+          <t>Saskatoon, SK, Canada</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
@@ -10858,29 +10858,29 @@
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>Seattle, WA</t>
+          <t>Saskatoon, SK</t>
         </is>
       </c>
       <c r="E329" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F329" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="330">
       <c r="A330" s="1" t="inlineStr">
         <is>
-          <t>FSD</t>
+          <t>SEA</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>Sioux Falls, SD, United States</t>
+          <t>Seattle, WA, United States</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
@@ -10890,7 +10890,7 @@
       </c>
       <c r="D330" t="inlineStr">
         <is>
-          <t>Sioux Falls, SD</t>
+          <t>Seattle, WA</t>
         </is>
       </c>
       <c r="E330" t="inlineStr">
@@ -10907,12 +10907,12 @@
     <row r="331">
       <c r="A331" s="1" t="inlineStr">
         <is>
-          <t>STL</t>
+          <t>FSD</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>St. Louis, MO, United States</t>
+          <t>Sioux Falls, SD, United States</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
@@ -10922,7 +10922,7 @@
       </c>
       <c r="D331" t="inlineStr">
         <is>
-          <t>St. Louis, MO</t>
+          <t>Sioux Falls, SD</t>
         </is>
       </c>
       <c r="E331" t="inlineStr">
@@ -10939,12 +10939,12 @@
     <row r="332">
       <c r="A332" s="1" t="inlineStr">
         <is>
-          <t>TLH</t>
+          <t>STL</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>Tallahassee, FL, United States</t>
+          <t>St. Louis, MO, United States</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
@@ -10954,7 +10954,7 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>Tallahassee, FL</t>
+          <t>St. Louis, MO</t>
         </is>
       </c>
       <c r="E332" t="inlineStr">
@@ -10971,12 +10971,12 @@
     <row r="333">
       <c r="A333" s="1" t="inlineStr">
         <is>
-          <t>TPA</t>
+          <t>TLH</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>Tampa, FL, United States</t>
+          <t>Tallahassee, FL, United States</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
@@ -10986,7 +10986,7 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>Tampa, FL</t>
+          <t>Tallahassee, FL</t>
         </is>
       </c>
       <c r="E333" t="inlineStr">
@@ -11003,12 +11003,12 @@
     <row r="334">
       <c r="A334" s="1" t="inlineStr">
         <is>
-          <t>YYZ</t>
+          <t>TPA</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>Toronto, ON, Canada</t>
+          <t>Tampa, FL, United States</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
@@ -11018,29 +11018,29 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>Toronto, ON</t>
+          <t>Tampa, FL</t>
         </is>
       </c>
       <c r="E334" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F334" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="335">
       <c r="A335" s="1" t="inlineStr">
         <is>
-          <t>YVR</t>
+          <t>YYZ</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>Vancouver, BC, Canada</t>
+          <t>Toronto, ON, Canada</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
@@ -11050,7 +11050,7 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Toronto, ON</t>
         </is>
       </c>
       <c r="E335" t="inlineStr">
@@ -11067,12 +11067,12 @@
     <row r="336">
       <c r="A336" s="1" t="inlineStr">
         <is>
-          <t>YWG</t>
+          <t>YVR</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>Winnipeg, MB, Canada</t>
+          <t>Vancouver, BC, Canada</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
@@ -11082,7 +11082,7 @@
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>Winnipeg, MB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="E336" t="inlineStr">
@@ -11099,30 +11099,62 @@
     <row r="337">
       <c r="A337" s="1" t="inlineStr">
         <is>
+          <t>YWG</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>Winnipeg, MB, Canada</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>North America</t>
+        </is>
+      </c>
+      <c r="D337" t="inlineStr">
+        <is>
+          <t>Winnipeg, MB</t>
+        </is>
+      </c>
+      <c r="E337" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="F337" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" s="1" t="inlineStr">
+        <is>
           <t>CVG</t>
         </is>
       </c>
-      <c r="B337" t="inlineStr">
+      <c r="B338" t="inlineStr">
         <is>
           <t>Cincinnati, United States</t>
         </is>
       </c>
-      <c r="C337" t="inlineStr">
+      <c r="C338" t="inlineStr">
         <is>
           <t>North America</t>
         </is>
       </c>
-      <c r="D337" t="inlineStr">
+      <c r="D338" t="inlineStr">
         <is>
           <t>Cincinnati</t>
         </is>
       </c>
-      <c r="E337" t="inlineStr">
+      <c r="E338" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="F337" t="inlineStr">
+      <c r="F338" t="inlineStr">
         <is>
           <t>US</t>
         </is>

</xml_diff>

<commit_message>
update generated data Triggered by 0324c78d429f65f1060a683ba5b0e85738a5a1f1
</commit_message>
<xml_diff>
--- a/DC-Colos.xlsx
+++ b/DC-Colos.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F338"/>
+  <dimension ref="A1:F339"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9275,44 +9275,44 @@
     <row r="280">
       <c r="A280" s="1" t="inlineStr">
         <is>
-          <t>ABQ</t>
+          <t>BDQ</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>Albuquerque, NM, United States</t>
+          <t>Jamnagar, India</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>North America</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>Albuquerque, NM</t>
+          <t>Jamnagar</t>
         </is>
       </c>
       <c r="E280" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F280" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="281">
       <c r="A281" s="1" t="inlineStr">
         <is>
-          <t>ANC</t>
+          <t>ABQ</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>Anchorage, AK, United States</t>
+          <t>Albuquerque, NM, United States</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
@@ -9322,7 +9322,7 @@
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>Anchorage, AK</t>
+          <t>Albuquerque, NM</t>
         </is>
       </c>
       <c r="E281" t="inlineStr">
@@ -9339,12 +9339,12 @@
     <row r="282">
       <c r="A282" s="1" t="inlineStr">
         <is>
-          <t>IAD</t>
+          <t>ANC</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>Ashburn, VA, United States</t>
+          <t>Anchorage, AK, United States</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
@@ -9354,7 +9354,7 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>Ashburn, VA</t>
+          <t>Anchorage, AK</t>
         </is>
       </c>
       <c r="E282" t="inlineStr">
@@ -9371,12 +9371,12 @@
     <row r="283">
       <c r="A283" s="1" t="inlineStr">
         <is>
-          <t>ATL</t>
+          <t>IAD</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>Atlanta, GA, United States</t>
+          <t>Ashburn, VA, United States</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
@@ -9386,7 +9386,7 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>Atlanta, GA</t>
+          <t>Ashburn, VA</t>
         </is>
       </c>
       <c r="E283" t="inlineStr">
@@ -9403,12 +9403,12 @@
     <row r="284">
       <c r="A284" s="1" t="inlineStr">
         <is>
-          <t>AUS</t>
+          <t>ATL</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>Austin, TX, United States</t>
+          <t>Atlanta, GA, United States</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
@@ -9418,7 +9418,7 @@
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>Austin, TX</t>
+          <t>Atlanta, GA</t>
         </is>
       </c>
       <c r="E284" t="inlineStr">
@@ -9435,12 +9435,12 @@
     <row r="285">
       <c r="A285" s="1" t="inlineStr">
         <is>
-          <t>BGR</t>
+          <t>AUS</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>Bangor, ME, United States</t>
+          <t>Austin, TX, United States</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
@@ -9450,7 +9450,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>Bangor, ME</t>
+          <t>Austin, TX</t>
         </is>
       </c>
       <c r="E285" t="inlineStr">
@@ -9467,12 +9467,12 @@
     <row r="286">
       <c r="A286" s="1" t="inlineStr">
         <is>
-          <t>BOS</t>
+          <t>BGR</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>Boston, MA, United States</t>
+          <t>Bangor, ME, United States</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
@@ -9482,7 +9482,7 @@
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>Boston, MA</t>
+          <t>Bangor, ME</t>
         </is>
       </c>
       <c r="E286" t="inlineStr">
@@ -9499,12 +9499,12 @@
     <row r="287">
       <c r="A287" s="1" t="inlineStr">
         <is>
-          <t>BUF</t>
+          <t>BOS</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>Buffalo, NY, United States</t>
+          <t>Boston, MA, United States</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
@@ -9514,7 +9514,7 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>Buffalo, NY</t>
+          <t>Boston, MA</t>
         </is>
       </c>
       <c r="E287" t="inlineStr">
@@ -9531,12 +9531,12 @@
     <row r="288">
       <c r="A288" s="1" t="inlineStr">
         <is>
-          <t>YYC</t>
+          <t>BUF</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>Calgary, AB, Canada</t>
+          <t>Buffalo, NY, United States</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
@@ -9546,29 +9546,29 @@
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Buffalo, NY</t>
         </is>
       </c>
       <c r="E288" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F288" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="289">
       <c r="A289" s="1" t="inlineStr">
         <is>
-          <t>CLT</t>
+          <t>YYC</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>Charlotte, NC, United States</t>
+          <t>Calgary, AB, Canada</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
@@ -9578,29 +9578,29 @@
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>Charlotte, NC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="E289" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F289" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="290">
       <c r="A290" s="1" t="inlineStr">
         <is>
-          <t>ORD</t>
+          <t>CLT</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>Chicago, IL, United States</t>
+          <t>Charlotte, NC, United States</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
@@ -9610,7 +9610,7 @@
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>Chicago, IL</t>
+          <t>Charlotte, NC</t>
         </is>
       </c>
       <c r="E290" t="inlineStr">
@@ -9627,12 +9627,12 @@
     <row r="291">
       <c r="A291" s="1" t="inlineStr">
         <is>
-          <t>CLE</t>
+          <t>ORD</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>Cleveland, OH, United States</t>
+          <t>Chicago, IL, United States</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
@@ -9642,7 +9642,7 @@
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>Cleveland, OH</t>
+          <t>Chicago, IL</t>
         </is>
       </c>
       <c r="E291" t="inlineStr">
@@ -9659,12 +9659,12 @@
     <row r="292">
       <c r="A292" s="1" t="inlineStr">
         <is>
-          <t>CMH</t>
+          <t>CLE</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>Columbus, OH, United States</t>
+          <t>Cleveland, OH, United States</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
@@ -9674,7 +9674,7 @@
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>Columbus, OH</t>
+          <t>Cleveland, OH</t>
         </is>
       </c>
       <c r="E292" t="inlineStr">
@@ -9691,12 +9691,12 @@
     <row r="293">
       <c r="A293" s="1" t="inlineStr">
         <is>
-          <t>DFW</t>
+          <t>CMH</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>Dallas, TX, United States</t>
+          <t>Columbus, OH, United States</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
@@ -9706,7 +9706,7 @@
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>Dallas, TX</t>
+          <t>Columbus, OH</t>
         </is>
       </c>
       <c r="E293" t="inlineStr">
@@ -9723,12 +9723,12 @@
     <row r="294">
       <c r="A294" s="1" t="inlineStr">
         <is>
-          <t>DEN</t>
+          <t>DFW</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>Denver, CO, United States</t>
+          <t>Dallas, TX, United States</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
@@ -9738,7 +9738,7 @@
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>Denver, CO</t>
+          <t>Dallas, TX</t>
         </is>
       </c>
       <c r="E294" t="inlineStr">
@@ -9755,12 +9755,12 @@
     <row r="295">
       <c r="A295" s="1" t="inlineStr">
         <is>
-          <t>DTW</t>
+          <t>DEN</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>Detroit, MI, United States</t>
+          <t>Denver, CO, United States</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -9770,7 +9770,7 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>Detroit, MI</t>
+          <t>Denver, CO</t>
         </is>
       </c>
       <c r="E295" t="inlineStr">
@@ -9787,12 +9787,12 @@
     <row r="296">
       <c r="A296" s="1" t="inlineStr">
         <is>
-          <t>RDU</t>
+          <t>DTW</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>Durham, NC, United States</t>
+          <t>Detroit, MI, United States</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -9802,7 +9802,7 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>Durham, NC</t>
+          <t>Detroit, MI</t>
         </is>
       </c>
       <c r="E296" t="inlineStr">
@@ -9819,12 +9819,12 @@
     <row r="297">
       <c r="A297" s="1" t="inlineStr">
         <is>
-          <t>GDL</t>
+          <t>RDU</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>Guadalajara, Mexico</t>
+          <t>Durham, NC, United States</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
@@ -9834,29 +9834,29 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>Guadalajara</t>
+          <t>Durham, NC</t>
         </is>
       </c>
       <c r="E297" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F297" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="298">
       <c r="A298" s="1" t="inlineStr">
         <is>
-          <t>YHZ</t>
+          <t>GDL</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>Halifax, Canada</t>
+          <t>Guadalajara, Mexico</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
@@ -9866,29 +9866,29 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>Halifax</t>
+          <t>Guadalajara</t>
         </is>
       </c>
       <c r="E298" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F298" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>MX</t>
         </is>
       </c>
     </row>
     <row r="299">
       <c r="A299" s="1" t="inlineStr">
         <is>
-          <t>HNL</t>
+          <t>YHZ</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>Honolulu, HI, United States</t>
+          <t>Halifax, Canada</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
@@ -9898,29 +9898,29 @@
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>Honolulu, HI</t>
+          <t>Halifax</t>
         </is>
       </c>
       <c r="E299" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F299" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="300">
       <c r="A300" s="1" t="inlineStr">
         <is>
-          <t>IAH</t>
+          <t>HNL</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>Houston, TX, United States</t>
+          <t>Honolulu, HI, United States</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
@@ -9930,7 +9930,7 @@
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>Houston, TX</t>
+          <t>Honolulu, HI</t>
         </is>
       </c>
       <c r="E300" t="inlineStr">
@@ -9947,12 +9947,12 @@
     <row r="301">
       <c r="A301" s="1" t="inlineStr">
         <is>
-          <t>IND</t>
+          <t>IAH</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>Indianapolis, IN, United States</t>
+          <t>Houston, TX, United States</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
@@ -9962,7 +9962,7 @@
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>Indianapolis, IN</t>
+          <t>Houston, TX</t>
         </is>
       </c>
       <c r="E301" t="inlineStr">
@@ -9979,12 +9979,12 @@
     <row r="302">
       <c r="A302" s="1" t="inlineStr">
         <is>
-          <t>JAX</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>Jacksonville, FL, United States</t>
+          <t>Indianapolis, IN, United States</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
@@ -9994,7 +9994,7 @@
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>Jacksonville, FL</t>
+          <t>Indianapolis, IN</t>
         </is>
       </c>
       <c r="E302" t="inlineStr">
@@ -10011,12 +10011,12 @@
     <row r="303">
       <c r="A303" s="1" t="inlineStr">
         <is>
-          <t>MCI</t>
+          <t>JAX</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>Kansas City, MO, United States</t>
+          <t>Jacksonville, FL, United States</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
@@ -10026,7 +10026,7 @@
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>Kansas City, MO</t>
+          <t>Jacksonville, FL</t>
         </is>
       </c>
       <c r="E303" t="inlineStr">
@@ -10043,12 +10043,12 @@
     <row r="304">
       <c r="A304" s="1" t="inlineStr">
         <is>
-          <t>KIN</t>
+          <t>MCI</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>Kingston, Jamaica</t>
+          <t>Kansas City, MO, United States</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
@@ -10058,29 +10058,29 @@
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>Kingston</t>
+          <t>Kansas City, MO</t>
         </is>
       </c>
       <c r="E304" t="inlineStr">
         <is>
-          <t>Jamaica</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F304" t="inlineStr">
         <is>
-          <t>JM</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="305">
       <c r="A305" s="1" t="inlineStr">
         <is>
-          <t>LAS</t>
+          <t>KIN</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>Las Vegas, NV, United States</t>
+          <t>Kingston, Jamaica</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
@@ -10090,29 +10090,29 @@
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>Las Vegas, NV</t>
+          <t>Kingston</t>
         </is>
       </c>
       <c r="E305" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Jamaica</t>
         </is>
       </c>
       <c r="F305" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>JM</t>
         </is>
       </c>
     </row>
     <row r="306">
       <c r="A306" s="1" t="inlineStr">
         <is>
-          <t>LAX</t>
+          <t>LAS</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>Los Angeles, CA, United States</t>
+          <t>Las Vegas, NV, United States</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
@@ -10122,7 +10122,7 @@
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t>Los Angeles, CA</t>
+          <t>Las Vegas, NV</t>
         </is>
       </c>
       <c r="E306" t="inlineStr">
@@ -10139,12 +10139,12 @@
     <row r="307">
       <c r="A307" s="1" t="inlineStr">
         <is>
-          <t>MEM</t>
+          <t>LAX</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>Memphis, TN, United States</t>
+          <t>Los Angeles, CA, United States</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
@@ -10154,7 +10154,7 @@
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>Memphis, TN</t>
+          <t>Los Angeles, CA</t>
         </is>
       </c>
       <c r="E307" t="inlineStr">
@@ -10171,12 +10171,12 @@
     <row r="308">
       <c r="A308" s="1" t="inlineStr">
         <is>
-          <t>MEX</t>
+          <t>MEM</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>Mexico City, Mexico</t>
+          <t>Memphis, TN, United States</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
@@ -10186,29 +10186,29 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>Mexico City</t>
+          <t>Memphis, TN</t>
         </is>
       </c>
       <c r="E308" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F308" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="309">
       <c r="A309" s="1" t="inlineStr">
         <is>
-          <t>MIA</t>
+          <t>MEX</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>Miami, FL, United States</t>
+          <t>Mexico City, Mexico</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
@@ -10218,29 +10218,29 @@
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>Miami, FL</t>
+          <t>Mexico City</t>
         </is>
       </c>
       <c r="E309" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F309" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
     </row>
     <row r="310">
       <c r="A310" s="1" t="inlineStr">
         <is>
-          <t>MSP</t>
+          <t>MIA</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>Minneapolis, MN, United States</t>
+          <t>Miami, FL, United States</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
@@ -10250,7 +10250,7 @@
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>Minneapolis, MN</t>
+          <t>Miami, FL</t>
         </is>
       </c>
       <c r="E310" t="inlineStr">
@@ -10267,12 +10267,12 @@
     <row r="311">
       <c r="A311" s="1" t="inlineStr">
         <is>
-          <t>YUL</t>
+          <t>MSP</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Montréal, QC, Canada</t>
+          <t>Minneapolis, MN, United States</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
@@ -10282,29 +10282,29 @@
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>Montréal, QC</t>
+          <t>Minneapolis, MN</t>
         </is>
       </c>
       <c r="E311" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F311" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="312">
       <c r="A312" s="1" t="inlineStr">
         <is>
-          <t>BNA</t>
+          <t>YUL</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>Nashville, United States</t>
+          <t>Montréal, QC, Canada</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
@@ -10314,29 +10314,29 @@
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>Nashville</t>
+          <t>Montréal, QC</t>
         </is>
       </c>
       <c r="E312" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F312" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="313">
       <c r="A313" s="1" t="inlineStr">
         <is>
-          <t>EWR</t>
+          <t>BNA</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Newark, NJ, United States</t>
+          <t>Nashville, United States</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
@@ -10346,7 +10346,7 @@
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>Newark, NJ</t>
+          <t>Nashville</t>
         </is>
       </c>
       <c r="E313" t="inlineStr">
@@ -10363,12 +10363,12 @@
     <row r="314">
       <c r="A314" s="1" t="inlineStr">
         <is>
-          <t>ORF</t>
+          <t>EWR</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Norfolk, VA, United States</t>
+          <t>Newark, NJ, United States</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -10378,7 +10378,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>Norfolk, VA</t>
+          <t>Newark, NJ</t>
         </is>
       </c>
       <c r="E314" t="inlineStr">
@@ -10395,12 +10395,12 @@
     <row r="315">
       <c r="A315" s="1" t="inlineStr">
         <is>
-          <t>OKC</t>
+          <t>ORF</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>Oklahoma City, OK, United States</t>
+          <t>Norfolk, VA, United States</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
@@ -10410,7 +10410,7 @@
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>Oklahoma City, OK</t>
+          <t>Norfolk, VA</t>
         </is>
       </c>
       <c r="E315" t="inlineStr">
@@ -10427,12 +10427,12 @@
     <row r="316">
       <c r="A316" s="1" t="inlineStr">
         <is>
-          <t>OMA</t>
+          <t>OKC</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Omaha, NE, United States</t>
+          <t>Oklahoma City, OK, United States</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
@@ -10442,7 +10442,7 @@
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>Omaha, NE</t>
+          <t>Oklahoma City, OK</t>
         </is>
       </c>
       <c r="E316" t="inlineStr">
@@ -10459,12 +10459,12 @@
     <row r="317">
       <c r="A317" s="1" t="inlineStr">
         <is>
-          <t>PHL</t>
+          <t>OMA</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Philadelphia, United States</t>
+          <t>Omaha, NE, United States</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -10474,7 +10474,7 @@
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t>Philadelphia</t>
+          <t>Omaha, NE</t>
         </is>
       </c>
       <c r="E317" t="inlineStr">
@@ -10491,12 +10491,12 @@
     <row r="318">
       <c r="A318" s="1" t="inlineStr">
         <is>
-          <t>PHX</t>
+          <t>PHL</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>Phoenix, AZ, United States</t>
+          <t>Philadelphia, United States</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
@@ -10506,7 +10506,7 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>Phoenix, AZ</t>
+          <t>Philadelphia</t>
         </is>
       </c>
       <c r="E318" t="inlineStr">
@@ -10523,12 +10523,12 @@
     <row r="319">
       <c r="A319" s="1" t="inlineStr">
         <is>
-          <t>PIT</t>
+          <t>PHX</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Pittsburgh, PA, United States</t>
+          <t>Phoenix, AZ, United States</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
@@ -10538,7 +10538,7 @@
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>Pittsburgh, PA</t>
+          <t>Phoenix, AZ</t>
         </is>
       </c>
       <c r="E319" t="inlineStr">
@@ -10555,12 +10555,12 @@
     <row r="320">
       <c r="A320" s="1" t="inlineStr">
         <is>
-          <t>PDX</t>
+          <t>PIT</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Portland, OR, United States</t>
+          <t>Pittsburgh, PA, United States</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -10570,7 +10570,7 @@
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t>Portland, OR</t>
+          <t>Pittsburgh, PA</t>
         </is>
       </c>
       <c r="E320" t="inlineStr">
@@ -10587,12 +10587,12 @@
     <row r="321">
       <c r="A321" s="1" t="inlineStr">
         <is>
-          <t>QRO</t>
+          <t>PDX</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>Queretaro, MX, Mexico</t>
+          <t>Portland, OR, United States</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
@@ -10602,29 +10602,29 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>Queretaro, MX</t>
+          <t>Portland, OR</t>
         </is>
       </c>
       <c r="E321" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F321" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="322">
       <c r="A322" s="1" t="inlineStr">
         <is>
-          <t>RIC</t>
+          <t>QRO</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>Richmond, VA, United States</t>
+          <t>Queretaro, MX, Mexico</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
@@ -10634,29 +10634,29 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>Richmond, VA</t>
+          <t>Queretaro, MX</t>
         </is>
       </c>
       <c r="E322" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F322" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
     </row>
     <row r="323">
       <c r="A323" s="1" t="inlineStr">
         <is>
-          <t>SMF</t>
+          <t>RIC</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>Sacramento, CA, United States</t>
+          <t>Richmond, VA, United States</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -10666,7 +10666,7 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>Sacramento, CA</t>
+          <t>Richmond, VA</t>
         </is>
       </c>
       <c r="E323" t="inlineStr">
@@ -10683,12 +10683,12 @@
     <row r="324">
       <c r="A324" s="1" t="inlineStr">
         <is>
-          <t>SLC</t>
+          <t>SMF</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>Salt Lake City, UT, United States</t>
+          <t>Sacramento, CA, United States</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -10698,7 +10698,7 @@
       </c>
       <c r="D324" t="inlineStr">
         <is>
-          <t>Salt Lake City, UT</t>
+          <t>Sacramento, CA</t>
         </is>
       </c>
       <c r="E324" t="inlineStr">
@@ -10715,12 +10715,12 @@
     <row r="325">
       <c r="A325" s="1" t="inlineStr">
         <is>
-          <t>SAT</t>
+          <t>SLC</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>San Antonio, TX, United States</t>
+          <t>Salt Lake City, UT, United States</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -10730,7 +10730,7 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>San Antonio, TX</t>
+          <t>Salt Lake City, UT</t>
         </is>
       </c>
       <c r="E325" t="inlineStr">
@@ -10747,12 +10747,12 @@
     <row r="326">
       <c r="A326" s="1" t="inlineStr">
         <is>
-          <t>SAN</t>
+          <t>SAT</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>San Diego, CA, United States</t>
+          <t>San Antonio, TX, United States</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
@@ -10762,7 +10762,7 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>San Diego, CA</t>
+          <t>San Antonio, TX</t>
         </is>
       </c>
       <c r="E326" t="inlineStr">
@@ -10779,12 +10779,12 @@
     <row r="327">
       <c r="A327" s="1" t="inlineStr">
         <is>
-          <t>SFO</t>
+          <t>SAN</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>San Francisco, CA, United States</t>
+          <t>San Diego, CA, United States</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
@@ -10794,7 +10794,7 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>San Francisco, CA</t>
+          <t>San Diego, CA</t>
         </is>
       </c>
       <c r="E327" t="inlineStr">
@@ -10811,12 +10811,12 @@
     <row r="328">
       <c r="A328" s="1" t="inlineStr">
         <is>
-          <t>SJC</t>
+          <t>SFO</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>San Jose, CA, United States</t>
+          <t>San Francisco, CA, United States</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
@@ -10826,7 +10826,7 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>San Jose, CA</t>
+          <t>San Francisco, CA</t>
         </is>
       </c>
       <c r="E328" t="inlineStr">
@@ -10843,12 +10843,12 @@
     <row r="329">
       <c r="A329" s="1" t="inlineStr">
         <is>
-          <t>YXE</t>
+          <t>SJC</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>Saskatoon, SK, Canada</t>
+          <t>San Jose, CA, United States</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
@@ -10858,29 +10858,29 @@
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>Saskatoon, SK</t>
+          <t>San Jose, CA</t>
         </is>
       </c>
       <c r="E329" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F329" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="330">
       <c r="A330" s="1" t="inlineStr">
         <is>
-          <t>SEA</t>
+          <t>YXE</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>Seattle, WA, United States</t>
+          <t>Saskatoon, SK, Canada</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
@@ -10890,29 +10890,29 @@
       </c>
       <c r="D330" t="inlineStr">
         <is>
-          <t>Seattle, WA</t>
+          <t>Saskatoon, SK</t>
         </is>
       </c>
       <c r="E330" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F330" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="331">
       <c r="A331" s="1" t="inlineStr">
         <is>
-          <t>FSD</t>
+          <t>SEA</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>Sioux Falls, SD, United States</t>
+          <t>Seattle, WA, United States</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
@@ -10922,7 +10922,7 @@
       </c>
       <c r="D331" t="inlineStr">
         <is>
-          <t>Sioux Falls, SD</t>
+          <t>Seattle, WA</t>
         </is>
       </c>
       <c r="E331" t="inlineStr">
@@ -10939,12 +10939,12 @@
     <row r="332">
       <c r="A332" s="1" t="inlineStr">
         <is>
-          <t>STL</t>
+          <t>FSD</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>St. Louis, MO, United States</t>
+          <t>Sioux Falls, SD, United States</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
@@ -10954,7 +10954,7 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>St. Louis, MO</t>
+          <t>Sioux Falls, SD</t>
         </is>
       </c>
       <c r="E332" t="inlineStr">
@@ -10971,12 +10971,12 @@
     <row r="333">
       <c r="A333" s="1" t="inlineStr">
         <is>
-          <t>TLH</t>
+          <t>STL</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>Tallahassee, FL, United States</t>
+          <t>St. Louis, MO, United States</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
@@ -10986,7 +10986,7 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>Tallahassee, FL</t>
+          <t>St. Louis, MO</t>
         </is>
       </c>
       <c r="E333" t="inlineStr">
@@ -11003,12 +11003,12 @@
     <row r="334">
       <c r="A334" s="1" t="inlineStr">
         <is>
-          <t>TPA</t>
+          <t>TLH</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>Tampa, FL, United States</t>
+          <t>Tallahassee, FL, United States</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
@@ -11018,7 +11018,7 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>Tampa, FL</t>
+          <t>Tallahassee, FL</t>
         </is>
       </c>
       <c r="E334" t="inlineStr">
@@ -11035,12 +11035,12 @@
     <row r="335">
       <c r="A335" s="1" t="inlineStr">
         <is>
-          <t>YYZ</t>
+          <t>TPA</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>Toronto, ON, Canada</t>
+          <t>Tampa, FL, United States</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
@@ -11050,29 +11050,29 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>Toronto, ON</t>
+          <t>Tampa, FL</t>
         </is>
       </c>
       <c r="E335" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F335" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="336">
       <c r="A336" s="1" t="inlineStr">
         <is>
-          <t>YVR</t>
+          <t>YYZ</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>Vancouver, BC, Canada</t>
+          <t>Toronto, ON, Canada</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
@@ -11082,7 +11082,7 @@
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Toronto, ON</t>
         </is>
       </c>
       <c r="E336" t="inlineStr">
@@ -11099,12 +11099,12 @@
     <row r="337">
       <c r="A337" s="1" t="inlineStr">
         <is>
-          <t>YWG</t>
+          <t>YVR</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>Winnipeg, MB, Canada</t>
+          <t>Vancouver, BC, Canada</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
@@ -11114,7 +11114,7 @@
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>Winnipeg, MB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="E337" t="inlineStr">
@@ -11131,30 +11131,62 @@
     <row r="338">
       <c r="A338" s="1" t="inlineStr">
         <is>
+          <t>YWG</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>Winnipeg, MB, Canada</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>North America</t>
+        </is>
+      </c>
+      <c r="D338" t="inlineStr">
+        <is>
+          <t>Winnipeg, MB</t>
+        </is>
+      </c>
+      <c r="E338" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="F338" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" s="1" t="inlineStr">
+        <is>
           <t>CVG</t>
         </is>
       </c>
-      <c r="B338" t="inlineStr">
+      <c r="B339" t="inlineStr">
         <is>
           <t>Cincinnati, United States</t>
         </is>
       </c>
-      <c r="C338" t="inlineStr">
+      <c r="C339" t="inlineStr">
         <is>
           <t>North America</t>
         </is>
       </c>
-      <c r="D338" t="inlineStr">
+      <c r="D339" t="inlineStr">
         <is>
           <t>Cincinnati</t>
         </is>
       </c>
-      <c r="E338" t="inlineStr">
+      <c r="E339" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="F338" t="inlineStr">
+      <c r="F339" t="inlineStr">
         <is>
           <t>US</t>
         </is>

</xml_diff>

<commit_message>
update generated data Triggered by 1d4e24b543e7f3c464e53ddfa6c74fd529549993
</commit_message>
<xml_diff>
--- a/DC-Colos.xlsx
+++ b/DC-Colos.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F339"/>
+  <dimension ref="A1:F340"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6283,44 +6283,44 @@
     <row r="185">
       <c r="A185" s="1" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>LLW</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>Ahmedabad, India</t>
+          <t>Lilongwe, Malawi</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>Asia</t>
+          <t>Africa</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>Ahmedabad</t>
+          <t>Lilongwe</t>
         </is>
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Malawi</t>
         </is>
       </c>
       <c r="F185" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>MW</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="1" t="inlineStr">
         <is>
-          <t>ALA</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>Almaty, Kazakhstan</t>
+          <t>Ahmedabad, India</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
@@ -6330,29 +6330,29 @@
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>Almaty</t>
+          <t>Ahmedabad</t>
         </is>
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>Kazakhstan</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F186" t="inlineStr">
         <is>
-          <t>KZ</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="1" t="inlineStr">
         <is>
-          <t>BLR</t>
+          <t>ALA</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>Bangalore, India</t>
+          <t>Almaty, Kazakhstan</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
@@ -6362,29 +6362,29 @@
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Almaty</t>
         </is>
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Kazakhstan</t>
         </is>
       </c>
       <c r="F187" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>KZ</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="1" t="inlineStr">
         <is>
-          <t>BKK</t>
+          <t>BLR</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>Bangkok, Thailand</t>
+          <t>Bangalore, India</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
@@ -6394,29 +6394,29 @@
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>Bangkok</t>
+          <t>Bangalore</t>
         </is>
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F188" t="inlineStr">
         <is>
-          <t>TH</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="1" t="inlineStr">
         <is>
-          <t>BWN</t>
+          <t>BKK</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>Bandar Seri Begawan, Brunei</t>
+          <t>Bangkok, Thailand</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
@@ -6426,29 +6426,29 @@
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>Bandar Seri Begawan</t>
+          <t>Bangkok</t>
         </is>
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>Brunei</t>
+          <t>Thailand</t>
         </is>
       </c>
       <c r="F189" t="inlineStr">
         <is>
-          <t>BN</t>
+          <t>TH</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" s="1" t="inlineStr">
         <is>
-          <t>CEB</t>
+          <t>BWN</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>Cebu, Philippines</t>
+          <t>Bandar Seri Begawan, Brunei</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
@@ -6458,29 +6458,29 @@
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>Cebu</t>
+          <t>Bandar Seri Begawan</t>
         </is>
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>Philippines</t>
+          <t>Brunei</t>
         </is>
       </c>
       <c r="F190" t="inlineStr">
         <is>
-          <t>PH</t>
+          <t>BN</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="1" t="inlineStr">
         <is>
-          <t>IXC</t>
+          <t>CEB</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>Chandigarh, India</t>
+          <t>Cebu, Philippines</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
@@ -6490,29 +6490,29 @@
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>Chandigarh</t>
+          <t>Cebu</t>
         </is>
       </c>
       <c r="E191" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Philippines</t>
         </is>
       </c>
       <c r="F191" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>PH</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="1" t="inlineStr">
         <is>
-          <t>CGD</t>
+          <t>IXC</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>Changde, China</t>
+          <t>Chandigarh, India</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
@@ -6522,29 +6522,29 @@
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>Changde</t>
+          <t>Chandigarh</t>
         </is>
       </c>
       <c r="E192" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F192" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="1" t="inlineStr">
         <is>
-          <t>MAA</t>
+          <t>CGD</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>Chennai, India</t>
+          <t>Changde, China</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
@@ -6554,29 +6554,29 @@
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>Chennai</t>
+          <t>Changde</t>
         </is>
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F193" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="1" t="inlineStr">
         <is>
-          <t>CGP</t>
+          <t>MAA</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>Chittagong, Bangladesh</t>
+          <t>Chennai, India</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
@@ -6586,29 +6586,29 @@
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>Chittagong</t>
+          <t>Chennai</t>
         </is>
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>Bangladesh</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F194" t="inlineStr">
         <is>
-          <t>BD</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" s="1" t="inlineStr">
         <is>
-          <t>CMB</t>
+          <t>CGP</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>Colombo, Sri Lanka</t>
+          <t>Chittagong, Bangladesh</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
@@ -6618,29 +6618,29 @@
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>Colombo</t>
+          <t>Chittagong</t>
         </is>
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>Sri Lanka</t>
+          <t>Bangladesh</t>
         </is>
       </c>
       <c r="F195" t="inlineStr">
         <is>
-          <t>LK</t>
+          <t>BD</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="1" t="inlineStr">
         <is>
-          <t>DAC</t>
+          <t>CMB</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>Dhaka, Bangladesh</t>
+          <t>Colombo, Sri Lanka</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
@@ -6650,29 +6650,29 @@
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>Dhaka</t>
+          <t>Colombo</t>
         </is>
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t>Bangladesh</t>
+          <t>Sri Lanka</t>
         </is>
       </c>
       <c r="F196" t="inlineStr">
         <is>
-          <t>BD</t>
+          <t>LK</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="1" t="inlineStr">
         <is>
-          <t>FUO</t>
+          <t>DAC</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>Foshan, China</t>
+          <t>Dhaka, Bangladesh</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
@@ -6682,29 +6682,29 @@
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>Foshan</t>
+          <t>Dhaka</t>
         </is>
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Bangladesh</t>
         </is>
       </c>
       <c r="F197" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>BD</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="1" t="inlineStr">
         <is>
-          <t>FUK</t>
+          <t>FUO</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>Fukuoka, Japan</t>
+          <t>Foshan, China</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
@@ -6714,29 +6714,29 @@
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>Fukuoka</t>
+          <t>Foshan</t>
         </is>
       </c>
       <c r="E198" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F198" t="inlineStr">
         <is>
-          <t>JP</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="1" t="inlineStr">
         <is>
-          <t>FOC</t>
+          <t>FUK</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>Fuzhou, China</t>
+          <t>Fukuoka, Japan</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
@@ -6746,29 +6746,29 @@
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>Fuzhou</t>
+          <t>Fukuoka</t>
         </is>
       </c>
       <c r="E199" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="F199" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>JP</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="1" t="inlineStr">
         <is>
-          <t>CAN</t>
+          <t>FOC</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>Guangzhou, China</t>
+          <t>Fuzhou, China</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
@@ -6778,7 +6778,7 @@
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>Guangzhou</t>
+          <t>Fuzhou</t>
         </is>
       </c>
       <c r="E200" t="inlineStr">
@@ -6795,12 +6795,12 @@
     <row r="201">
       <c r="A201" s="1" t="inlineStr">
         <is>
-          <t>HAK</t>
+          <t>CAN</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>Haikou, China</t>
+          <t>Guangzhou, China</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
@@ -6810,7 +6810,7 @@
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>Haikou</t>
+          <t>Guangzhou</t>
         </is>
       </c>
       <c r="E201" t="inlineStr">
@@ -6827,12 +6827,12 @@
     <row r="202">
       <c r="A202" s="1" t="inlineStr">
         <is>
-          <t>HAN</t>
+          <t>HAK</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>Hanoi, Vietnam</t>
+          <t>Haikou, China</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
@@ -6842,29 +6842,29 @@
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Haikou</t>
         </is>
       </c>
       <c r="E202" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F202" t="inlineStr">
         <is>
-          <t>VN</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="1" t="inlineStr">
         <is>
-          <t>SJW</t>
+          <t>HAN</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>Hengshui, China</t>
+          <t>Hanoi, Vietnam</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
@@ -6874,29 +6874,29 @@
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>Hengshui</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="E203" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Vietnam</t>
         </is>
       </c>
       <c r="F203" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>VN</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="1" t="inlineStr">
         <is>
-          <t>SGN</t>
+          <t>SJW</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City, Vietnam</t>
+          <t>Hengshui, China</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
@@ -6906,29 +6906,29 @@
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City</t>
+          <t>Hengshui</t>
         </is>
       </c>
       <c r="E204" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F204" t="inlineStr">
         <is>
-          <t>VN</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="1" t="inlineStr">
         <is>
-          <t>HKG</t>
+          <t>SGN</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>Hong Kong</t>
+          <t>Ho Chi Minh City, Vietnam</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
@@ -6936,19 +6936,31 @@
           <t>Asia</t>
         </is>
       </c>
-      <c r="D205" t="inlineStr"/>
-      <c r="E205" t="inlineStr"/>
-      <c r="F205" t="inlineStr"/>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>Ho Chi Minh City</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>Vietnam</t>
+        </is>
+      </c>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>VN</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" s="1" t="inlineStr">
         <is>
-          <t>HYD</t>
+          <t>HKG</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>Hyderabad, India</t>
+          <t>Hong Kong</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
@@ -6956,31 +6968,19 @@
           <t>Asia</t>
         </is>
       </c>
-      <c r="D206" t="inlineStr">
-        <is>
-          <t>Hyderabad</t>
-        </is>
-      </c>
-      <c r="E206" t="inlineStr">
-        <is>
-          <t>India</t>
-        </is>
-      </c>
-      <c r="F206" t="inlineStr">
-        <is>
-          <t>IN</t>
-        </is>
-      </c>
+      <c r="D206" t="inlineStr"/>
+      <c r="E206" t="inlineStr"/>
+      <c r="F206" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" s="1" t="inlineStr">
         <is>
-          <t>ISB</t>
+          <t>HYD</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>Islamabad, Pakistan</t>
+          <t>Hyderabad, India</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
@@ -6990,29 +6990,29 @@
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>Islamabad</t>
+          <t>Hyderabad</t>
         </is>
       </c>
       <c r="E207" t="inlineStr">
         <is>
-          <t>Pakistan</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F207" t="inlineStr">
         <is>
-          <t>PK</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="1" t="inlineStr">
         <is>
-          <t>CGK</t>
+          <t>ISB</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>Jakarta, Indonesia</t>
+          <t>Islamabad, Pakistan</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
@@ -7022,29 +7022,29 @@
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t>Jakarta</t>
+          <t>Islamabad</t>
         </is>
       </c>
       <c r="E208" t="inlineStr">
         <is>
-          <t>Indonesia</t>
+          <t>Pakistan</t>
         </is>
       </c>
       <c r="F208" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>PK</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="1" t="inlineStr">
         <is>
-          <t>TNA</t>
+          <t>CGK</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>Jinan, China</t>
+          <t>Jakarta, Indonesia</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
@@ -7054,29 +7054,29 @@
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t>Jinan</t>
+          <t>Jakarta</t>
         </is>
       </c>
       <c r="E209" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Indonesia</t>
         </is>
       </c>
       <c r="F209" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>ID</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" s="1" t="inlineStr">
         <is>
-          <t>JHB</t>
+          <t>TNA</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>Johor Bahru, Malaysia</t>
+          <t>Jinan, China</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
@@ -7086,29 +7086,29 @@
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>Johor Bahru</t>
+          <t>Jinan</t>
         </is>
       </c>
       <c r="E210" t="inlineStr">
         <is>
-          <t>Malaysia</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F210" t="inlineStr">
         <is>
-          <t>MY</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" s="1" t="inlineStr">
         <is>
-          <t>KNU</t>
+          <t>JHB</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>Kanpur, India</t>
+          <t>Johor Bahru, Malaysia</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
@@ -7118,29 +7118,29 @@
       </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t>Kanpur</t>
+          <t>Johor Bahru</t>
         </is>
       </c>
       <c r="E211" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Malaysia</t>
         </is>
       </c>
       <c r="F211" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>MY</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" s="1" t="inlineStr">
         <is>
-          <t>KHH</t>
+          <t>KNU</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>Kaohsiung City</t>
+          <t>Kanpur, India</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
@@ -7148,19 +7148,31 @@
           <t>Asia</t>
         </is>
       </c>
-      <c r="D212" t="inlineStr"/>
-      <c r="E212" t="inlineStr"/>
-      <c r="F212" t="inlineStr"/>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>Kanpur</t>
+        </is>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
     </row>
     <row r="213">
       <c r="A213" s="1" t="inlineStr">
         <is>
-          <t>KHI</t>
+          <t>KHH</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>Karachi, Pakistan</t>
+          <t>Kaohsiung City</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
@@ -7168,31 +7180,19 @@
           <t>Asia</t>
         </is>
       </c>
-      <c r="D213" t="inlineStr">
-        <is>
-          <t>Karachi</t>
-        </is>
-      </c>
-      <c r="E213" t="inlineStr">
-        <is>
-          <t>Pakistan</t>
-        </is>
-      </c>
-      <c r="F213" t="inlineStr">
-        <is>
-          <t>PK</t>
-        </is>
-      </c>
+      <c r="D213" t="inlineStr"/>
+      <c r="E213" t="inlineStr"/>
+      <c r="F213" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" s="1" t="inlineStr">
         <is>
-          <t>KTM</t>
+          <t>KHI</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>Kathmandu, Nepal</t>
+          <t>Karachi, Pakistan</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
@@ -7202,29 +7202,29 @@
       </c>
       <c r="D214" t="inlineStr">
         <is>
-          <t>Kathmandu</t>
+          <t>Karachi</t>
         </is>
       </c>
       <c r="E214" t="inlineStr">
         <is>
-          <t>Nepal</t>
+          <t>Pakistan</t>
         </is>
       </c>
       <c r="F214" t="inlineStr">
         <is>
-          <t>NP</t>
+          <t>PK</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" s="1" t="inlineStr">
         <is>
-          <t>CCU</t>
+          <t>KTM</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>Kolkata, India</t>
+          <t>Kathmandu, Nepal</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
@@ -7234,29 +7234,29 @@
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>Kolkata</t>
+          <t>Kathmandu</t>
         </is>
       </c>
       <c r="E215" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Nepal</t>
         </is>
       </c>
       <c r="F215" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>NP</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="1" t="inlineStr">
         <is>
-          <t>KJA</t>
+          <t>CCU</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>Krasnoyarsk, Russia</t>
+          <t>Kolkata, India</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
@@ -7266,29 +7266,29 @@
       </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t>Krasnoyarsk</t>
+          <t>Kolkata</t>
         </is>
       </c>
       <c r="E216" t="inlineStr">
         <is>
-          <t>Russia</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F216" t="inlineStr">
         <is>
-          <t>RU</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="1" t="inlineStr">
         <is>
-          <t>KUL</t>
+          <t>KJA</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>Kuala Lumpur, Malaysia</t>
+          <t>Krasnoyarsk, Russia</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
@@ -7298,29 +7298,29 @@
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>Kuala Lumpur</t>
+          <t>Krasnoyarsk</t>
         </is>
       </c>
       <c r="E217" t="inlineStr">
         <is>
-          <t>Malaysia</t>
+          <t>Russia</t>
         </is>
       </c>
       <c r="F217" t="inlineStr">
         <is>
-          <t>MY</t>
+          <t>RU</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="1" t="inlineStr">
         <is>
-          <t>PKX</t>
+          <t>KUL</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>Langfang, China</t>
+          <t>Kuala Lumpur, Malaysia</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
@@ -7330,29 +7330,29 @@
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>Langfang</t>
+          <t>Kuala Lumpur</t>
         </is>
       </c>
       <c r="E218" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Malaysia</t>
         </is>
       </c>
       <c r="F218" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>MY</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="1" t="inlineStr">
         <is>
-          <t>MFM</t>
+          <t>PKX</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>Macau</t>
+          <t>Langfang, China</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
@@ -7360,19 +7360,31 @@
           <t>Asia</t>
         </is>
       </c>
-      <c r="D219" t="inlineStr"/>
-      <c r="E219" t="inlineStr"/>
-      <c r="F219" t="inlineStr"/>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>Langfang</t>
+        </is>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" s="1" t="inlineStr">
         <is>
-          <t>MLE</t>
+          <t>MFM</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>Malé, Maldives</t>
+          <t>Macau</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
@@ -7380,31 +7392,19 @@
           <t>Asia</t>
         </is>
       </c>
-      <c r="D220" t="inlineStr">
-        <is>
-          <t>Malé</t>
-        </is>
-      </c>
-      <c r="E220" t="inlineStr">
-        <is>
-          <t>Maldives</t>
-        </is>
-      </c>
-      <c r="F220" t="inlineStr">
-        <is>
-          <t>MV</t>
-        </is>
-      </c>
+      <c r="D220" t="inlineStr"/>
+      <c r="E220" t="inlineStr"/>
+      <c r="F220" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" s="1" t="inlineStr">
         <is>
-          <t>MNL</t>
+          <t>MLE</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>Manila, Philippines</t>
+          <t>Malé, Maldives</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
@@ -7414,29 +7414,29 @@
       </c>
       <c r="D221" t="inlineStr">
         <is>
-          <t>Manila</t>
+          <t>Malé</t>
         </is>
       </c>
       <c r="E221" t="inlineStr">
         <is>
-          <t>Philippines</t>
+          <t>Maldives</t>
         </is>
       </c>
       <c r="F221" t="inlineStr">
         <is>
-          <t>PH</t>
+          <t>MV</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="1" t="inlineStr">
         <is>
-          <t>BOM</t>
+          <t>MNL</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>Mumbai, India</t>
+          <t>Manila, Philippines</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
@@ -7446,29 +7446,29 @@
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t>Mumbai</t>
+          <t>Manila</t>
         </is>
       </c>
       <c r="E222" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Philippines</t>
         </is>
       </c>
       <c r="F222" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>PH</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="1" t="inlineStr">
         <is>
-          <t>NAG</t>
+          <t>BOM</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>Nagpur, India</t>
+          <t>Mumbai, India</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
@@ -7478,7 +7478,7 @@
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>Nagpur</t>
+          <t>Mumbai</t>
         </is>
       </c>
       <c r="E223" t="inlineStr">
@@ -7495,12 +7495,12 @@
     <row r="224">
       <c r="A224" s="1" t="inlineStr">
         <is>
-          <t>OKA</t>
+          <t>NAG</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>Naha, Japan</t>
+          <t>Nagpur, India</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
@@ -7510,29 +7510,29 @@
       </c>
       <c r="D224" t="inlineStr">
         <is>
-          <t>Naha</t>
+          <t>Nagpur</t>
         </is>
       </c>
       <c r="E224" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F224" t="inlineStr">
         <is>
-          <t>JP</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" s="1" t="inlineStr">
         <is>
-          <t>DEL</t>
+          <t>OKA</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>New Delhi, India</t>
+          <t>Naha, Japan</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
@@ -7542,29 +7542,29 @@
       </c>
       <c r="D225" t="inlineStr">
         <is>
-          <t>New Delhi</t>
+          <t>Naha</t>
         </is>
       </c>
       <c r="E225" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="F225" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>JP</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" s="1" t="inlineStr">
         <is>
-          <t>KIX</t>
+          <t>DEL</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>Osaka, Japan</t>
+          <t>New Delhi, India</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
@@ -7574,29 +7574,29 @@
       </c>
       <c r="D226" t="inlineStr">
         <is>
-          <t>Osaka</t>
+          <t>New Delhi</t>
         </is>
       </c>
       <c r="E226" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F226" t="inlineStr">
         <is>
-          <t>JP</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" s="1" t="inlineStr">
         <is>
-          <t>PAT</t>
+          <t>KIX</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>Patna, India</t>
+          <t>Osaka, Japan</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
@@ -7606,29 +7606,29 @@
       </c>
       <c r="D227" t="inlineStr">
         <is>
-          <t>Patna</t>
+          <t>Osaka</t>
         </is>
       </c>
       <c r="E227" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="F227" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>JP</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" s="1" t="inlineStr">
         <is>
-          <t>PNH</t>
+          <t>PAT</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>Phnom Penh, Cambodia</t>
+          <t>Patna, India</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
@@ -7638,29 +7638,29 @@
       </c>
       <c r="D228" t="inlineStr">
         <is>
-          <t>Phnom Penh</t>
+          <t>Patna</t>
         </is>
       </c>
       <c r="E228" t="inlineStr">
         <is>
-          <t>Cambodia</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F228" t="inlineStr">
         <is>
-          <t>KH</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" s="1" t="inlineStr">
         <is>
-          <t>TAO</t>
+          <t>PNH</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>Qingdao, China</t>
+          <t>Phnom Penh, Cambodia</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
@@ -7670,29 +7670,29 @@
       </c>
       <c r="D229" t="inlineStr">
         <is>
-          <t>Qingdao</t>
+          <t>Phnom Penh</t>
         </is>
       </c>
       <c r="E229" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Cambodia</t>
         </is>
       </c>
       <c r="F229" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>KH</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" s="1" t="inlineStr">
         <is>
-          <t>ICN</t>
+          <t>TAO</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>Seoul, South Korea</t>
+          <t>Qingdao, China</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
@@ -7702,29 +7702,29 @@
       </c>
       <c r="D230" t="inlineStr">
         <is>
-          <t>Seoul</t>
+          <t>Qingdao</t>
         </is>
       </c>
       <c r="E230" t="inlineStr">
         <is>
-          <t>South Korea</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F230" t="inlineStr">
         <is>
-          <t>KR</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" s="1" t="inlineStr">
         <is>
-          <t>SHA</t>
+          <t>ICN</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>Shanghai, China</t>
+          <t>Seoul, South Korea</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
@@ -7734,29 +7734,29 @@
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>Shanghai</t>
+          <t>Seoul</t>
         </is>
       </c>
       <c r="E231" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>South Korea</t>
         </is>
       </c>
       <c r="F231" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>KR</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" s="1" t="inlineStr">
         <is>
-          <t>SIN</t>
+          <t>SHA</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>Singapore, Singapore</t>
+          <t>Shanghai, China</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
@@ -7766,29 +7766,29 @@
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Shanghai</t>
         </is>
       </c>
       <c r="E232" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F232" t="inlineStr">
         <is>
-          <t>SG</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" s="1" t="inlineStr">
         <is>
-          <t>URT</t>
+          <t>SIN</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>Surat Thani, Thailand</t>
+          <t>Singapore, Singapore</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
@@ -7798,29 +7798,29 @@
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>Surat Thani</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="E233" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="F233" t="inlineStr">
         <is>
-          <t>TH</t>
+          <t>SG</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" s="1" t="inlineStr">
         <is>
-          <t>TPE</t>
+          <t>URT</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>Taipei</t>
+          <t>Surat Thani, Thailand</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
@@ -7828,19 +7828,31 @@
           <t>Asia</t>
         </is>
       </c>
-      <c r="D234" t="inlineStr"/>
-      <c r="E234" t="inlineStr"/>
-      <c r="F234" t="inlineStr"/>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>Surat Thani</t>
+        </is>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>Thailand</t>
+        </is>
+      </c>
+      <c r="F234" t="inlineStr">
+        <is>
+          <t>TH</t>
+        </is>
+      </c>
     </row>
     <row r="235">
       <c r="A235" s="1" t="inlineStr">
         <is>
-          <t>NRT</t>
+          <t>TPE</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>Tokyo, Japan</t>
+          <t>Taipei</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
@@ -7848,31 +7860,19 @@
           <t>Asia</t>
         </is>
       </c>
-      <c r="D235" t="inlineStr">
-        <is>
-          <t>Tokyo</t>
-        </is>
-      </c>
-      <c r="E235" t="inlineStr">
-        <is>
-          <t>Japan</t>
-        </is>
-      </c>
-      <c r="F235" t="inlineStr">
-        <is>
-          <t>JP</t>
-        </is>
-      </c>
+      <c r="D235" t="inlineStr"/>
+      <c r="E235" t="inlineStr"/>
+      <c r="F235" t="inlineStr"/>
     </row>
     <row r="236">
       <c r="A236" s="1" t="inlineStr">
         <is>
-          <t>ULN</t>
+          <t>NRT</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>Ulaanbaatar, Mongolia</t>
+          <t>Tokyo, Japan</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
@@ -7882,29 +7882,29 @@
       </c>
       <c r="D236" t="inlineStr">
         <is>
-          <t>Ulaanbaatar</t>
+          <t>Tokyo</t>
         </is>
       </c>
       <c r="E236" t="inlineStr">
         <is>
-          <t>Mongolia</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="F236" t="inlineStr">
         <is>
-          <t>MN</t>
+          <t>JP</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" s="1" t="inlineStr">
         <is>
-          <t>VTE</t>
+          <t>ULN</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>Vientiane, Laos</t>
+          <t>Ulaanbaatar, Mongolia</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
@@ -7914,29 +7914,29 @@
       </c>
       <c r="D237" t="inlineStr">
         <is>
-          <t>Vientiane</t>
+          <t>Ulaanbaatar</t>
         </is>
       </c>
       <c r="E237" t="inlineStr">
         <is>
-          <t>Laos</t>
+          <t>Mongolia</t>
         </is>
       </c>
       <c r="F237" t="inlineStr">
         <is>
-          <t>LA</t>
+          <t>MN</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" s="1" t="inlineStr">
         <is>
-          <t>KHN</t>
+          <t>VTE</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>Xinyu, China</t>
+          <t>Vientiane, Laos</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
@@ -7946,29 +7946,29 @@
       </c>
       <c r="D238" t="inlineStr">
         <is>
-          <t>Xinyu</t>
+          <t>Vientiane</t>
         </is>
       </c>
       <c r="E238" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Laos</t>
         </is>
       </c>
       <c r="F238" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>LA</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" s="1" t="inlineStr">
         <is>
-          <t>EVN</t>
+          <t>KHN</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>Yerevan, Armenia</t>
+          <t>Xinyu, China</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
@@ -7978,29 +7978,29 @@
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>Yerevan</t>
+          <t>Xinyu</t>
         </is>
       </c>
       <c r="E239" t="inlineStr">
         <is>
-          <t>Armenia</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F239" t="inlineStr">
         <is>
-          <t>AM</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" s="1" t="inlineStr">
         <is>
-          <t>JOG</t>
+          <t>EVN</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>Yogyakarta, Indonesia</t>
+          <t>Yerevan, Armenia</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
@@ -8010,29 +8010,29 @@
       </c>
       <c r="D240" t="inlineStr">
         <is>
-          <t>Yogyakarta</t>
+          <t>Yerevan</t>
         </is>
       </c>
       <c r="E240" t="inlineStr">
         <is>
-          <t>Indonesia</t>
+          <t>Armenia</t>
         </is>
       </c>
       <c r="F240" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>AM</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" s="1" t="inlineStr">
         <is>
-          <t>CGY</t>
+          <t>JOG</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>Cagayan de Oro, Philippines</t>
+          <t>Yogyakarta, Indonesia</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
@@ -8042,29 +8042,29 @@
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t>Cagayan de Oro</t>
+          <t>Yogyakarta</t>
         </is>
       </c>
       <c r="E241" t="inlineStr">
         <is>
-          <t>Philippines</t>
+          <t>Indonesia</t>
         </is>
       </c>
       <c r="F241" t="inlineStr">
         <is>
-          <t>PH</t>
+          <t>ID</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" s="1" t="inlineStr">
         <is>
-          <t>COK</t>
+          <t>CGY</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>Kochi, India</t>
+          <t>Cagayan de Oro, Philippines</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
@@ -8074,29 +8074,29 @@
       </c>
       <c r="D242" t="inlineStr">
         <is>
-          <t>Kochi</t>
+          <t>Cagayan de Oro</t>
         </is>
       </c>
       <c r="E242" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Philippines</t>
         </is>
       </c>
       <c r="F242" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>PH</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" s="1" t="inlineStr">
         <is>
-          <t>DPS</t>
+          <t>COK</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>Denpasar, Indonesia</t>
+          <t>Kochi, India</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
@@ -8106,29 +8106,29 @@
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>Denpasar</t>
+          <t>Kochi</t>
         </is>
       </c>
       <c r="E243" t="inlineStr">
         <is>
-          <t>Indonesia</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F243" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" s="1" t="inlineStr">
         <is>
-          <t>CNN</t>
+          <t>DPS</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>Kannur, India</t>
+          <t>Denpasar, Indonesia</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
@@ -8138,29 +8138,29 @@
       </c>
       <c r="D244" t="inlineStr">
         <is>
-          <t>Kannur</t>
+          <t>Denpasar</t>
         </is>
       </c>
       <c r="E244" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Indonesia</t>
         </is>
       </c>
       <c r="F244" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>ID</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" s="1" t="inlineStr">
         <is>
-          <t>SZX</t>
+          <t>CNN</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>Shenzhen, China</t>
+          <t>Kannur, India</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
@@ -8170,29 +8170,29 @@
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>Shenzhen</t>
+          <t>Kannur</t>
         </is>
       </c>
       <c r="E245" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F245" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" s="1" t="inlineStr">
         <is>
-          <t>KWE</t>
+          <t>SZX</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>Guiyang, China</t>
+          <t>Shenzhen, China</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
@@ -8202,7 +8202,7 @@
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>Guiyang</t>
+          <t>Shenzhen</t>
         </is>
       </c>
       <c r="E246" t="inlineStr">
@@ -8219,12 +8219,12 @@
     <row r="247">
       <c r="A247" s="1" t="inlineStr">
         <is>
-          <t>HGH</t>
+          <t>KWE</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>Shaoxing, China</t>
+          <t>Guiyang, China</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
@@ -8234,7 +8234,7 @@
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>Shaoxing</t>
+          <t>Guiyang</t>
         </is>
       </c>
       <c r="E247" t="inlineStr">
@@ -8251,12 +8251,12 @@
     <row r="248">
       <c r="A248" s="1" t="inlineStr">
         <is>
-          <t>CZX</t>
+          <t>HGH</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>Changzhou, China</t>
+          <t>Shaoxing, China</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
@@ -8266,7 +8266,7 @@
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>Changzhou</t>
+          <t>Shaoxing</t>
         </is>
       </c>
       <c r="E248" t="inlineStr">
@@ -8283,12 +8283,12 @@
     <row r="249">
       <c r="A249" s="1" t="inlineStr">
         <is>
-          <t>KMG</t>
+          <t>CZX</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>Kunming, China</t>
+          <t>Changzhou, China</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
@@ -8298,7 +8298,7 @@
       </c>
       <c r="D249" t="inlineStr">
         <is>
-          <t>Kunming</t>
+          <t>Changzhou</t>
         </is>
       </c>
       <c r="E249" t="inlineStr">
@@ -8315,12 +8315,12 @@
     <row r="250">
       <c r="A250" s="1" t="inlineStr">
         <is>
-          <t>CNX</t>
+          <t>KMG</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>Chiang Mai, Thailand</t>
+          <t>Kunming, China</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
@@ -8330,29 +8330,29 @@
       </c>
       <c r="D250" t="inlineStr">
         <is>
-          <t>Chiang Mai</t>
+          <t>Kunming</t>
         </is>
       </c>
       <c r="E250" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F250" t="inlineStr">
         <is>
-          <t>TH</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" s="1" t="inlineStr">
         <is>
-          <t>CGO</t>
+          <t>CNX</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>Zhengzhou, China</t>
+          <t>Chiang Mai, Thailand</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
@@ -8362,29 +8362,29 @@
       </c>
       <c r="D251" t="inlineStr">
         <is>
-          <t>Zhengzhou</t>
+          <t>Chiang Mai</t>
         </is>
       </c>
       <c r="E251" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Thailand</t>
         </is>
       </c>
       <c r="F251" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>TH</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" s="1" t="inlineStr">
         <is>
-          <t>TYN</t>
+          <t>CGO</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>Yangquan, China</t>
+          <t>Zhengzhou, China</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
@@ -8394,7 +8394,7 @@
       </c>
       <c r="D252" t="inlineStr">
         <is>
-          <t>Yangquan</t>
+          <t>Zhengzhou</t>
         </is>
       </c>
       <c r="E252" t="inlineStr">
@@ -8411,12 +8411,12 @@
     <row r="253">
       <c r="A253" s="1" t="inlineStr">
         <is>
-          <t>CSX</t>
+          <t>TYN</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>Changsha, China</t>
+          <t>Yangquan, China</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
@@ -8426,7 +8426,7 @@
       </c>
       <c r="D253" t="inlineStr">
         <is>
-          <t>Changsha</t>
+          <t>Yangquan</t>
         </is>
       </c>
       <c r="E253" t="inlineStr">
@@ -8443,12 +8443,12 @@
     <row r="254">
       <c r="A254" s="1" t="inlineStr">
         <is>
-          <t>DLC</t>
+          <t>CSX</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>Dalian, China</t>
+          <t>Changsha, China</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
@@ -8458,7 +8458,7 @@
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t>Dalian</t>
+          <t>Changsha</t>
         </is>
       </c>
       <c r="E254" t="inlineStr">
@@ -8475,12 +8475,12 @@
     <row r="255">
       <c r="A255" s="1" t="inlineStr">
         <is>
-          <t>BHY</t>
+          <t>DLC</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>Beihai, China</t>
+          <t>Dalian, China</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
@@ -8490,7 +8490,7 @@
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>Beihai</t>
+          <t>Dalian</t>
         </is>
       </c>
       <c r="E255" t="inlineStr">
@@ -8507,12 +8507,12 @@
     <row r="256">
       <c r="A256" s="1" t="inlineStr">
         <is>
-          <t>CKG</t>
+          <t>BHY</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>Chongqing, China</t>
+          <t>Beihai, China</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
@@ -8522,7 +8522,7 @@
       </c>
       <c r="D256" t="inlineStr">
         <is>
-          <t>Chongqing</t>
+          <t>Beihai</t>
         </is>
       </c>
       <c r="E256" t="inlineStr">
@@ -8539,12 +8539,12 @@
     <row r="257">
       <c r="A257" s="1" t="inlineStr">
         <is>
-          <t>XFN</t>
+          <t>CKG</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>Xiangyang, China</t>
+          <t>Chongqing, China</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
@@ -8554,7 +8554,7 @@
       </c>
       <c r="D257" t="inlineStr">
         <is>
-          <t>Xiangyang</t>
+          <t>Chongqing</t>
         </is>
       </c>
       <c r="E257" t="inlineStr">
@@ -8571,12 +8571,12 @@
     <row r="258">
       <c r="A258" s="1" t="inlineStr">
         <is>
-          <t>DAD</t>
+          <t>XFN</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>Da Nang, Vietnam</t>
+          <t>Xiangyang, China</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
@@ -8586,29 +8586,29 @@
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>Da Nang</t>
+          <t>Xiangyang</t>
         </is>
       </c>
       <c r="E258" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F258" t="inlineStr">
         <is>
-          <t>VN</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" s="1" t="inlineStr">
         <is>
-          <t>JXG</t>
+          <t>DAD</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>Jiaxing, China</t>
+          <t>Da Nang, Vietnam</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
@@ -8618,29 +8618,29 @@
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>Jiaxing</t>
+          <t>Da Nang</t>
         </is>
       </c>
       <c r="E259" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Vietnam</t>
         </is>
       </c>
       <c r="F259" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>VN</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" s="1" t="inlineStr">
         <is>
-          <t>CRK</t>
+          <t>JXG</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>Tarlac City, Philippines</t>
+          <t>Jiaxing, China</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
@@ -8650,29 +8650,29 @@
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>Tarlac City</t>
+          <t>Jiaxing</t>
         </is>
       </c>
       <c r="E260" t="inlineStr">
         <is>
-          <t>Philippines</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F260" t="inlineStr">
         <is>
-          <t>PH</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" s="1" t="inlineStr">
         <is>
-          <t>PBH</t>
+          <t>CRK</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>Thimphu, Bhutan</t>
+          <t>Tarlac City, Philippines</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
@@ -8682,29 +8682,29 @@
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>Thimphu</t>
+          <t>Tarlac City</t>
         </is>
       </c>
       <c r="E261" t="inlineStr">
         <is>
-          <t>Bhutan</t>
+          <t>Philippines</t>
         </is>
       </c>
       <c r="F261" t="inlineStr">
         <is>
-          <t>BT</t>
+          <t>PH</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" s="1" t="inlineStr">
         <is>
-          <t>XIY</t>
+          <t>PBH</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>Baoji, China</t>
+          <t>Thimphu, Bhutan</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
@@ -8714,29 +8714,29 @@
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t>Baoji</t>
+          <t>Thimphu</t>
         </is>
       </c>
       <c r="E262" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Bhutan</t>
         </is>
       </c>
       <c r="F262" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>BT</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" s="1" t="inlineStr">
         <is>
-          <t>KCH</t>
+          <t>XIY</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>Kuching, Malaysia</t>
+          <t>Baoji, China</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
@@ -8746,29 +8746,29 @@
       </c>
       <c r="D263" t="inlineStr">
         <is>
-          <t>Kuching</t>
+          <t>Baoji</t>
         </is>
       </c>
       <c r="E263" t="inlineStr">
         <is>
-          <t>Malaysia</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F263" t="inlineStr">
         <is>
-          <t>MY</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" s="1" t="inlineStr">
         <is>
-          <t>AKX</t>
+          <t>KCH</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>Aktobe, Kazakhstan</t>
+          <t>Kuching, Malaysia</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
@@ -8778,29 +8778,29 @@
       </c>
       <c r="D264" t="inlineStr">
         <is>
-          <t>Aktobe</t>
+          <t>Kuching</t>
         </is>
       </c>
       <c r="E264" t="inlineStr">
         <is>
-          <t>Kazakhstan</t>
+          <t>Malaysia</t>
         </is>
       </c>
       <c r="F264" t="inlineStr">
         <is>
-          <t>KZ</t>
+          <t>MY</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" s="1" t="inlineStr">
         <is>
-          <t>TEN</t>
+          <t>AKX</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>Tongren, China</t>
+          <t>Aktobe, Kazakhstan</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
@@ -8810,29 +8810,29 @@
       </c>
       <c r="D265" t="inlineStr">
         <is>
-          <t>Tongren</t>
+          <t>Aktobe</t>
         </is>
       </c>
       <c r="E265" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Kazakhstan</t>
         </is>
       </c>
       <c r="F265" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>KZ</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" s="1" t="inlineStr">
         <is>
-          <t>HYN</t>
+          <t>TEN</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>Taizhou, China</t>
+          <t>Tongren, China</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
@@ -8842,7 +8842,7 @@
       </c>
       <c r="D266" t="inlineStr">
         <is>
-          <t>Taizhou</t>
+          <t>Tongren</t>
         </is>
       </c>
       <c r="E266" t="inlineStr">
@@ -8859,12 +8859,12 @@
     <row r="267">
       <c r="A267" s="1" t="inlineStr">
         <is>
-          <t>FRU</t>
+          <t>HYN</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>Bishkek, Kyrgyzstan</t>
+          <t>Taizhou, China</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
@@ -8874,29 +8874,29 @@
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>Bishkek</t>
+          <t>Taizhou</t>
         </is>
       </c>
       <c r="E267" t="inlineStr">
         <is>
-          <t>Kyrgyzstan</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F267" t="inlineStr">
         <is>
-          <t>KG</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" s="1" t="inlineStr">
         <is>
-          <t>MLG</t>
+          <t>FRU</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>Malang, Indonesia</t>
+          <t>Bishkek, Kyrgyzstan</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
@@ -8906,29 +8906,29 @@
       </c>
       <c r="D268" t="inlineStr">
         <is>
-          <t>Malang</t>
+          <t>Bishkek</t>
         </is>
       </c>
       <c r="E268" t="inlineStr">
         <is>
-          <t>Indonesia</t>
+          <t>Kyrgyzstan</t>
         </is>
       </c>
       <c r="F268" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>KG</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" s="1" t="inlineStr">
         <is>
-          <t>LHE</t>
+          <t>MLG</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>Lahore, Pakistan</t>
+          <t>Malang, Indonesia</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
@@ -8938,29 +8938,29 @@
       </c>
       <c r="D269" t="inlineStr">
         <is>
-          <t>Lahore</t>
+          <t>Malang</t>
         </is>
       </c>
       <c r="E269" t="inlineStr">
         <is>
-          <t>Pakistan</t>
+          <t>Indonesia</t>
         </is>
       </c>
       <c r="F269" t="inlineStr">
         <is>
-          <t>PK</t>
+          <t>ID</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" s="1" t="inlineStr">
         <is>
-          <t>CTU</t>
+          <t>LHE</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>Chengdu, China</t>
+          <t>Lahore, Pakistan</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
@@ -8970,29 +8970,29 @@
       </c>
       <c r="D270" t="inlineStr">
         <is>
-          <t>Chengdu</t>
+          <t>Lahore</t>
         </is>
       </c>
       <c r="E270" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Pakistan</t>
         </is>
       </c>
       <c r="F270" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>PK</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" s="1" t="inlineStr">
         <is>
-          <t>AGR</t>
+          <t>CTU</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>Agra, India</t>
+          <t>Chengdu, China</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
@@ -9002,29 +9002,29 @@
       </c>
       <c r="D271" t="inlineStr">
         <is>
-          <t>Agra</t>
+          <t>Chengdu</t>
         </is>
       </c>
       <c r="E271" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F271" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" s="1" t="inlineStr">
         <is>
-          <t>CJB</t>
+          <t>AGR</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>Coimbatore, India</t>
+          <t>Agra, India</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
@@ -9034,7 +9034,7 @@
       </c>
       <c r="D272" t="inlineStr">
         <is>
-          <t>Coimbatore</t>
+          <t>Agra</t>
         </is>
       </c>
       <c r="E272" t="inlineStr">
@@ -9051,12 +9051,12 @@
     <row r="273">
       <c r="A273" s="1" t="inlineStr">
         <is>
-          <t>ACX</t>
+          <t>CJB</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>Xingyi, China</t>
+          <t>Coimbatore, India</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
@@ -9066,29 +9066,29 @@
       </c>
       <c r="D273" t="inlineStr">
         <is>
-          <t>Xingyi</t>
+          <t>Coimbatore</t>
         </is>
       </c>
       <c r="E273" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F273" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="274">
       <c r="A274" s="1" t="inlineStr">
         <is>
-          <t>BBI</t>
+          <t>ACX</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>Bhubaneswar, India</t>
+          <t>Xingyi, China</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
@@ -9098,29 +9098,29 @@
       </c>
       <c r="D274" t="inlineStr">
         <is>
-          <t>Bhubaneswar</t>
+          <t>Xingyi</t>
         </is>
       </c>
       <c r="E274" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F274" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="275">
       <c r="A275" s="1" t="inlineStr">
         <is>
-          <t>LYA</t>
+          <t>BBI</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>Luoyang, China</t>
+          <t>Bhubaneswar, India</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
@@ -9130,29 +9130,29 @@
       </c>
       <c r="D275" t="inlineStr">
         <is>
-          <t>Luoyang</t>
+          <t>Bhubaneswar</t>
         </is>
       </c>
       <c r="E275" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F275" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="276">
       <c r="A276" s="1" t="inlineStr">
         <is>
-          <t>PNQ</t>
+          <t>LYA</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>Pune, India</t>
+          <t>Luoyang, China</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
@@ -9162,29 +9162,29 @@
       </c>
       <c r="D276" t="inlineStr">
         <is>
-          <t>Pune</t>
+          <t>Luoyang</t>
         </is>
       </c>
       <c r="E276" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F276" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="277">
       <c r="A277" s="1" t="inlineStr">
         <is>
-          <t>JRG</t>
+          <t>PNQ</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>Sambalpur, India</t>
+          <t>Pune, India</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
@@ -9194,7 +9194,7 @@
       </c>
       <c r="D277" t="inlineStr">
         <is>
-          <t>Sambalpur</t>
+          <t>Pune</t>
         </is>
       </c>
       <c r="E277" t="inlineStr">
@@ -9211,12 +9211,12 @@
     <row r="278">
       <c r="A278" s="1" t="inlineStr">
         <is>
-          <t>AVA</t>
+          <t>JRG</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>Anshun, China</t>
+          <t>Sambalpur, India</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
@@ -9226,29 +9226,29 @@
       </c>
       <c r="D278" t="inlineStr">
         <is>
-          <t>Anshun</t>
+          <t>Sambalpur</t>
         </is>
       </c>
       <c r="E278" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F278" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="279">
       <c r="A279" s="1" t="inlineStr">
         <is>
-          <t>NQZ</t>
+          <t>AVA</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>Astana, Kazakhstan</t>
+          <t>Anshun, China</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
@@ -9258,29 +9258,29 @@
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>Astana</t>
+          <t>Anshun</t>
         </is>
       </c>
       <c r="E279" t="inlineStr">
         <is>
-          <t>Kazakhstan</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F279" t="inlineStr">
         <is>
-          <t>KZ</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" s="1" t="inlineStr">
         <is>
-          <t>BDQ</t>
+          <t>NQZ</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>Jamnagar, India</t>
+          <t>Astana, Kazakhstan</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
@@ -9290,61 +9290,61 @@
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>Jamnagar</t>
+          <t>Astana</t>
         </is>
       </c>
       <c r="E280" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Kazakhstan</t>
         </is>
       </c>
       <c r="F280" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>KZ</t>
         </is>
       </c>
     </row>
     <row r="281">
       <c r="A281" s="1" t="inlineStr">
         <is>
-          <t>ABQ</t>
+          <t>BDQ</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>Albuquerque, NM, United States</t>
+          <t>Jamnagar, India</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>North America</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>Albuquerque, NM</t>
+          <t>Jamnagar</t>
         </is>
       </c>
       <c r="E281" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F281" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="282">
       <c r="A282" s="1" t="inlineStr">
         <is>
-          <t>ANC</t>
+          <t>ABQ</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>Anchorage, AK, United States</t>
+          <t>Albuquerque, NM, United States</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
@@ -9354,7 +9354,7 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>Anchorage, AK</t>
+          <t>Albuquerque, NM</t>
         </is>
       </c>
       <c r="E282" t="inlineStr">
@@ -9371,12 +9371,12 @@
     <row r="283">
       <c r="A283" s="1" t="inlineStr">
         <is>
-          <t>IAD</t>
+          <t>ANC</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>Ashburn, VA, United States</t>
+          <t>Anchorage, AK, United States</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
@@ -9386,7 +9386,7 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>Ashburn, VA</t>
+          <t>Anchorage, AK</t>
         </is>
       </c>
       <c r="E283" t="inlineStr">
@@ -9403,12 +9403,12 @@
     <row r="284">
       <c r="A284" s="1" t="inlineStr">
         <is>
-          <t>ATL</t>
+          <t>IAD</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>Atlanta, GA, United States</t>
+          <t>Ashburn, VA, United States</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
@@ -9418,7 +9418,7 @@
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>Atlanta, GA</t>
+          <t>Ashburn, VA</t>
         </is>
       </c>
       <c r="E284" t="inlineStr">
@@ -9435,12 +9435,12 @@
     <row r="285">
       <c r="A285" s="1" t="inlineStr">
         <is>
-          <t>AUS</t>
+          <t>ATL</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>Austin, TX, United States</t>
+          <t>Atlanta, GA, United States</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
@@ -9450,7 +9450,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>Austin, TX</t>
+          <t>Atlanta, GA</t>
         </is>
       </c>
       <c r="E285" t="inlineStr">
@@ -9467,12 +9467,12 @@
     <row r="286">
       <c r="A286" s="1" t="inlineStr">
         <is>
-          <t>BGR</t>
+          <t>AUS</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>Bangor, ME, United States</t>
+          <t>Austin, TX, United States</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
@@ -9482,7 +9482,7 @@
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>Bangor, ME</t>
+          <t>Austin, TX</t>
         </is>
       </c>
       <c r="E286" t="inlineStr">
@@ -9499,12 +9499,12 @@
     <row r="287">
       <c r="A287" s="1" t="inlineStr">
         <is>
-          <t>BOS</t>
+          <t>BGR</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>Boston, MA, United States</t>
+          <t>Bangor, ME, United States</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
@@ -9514,7 +9514,7 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>Boston, MA</t>
+          <t>Bangor, ME</t>
         </is>
       </c>
       <c r="E287" t="inlineStr">
@@ -9531,12 +9531,12 @@
     <row r="288">
       <c r="A288" s="1" t="inlineStr">
         <is>
-          <t>BUF</t>
+          <t>BOS</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>Buffalo, NY, United States</t>
+          <t>Boston, MA, United States</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
@@ -9546,7 +9546,7 @@
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>Buffalo, NY</t>
+          <t>Boston, MA</t>
         </is>
       </c>
       <c r="E288" t="inlineStr">
@@ -9563,12 +9563,12 @@
     <row r="289">
       <c r="A289" s="1" t="inlineStr">
         <is>
-          <t>YYC</t>
+          <t>BUF</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>Calgary, AB, Canada</t>
+          <t>Buffalo, NY, United States</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
@@ -9578,29 +9578,29 @@
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Buffalo, NY</t>
         </is>
       </c>
       <c r="E289" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F289" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="290">
       <c r="A290" s="1" t="inlineStr">
         <is>
-          <t>CLT</t>
+          <t>YYC</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>Charlotte, NC, United States</t>
+          <t>Calgary, AB, Canada</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
@@ -9610,29 +9610,29 @@
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>Charlotte, NC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="E290" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F290" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="291">
       <c r="A291" s="1" t="inlineStr">
         <is>
-          <t>ORD</t>
+          <t>CLT</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>Chicago, IL, United States</t>
+          <t>Charlotte, NC, United States</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
@@ -9642,7 +9642,7 @@
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>Chicago, IL</t>
+          <t>Charlotte, NC</t>
         </is>
       </c>
       <c r="E291" t="inlineStr">
@@ -9659,12 +9659,12 @@
     <row r="292">
       <c r="A292" s="1" t="inlineStr">
         <is>
-          <t>CLE</t>
+          <t>ORD</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>Cleveland, OH, United States</t>
+          <t>Chicago, IL, United States</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
@@ -9674,7 +9674,7 @@
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>Cleveland, OH</t>
+          <t>Chicago, IL</t>
         </is>
       </c>
       <c r="E292" t="inlineStr">
@@ -9691,12 +9691,12 @@
     <row r="293">
       <c r="A293" s="1" t="inlineStr">
         <is>
-          <t>CMH</t>
+          <t>CLE</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>Columbus, OH, United States</t>
+          <t>Cleveland, OH, United States</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
@@ -9706,7 +9706,7 @@
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>Columbus, OH</t>
+          <t>Cleveland, OH</t>
         </is>
       </c>
       <c r="E293" t="inlineStr">
@@ -9723,12 +9723,12 @@
     <row r="294">
       <c r="A294" s="1" t="inlineStr">
         <is>
-          <t>DFW</t>
+          <t>CMH</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>Dallas, TX, United States</t>
+          <t>Columbus, OH, United States</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
@@ -9738,7 +9738,7 @@
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>Dallas, TX</t>
+          <t>Columbus, OH</t>
         </is>
       </c>
       <c r="E294" t="inlineStr">
@@ -9755,12 +9755,12 @@
     <row r="295">
       <c r="A295" s="1" t="inlineStr">
         <is>
-          <t>DEN</t>
+          <t>DFW</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>Denver, CO, United States</t>
+          <t>Dallas, TX, United States</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -9770,7 +9770,7 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>Denver, CO</t>
+          <t>Dallas, TX</t>
         </is>
       </c>
       <c r="E295" t="inlineStr">
@@ -9787,12 +9787,12 @@
     <row r="296">
       <c r="A296" s="1" t="inlineStr">
         <is>
-          <t>DTW</t>
+          <t>DEN</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>Detroit, MI, United States</t>
+          <t>Denver, CO, United States</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -9802,7 +9802,7 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>Detroit, MI</t>
+          <t>Denver, CO</t>
         </is>
       </c>
       <c r="E296" t="inlineStr">
@@ -9819,12 +9819,12 @@
     <row r="297">
       <c r="A297" s="1" t="inlineStr">
         <is>
-          <t>RDU</t>
+          <t>DTW</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>Durham, NC, United States</t>
+          <t>Detroit, MI, United States</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
@@ -9834,7 +9834,7 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>Durham, NC</t>
+          <t>Detroit, MI</t>
         </is>
       </c>
       <c r="E297" t="inlineStr">
@@ -9851,12 +9851,12 @@
     <row r="298">
       <c r="A298" s="1" t="inlineStr">
         <is>
-          <t>GDL</t>
+          <t>RDU</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>Guadalajara, Mexico</t>
+          <t>Durham, NC, United States</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
@@ -9866,29 +9866,29 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>Guadalajara</t>
+          <t>Durham, NC</t>
         </is>
       </c>
       <c r="E298" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F298" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="299">
       <c r="A299" s="1" t="inlineStr">
         <is>
-          <t>YHZ</t>
+          <t>GDL</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>Halifax, Canada</t>
+          <t>Guadalajara, Mexico</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
@@ -9898,29 +9898,29 @@
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>Halifax</t>
+          <t>Guadalajara</t>
         </is>
       </c>
       <c r="E299" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F299" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>MX</t>
         </is>
       </c>
     </row>
     <row r="300">
       <c r="A300" s="1" t="inlineStr">
         <is>
-          <t>HNL</t>
+          <t>YHZ</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>Honolulu, HI, United States</t>
+          <t>Halifax, Canada</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
@@ -9930,29 +9930,29 @@
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>Honolulu, HI</t>
+          <t>Halifax</t>
         </is>
       </c>
       <c r="E300" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F300" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="301">
       <c r="A301" s="1" t="inlineStr">
         <is>
-          <t>IAH</t>
+          <t>HNL</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>Houston, TX, United States</t>
+          <t>Honolulu, HI, United States</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
@@ -9962,7 +9962,7 @@
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>Houston, TX</t>
+          <t>Honolulu, HI</t>
         </is>
       </c>
       <c r="E301" t="inlineStr">
@@ -9979,12 +9979,12 @@
     <row r="302">
       <c r="A302" s="1" t="inlineStr">
         <is>
-          <t>IND</t>
+          <t>IAH</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>Indianapolis, IN, United States</t>
+          <t>Houston, TX, United States</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
@@ -9994,7 +9994,7 @@
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>Indianapolis, IN</t>
+          <t>Houston, TX</t>
         </is>
       </c>
       <c r="E302" t="inlineStr">
@@ -10011,12 +10011,12 @@
     <row r="303">
       <c r="A303" s="1" t="inlineStr">
         <is>
-          <t>JAX</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>Jacksonville, FL, United States</t>
+          <t>Indianapolis, IN, United States</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
@@ -10026,7 +10026,7 @@
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>Jacksonville, FL</t>
+          <t>Indianapolis, IN</t>
         </is>
       </c>
       <c r="E303" t="inlineStr">
@@ -10043,12 +10043,12 @@
     <row r="304">
       <c r="A304" s="1" t="inlineStr">
         <is>
-          <t>MCI</t>
+          <t>JAX</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>Kansas City, MO, United States</t>
+          <t>Jacksonville, FL, United States</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
@@ -10058,7 +10058,7 @@
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>Kansas City, MO</t>
+          <t>Jacksonville, FL</t>
         </is>
       </c>
       <c r="E304" t="inlineStr">
@@ -10075,12 +10075,12 @@
     <row r="305">
       <c r="A305" s="1" t="inlineStr">
         <is>
-          <t>KIN</t>
+          <t>MCI</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>Kingston, Jamaica</t>
+          <t>Kansas City, MO, United States</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
@@ -10090,29 +10090,29 @@
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>Kingston</t>
+          <t>Kansas City, MO</t>
         </is>
       </c>
       <c r="E305" t="inlineStr">
         <is>
-          <t>Jamaica</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F305" t="inlineStr">
         <is>
-          <t>JM</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="306">
       <c r="A306" s="1" t="inlineStr">
         <is>
-          <t>LAS</t>
+          <t>KIN</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>Las Vegas, NV, United States</t>
+          <t>Kingston, Jamaica</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
@@ -10122,29 +10122,29 @@
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t>Las Vegas, NV</t>
+          <t>Kingston</t>
         </is>
       </c>
       <c r="E306" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Jamaica</t>
         </is>
       </c>
       <c r="F306" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>JM</t>
         </is>
       </c>
     </row>
     <row r="307">
       <c r="A307" s="1" t="inlineStr">
         <is>
-          <t>LAX</t>
+          <t>LAS</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>Los Angeles, CA, United States</t>
+          <t>Las Vegas, NV, United States</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
@@ -10154,7 +10154,7 @@
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>Los Angeles, CA</t>
+          <t>Las Vegas, NV</t>
         </is>
       </c>
       <c r="E307" t="inlineStr">
@@ -10171,12 +10171,12 @@
     <row r="308">
       <c r="A308" s="1" t="inlineStr">
         <is>
-          <t>MEM</t>
+          <t>LAX</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>Memphis, TN, United States</t>
+          <t>Los Angeles, CA, United States</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
@@ -10186,7 +10186,7 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>Memphis, TN</t>
+          <t>Los Angeles, CA</t>
         </is>
       </c>
       <c r="E308" t="inlineStr">
@@ -10203,12 +10203,12 @@
     <row r="309">
       <c r="A309" s="1" t="inlineStr">
         <is>
-          <t>MEX</t>
+          <t>MEM</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>Mexico City, Mexico</t>
+          <t>Memphis, TN, United States</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
@@ -10218,29 +10218,29 @@
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>Mexico City</t>
+          <t>Memphis, TN</t>
         </is>
       </c>
       <c r="E309" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F309" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="310">
       <c r="A310" s="1" t="inlineStr">
         <is>
-          <t>MIA</t>
+          <t>MEX</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>Miami, FL, United States</t>
+          <t>Mexico City, Mexico</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
@@ -10250,29 +10250,29 @@
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>Miami, FL</t>
+          <t>Mexico City</t>
         </is>
       </c>
       <c r="E310" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F310" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
     </row>
     <row r="311">
       <c r="A311" s="1" t="inlineStr">
         <is>
-          <t>MSP</t>
+          <t>MIA</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Minneapolis, MN, United States</t>
+          <t>Miami, FL, United States</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
@@ -10282,7 +10282,7 @@
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>Minneapolis, MN</t>
+          <t>Miami, FL</t>
         </is>
       </c>
       <c r="E311" t="inlineStr">
@@ -10299,12 +10299,12 @@
     <row r="312">
       <c r="A312" s="1" t="inlineStr">
         <is>
-          <t>YUL</t>
+          <t>MSP</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>Montréal, QC, Canada</t>
+          <t>Minneapolis, MN, United States</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
@@ -10314,29 +10314,29 @@
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>Montréal, QC</t>
+          <t>Minneapolis, MN</t>
         </is>
       </c>
       <c r="E312" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F312" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="313">
       <c r="A313" s="1" t="inlineStr">
         <is>
-          <t>BNA</t>
+          <t>YUL</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Nashville, United States</t>
+          <t>Montréal, QC, Canada</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
@@ -10346,29 +10346,29 @@
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>Nashville</t>
+          <t>Montréal, QC</t>
         </is>
       </c>
       <c r="E313" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F313" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="314">
       <c r="A314" s="1" t="inlineStr">
         <is>
-          <t>EWR</t>
+          <t>BNA</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Newark, NJ, United States</t>
+          <t>Nashville, United States</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -10378,7 +10378,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>Newark, NJ</t>
+          <t>Nashville</t>
         </is>
       </c>
       <c r="E314" t="inlineStr">
@@ -10395,12 +10395,12 @@
     <row r="315">
       <c r="A315" s="1" t="inlineStr">
         <is>
-          <t>ORF</t>
+          <t>EWR</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>Norfolk, VA, United States</t>
+          <t>Newark, NJ, United States</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
@@ -10410,7 +10410,7 @@
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>Norfolk, VA</t>
+          <t>Newark, NJ</t>
         </is>
       </c>
       <c r="E315" t="inlineStr">
@@ -10427,12 +10427,12 @@
     <row r="316">
       <c r="A316" s="1" t="inlineStr">
         <is>
-          <t>OKC</t>
+          <t>ORF</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Oklahoma City, OK, United States</t>
+          <t>Norfolk, VA, United States</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
@@ -10442,7 +10442,7 @@
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>Oklahoma City, OK</t>
+          <t>Norfolk, VA</t>
         </is>
       </c>
       <c r="E316" t="inlineStr">
@@ -10459,12 +10459,12 @@
     <row r="317">
       <c r="A317" s="1" t="inlineStr">
         <is>
-          <t>OMA</t>
+          <t>OKC</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Omaha, NE, United States</t>
+          <t>Oklahoma City, OK, United States</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -10474,7 +10474,7 @@
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t>Omaha, NE</t>
+          <t>Oklahoma City, OK</t>
         </is>
       </c>
       <c r="E317" t="inlineStr">
@@ -10491,12 +10491,12 @@
     <row r="318">
       <c r="A318" s="1" t="inlineStr">
         <is>
-          <t>PHL</t>
+          <t>OMA</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>Philadelphia, United States</t>
+          <t>Omaha, NE, United States</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
@@ -10506,7 +10506,7 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>Philadelphia</t>
+          <t>Omaha, NE</t>
         </is>
       </c>
       <c r="E318" t="inlineStr">
@@ -10523,12 +10523,12 @@
     <row r="319">
       <c r="A319" s="1" t="inlineStr">
         <is>
-          <t>PHX</t>
+          <t>PHL</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Phoenix, AZ, United States</t>
+          <t>Philadelphia, United States</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
@@ -10538,7 +10538,7 @@
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>Phoenix, AZ</t>
+          <t>Philadelphia</t>
         </is>
       </c>
       <c r="E319" t="inlineStr">
@@ -10555,12 +10555,12 @@
     <row r="320">
       <c r="A320" s="1" t="inlineStr">
         <is>
-          <t>PIT</t>
+          <t>PHX</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Pittsburgh, PA, United States</t>
+          <t>Phoenix, AZ, United States</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -10570,7 +10570,7 @@
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t>Pittsburgh, PA</t>
+          <t>Phoenix, AZ</t>
         </is>
       </c>
       <c r="E320" t="inlineStr">
@@ -10587,12 +10587,12 @@
     <row r="321">
       <c r="A321" s="1" t="inlineStr">
         <is>
-          <t>PDX</t>
+          <t>PIT</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>Portland, OR, United States</t>
+          <t>Pittsburgh, PA, United States</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
@@ -10602,7 +10602,7 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>Portland, OR</t>
+          <t>Pittsburgh, PA</t>
         </is>
       </c>
       <c r="E321" t="inlineStr">
@@ -10619,12 +10619,12 @@
     <row r="322">
       <c r="A322" s="1" t="inlineStr">
         <is>
-          <t>QRO</t>
+          <t>PDX</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>Queretaro, MX, Mexico</t>
+          <t>Portland, OR, United States</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
@@ -10634,29 +10634,29 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>Queretaro, MX</t>
+          <t>Portland, OR</t>
         </is>
       </c>
       <c r="E322" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F322" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="323">
       <c r="A323" s="1" t="inlineStr">
         <is>
-          <t>RIC</t>
+          <t>QRO</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>Richmond, VA, United States</t>
+          <t>Queretaro, MX, Mexico</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -10666,29 +10666,29 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>Richmond, VA</t>
+          <t>Queretaro, MX</t>
         </is>
       </c>
       <c r="E323" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F323" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
     </row>
     <row r="324">
       <c r="A324" s="1" t="inlineStr">
         <is>
-          <t>SMF</t>
+          <t>RIC</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>Sacramento, CA, United States</t>
+          <t>Richmond, VA, United States</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -10698,7 +10698,7 @@
       </c>
       <c r="D324" t="inlineStr">
         <is>
-          <t>Sacramento, CA</t>
+          <t>Richmond, VA</t>
         </is>
       </c>
       <c r="E324" t="inlineStr">
@@ -10715,12 +10715,12 @@
     <row r="325">
       <c r="A325" s="1" t="inlineStr">
         <is>
-          <t>SLC</t>
+          <t>SMF</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>Salt Lake City, UT, United States</t>
+          <t>Sacramento, CA, United States</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -10730,7 +10730,7 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>Salt Lake City, UT</t>
+          <t>Sacramento, CA</t>
         </is>
       </c>
       <c r="E325" t="inlineStr">
@@ -10747,12 +10747,12 @@
     <row r="326">
       <c r="A326" s="1" t="inlineStr">
         <is>
-          <t>SAT</t>
+          <t>SLC</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>San Antonio, TX, United States</t>
+          <t>Salt Lake City, UT, United States</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
@@ -10762,7 +10762,7 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>San Antonio, TX</t>
+          <t>Salt Lake City, UT</t>
         </is>
       </c>
       <c r="E326" t="inlineStr">
@@ -10779,12 +10779,12 @@
     <row r="327">
       <c r="A327" s="1" t="inlineStr">
         <is>
-          <t>SAN</t>
+          <t>SAT</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>San Diego, CA, United States</t>
+          <t>San Antonio, TX, United States</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
@@ -10794,7 +10794,7 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>San Diego, CA</t>
+          <t>San Antonio, TX</t>
         </is>
       </c>
       <c r="E327" t="inlineStr">
@@ -10811,12 +10811,12 @@
     <row r="328">
       <c r="A328" s="1" t="inlineStr">
         <is>
-          <t>SFO</t>
+          <t>SAN</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>San Francisco, CA, United States</t>
+          <t>San Diego, CA, United States</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
@@ -10826,7 +10826,7 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>San Francisco, CA</t>
+          <t>San Diego, CA</t>
         </is>
       </c>
       <c r="E328" t="inlineStr">
@@ -10843,12 +10843,12 @@
     <row r="329">
       <c r="A329" s="1" t="inlineStr">
         <is>
-          <t>SJC</t>
+          <t>SFO</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>San Jose, CA, United States</t>
+          <t>San Francisco, CA, United States</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
@@ -10858,7 +10858,7 @@
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>San Jose, CA</t>
+          <t>San Francisco, CA</t>
         </is>
       </c>
       <c r="E329" t="inlineStr">
@@ -10875,12 +10875,12 @@
     <row r="330">
       <c r="A330" s="1" t="inlineStr">
         <is>
-          <t>YXE</t>
+          <t>SJC</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>Saskatoon, SK, Canada</t>
+          <t>San Jose, CA, United States</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
@@ -10890,29 +10890,29 @@
       </c>
       <c r="D330" t="inlineStr">
         <is>
-          <t>Saskatoon, SK</t>
+          <t>San Jose, CA</t>
         </is>
       </c>
       <c r="E330" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F330" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="331">
       <c r="A331" s="1" t="inlineStr">
         <is>
-          <t>SEA</t>
+          <t>YXE</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>Seattle, WA, United States</t>
+          <t>Saskatoon, SK, Canada</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
@@ -10922,29 +10922,29 @@
       </c>
       <c r="D331" t="inlineStr">
         <is>
-          <t>Seattle, WA</t>
+          <t>Saskatoon, SK</t>
         </is>
       </c>
       <c r="E331" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F331" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="332">
       <c r="A332" s="1" t="inlineStr">
         <is>
-          <t>FSD</t>
+          <t>SEA</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>Sioux Falls, SD, United States</t>
+          <t>Seattle, WA, United States</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
@@ -10954,7 +10954,7 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>Sioux Falls, SD</t>
+          <t>Seattle, WA</t>
         </is>
       </c>
       <c r="E332" t="inlineStr">
@@ -10971,12 +10971,12 @@
     <row r="333">
       <c r="A333" s="1" t="inlineStr">
         <is>
-          <t>STL</t>
+          <t>FSD</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>St. Louis, MO, United States</t>
+          <t>Sioux Falls, SD, United States</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
@@ -10986,7 +10986,7 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>St. Louis, MO</t>
+          <t>Sioux Falls, SD</t>
         </is>
       </c>
       <c r="E333" t="inlineStr">
@@ -11003,12 +11003,12 @@
     <row r="334">
       <c r="A334" s="1" t="inlineStr">
         <is>
-          <t>TLH</t>
+          <t>STL</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>Tallahassee, FL, United States</t>
+          <t>St. Louis, MO, United States</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
@@ -11018,7 +11018,7 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>Tallahassee, FL</t>
+          <t>St. Louis, MO</t>
         </is>
       </c>
       <c r="E334" t="inlineStr">
@@ -11035,12 +11035,12 @@
     <row r="335">
       <c r="A335" s="1" t="inlineStr">
         <is>
-          <t>TPA</t>
+          <t>TLH</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>Tampa, FL, United States</t>
+          <t>Tallahassee, FL, United States</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
@@ -11050,7 +11050,7 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>Tampa, FL</t>
+          <t>Tallahassee, FL</t>
         </is>
       </c>
       <c r="E335" t="inlineStr">
@@ -11067,12 +11067,12 @@
     <row r="336">
       <c r="A336" s="1" t="inlineStr">
         <is>
-          <t>YYZ</t>
+          <t>TPA</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>Toronto, ON, Canada</t>
+          <t>Tampa, FL, United States</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
@@ -11082,29 +11082,29 @@
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>Toronto, ON</t>
+          <t>Tampa, FL</t>
         </is>
       </c>
       <c r="E336" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F336" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="337">
       <c r="A337" s="1" t="inlineStr">
         <is>
-          <t>YVR</t>
+          <t>YYZ</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>Vancouver, BC, Canada</t>
+          <t>Toronto, ON, Canada</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
@@ -11114,7 +11114,7 @@
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Toronto, ON</t>
         </is>
       </c>
       <c r="E337" t="inlineStr">
@@ -11131,12 +11131,12 @@
     <row r="338">
       <c r="A338" s="1" t="inlineStr">
         <is>
-          <t>YWG</t>
+          <t>YVR</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>Winnipeg, MB, Canada</t>
+          <t>Vancouver, BC, Canada</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
@@ -11146,7 +11146,7 @@
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>Winnipeg, MB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="E338" t="inlineStr">
@@ -11163,30 +11163,62 @@
     <row r="339">
       <c r="A339" s="1" t="inlineStr">
         <is>
+          <t>YWG</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>Winnipeg, MB, Canada</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>North America</t>
+        </is>
+      </c>
+      <c r="D339" t="inlineStr">
+        <is>
+          <t>Winnipeg, MB</t>
+        </is>
+      </c>
+      <c r="E339" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="F339" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" s="1" t="inlineStr">
+        <is>
           <t>CVG</t>
         </is>
       </c>
-      <c r="B339" t="inlineStr">
+      <c r="B340" t="inlineStr">
         <is>
           <t>Cincinnati, United States</t>
         </is>
       </c>
-      <c r="C339" t="inlineStr">
+      <c r="C340" t="inlineStr">
         <is>
           <t>North America</t>
         </is>
       </c>
-      <c r="D339" t="inlineStr">
+      <c r="D340" t="inlineStr">
         <is>
           <t>Cincinnati</t>
         </is>
       </c>
-      <c r="E339" t="inlineStr">
+      <c r="E340" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="F339" t="inlineStr">
+      <c r="F340" t="inlineStr">
         <is>
           <t>US</t>
         </is>

</xml_diff>

<commit_message>
update generated data Triggered by a1fd5cb928c1501faf5c668f7ccd92c2a2e5332a
</commit_message>
<xml_diff>
--- a/DC-Colos.xlsx
+++ b/DC-Colos.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F340"/>
+  <dimension ref="A1:F339"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8507,12 +8507,12 @@
     <row r="256">
       <c r="A256" s="1" t="inlineStr">
         <is>
-          <t>BHY</t>
+          <t>CKG</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>Beihai, China</t>
+          <t>Chongqing, China</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
@@ -8522,7 +8522,7 @@
       </c>
       <c r="D256" t="inlineStr">
         <is>
-          <t>Beihai</t>
+          <t>Chongqing</t>
         </is>
       </c>
       <c r="E256" t="inlineStr">
@@ -8539,12 +8539,12 @@
     <row r="257">
       <c r="A257" s="1" t="inlineStr">
         <is>
-          <t>CKG</t>
+          <t>XFN</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>Chongqing, China</t>
+          <t>Xiangyang, China</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
@@ -8554,7 +8554,7 @@
       </c>
       <c r="D257" t="inlineStr">
         <is>
-          <t>Chongqing</t>
+          <t>Xiangyang</t>
         </is>
       </c>
       <c r="E257" t="inlineStr">
@@ -8571,12 +8571,12 @@
     <row r="258">
       <c r="A258" s="1" t="inlineStr">
         <is>
-          <t>XFN</t>
+          <t>DAD</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>Xiangyang, China</t>
+          <t>Da Nang, Vietnam</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
@@ -8586,29 +8586,29 @@
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>Xiangyang</t>
+          <t>Da Nang</t>
         </is>
       </c>
       <c r="E258" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Vietnam</t>
         </is>
       </c>
       <c r="F258" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>VN</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" s="1" t="inlineStr">
         <is>
-          <t>DAD</t>
+          <t>JXG</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>Da Nang, Vietnam</t>
+          <t>Jiaxing, China</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
@@ -8618,29 +8618,29 @@
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>Da Nang</t>
+          <t>Jiaxing</t>
         </is>
       </c>
       <c r="E259" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F259" t="inlineStr">
         <is>
-          <t>VN</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" s="1" t="inlineStr">
         <is>
-          <t>JXG</t>
+          <t>CRK</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>Jiaxing, China</t>
+          <t>Tarlac City, Philippines</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
@@ -8650,29 +8650,29 @@
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>Jiaxing</t>
+          <t>Tarlac City</t>
         </is>
       </c>
       <c r="E260" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Philippines</t>
         </is>
       </c>
       <c r="F260" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>PH</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" s="1" t="inlineStr">
         <is>
-          <t>CRK</t>
+          <t>PBH</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>Tarlac City, Philippines</t>
+          <t>Thimphu, Bhutan</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
@@ -8682,29 +8682,29 @@
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>Tarlac City</t>
+          <t>Thimphu</t>
         </is>
       </c>
       <c r="E261" t="inlineStr">
         <is>
-          <t>Philippines</t>
+          <t>Bhutan</t>
         </is>
       </c>
       <c r="F261" t="inlineStr">
         <is>
-          <t>PH</t>
+          <t>BT</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" s="1" t="inlineStr">
         <is>
-          <t>PBH</t>
+          <t>XIY</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>Thimphu, Bhutan</t>
+          <t>Baoji, China</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
@@ -8714,29 +8714,29 @@
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t>Thimphu</t>
+          <t>Baoji</t>
         </is>
       </c>
       <c r="E262" t="inlineStr">
         <is>
-          <t>Bhutan</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F262" t="inlineStr">
         <is>
-          <t>BT</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" s="1" t="inlineStr">
         <is>
-          <t>XIY</t>
+          <t>KCH</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>Baoji, China</t>
+          <t>Kuching, Malaysia</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
@@ -8746,29 +8746,29 @@
       </c>
       <c r="D263" t="inlineStr">
         <is>
-          <t>Baoji</t>
+          <t>Kuching</t>
         </is>
       </c>
       <c r="E263" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Malaysia</t>
         </is>
       </c>
       <c r="F263" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>MY</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" s="1" t="inlineStr">
         <is>
-          <t>KCH</t>
+          <t>AKX</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>Kuching, Malaysia</t>
+          <t>Aktobe, Kazakhstan</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
@@ -8778,29 +8778,29 @@
       </c>
       <c r="D264" t="inlineStr">
         <is>
-          <t>Kuching</t>
+          <t>Aktobe</t>
         </is>
       </c>
       <c r="E264" t="inlineStr">
         <is>
-          <t>Malaysia</t>
+          <t>Kazakhstan</t>
         </is>
       </c>
       <c r="F264" t="inlineStr">
         <is>
-          <t>MY</t>
+          <t>KZ</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" s="1" t="inlineStr">
         <is>
-          <t>AKX</t>
+          <t>TEN</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>Aktobe, Kazakhstan</t>
+          <t>Tongren, China</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
@@ -8810,29 +8810,29 @@
       </c>
       <c r="D265" t="inlineStr">
         <is>
-          <t>Aktobe</t>
+          <t>Tongren</t>
         </is>
       </c>
       <c r="E265" t="inlineStr">
         <is>
-          <t>Kazakhstan</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F265" t="inlineStr">
         <is>
-          <t>KZ</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" s="1" t="inlineStr">
         <is>
-          <t>TEN</t>
+          <t>HYN</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>Tongren, China</t>
+          <t>Taizhou, China</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
@@ -8842,7 +8842,7 @@
       </c>
       <c r="D266" t="inlineStr">
         <is>
-          <t>Tongren</t>
+          <t>Taizhou</t>
         </is>
       </c>
       <c r="E266" t="inlineStr">
@@ -8859,12 +8859,12 @@
     <row r="267">
       <c r="A267" s="1" t="inlineStr">
         <is>
-          <t>HYN</t>
+          <t>FRU</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>Taizhou, China</t>
+          <t>Bishkek, Kyrgyzstan</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
@@ -8874,29 +8874,29 @@
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>Taizhou</t>
+          <t>Bishkek</t>
         </is>
       </c>
       <c r="E267" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Kyrgyzstan</t>
         </is>
       </c>
       <c r="F267" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>KG</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" s="1" t="inlineStr">
         <is>
-          <t>FRU</t>
+          <t>MLG</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>Bishkek, Kyrgyzstan</t>
+          <t>Malang, Indonesia</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
@@ -8906,29 +8906,29 @@
       </c>
       <c r="D268" t="inlineStr">
         <is>
-          <t>Bishkek</t>
+          <t>Malang</t>
         </is>
       </c>
       <c r="E268" t="inlineStr">
         <is>
-          <t>Kyrgyzstan</t>
+          <t>Indonesia</t>
         </is>
       </c>
       <c r="F268" t="inlineStr">
         <is>
-          <t>KG</t>
+          <t>ID</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" s="1" t="inlineStr">
         <is>
-          <t>MLG</t>
+          <t>LHE</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>Malang, Indonesia</t>
+          <t>Lahore, Pakistan</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
@@ -8938,29 +8938,29 @@
       </c>
       <c r="D269" t="inlineStr">
         <is>
-          <t>Malang</t>
+          <t>Lahore</t>
         </is>
       </c>
       <c r="E269" t="inlineStr">
         <is>
-          <t>Indonesia</t>
+          <t>Pakistan</t>
         </is>
       </c>
       <c r="F269" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>PK</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" s="1" t="inlineStr">
         <is>
-          <t>LHE</t>
+          <t>CTU</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>Lahore, Pakistan</t>
+          <t>Chengdu, China</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
@@ -8970,29 +8970,29 @@
       </c>
       <c r="D270" t="inlineStr">
         <is>
-          <t>Lahore</t>
+          <t>Chengdu</t>
         </is>
       </c>
       <c r="E270" t="inlineStr">
         <is>
-          <t>Pakistan</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F270" t="inlineStr">
         <is>
-          <t>PK</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" s="1" t="inlineStr">
         <is>
-          <t>CTU</t>
+          <t>AGR</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>Chengdu, China</t>
+          <t>Agra, India</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
@@ -9002,29 +9002,29 @@
       </c>
       <c r="D271" t="inlineStr">
         <is>
-          <t>Chengdu</t>
+          <t>Agra</t>
         </is>
       </c>
       <c r="E271" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F271" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" s="1" t="inlineStr">
         <is>
-          <t>AGR</t>
+          <t>CJB</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>Agra, India</t>
+          <t>Coimbatore, India</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
@@ -9034,7 +9034,7 @@
       </c>
       <c r="D272" t="inlineStr">
         <is>
-          <t>Agra</t>
+          <t>Coimbatore</t>
         </is>
       </c>
       <c r="E272" t="inlineStr">
@@ -9051,12 +9051,12 @@
     <row r="273">
       <c r="A273" s="1" t="inlineStr">
         <is>
-          <t>CJB</t>
+          <t>ACX</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>Coimbatore, India</t>
+          <t>Xingyi, China</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
@@ -9066,29 +9066,29 @@
       </c>
       <c r="D273" t="inlineStr">
         <is>
-          <t>Coimbatore</t>
+          <t>Xingyi</t>
         </is>
       </c>
       <c r="E273" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F273" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="274">
       <c r="A274" s="1" t="inlineStr">
         <is>
-          <t>ACX</t>
+          <t>BBI</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>Xingyi, China</t>
+          <t>Bhubaneswar, India</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
@@ -9098,29 +9098,29 @@
       </c>
       <c r="D274" t="inlineStr">
         <is>
-          <t>Xingyi</t>
+          <t>Bhubaneswar</t>
         </is>
       </c>
       <c r="E274" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F274" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="275">
       <c r="A275" s="1" t="inlineStr">
         <is>
-          <t>BBI</t>
+          <t>LYA</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>Bhubaneswar, India</t>
+          <t>Luoyang, China</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
@@ -9130,29 +9130,29 @@
       </c>
       <c r="D275" t="inlineStr">
         <is>
-          <t>Bhubaneswar</t>
+          <t>Luoyang</t>
         </is>
       </c>
       <c r="E275" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F275" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="276">
       <c r="A276" s="1" t="inlineStr">
         <is>
-          <t>LYA</t>
+          <t>PNQ</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>Luoyang, China</t>
+          <t>Pune, India</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
@@ -9162,29 +9162,29 @@
       </c>
       <c r="D276" t="inlineStr">
         <is>
-          <t>Luoyang</t>
+          <t>Pune</t>
         </is>
       </c>
       <c r="E276" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F276" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="277">
       <c r="A277" s="1" t="inlineStr">
         <is>
-          <t>PNQ</t>
+          <t>JRG</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>Pune, India</t>
+          <t>Sambalpur, India</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
@@ -9194,7 +9194,7 @@
       </c>
       <c r="D277" t="inlineStr">
         <is>
-          <t>Pune</t>
+          <t>Sambalpur</t>
         </is>
       </c>
       <c r="E277" t="inlineStr">
@@ -9211,12 +9211,12 @@
     <row r="278">
       <c r="A278" s="1" t="inlineStr">
         <is>
-          <t>JRG</t>
+          <t>AVA</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>Sambalpur, India</t>
+          <t>Anshun, China</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
@@ -9226,29 +9226,29 @@
       </c>
       <c r="D278" t="inlineStr">
         <is>
-          <t>Sambalpur</t>
+          <t>Anshun</t>
         </is>
       </c>
       <c r="E278" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F278" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="279">
       <c r="A279" s="1" t="inlineStr">
         <is>
-          <t>AVA</t>
+          <t>NQZ</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>Anshun, China</t>
+          <t>Astana, Kazakhstan</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
@@ -9258,29 +9258,29 @@
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>Anshun</t>
+          <t>Astana</t>
         </is>
       </c>
       <c r="E279" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Kazakhstan</t>
         </is>
       </c>
       <c r="F279" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>KZ</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" s="1" t="inlineStr">
         <is>
-          <t>NQZ</t>
+          <t>BDQ</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>Astana, Kazakhstan</t>
+          <t>Jamnagar, India</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
@@ -9290,61 +9290,61 @@
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>Astana</t>
+          <t>Jamnagar</t>
         </is>
       </c>
       <c r="E280" t="inlineStr">
         <is>
-          <t>Kazakhstan</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F280" t="inlineStr">
         <is>
-          <t>KZ</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="281">
       <c r="A281" s="1" t="inlineStr">
         <is>
-          <t>BDQ</t>
+          <t>ABQ</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>Jamnagar, India</t>
+          <t>Albuquerque, NM, United States</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>Asia</t>
+          <t>North America</t>
         </is>
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>Jamnagar</t>
+          <t>Albuquerque, NM</t>
         </is>
       </c>
       <c r="E281" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F281" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="282">
       <c r="A282" s="1" t="inlineStr">
         <is>
-          <t>ABQ</t>
+          <t>ANC</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>Albuquerque, NM, United States</t>
+          <t>Anchorage, AK, United States</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
@@ -9354,7 +9354,7 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>Albuquerque, NM</t>
+          <t>Anchorage, AK</t>
         </is>
       </c>
       <c r="E282" t="inlineStr">
@@ -9371,12 +9371,12 @@
     <row r="283">
       <c r="A283" s="1" t="inlineStr">
         <is>
-          <t>ANC</t>
+          <t>IAD</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>Anchorage, AK, United States</t>
+          <t>Ashburn, VA, United States</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
@@ -9386,7 +9386,7 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>Anchorage, AK</t>
+          <t>Ashburn, VA</t>
         </is>
       </c>
       <c r="E283" t="inlineStr">
@@ -9403,12 +9403,12 @@
     <row r="284">
       <c r="A284" s="1" t="inlineStr">
         <is>
-          <t>IAD</t>
+          <t>ATL</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>Ashburn, VA, United States</t>
+          <t>Atlanta, GA, United States</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
@@ -9418,7 +9418,7 @@
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>Ashburn, VA</t>
+          <t>Atlanta, GA</t>
         </is>
       </c>
       <c r="E284" t="inlineStr">
@@ -9435,12 +9435,12 @@
     <row r="285">
       <c r="A285" s="1" t="inlineStr">
         <is>
-          <t>ATL</t>
+          <t>AUS</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>Atlanta, GA, United States</t>
+          <t>Austin, TX, United States</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
@@ -9450,7 +9450,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>Atlanta, GA</t>
+          <t>Austin, TX</t>
         </is>
       </c>
       <c r="E285" t="inlineStr">
@@ -9467,12 +9467,12 @@
     <row r="286">
       <c r="A286" s="1" t="inlineStr">
         <is>
-          <t>AUS</t>
+          <t>BGR</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>Austin, TX, United States</t>
+          <t>Bangor, ME, United States</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
@@ -9482,7 +9482,7 @@
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>Austin, TX</t>
+          <t>Bangor, ME</t>
         </is>
       </c>
       <c r="E286" t="inlineStr">
@@ -9499,12 +9499,12 @@
     <row r="287">
       <c r="A287" s="1" t="inlineStr">
         <is>
-          <t>BGR</t>
+          <t>BOS</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>Bangor, ME, United States</t>
+          <t>Boston, MA, United States</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
@@ -9514,7 +9514,7 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>Bangor, ME</t>
+          <t>Boston, MA</t>
         </is>
       </c>
       <c r="E287" t="inlineStr">
@@ -9531,12 +9531,12 @@
     <row r="288">
       <c r="A288" s="1" t="inlineStr">
         <is>
-          <t>BOS</t>
+          <t>BUF</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>Boston, MA, United States</t>
+          <t>Buffalo, NY, United States</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
@@ -9546,7 +9546,7 @@
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>Boston, MA</t>
+          <t>Buffalo, NY</t>
         </is>
       </c>
       <c r="E288" t="inlineStr">
@@ -9563,12 +9563,12 @@
     <row r="289">
       <c r="A289" s="1" t="inlineStr">
         <is>
-          <t>BUF</t>
+          <t>YYC</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>Buffalo, NY, United States</t>
+          <t>Calgary, AB, Canada</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
@@ -9578,29 +9578,29 @@
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>Buffalo, NY</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="E289" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F289" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="290">
       <c r="A290" s="1" t="inlineStr">
         <is>
-          <t>YYC</t>
+          <t>CLT</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>Calgary, AB, Canada</t>
+          <t>Charlotte, NC, United States</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
@@ -9610,29 +9610,29 @@
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Charlotte, NC</t>
         </is>
       </c>
       <c r="E290" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F290" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="291">
       <c r="A291" s="1" t="inlineStr">
         <is>
-          <t>CLT</t>
+          <t>ORD</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>Charlotte, NC, United States</t>
+          <t>Chicago, IL, United States</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
@@ -9642,7 +9642,7 @@
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>Charlotte, NC</t>
+          <t>Chicago, IL</t>
         </is>
       </c>
       <c r="E291" t="inlineStr">
@@ -9659,12 +9659,12 @@
     <row r="292">
       <c r="A292" s="1" t="inlineStr">
         <is>
-          <t>ORD</t>
+          <t>CLE</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>Chicago, IL, United States</t>
+          <t>Cleveland, OH, United States</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
@@ -9674,7 +9674,7 @@
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>Chicago, IL</t>
+          <t>Cleveland, OH</t>
         </is>
       </c>
       <c r="E292" t="inlineStr">
@@ -9691,12 +9691,12 @@
     <row r="293">
       <c r="A293" s="1" t="inlineStr">
         <is>
-          <t>CLE</t>
+          <t>CMH</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>Cleveland, OH, United States</t>
+          <t>Columbus, OH, United States</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
@@ -9706,7 +9706,7 @@
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>Cleveland, OH</t>
+          <t>Columbus, OH</t>
         </is>
       </c>
       <c r="E293" t="inlineStr">
@@ -9723,12 +9723,12 @@
     <row r="294">
       <c r="A294" s="1" t="inlineStr">
         <is>
-          <t>CMH</t>
+          <t>DFW</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>Columbus, OH, United States</t>
+          <t>Dallas, TX, United States</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
@@ -9738,7 +9738,7 @@
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>Columbus, OH</t>
+          <t>Dallas, TX</t>
         </is>
       </c>
       <c r="E294" t="inlineStr">
@@ -9755,12 +9755,12 @@
     <row r="295">
       <c r="A295" s="1" t="inlineStr">
         <is>
-          <t>DFW</t>
+          <t>DEN</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>Dallas, TX, United States</t>
+          <t>Denver, CO, United States</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -9770,7 +9770,7 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>Dallas, TX</t>
+          <t>Denver, CO</t>
         </is>
       </c>
       <c r="E295" t="inlineStr">
@@ -9787,12 +9787,12 @@
     <row r="296">
       <c r="A296" s="1" t="inlineStr">
         <is>
-          <t>DEN</t>
+          <t>DTW</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>Denver, CO, United States</t>
+          <t>Detroit, MI, United States</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -9802,7 +9802,7 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>Denver, CO</t>
+          <t>Detroit, MI</t>
         </is>
       </c>
       <c r="E296" t="inlineStr">
@@ -9819,12 +9819,12 @@
     <row r="297">
       <c r="A297" s="1" t="inlineStr">
         <is>
-          <t>DTW</t>
+          <t>RDU</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>Detroit, MI, United States</t>
+          <t>Durham, NC, United States</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
@@ -9834,7 +9834,7 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>Detroit, MI</t>
+          <t>Durham, NC</t>
         </is>
       </c>
       <c r="E297" t="inlineStr">
@@ -9851,12 +9851,12 @@
     <row r="298">
       <c r="A298" s="1" t="inlineStr">
         <is>
-          <t>RDU</t>
+          <t>GDL</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>Durham, NC, United States</t>
+          <t>Guadalajara, Mexico</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
@@ -9866,29 +9866,29 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>Durham, NC</t>
+          <t>Guadalajara</t>
         </is>
       </c>
       <c r="E298" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F298" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
     </row>
     <row r="299">
       <c r="A299" s="1" t="inlineStr">
         <is>
-          <t>GDL</t>
+          <t>YHZ</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>Guadalajara, Mexico</t>
+          <t>Halifax, Canada</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
@@ -9898,29 +9898,29 @@
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>Guadalajara</t>
+          <t>Halifax</t>
         </is>
       </c>
       <c r="E299" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F299" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="300">
       <c r="A300" s="1" t="inlineStr">
         <is>
-          <t>YHZ</t>
+          <t>HNL</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>Halifax, Canada</t>
+          <t>Honolulu, HI, United States</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
@@ -9930,29 +9930,29 @@
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>Halifax</t>
+          <t>Honolulu, HI</t>
         </is>
       </c>
       <c r="E300" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F300" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="301">
       <c r="A301" s="1" t="inlineStr">
         <is>
-          <t>HNL</t>
+          <t>IAH</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>Honolulu, HI, United States</t>
+          <t>Houston, TX, United States</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
@@ -9962,7 +9962,7 @@
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>Honolulu, HI</t>
+          <t>Houston, TX</t>
         </is>
       </c>
       <c r="E301" t="inlineStr">
@@ -9979,12 +9979,12 @@
     <row r="302">
       <c r="A302" s="1" t="inlineStr">
         <is>
-          <t>IAH</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>Houston, TX, United States</t>
+          <t>Indianapolis, IN, United States</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
@@ -9994,7 +9994,7 @@
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>Houston, TX</t>
+          <t>Indianapolis, IN</t>
         </is>
       </c>
       <c r="E302" t="inlineStr">
@@ -10011,12 +10011,12 @@
     <row r="303">
       <c r="A303" s="1" t="inlineStr">
         <is>
-          <t>IND</t>
+          <t>JAX</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>Indianapolis, IN, United States</t>
+          <t>Jacksonville, FL, United States</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
@@ -10026,7 +10026,7 @@
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>Indianapolis, IN</t>
+          <t>Jacksonville, FL</t>
         </is>
       </c>
       <c r="E303" t="inlineStr">
@@ -10043,12 +10043,12 @@
     <row r="304">
       <c r="A304" s="1" t="inlineStr">
         <is>
-          <t>JAX</t>
+          <t>MCI</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>Jacksonville, FL, United States</t>
+          <t>Kansas City, MO, United States</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
@@ -10058,7 +10058,7 @@
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>Jacksonville, FL</t>
+          <t>Kansas City, MO</t>
         </is>
       </c>
       <c r="E304" t="inlineStr">
@@ -10075,12 +10075,12 @@
     <row r="305">
       <c r="A305" s="1" t="inlineStr">
         <is>
-          <t>MCI</t>
+          <t>KIN</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>Kansas City, MO, United States</t>
+          <t>Kingston, Jamaica</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
@@ -10090,29 +10090,29 @@
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>Kansas City, MO</t>
+          <t>Kingston</t>
         </is>
       </c>
       <c r="E305" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Jamaica</t>
         </is>
       </c>
       <c r="F305" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>JM</t>
         </is>
       </c>
     </row>
     <row r="306">
       <c r="A306" s="1" t="inlineStr">
         <is>
-          <t>KIN</t>
+          <t>LAS</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>Kingston, Jamaica</t>
+          <t>Las Vegas, NV, United States</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
@@ -10122,29 +10122,29 @@
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t>Kingston</t>
+          <t>Las Vegas, NV</t>
         </is>
       </c>
       <c r="E306" t="inlineStr">
         <is>
-          <t>Jamaica</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F306" t="inlineStr">
         <is>
-          <t>JM</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="307">
       <c r="A307" s="1" t="inlineStr">
         <is>
-          <t>LAS</t>
+          <t>LAX</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>Las Vegas, NV, United States</t>
+          <t>Los Angeles, CA, United States</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
@@ -10154,7 +10154,7 @@
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>Las Vegas, NV</t>
+          <t>Los Angeles, CA</t>
         </is>
       </c>
       <c r="E307" t="inlineStr">
@@ -10171,12 +10171,12 @@
     <row r="308">
       <c r="A308" s="1" t="inlineStr">
         <is>
-          <t>LAX</t>
+          <t>MEM</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>Los Angeles, CA, United States</t>
+          <t>Memphis, TN, United States</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
@@ -10186,7 +10186,7 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>Los Angeles, CA</t>
+          <t>Memphis, TN</t>
         </is>
       </c>
       <c r="E308" t="inlineStr">
@@ -10203,12 +10203,12 @@
     <row r="309">
       <c r="A309" s="1" t="inlineStr">
         <is>
-          <t>MEM</t>
+          <t>MEX</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>Memphis, TN, United States</t>
+          <t>Mexico City, Mexico</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
@@ -10218,29 +10218,29 @@
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>Memphis, TN</t>
+          <t>Mexico City</t>
         </is>
       </c>
       <c r="E309" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F309" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
     </row>
     <row r="310">
       <c r="A310" s="1" t="inlineStr">
         <is>
-          <t>MEX</t>
+          <t>MIA</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>Mexico City, Mexico</t>
+          <t>Miami, FL, United States</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
@@ -10250,29 +10250,29 @@
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>Mexico City</t>
+          <t>Miami, FL</t>
         </is>
       </c>
       <c r="E310" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F310" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="311">
       <c r="A311" s="1" t="inlineStr">
         <is>
-          <t>MIA</t>
+          <t>MSP</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Miami, FL, United States</t>
+          <t>Minneapolis, MN, United States</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
@@ -10282,7 +10282,7 @@
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>Miami, FL</t>
+          <t>Minneapolis, MN</t>
         </is>
       </c>
       <c r="E311" t="inlineStr">
@@ -10299,12 +10299,12 @@
     <row r="312">
       <c r="A312" s="1" t="inlineStr">
         <is>
-          <t>MSP</t>
+          <t>YUL</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>Minneapolis, MN, United States</t>
+          <t>Montréal, QC, Canada</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
@@ -10314,29 +10314,29 @@
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>Minneapolis, MN</t>
+          <t>Montréal, QC</t>
         </is>
       </c>
       <c r="E312" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F312" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="313">
       <c r="A313" s="1" t="inlineStr">
         <is>
-          <t>YUL</t>
+          <t>BNA</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Montréal, QC, Canada</t>
+          <t>Nashville, United States</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
@@ -10346,29 +10346,29 @@
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>Montréal, QC</t>
+          <t>Nashville</t>
         </is>
       </c>
       <c r="E313" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F313" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="314">
       <c r="A314" s="1" t="inlineStr">
         <is>
-          <t>BNA</t>
+          <t>EWR</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Nashville, United States</t>
+          <t>Newark, NJ, United States</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -10378,7 +10378,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>Nashville</t>
+          <t>Newark, NJ</t>
         </is>
       </c>
       <c r="E314" t="inlineStr">
@@ -10395,12 +10395,12 @@
     <row r="315">
       <c r="A315" s="1" t="inlineStr">
         <is>
-          <t>EWR</t>
+          <t>ORF</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>Newark, NJ, United States</t>
+          <t>Norfolk, VA, United States</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
@@ -10410,7 +10410,7 @@
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>Newark, NJ</t>
+          <t>Norfolk, VA</t>
         </is>
       </c>
       <c r="E315" t="inlineStr">
@@ -10427,12 +10427,12 @@
     <row r="316">
       <c r="A316" s="1" t="inlineStr">
         <is>
-          <t>ORF</t>
+          <t>OKC</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Norfolk, VA, United States</t>
+          <t>Oklahoma City, OK, United States</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
@@ -10442,7 +10442,7 @@
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>Norfolk, VA</t>
+          <t>Oklahoma City, OK</t>
         </is>
       </c>
       <c r="E316" t="inlineStr">
@@ -10459,12 +10459,12 @@
     <row r="317">
       <c r="A317" s="1" t="inlineStr">
         <is>
-          <t>OKC</t>
+          <t>OMA</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Oklahoma City, OK, United States</t>
+          <t>Omaha, NE, United States</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -10474,7 +10474,7 @@
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t>Oklahoma City, OK</t>
+          <t>Omaha, NE</t>
         </is>
       </c>
       <c r="E317" t="inlineStr">
@@ -10491,12 +10491,12 @@
     <row r="318">
       <c r="A318" s="1" t="inlineStr">
         <is>
-          <t>OMA</t>
+          <t>PHL</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>Omaha, NE, United States</t>
+          <t>Philadelphia, United States</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
@@ -10506,7 +10506,7 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>Omaha, NE</t>
+          <t>Philadelphia</t>
         </is>
       </c>
       <c r="E318" t="inlineStr">
@@ -10523,12 +10523,12 @@
     <row r="319">
       <c r="A319" s="1" t="inlineStr">
         <is>
-          <t>PHL</t>
+          <t>PHX</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Philadelphia, United States</t>
+          <t>Phoenix, AZ, United States</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
@@ -10538,7 +10538,7 @@
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>Philadelphia</t>
+          <t>Phoenix, AZ</t>
         </is>
       </c>
       <c r="E319" t="inlineStr">
@@ -10555,12 +10555,12 @@
     <row r="320">
       <c r="A320" s="1" t="inlineStr">
         <is>
-          <t>PHX</t>
+          <t>PIT</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Phoenix, AZ, United States</t>
+          <t>Pittsburgh, PA, United States</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -10570,7 +10570,7 @@
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t>Phoenix, AZ</t>
+          <t>Pittsburgh, PA</t>
         </is>
       </c>
       <c r="E320" t="inlineStr">
@@ -10587,12 +10587,12 @@
     <row r="321">
       <c r="A321" s="1" t="inlineStr">
         <is>
-          <t>PIT</t>
+          <t>PDX</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>Pittsburgh, PA, United States</t>
+          <t>Portland, OR, United States</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
@@ -10602,7 +10602,7 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>Pittsburgh, PA</t>
+          <t>Portland, OR</t>
         </is>
       </c>
       <c r="E321" t="inlineStr">
@@ -10619,12 +10619,12 @@
     <row r="322">
       <c r="A322" s="1" t="inlineStr">
         <is>
-          <t>PDX</t>
+          <t>QRO</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>Portland, OR, United States</t>
+          <t>Queretaro, MX, Mexico</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
@@ -10634,29 +10634,29 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>Portland, OR</t>
+          <t>Queretaro, MX</t>
         </is>
       </c>
       <c r="E322" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F322" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
     </row>
     <row r="323">
       <c r="A323" s="1" t="inlineStr">
         <is>
-          <t>QRO</t>
+          <t>RIC</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>Queretaro, MX, Mexico</t>
+          <t>Richmond, VA, United States</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -10666,29 +10666,29 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>Queretaro, MX</t>
+          <t>Richmond, VA</t>
         </is>
       </c>
       <c r="E323" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F323" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="324">
       <c r="A324" s="1" t="inlineStr">
         <is>
-          <t>RIC</t>
+          <t>SMF</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>Richmond, VA, United States</t>
+          <t>Sacramento, CA, United States</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -10698,7 +10698,7 @@
       </c>
       <c r="D324" t="inlineStr">
         <is>
-          <t>Richmond, VA</t>
+          <t>Sacramento, CA</t>
         </is>
       </c>
       <c r="E324" t="inlineStr">
@@ -10715,12 +10715,12 @@
     <row r="325">
       <c r="A325" s="1" t="inlineStr">
         <is>
-          <t>SMF</t>
+          <t>SLC</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>Sacramento, CA, United States</t>
+          <t>Salt Lake City, UT, United States</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -10730,7 +10730,7 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>Sacramento, CA</t>
+          <t>Salt Lake City, UT</t>
         </is>
       </c>
       <c r="E325" t="inlineStr">
@@ -10747,12 +10747,12 @@
     <row r="326">
       <c r="A326" s="1" t="inlineStr">
         <is>
-          <t>SLC</t>
+          <t>SAT</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>Salt Lake City, UT, United States</t>
+          <t>San Antonio, TX, United States</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
@@ -10762,7 +10762,7 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>Salt Lake City, UT</t>
+          <t>San Antonio, TX</t>
         </is>
       </c>
       <c r="E326" t="inlineStr">
@@ -10779,12 +10779,12 @@
     <row r="327">
       <c r="A327" s="1" t="inlineStr">
         <is>
-          <t>SAT</t>
+          <t>SAN</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>San Antonio, TX, United States</t>
+          <t>San Diego, CA, United States</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
@@ -10794,7 +10794,7 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>San Antonio, TX</t>
+          <t>San Diego, CA</t>
         </is>
       </c>
       <c r="E327" t="inlineStr">
@@ -10811,12 +10811,12 @@
     <row r="328">
       <c r="A328" s="1" t="inlineStr">
         <is>
-          <t>SAN</t>
+          <t>SFO</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>San Diego, CA, United States</t>
+          <t>San Francisco, CA, United States</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
@@ -10826,7 +10826,7 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>San Diego, CA</t>
+          <t>San Francisco, CA</t>
         </is>
       </c>
       <c r="E328" t="inlineStr">
@@ -10843,12 +10843,12 @@
     <row r="329">
       <c r="A329" s="1" t="inlineStr">
         <is>
-          <t>SFO</t>
+          <t>SJC</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>San Francisco, CA, United States</t>
+          <t>San Jose, CA, United States</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
@@ -10858,7 +10858,7 @@
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>San Francisco, CA</t>
+          <t>San Jose, CA</t>
         </is>
       </c>
       <c r="E329" t="inlineStr">
@@ -10875,12 +10875,12 @@
     <row r="330">
       <c r="A330" s="1" t="inlineStr">
         <is>
-          <t>SJC</t>
+          <t>YXE</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>San Jose, CA, United States</t>
+          <t>Saskatoon, SK, Canada</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
@@ -10890,29 +10890,29 @@
       </c>
       <c r="D330" t="inlineStr">
         <is>
-          <t>San Jose, CA</t>
+          <t>Saskatoon, SK</t>
         </is>
       </c>
       <c r="E330" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F330" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="331">
       <c r="A331" s="1" t="inlineStr">
         <is>
-          <t>YXE</t>
+          <t>SEA</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>Saskatoon, SK, Canada</t>
+          <t>Seattle, WA, United States</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
@@ -10922,29 +10922,29 @@
       </c>
       <c r="D331" t="inlineStr">
         <is>
-          <t>Saskatoon, SK</t>
+          <t>Seattle, WA</t>
         </is>
       </c>
       <c r="E331" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F331" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="332">
       <c r="A332" s="1" t="inlineStr">
         <is>
-          <t>SEA</t>
+          <t>FSD</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>Seattle, WA, United States</t>
+          <t>Sioux Falls, SD, United States</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
@@ -10954,7 +10954,7 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>Seattle, WA</t>
+          <t>Sioux Falls, SD</t>
         </is>
       </c>
       <c r="E332" t="inlineStr">
@@ -10971,12 +10971,12 @@
     <row r="333">
       <c r="A333" s="1" t="inlineStr">
         <is>
-          <t>FSD</t>
+          <t>STL</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>Sioux Falls, SD, United States</t>
+          <t>St. Louis, MO, United States</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
@@ -10986,7 +10986,7 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>Sioux Falls, SD</t>
+          <t>St. Louis, MO</t>
         </is>
       </c>
       <c r="E333" t="inlineStr">
@@ -11003,12 +11003,12 @@
     <row r="334">
       <c r="A334" s="1" t="inlineStr">
         <is>
-          <t>STL</t>
+          <t>TLH</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>St. Louis, MO, United States</t>
+          <t>Tallahassee, FL, United States</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
@@ -11018,7 +11018,7 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>St. Louis, MO</t>
+          <t>Tallahassee, FL</t>
         </is>
       </c>
       <c r="E334" t="inlineStr">
@@ -11035,12 +11035,12 @@
     <row r="335">
       <c r="A335" s="1" t="inlineStr">
         <is>
-          <t>TLH</t>
+          <t>TPA</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>Tallahassee, FL, United States</t>
+          <t>Tampa, FL, United States</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
@@ -11050,7 +11050,7 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>Tallahassee, FL</t>
+          <t>Tampa, FL</t>
         </is>
       </c>
       <c r="E335" t="inlineStr">
@@ -11067,12 +11067,12 @@
     <row r="336">
       <c r="A336" s="1" t="inlineStr">
         <is>
-          <t>TPA</t>
+          <t>YYZ</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>Tampa, FL, United States</t>
+          <t>Toronto, ON, Canada</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
@@ -11082,29 +11082,29 @@
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>Tampa, FL</t>
+          <t>Toronto, ON</t>
         </is>
       </c>
       <c r="E336" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F336" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="337">
       <c r="A337" s="1" t="inlineStr">
         <is>
-          <t>YYZ</t>
+          <t>YVR</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>Toronto, ON, Canada</t>
+          <t>Vancouver, BC, Canada</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
@@ -11114,7 +11114,7 @@
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>Toronto, ON</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="E337" t="inlineStr">
@@ -11131,12 +11131,12 @@
     <row r="338">
       <c r="A338" s="1" t="inlineStr">
         <is>
-          <t>YVR</t>
+          <t>YWG</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>Vancouver, BC, Canada</t>
+          <t>Winnipeg, MB, Canada</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
@@ -11146,7 +11146,7 @@
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Winnipeg, MB</t>
         </is>
       </c>
       <c r="E338" t="inlineStr">
@@ -11163,12 +11163,12 @@
     <row r="339">
       <c r="A339" s="1" t="inlineStr">
         <is>
-          <t>YWG</t>
+          <t>CVG</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>Winnipeg, MB, Canada</t>
+          <t>Cincinnati, United States</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
@@ -11178,47 +11178,15 @@
       </c>
       <c r="D339" t="inlineStr">
         <is>
-          <t>Winnipeg, MB</t>
+          <t>Cincinnati</t>
         </is>
       </c>
       <c r="E339" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F339" t="inlineStr">
-        <is>
-          <t>CA</t>
-        </is>
-      </c>
-    </row>
-    <row r="340">
-      <c r="A340" s="1" t="inlineStr">
-        <is>
-          <t>CVG</t>
-        </is>
-      </c>
-      <c r="B340" t="inlineStr">
-        <is>
-          <t>Cincinnati, United States</t>
-        </is>
-      </c>
-      <c r="C340" t="inlineStr">
-        <is>
-          <t>North America</t>
-        </is>
-      </c>
-      <c r="D340" t="inlineStr">
-        <is>
-          <t>Cincinnati</t>
-        </is>
-      </c>
-      <c r="E340" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="F340" t="inlineStr">
         <is>
           <t>US</t>
         </is>

</xml_diff>

<commit_message>
update generated data Triggered by 651048d847ef7c7a3caf19f5ae1ad56677f3599c
</commit_message>
<xml_diff>
--- a/DC-Colos.xlsx
+++ b/DC-Colos.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F339"/>
+  <dimension ref="A1:F340"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9307,44 +9307,44 @@
     <row r="281">
       <c r="A281" s="1" t="inlineStr">
         <is>
-          <t>ABQ</t>
+          <t>UDR</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>Albuquerque, NM, United States</t>
+          <t>Udaipur, India</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>North America</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>Albuquerque, NM</t>
+          <t>Udaipur</t>
         </is>
       </c>
       <c r="E281" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F281" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="282">
       <c r="A282" s="1" t="inlineStr">
         <is>
-          <t>ANC</t>
+          <t>ABQ</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>Anchorage, AK, United States</t>
+          <t>Albuquerque, NM, United States</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
@@ -9354,7 +9354,7 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>Anchorage, AK</t>
+          <t>Albuquerque, NM</t>
         </is>
       </c>
       <c r="E282" t="inlineStr">
@@ -9371,12 +9371,12 @@
     <row r="283">
       <c r="A283" s="1" t="inlineStr">
         <is>
-          <t>IAD</t>
+          <t>ANC</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>Ashburn, VA, United States</t>
+          <t>Anchorage, AK, United States</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
@@ -9386,7 +9386,7 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>Ashburn, VA</t>
+          <t>Anchorage, AK</t>
         </is>
       </c>
       <c r="E283" t="inlineStr">
@@ -9403,12 +9403,12 @@
     <row r="284">
       <c r="A284" s="1" t="inlineStr">
         <is>
-          <t>ATL</t>
+          <t>IAD</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>Atlanta, GA, United States</t>
+          <t>Ashburn, VA, United States</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
@@ -9418,7 +9418,7 @@
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>Atlanta, GA</t>
+          <t>Ashburn, VA</t>
         </is>
       </c>
       <c r="E284" t="inlineStr">
@@ -9435,12 +9435,12 @@
     <row r="285">
       <c r="A285" s="1" t="inlineStr">
         <is>
-          <t>AUS</t>
+          <t>ATL</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>Austin, TX, United States</t>
+          <t>Atlanta, GA, United States</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
@@ -9450,7 +9450,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>Austin, TX</t>
+          <t>Atlanta, GA</t>
         </is>
       </c>
       <c r="E285" t="inlineStr">
@@ -9467,12 +9467,12 @@
     <row r="286">
       <c r="A286" s="1" t="inlineStr">
         <is>
-          <t>BGR</t>
+          <t>AUS</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>Bangor, ME, United States</t>
+          <t>Austin, TX, United States</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
@@ -9482,7 +9482,7 @@
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>Bangor, ME</t>
+          <t>Austin, TX</t>
         </is>
       </c>
       <c r="E286" t="inlineStr">
@@ -9499,12 +9499,12 @@
     <row r="287">
       <c r="A287" s="1" t="inlineStr">
         <is>
-          <t>BOS</t>
+          <t>BGR</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>Boston, MA, United States</t>
+          <t>Bangor, ME, United States</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
@@ -9514,7 +9514,7 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>Boston, MA</t>
+          <t>Bangor, ME</t>
         </is>
       </c>
       <c r="E287" t="inlineStr">
@@ -9531,12 +9531,12 @@
     <row r="288">
       <c r="A288" s="1" t="inlineStr">
         <is>
-          <t>BUF</t>
+          <t>BOS</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>Buffalo, NY, United States</t>
+          <t>Boston, MA, United States</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
@@ -9546,7 +9546,7 @@
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>Buffalo, NY</t>
+          <t>Boston, MA</t>
         </is>
       </c>
       <c r="E288" t="inlineStr">
@@ -9563,12 +9563,12 @@
     <row r="289">
       <c r="A289" s="1" t="inlineStr">
         <is>
-          <t>YYC</t>
+          <t>BUF</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>Calgary, AB, Canada</t>
+          <t>Buffalo, NY, United States</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
@@ -9578,29 +9578,29 @@
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Buffalo, NY</t>
         </is>
       </c>
       <c r="E289" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F289" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="290">
       <c r="A290" s="1" t="inlineStr">
         <is>
-          <t>CLT</t>
+          <t>YYC</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>Charlotte, NC, United States</t>
+          <t>Calgary, AB, Canada</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
@@ -9610,29 +9610,29 @@
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>Charlotte, NC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="E290" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F290" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="291">
       <c r="A291" s="1" t="inlineStr">
         <is>
-          <t>ORD</t>
+          <t>CLT</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>Chicago, IL, United States</t>
+          <t>Charlotte, NC, United States</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
@@ -9642,7 +9642,7 @@
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>Chicago, IL</t>
+          <t>Charlotte, NC</t>
         </is>
       </c>
       <c r="E291" t="inlineStr">
@@ -9659,12 +9659,12 @@
     <row r="292">
       <c r="A292" s="1" t="inlineStr">
         <is>
-          <t>CLE</t>
+          <t>ORD</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>Cleveland, OH, United States</t>
+          <t>Chicago, IL, United States</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
@@ -9674,7 +9674,7 @@
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>Cleveland, OH</t>
+          <t>Chicago, IL</t>
         </is>
       </c>
       <c r="E292" t="inlineStr">
@@ -9691,12 +9691,12 @@
     <row r="293">
       <c r="A293" s="1" t="inlineStr">
         <is>
-          <t>CMH</t>
+          <t>CLE</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>Columbus, OH, United States</t>
+          <t>Cleveland, OH, United States</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
@@ -9706,7 +9706,7 @@
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>Columbus, OH</t>
+          <t>Cleveland, OH</t>
         </is>
       </c>
       <c r="E293" t="inlineStr">
@@ -9723,12 +9723,12 @@
     <row r="294">
       <c r="A294" s="1" t="inlineStr">
         <is>
-          <t>DFW</t>
+          <t>CMH</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>Dallas, TX, United States</t>
+          <t>Columbus, OH, United States</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
@@ -9738,7 +9738,7 @@
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>Dallas, TX</t>
+          <t>Columbus, OH</t>
         </is>
       </c>
       <c r="E294" t="inlineStr">
@@ -9755,12 +9755,12 @@
     <row r="295">
       <c r="A295" s="1" t="inlineStr">
         <is>
-          <t>DEN</t>
+          <t>DFW</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>Denver, CO, United States</t>
+          <t>Dallas, TX, United States</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -9770,7 +9770,7 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>Denver, CO</t>
+          <t>Dallas, TX</t>
         </is>
       </c>
       <c r="E295" t="inlineStr">
@@ -9787,12 +9787,12 @@
     <row r="296">
       <c r="A296" s="1" t="inlineStr">
         <is>
-          <t>DTW</t>
+          <t>DEN</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>Detroit, MI, United States</t>
+          <t>Denver, CO, United States</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -9802,7 +9802,7 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>Detroit, MI</t>
+          <t>Denver, CO</t>
         </is>
       </c>
       <c r="E296" t="inlineStr">
@@ -9819,12 +9819,12 @@
     <row r="297">
       <c r="A297" s="1" t="inlineStr">
         <is>
-          <t>RDU</t>
+          <t>DTW</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>Durham, NC, United States</t>
+          <t>Detroit, MI, United States</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
@@ -9834,7 +9834,7 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>Durham, NC</t>
+          <t>Detroit, MI</t>
         </is>
       </c>
       <c r="E297" t="inlineStr">
@@ -9851,12 +9851,12 @@
     <row r="298">
       <c r="A298" s="1" t="inlineStr">
         <is>
-          <t>GDL</t>
+          <t>RDU</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>Guadalajara, Mexico</t>
+          <t>Durham, NC, United States</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
@@ -9866,29 +9866,29 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>Guadalajara</t>
+          <t>Durham, NC</t>
         </is>
       </c>
       <c r="E298" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F298" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="299">
       <c r="A299" s="1" t="inlineStr">
         <is>
-          <t>YHZ</t>
+          <t>GDL</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>Halifax, Canada</t>
+          <t>Guadalajara, Mexico</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
@@ -9898,29 +9898,29 @@
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>Halifax</t>
+          <t>Guadalajara</t>
         </is>
       </c>
       <c r="E299" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F299" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>MX</t>
         </is>
       </c>
     </row>
     <row r="300">
       <c r="A300" s="1" t="inlineStr">
         <is>
-          <t>HNL</t>
+          <t>YHZ</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>Honolulu, HI, United States</t>
+          <t>Halifax, Canada</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
@@ -9930,29 +9930,29 @@
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>Honolulu, HI</t>
+          <t>Halifax</t>
         </is>
       </c>
       <c r="E300" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F300" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="301">
       <c r="A301" s="1" t="inlineStr">
         <is>
-          <t>IAH</t>
+          <t>HNL</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>Houston, TX, United States</t>
+          <t>Honolulu, HI, United States</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
@@ -9962,7 +9962,7 @@
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>Houston, TX</t>
+          <t>Honolulu, HI</t>
         </is>
       </c>
       <c r="E301" t="inlineStr">
@@ -9979,12 +9979,12 @@
     <row r="302">
       <c r="A302" s="1" t="inlineStr">
         <is>
-          <t>IND</t>
+          <t>IAH</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>Indianapolis, IN, United States</t>
+          <t>Houston, TX, United States</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
@@ -9994,7 +9994,7 @@
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>Indianapolis, IN</t>
+          <t>Houston, TX</t>
         </is>
       </c>
       <c r="E302" t="inlineStr">
@@ -10011,12 +10011,12 @@
     <row r="303">
       <c r="A303" s="1" t="inlineStr">
         <is>
-          <t>JAX</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>Jacksonville, FL, United States</t>
+          <t>Indianapolis, IN, United States</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
@@ -10026,7 +10026,7 @@
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>Jacksonville, FL</t>
+          <t>Indianapolis, IN</t>
         </is>
       </c>
       <c r="E303" t="inlineStr">
@@ -10043,12 +10043,12 @@
     <row r="304">
       <c r="A304" s="1" t="inlineStr">
         <is>
-          <t>MCI</t>
+          <t>JAX</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>Kansas City, MO, United States</t>
+          <t>Jacksonville, FL, United States</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
@@ -10058,7 +10058,7 @@
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>Kansas City, MO</t>
+          <t>Jacksonville, FL</t>
         </is>
       </c>
       <c r="E304" t="inlineStr">
@@ -10075,12 +10075,12 @@
     <row r="305">
       <c r="A305" s="1" t="inlineStr">
         <is>
-          <t>KIN</t>
+          <t>MCI</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>Kingston, Jamaica</t>
+          <t>Kansas City, MO, United States</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
@@ -10090,29 +10090,29 @@
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>Kingston</t>
+          <t>Kansas City, MO</t>
         </is>
       </c>
       <c r="E305" t="inlineStr">
         <is>
-          <t>Jamaica</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F305" t="inlineStr">
         <is>
-          <t>JM</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="306">
       <c r="A306" s="1" t="inlineStr">
         <is>
-          <t>LAS</t>
+          <t>KIN</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>Las Vegas, NV, United States</t>
+          <t>Kingston, Jamaica</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
@@ -10122,29 +10122,29 @@
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t>Las Vegas, NV</t>
+          <t>Kingston</t>
         </is>
       </c>
       <c r="E306" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Jamaica</t>
         </is>
       </c>
       <c r="F306" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>JM</t>
         </is>
       </c>
     </row>
     <row r="307">
       <c r="A307" s="1" t="inlineStr">
         <is>
-          <t>LAX</t>
+          <t>LAS</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>Los Angeles, CA, United States</t>
+          <t>Las Vegas, NV, United States</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
@@ -10154,7 +10154,7 @@
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>Los Angeles, CA</t>
+          <t>Las Vegas, NV</t>
         </is>
       </c>
       <c r="E307" t="inlineStr">
@@ -10171,12 +10171,12 @@
     <row r="308">
       <c r="A308" s="1" t="inlineStr">
         <is>
-          <t>MEM</t>
+          <t>LAX</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>Memphis, TN, United States</t>
+          <t>Los Angeles, CA, United States</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
@@ -10186,7 +10186,7 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>Memphis, TN</t>
+          <t>Los Angeles, CA</t>
         </is>
       </c>
       <c r="E308" t="inlineStr">
@@ -10203,12 +10203,12 @@
     <row r="309">
       <c r="A309" s="1" t="inlineStr">
         <is>
-          <t>MEX</t>
+          <t>MEM</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>Mexico City, Mexico</t>
+          <t>Memphis, TN, United States</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
@@ -10218,29 +10218,29 @@
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>Mexico City</t>
+          <t>Memphis, TN</t>
         </is>
       </c>
       <c r="E309" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F309" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="310">
       <c r="A310" s="1" t="inlineStr">
         <is>
-          <t>MIA</t>
+          <t>MEX</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>Miami, FL, United States</t>
+          <t>Mexico City, Mexico</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
@@ -10250,29 +10250,29 @@
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>Miami, FL</t>
+          <t>Mexico City</t>
         </is>
       </c>
       <c r="E310" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F310" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
     </row>
     <row r="311">
       <c r="A311" s="1" t="inlineStr">
         <is>
-          <t>MSP</t>
+          <t>MIA</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Minneapolis, MN, United States</t>
+          <t>Miami, FL, United States</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
@@ -10282,7 +10282,7 @@
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>Minneapolis, MN</t>
+          <t>Miami, FL</t>
         </is>
       </c>
       <c r="E311" t="inlineStr">
@@ -10299,12 +10299,12 @@
     <row r="312">
       <c r="A312" s="1" t="inlineStr">
         <is>
-          <t>YUL</t>
+          <t>MSP</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>Montréal, QC, Canada</t>
+          <t>Minneapolis, MN, United States</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
@@ -10314,29 +10314,29 @@
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>Montréal, QC</t>
+          <t>Minneapolis, MN</t>
         </is>
       </c>
       <c r="E312" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F312" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="313">
       <c r="A313" s="1" t="inlineStr">
         <is>
-          <t>BNA</t>
+          <t>YUL</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Nashville, United States</t>
+          <t>Montréal, QC, Canada</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
@@ -10346,29 +10346,29 @@
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>Nashville</t>
+          <t>Montréal, QC</t>
         </is>
       </c>
       <c r="E313" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F313" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="314">
       <c r="A314" s="1" t="inlineStr">
         <is>
-          <t>EWR</t>
+          <t>BNA</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Newark, NJ, United States</t>
+          <t>Nashville, United States</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -10378,7 +10378,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>Newark, NJ</t>
+          <t>Nashville</t>
         </is>
       </c>
       <c r="E314" t="inlineStr">
@@ -10395,12 +10395,12 @@
     <row r="315">
       <c r="A315" s="1" t="inlineStr">
         <is>
-          <t>ORF</t>
+          <t>EWR</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>Norfolk, VA, United States</t>
+          <t>Newark, NJ, United States</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
@@ -10410,7 +10410,7 @@
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>Norfolk, VA</t>
+          <t>Newark, NJ</t>
         </is>
       </c>
       <c r="E315" t="inlineStr">
@@ -10427,12 +10427,12 @@
     <row r="316">
       <c r="A316" s="1" t="inlineStr">
         <is>
-          <t>OKC</t>
+          <t>ORF</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Oklahoma City, OK, United States</t>
+          <t>Norfolk, VA, United States</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
@@ -10442,7 +10442,7 @@
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>Oklahoma City, OK</t>
+          <t>Norfolk, VA</t>
         </is>
       </c>
       <c r="E316" t="inlineStr">
@@ -10459,12 +10459,12 @@
     <row r="317">
       <c r="A317" s="1" t="inlineStr">
         <is>
-          <t>OMA</t>
+          <t>OKC</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Omaha, NE, United States</t>
+          <t>Oklahoma City, OK, United States</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -10474,7 +10474,7 @@
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t>Omaha, NE</t>
+          <t>Oklahoma City, OK</t>
         </is>
       </c>
       <c r="E317" t="inlineStr">
@@ -10491,12 +10491,12 @@
     <row r="318">
       <c r="A318" s="1" t="inlineStr">
         <is>
-          <t>PHL</t>
+          <t>OMA</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>Philadelphia, United States</t>
+          <t>Omaha, NE, United States</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
@@ -10506,7 +10506,7 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>Philadelphia</t>
+          <t>Omaha, NE</t>
         </is>
       </c>
       <c r="E318" t="inlineStr">
@@ -10523,12 +10523,12 @@
     <row r="319">
       <c r="A319" s="1" t="inlineStr">
         <is>
-          <t>PHX</t>
+          <t>PHL</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Phoenix, AZ, United States</t>
+          <t>Philadelphia, United States</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
@@ -10538,7 +10538,7 @@
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>Phoenix, AZ</t>
+          <t>Philadelphia</t>
         </is>
       </c>
       <c r="E319" t="inlineStr">
@@ -10555,12 +10555,12 @@
     <row r="320">
       <c r="A320" s="1" t="inlineStr">
         <is>
-          <t>PIT</t>
+          <t>PHX</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Pittsburgh, PA, United States</t>
+          <t>Phoenix, AZ, United States</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -10570,7 +10570,7 @@
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t>Pittsburgh, PA</t>
+          <t>Phoenix, AZ</t>
         </is>
       </c>
       <c r="E320" t="inlineStr">
@@ -10587,12 +10587,12 @@
     <row r="321">
       <c r="A321" s="1" t="inlineStr">
         <is>
-          <t>PDX</t>
+          <t>PIT</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>Portland, OR, United States</t>
+          <t>Pittsburgh, PA, United States</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
@@ -10602,7 +10602,7 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>Portland, OR</t>
+          <t>Pittsburgh, PA</t>
         </is>
       </c>
       <c r="E321" t="inlineStr">
@@ -10619,12 +10619,12 @@
     <row r="322">
       <c r="A322" s="1" t="inlineStr">
         <is>
-          <t>QRO</t>
+          <t>PDX</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>Queretaro, MX, Mexico</t>
+          <t>Portland, OR, United States</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
@@ -10634,29 +10634,29 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>Queretaro, MX</t>
+          <t>Portland, OR</t>
         </is>
       </c>
       <c r="E322" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F322" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="323">
       <c r="A323" s="1" t="inlineStr">
         <is>
-          <t>RIC</t>
+          <t>QRO</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>Richmond, VA, United States</t>
+          <t>Queretaro, MX, Mexico</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -10666,29 +10666,29 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>Richmond, VA</t>
+          <t>Queretaro, MX</t>
         </is>
       </c>
       <c r="E323" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F323" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
     </row>
     <row r="324">
       <c r="A324" s="1" t="inlineStr">
         <is>
-          <t>SMF</t>
+          <t>RIC</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>Sacramento, CA, United States</t>
+          <t>Richmond, VA, United States</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -10698,7 +10698,7 @@
       </c>
       <c r="D324" t="inlineStr">
         <is>
-          <t>Sacramento, CA</t>
+          <t>Richmond, VA</t>
         </is>
       </c>
       <c r="E324" t="inlineStr">
@@ -10715,12 +10715,12 @@
     <row r="325">
       <c r="A325" s="1" t="inlineStr">
         <is>
-          <t>SLC</t>
+          <t>SMF</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>Salt Lake City, UT, United States</t>
+          <t>Sacramento, CA, United States</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -10730,7 +10730,7 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>Salt Lake City, UT</t>
+          <t>Sacramento, CA</t>
         </is>
       </c>
       <c r="E325" t="inlineStr">
@@ -10747,12 +10747,12 @@
     <row r="326">
       <c r="A326" s="1" t="inlineStr">
         <is>
-          <t>SAT</t>
+          <t>SLC</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>San Antonio, TX, United States</t>
+          <t>Salt Lake City, UT, United States</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
@@ -10762,7 +10762,7 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>San Antonio, TX</t>
+          <t>Salt Lake City, UT</t>
         </is>
       </c>
       <c r="E326" t="inlineStr">
@@ -10779,12 +10779,12 @@
     <row r="327">
       <c r="A327" s="1" t="inlineStr">
         <is>
-          <t>SAN</t>
+          <t>SAT</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>San Diego, CA, United States</t>
+          <t>San Antonio, TX, United States</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
@@ -10794,7 +10794,7 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>San Diego, CA</t>
+          <t>San Antonio, TX</t>
         </is>
       </c>
       <c r="E327" t="inlineStr">
@@ -10811,12 +10811,12 @@
     <row r="328">
       <c r="A328" s="1" t="inlineStr">
         <is>
-          <t>SFO</t>
+          <t>SAN</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>San Francisco, CA, United States</t>
+          <t>San Diego, CA, United States</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
@@ -10826,7 +10826,7 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>San Francisco, CA</t>
+          <t>San Diego, CA</t>
         </is>
       </c>
       <c r="E328" t="inlineStr">
@@ -10843,12 +10843,12 @@
     <row r="329">
       <c r="A329" s="1" t="inlineStr">
         <is>
-          <t>SJC</t>
+          <t>SFO</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>San Jose, CA, United States</t>
+          <t>San Francisco, CA, United States</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
@@ -10858,7 +10858,7 @@
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>San Jose, CA</t>
+          <t>San Francisco, CA</t>
         </is>
       </c>
       <c r="E329" t="inlineStr">
@@ -10875,12 +10875,12 @@
     <row r="330">
       <c r="A330" s="1" t="inlineStr">
         <is>
-          <t>YXE</t>
+          <t>SJC</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>Saskatoon, SK, Canada</t>
+          <t>San Jose, CA, United States</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
@@ -10890,29 +10890,29 @@
       </c>
       <c r="D330" t="inlineStr">
         <is>
-          <t>Saskatoon, SK</t>
+          <t>San Jose, CA</t>
         </is>
       </c>
       <c r="E330" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F330" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="331">
       <c r="A331" s="1" t="inlineStr">
         <is>
-          <t>SEA</t>
+          <t>YXE</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>Seattle, WA, United States</t>
+          <t>Saskatoon, SK, Canada</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
@@ -10922,29 +10922,29 @@
       </c>
       <c r="D331" t="inlineStr">
         <is>
-          <t>Seattle, WA</t>
+          <t>Saskatoon, SK</t>
         </is>
       </c>
       <c r="E331" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F331" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="332">
       <c r="A332" s="1" t="inlineStr">
         <is>
-          <t>FSD</t>
+          <t>SEA</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>Sioux Falls, SD, United States</t>
+          <t>Seattle, WA, United States</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
@@ -10954,7 +10954,7 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>Sioux Falls, SD</t>
+          <t>Seattle, WA</t>
         </is>
       </c>
       <c r="E332" t="inlineStr">
@@ -10971,12 +10971,12 @@
     <row r="333">
       <c r="A333" s="1" t="inlineStr">
         <is>
-          <t>STL</t>
+          <t>FSD</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>St. Louis, MO, United States</t>
+          <t>Sioux Falls, SD, United States</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
@@ -10986,7 +10986,7 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>St. Louis, MO</t>
+          <t>Sioux Falls, SD</t>
         </is>
       </c>
       <c r="E333" t="inlineStr">
@@ -11003,12 +11003,12 @@
     <row r="334">
       <c r="A334" s="1" t="inlineStr">
         <is>
-          <t>TLH</t>
+          <t>STL</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>Tallahassee, FL, United States</t>
+          <t>St. Louis, MO, United States</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
@@ -11018,7 +11018,7 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>Tallahassee, FL</t>
+          <t>St. Louis, MO</t>
         </is>
       </c>
       <c r="E334" t="inlineStr">
@@ -11035,12 +11035,12 @@
     <row r="335">
       <c r="A335" s="1" t="inlineStr">
         <is>
-          <t>TPA</t>
+          <t>TLH</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>Tampa, FL, United States</t>
+          <t>Tallahassee, FL, United States</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
@@ -11050,7 +11050,7 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>Tampa, FL</t>
+          <t>Tallahassee, FL</t>
         </is>
       </c>
       <c r="E335" t="inlineStr">
@@ -11067,12 +11067,12 @@
     <row r="336">
       <c r="A336" s="1" t="inlineStr">
         <is>
-          <t>YYZ</t>
+          <t>TPA</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>Toronto, ON, Canada</t>
+          <t>Tampa, FL, United States</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
@@ -11082,29 +11082,29 @@
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>Toronto, ON</t>
+          <t>Tampa, FL</t>
         </is>
       </c>
       <c r="E336" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F336" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="337">
       <c r="A337" s="1" t="inlineStr">
         <is>
-          <t>YVR</t>
+          <t>YYZ</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>Vancouver, BC, Canada</t>
+          <t>Toronto, ON, Canada</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
@@ -11114,7 +11114,7 @@
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Toronto, ON</t>
         </is>
       </c>
       <c r="E337" t="inlineStr">
@@ -11131,12 +11131,12 @@
     <row r="338">
       <c r="A338" s="1" t="inlineStr">
         <is>
-          <t>YWG</t>
+          <t>YVR</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>Winnipeg, MB, Canada</t>
+          <t>Vancouver, BC, Canada</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
@@ -11146,7 +11146,7 @@
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>Winnipeg, MB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="E338" t="inlineStr">
@@ -11163,30 +11163,62 @@
     <row r="339">
       <c r="A339" s="1" t="inlineStr">
         <is>
+          <t>YWG</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>Winnipeg, MB, Canada</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>North America</t>
+        </is>
+      </c>
+      <c r="D339" t="inlineStr">
+        <is>
+          <t>Winnipeg, MB</t>
+        </is>
+      </c>
+      <c r="E339" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="F339" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" s="1" t="inlineStr">
+        <is>
           <t>CVG</t>
         </is>
       </c>
-      <c r="B339" t="inlineStr">
+      <c r="B340" t="inlineStr">
         <is>
           <t>Cincinnati, United States</t>
         </is>
       </c>
-      <c r="C339" t="inlineStr">
+      <c r="C340" t="inlineStr">
         <is>
           <t>North America</t>
         </is>
       </c>
-      <c r="D339" t="inlineStr">
+      <c r="D340" t="inlineStr">
         <is>
           <t>Cincinnati</t>
         </is>
       </c>
-      <c r="E339" t="inlineStr">
+      <c r="E340" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="F339" t="inlineStr">
+      <c r="F340" t="inlineStr">
         <is>
           <t>US</t>
         </is>

</xml_diff>

<commit_message>
update generated data Triggered by 8780defb2999a42ee2b397e88b6f8b80bb99de55
</commit_message>
<xml_diff>
--- a/DC-Colos.xlsx
+++ b/DC-Colos.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F340"/>
+  <dimension ref="A1:F341"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9339,44 +9339,44 @@
     <row r="282">
       <c r="A282" s="1" t="inlineStr">
         <is>
-          <t>ABQ</t>
+          <t>AIP</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>Albuquerque, NM, United States</t>
+          <t>Jalandhar, India</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>North America</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>Albuquerque, NM</t>
+          <t>Jalandhar</t>
         </is>
       </c>
       <c r="E282" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F282" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="283">
       <c r="A283" s="1" t="inlineStr">
         <is>
-          <t>ANC</t>
+          <t>ABQ</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>Anchorage, AK, United States</t>
+          <t>Albuquerque, NM, United States</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
@@ -9386,7 +9386,7 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>Anchorage, AK</t>
+          <t>Albuquerque, NM</t>
         </is>
       </c>
       <c r="E283" t="inlineStr">
@@ -9403,12 +9403,12 @@
     <row r="284">
       <c r="A284" s="1" t="inlineStr">
         <is>
-          <t>IAD</t>
+          <t>ANC</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>Ashburn, VA, United States</t>
+          <t>Anchorage, AK, United States</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
@@ -9418,7 +9418,7 @@
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>Ashburn, VA</t>
+          <t>Anchorage, AK</t>
         </is>
       </c>
       <c r="E284" t="inlineStr">
@@ -9435,12 +9435,12 @@
     <row r="285">
       <c r="A285" s="1" t="inlineStr">
         <is>
-          <t>ATL</t>
+          <t>IAD</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>Atlanta, GA, United States</t>
+          <t>Ashburn, VA, United States</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
@@ -9450,7 +9450,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>Atlanta, GA</t>
+          <t>Ashburn, VA</t>
         </is>
       </c>
       <c r="E285" t="inlineStr">
@@ -9467,12 +9467,12 @@
     <row r="286">
       <c r="A286" s="1" t="inlineStr">
         <is>
-          <t>AUS</t>
+          <t>ATL</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>Austin, TX, United States</t>
+          <t>Atlanta, GA, United States</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
@@ -9482,7 +9482,7 @@
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>Austin, TX</t>
+          <t>Atlanta, GA</t>
         </is>
       </c>
       <c r="E286" t="inlineStr">
@@ -9499,12 +9499,12 @@
     <row r="287">
       <c r="A287" s="1" t="inlineStr">
         <is>
-          <t>BGR</t>
+          <t>AUS</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>Bangor, ME, United States</t>
+          <t>Austin, TX, United States</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
@@ -9514,7 +9514,7 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>Bangor, ME</t>
+          <t>Austin, TX</t>
         </is>
       </c>
       <c r="E287" t="inlineStr">
@@ -9531,12 +9531,12 @@
     <row r="288">
       <c r="A288" s="1" t="inlineStr">
         <is>
-          <t>BOS</t>
+          <t>BGR</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>Boston, MA, United States</t>
+          <t>Bangor, ME, United States</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
@@ -9546,7 +9546,7 @@
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>Boston, MA</t>
+          <t>Bangor, ME</t>
         </is>
       </c>
       <c r="E288" t="inlineStr">
@@ -9563,12 +9563,12 @@
     <row r="289">
       <c r="A289" s="1" t="inlineStr">
         <is>
-          <t>BUF</t>
+          <t>BOS</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>Buffalo, NY, United States</t>
+          <t>Boston, MA, United States</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
@@ -9578,7 +9578,7 @@
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>Buffalo, NY</t>
+          <t>Boston, MA</t>
         </is>
       </c>
       <c r="E289" t="inlineStr">
@@ -9595,12 +9595,12 @@
     <row r="290">
       <c r="A290" s="1" t="inlineStr">
         <is>
-          <t>YYC</t>
+          <t>BUF</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>Calgary, AB, Canada</t>
+          <t>Buffalo, NY, United States</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
@@ -9610,29 +9610,29 @@
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Buffalo, NY</t>
         </is>
       </c>
       <c r="E290" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F290" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="291">
       <c r="A291" s="1" t="inlineStr">
         <is>
-          <t>CLT</t>
+          <t>YYC</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>Charlotte, NC, United States</t>
+          <t>Calgary, AB, Canada</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
@@ -9642,29 +9642,29 @@
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>Charlotte, NC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="E291" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F291" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="292">
       <c r="A292" s="1" t="inlineStr">
         <is>
-          <t>ORD</t>
+          <t>CLT</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>Chicago, IL, United States</t>
+          <t>Charlotte, NC, United States</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
@@ -9674,7 +9674,7 @@
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>Chicago, IL</t>
+          <t>Charlotte, NC</t>
         </is>
       </c>
       <c r="E292" t="inlineStr">
@@ -9691,12 +9691,12 @@
     <row r="293">
       <c r="A293" s="1" t="inlineStr">
         <is>
-          <t>CLE</t>
+          <t>ORD</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>Cleveland, OH, United States</t>
+          <t>Chicago, IL, United States</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
@@ -9706,7 +9706,7 @@
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>Cleveland, OH</t>
+          <t>Chicago, IL</t>
         </is>
       </c>
       <c r="E293" t="inlineStr">
@@ -9723,12 +9723,12 @@
     <row r="294">
       <c r="A294" s="1" t="inlineStr">
         <is>
-          <t>CMH</t>
+          <t>CLE</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>Columbus, OH, United States</t>
+          <t>Cleveland, OH, United States</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
@@ -9738,7 +9738,7 @@
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>Columbus, OH</t>
+          <t>Cleveland, OH</t>
         </is>
       </c>
       <c r="E294" t="inlineStr">
@@ -9755,12 +9755,12 @@
     <row r="295">
       <c r="A295" s="1" t="inlineStr">
         <is>
-          <t>DFW</t>
+          <t>CMH</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>Dallas, TX, United States</t>
+          <t>Columbus, OH, United States</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -9770,7 +9770,7 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>Dallas, TX</t>
+          <t>Columbus, OH</t>
         </is>
       </c>
       <c r="E295" t="inlineStr">
@@ -9787,12 +9787,12 @@
     <row r="296">
       <c r="A296" s="1" t="inlineStr">
         <is>
-          <t>DEN</t>
+          <t>DFW</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>Denver, CO, United States</t>
+          <t>Dallas, TX, United States</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -9802,7 +9802,7 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>Denver, CO</t>
+          <t>Dallas, TX</t>
         </is>
       </c>
       <c r="E296" t="inlineStr">
@@ -9819,12 +9819,12 @@
     <row r="297">
       <c r="A297" s="1" t="inlineStr">
         <is>
-          <t>DTW</t>
+          <t>DEN</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>Detroit, MI, United States</t>
+          <t>Denver, CO, United States</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
@@ -9834,7 +9834,7 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>Detroit, MI</t>
+          <t>Denver, CO</t>
         </is>
       </c>
       <c r="E297" t="inlineStr">
@@ -9851,12 +9851,12 @@
     <row r="298">
       <c r="A298" s="1" t="inlineStr">
         <is>
-          <t>RDU</t>
+          <t>DTW</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>Durham, NC, United States</t>
+          <t>Detroit, MI, United States</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
@@ -9866,7 +9866,7 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>Durham, NC</t>
+          <t>Detroit, MI</t>
         </is>
       </c>
       <c r="E298" t="inlineStr">
@@ -9883,12 +9883,12 @@
     <row r="299">
       <c r="A299" s="1" t="inlineStr">
         <is>
-          <t>GDL</t>
+          <t>RDU</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>Guadalajara, Mexico</t>
+          <t>Durham, NC, United States</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
@@ -9898,29 +9898,29 @@
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>Guadalajara</t>
+          <t>Durham, NC</t>
         </is>
       </c>
       <c r="E299" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F299" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="300">
       <c r="A300" s="1" t="inlineStr">
         <is>
-          <t>YHZ</t>
+          <t>GDL</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>Halifax, Canada</t>
+          <t>Guadalajara, Mexico</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
@@ -9930,29 +9930,29 @@
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>Halifax</t>
+          <t>Guadalajara</t>
         </is>
       </c>
       <c r="E300" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F300" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>MX</t>
         </is>
       </c>
     </row>
     <row r="301">
       <c r="A301" s="1" t="inlineStr">
         <is>
-          <t>HNL</t>
+          <t>YHZ</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>Honolulu, HI, United States</t>
+          <t>Halifax, Canada</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
@@ -9962,29 +9962,29 @@
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>Honolulu, HI</t>
+          <t>Halifax</t>
         </is>
       </c>
       <c r="E301" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F301" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="302">
       <c r="A302" s="1" t="inlineStr">
         <is>
-          <t>IAH</t>
+          <t>HNL</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>Houston, TX, United States</t>
+          <t>Honolulu, HI, United States</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
@@ -9994,7 +9994,7 @@
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>Houston, TX</t>
+          <t>Honolulu, HI</t>
         </is>
       </c>
       <c r="E302" t="inlineStr">
@@ -10011,12 +10011,12 @@
     <row r="303">
       <c r="A303" s="1" t="inlineStr">
         <is>
-          <t>IND</t>
+          <t>IAH</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>Indianapolis, IN, United States</t>
+          <t>Houston, TX, United States</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
@@ -10026,7 +10026,7 @@
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>Indianapolis, IN</t>
+          <t>Houston, TX</t>
         </is>
       </c>
       <c r="E303" t="inlineStr">
@@ -10043,12 +10043,12 @@
     <row r="304">
       <c r="A304" s="1" t="inlineStr">
         <is>
-          <t>JAX</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>Jacksonville, FL, United States</t>
+          <t>Indianapolis, IN, United States</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
@@ -10058,7 +10058,7 @@
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>Jacksonville, FL</t>
+          <t>Indianapolis, IN</t>
         </is>
       </c>
       <c r="E304" t="inlineStr">
@@ -10075,12 +10075,12 @@
     <row r="305">
       <c r="A305" s="1" t="inlineStr">
         <is>
-          <t>MCI</t>
+          <t>JAX</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>Kansas City, MO, United States</t>
+          <t>Jacksonville, FL, United States</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
@@ -10090,7 +10090,7 @@
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>Kansas City, MO</t>
+          <t>Jacksonville, FL</t>
         </is>
       </c>
       <c r="E305" t="inlineStr">
@@ -10107,12 +10107,12 @@
     <row r="306">
       <c r="A306" s="1" t="inlineStr">
         <is>
-          <t>KIN</t>
+          <t>MCI</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>Kingston, Jamaica</t>
+          <t>Kansas City, MO, United States</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
@@ -10122,29 +10122,29 @@
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t>Kingston</t>
+          <t>Kansas City, MO</t>
         </is>
       </c>
       <c r="E306" t="inlineStr">
         <is>
-          <t>Jamaica</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F306" t="inlineStr">
         <is>
-          <t>JM</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="307">
       <c r="A307" s="1" t="inlineStr">
         <is>
-          <t>LAS</t>
+          <t>KIN</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>Las Vegas, NV, United States</t>
+          <t>Kingston, Jamaica</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
@@ -10154,29 +10154,29 @@
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>Las Vegas, NV</t>
+          <t>Kingston</t>
         </is>
       </c>
       <c r="E307" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Jamaica</t>
         </is>
       </c>
       <c r="F307" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>JM</t>
         </is>
       </c>
     </row>
     <row r="308">
       <c r="A308" s="1" t="inlineStr">
         <is>
-          <t>LAX</t>
+          <t>LAS</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>Los Angeles, CA, United States</t>
+          <t>Las Vegas, NV, United States</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
@@ -10186,7 +10186,7 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>Los Angeles, CA</t>
+          <t>Las Vegas, NV</t>
         </is>
       </c>
       <c r="E308" t="inlineStr">
@@ -10203,12 +10203,12 @@
     <row r="309">
       <c r="A309" s="1" t="inlineStr">
         <is>
-          <t>MEM</t>
+          <t>LAX</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>Memphis, TN, United States</t>
+          <t>Los Angeles, CA, United States</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
@@ -10218,7 +10218,7 @@
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>Memphis, TN</t>
+          <t>Los Angeles, CA</t>
         </is>
       </c>
       <c r="E309" t="inlineStr">
@@ -10235,12 +10235,12 @@
     <row r="310">
       <c r="A310" s="1" t="inlineStr">
         <is>
-          <t>MEX</t>
+          <t>MEM</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>Mexico City, Mexico</t>
+          <t>Memphis, TN, United States</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
@@ -10250,29 +10250,29 @@
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>Mexico City</t>
+          <t>Memphis, TN</t>
         </is>
       </c>
       <c r="E310" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F310" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="311">
       <c r="A311" s="1" t="inlineStr">
         <is>
-          <t>MIA</t>
+          <t>MEX</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Miami, FL, United States</t>
+          <t>Mexico City, Mexico</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
@@ -10282,29 +10282,29 @@
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>Miami, FL</t>
+          <t>Mexico City</t>
         </is>
       </c>
       <c r="E311" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F311" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
     </row>
     <row r="312">
       <c r="A312" s="1" t="inlineStr">
         <is>
-          <t>MSP</t>
+          <t>MIA</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>Minneapolis, MN, United States</t>
+          <t>Miami, FL, United States</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
@@ -10314,7 +10314,7 @@
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>Minneapolis, MN</t>
+          <t>Miami, FL</t>
         </is>
       </c>
       <c r="E312" t="inlineStr">
@@ -10331,12 +10331,12 @@
     <row r="313">
       <c r="A313" s="1" t="inlineStr">
         <is>
-          <t>YUL</t>
+          <t>MSP</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Montréal, QC, Canada</t>
+          <t>Minneapolis, MN, United States</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
@@ -10346,29 +10346,29 @@
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>Montréal, QC</t>
+          <t>Minneapolis, MN</t>
         </is>
       </c>
       <c r="E313" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F313" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="314">
       <c r="A314" s="1" t="inlineStr">
         <is>
-          <t>BNA</t>
+          <t>YUL</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Nashville, United States</t>
+          <t>Montréal, QC, Canada</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -10378,29 +10378,29 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>Nashville</t>
+          <t>Montréal, QC</t>
         </is>
       </c>
       <c r="E314" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F314" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="315">
       <c r="A315" s="1" t="inlineStr">
         <is>
-          <t>EWR</t>
+          <t>BNA</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>Newark, NJ, United States</t>
+          <t>Nashville, United States</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
@@ -10410,7 +10410,7 @@
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>Newark, NJ</t>
+          <t>Nashville</t>
         </is>
       </c>
       <c r="E315" t="inlineStr">
@@ -10427,12 +10427,12 @@
     <row r="316">
       <c r="A316" s="1" t="inlineStr">
         <is>
-          <t>ORF</t>
+          <t>EWR</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Norfolk, VA, United States</t>
+          <t>Newark, NJ, United States</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
@@ -10442,7 +10442,7 @@
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>Norfolk, VA</t>
+          <t>Newark, NJ</t>
         </is>
       </c>
       <c r="E316" t="inlineStr">
@@ -10459,12 +10459,12 @@
     <row r="317">
       <c r="A317" s="1" t="inlineStr">
         <is>
-          <t>OKC</t>
+          <t>ORF</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Oklahoma City, OK, United States</t>
+          <t>Norfolk, VA, United States</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -10474,7 +10474,7 @@
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t>Oklahoma City, OK</t>
+          <t>Norfolk, VA</t>
         </is>
       </c>
       <c r="E317" t="inlineStr">
@@ -10491,12 +10491,12 @@
     <row r="318">
       <c r="A318" s="1" t="inlineStr">
         <is>
-          <t>OMA</t>
+          <t>OKC</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>Omaha, NE, United States</t>
+          <t>Oklahoma City, OK, United States</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
@@ -10506,7 +10506,7 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>Omaha, NE</t>
+          <t>Oklahoma City, OK</t>
         </is>
       </c>
       <c r="E318" t="inlineStr">
@@ -10523,12 +10523,12 @@
     <row r="319">
       <c r="A319" s="1" t="inlineStr">
         <is>
-          <t>PHL</t>
+          <t>OMA</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Philadelphia, United States</t>
+          <t>Omaha, NE, United States</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
@@ -10538,7 +10538,7 @@
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>Philadelphia</t>
+          <t>Omaha, NE</t>
         </is>
       </c>
       <c r="E319" t="inlineStr">
@@ -10555,12 +10555,12 @@
     <row r="320">
       <c r="A320" s="1" t="inlineStr">
         <is>
-          <t>PHX</t>
+          <t>PHL</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Phoenix, AZ, United States</t>
+          <t>Philadelphia, United States</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -10570,7 +10570,7 @@
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t>Phoenix, AZ</t>
+          <t>Philadelphia</t>
         </is>
       </c>
       <c r="E320" t="inlineStr">
@@ -10587,12 +10587,12 @@
     <row r="321">
       <c r="A321" s="1" t="inlineStr">
         <is>
-          <t>PIT</t>
+          <t>PHX</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>Pittsburgh, PA, United States</t>
+          <t>Phoenix, AZ, United States</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
@@ -10602,7 +10602,7 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>Pittsburgh, PA</t>
+          <t>Phoenix, AZ</t>
         </is>
       </c>
       <c r="E321" t="inlineStr">
@@ -10619,12 +10619,12 @@
     <row r="322">
       <c r="A322" s="1" t="inlineStr">
         <is>
-          <t>PDX</t>
+          <t>PIT</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>Portland, OR, United States</t>
+          <t>Pittsburgh, PA, United States</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
@@ -10634,7 +10634,7 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>Portland, OR</t>
+          <t>Pittsburgh, PA</t>
         </is>
       </c>
       <c r="E322" t="inlineStr">
@@ -10651,12 +10651,12 @@
     <row r="323">
       <c r="A323" s="1" t="inlineStr">
         <is>
-          <t>QRO</t>
+          <t>PDX</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>Queretaro, MX, Mexico</t>
+          <t>Portland, OR, United States</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -10666,29 +10666,29 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>Queretaro, MX</t>
+          <t>Portland, OR</t>
         </is>
       </c>
       <c r="E323" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F323" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="324">
       <c r="A324" s="1" t="inlineStr">
         <is>
-          <t>RIC</t>
+          <t>QRO</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>Richmond, VA, United States</t>
+          <t>Queretaro, MX, Mexico</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -10698,29 +10698,29 @@
       </c>
       <c r="D324" t="inlineStr">
         <is>
-          <t>Richmond, VA</t>
+          <t>Queretaro, MX</t>
         </is>
       </c>
       <c r="E324" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F324" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
     </row>
     <row r="325">
       <c r="A325" s="1" t="inlineStr">
         <is>
-          <t>SMF</t>
+          <t>RIC</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>Sacramento, CA, United States</t>
+          <t>Richmond, VA, United States</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -10730,7 +10730,7 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>Sacramento, CA</t>
+          <t>Richmond, VA</t>
         </is>
       </c>
       <c r="E325" t="inlineStr">
@@ -10747,12 +10747,12 @@
     <row r="326">
       <c r="A326" s="1" t="inlineStr">
         <is>
-          <t>SLC</t>
+          <t>SMF</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>Salt Lake City, UT, United States</t>
+          <t>Sacramento, CA, United States</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
@@ -10762,7 +10762,7 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>Salt Lake City, UT</t>
+          <t>Sacramento, CA</t>
         </is>
       </c>
       <c r="E326" t="inlineStr">
@@ -10779,12 +10779,12 @@
     <row r="327">
       <c r="A327" s="1" t="inlineStr">
         <is>
-          <t>SAT</t>
+          <t>SLC</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>San Antonio, TX, United States</t>
+          <t>Salt Lake City, UT, United States</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
@@ -10794,7 +10794,7 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>San Antonio, TX</t>
+          <t>Salt Lake City, UT</t>
         </is>
       </c>
       <c r="E327" t="inlineStr">
@@ -10811,12 +10811,12 @@
     <row r="328">
       <c r="A328" s="1" t="inlineStr">
         <is>
-          <t>SAN</t>
+          <t>SAT</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>San Diego, CA, United States</t>
+          <t>San Antonio, TX, United States</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
@@ -10826,7 +10826,7 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>San Diego, CA</t>
+          <t>San Antonio, TX</t>
         </is>
       </c>
       <c r="E328" t="inlineStr">
@@ -10843,12 +10843,12 @@
     <row r="329">
       <c r="A329" s="1" t="inlineStr">
         <is>
-          <t>SFO</t>
+          <t>SAN</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>San Francisco, CA, United States</t>
+          <t>San Diego, CA, United States</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
@@ -10858,7 +10858,7 @@
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>San Francisco, CA</t>
+          <t>San Diego, CA</t>
         </is>
       </c>
       <c r="E329" t="inlineStr">
@@ -10875,12 +10875,12 @@
     <row r="330">
       <c r="A330" s="1" t="inlineStr">
         <is>
-          <t>SJC</t>
+          <t>SFO</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>San Jose, CA, United States</t>
+          <t>San Francisco, CA, United States</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
@@ -10890,7 +10890,7 @@
       </c>
       <c r="D330" t="inlineStr">
         <is>
-          <t>San Jose, CA</t>
+          <t>San Francisco, CA</t>
         </is>
       </c>
       <c r="E330" t="inlineStr">
@@ -10907,12 +10907,12 @@
     <row r="331">
       <c r="A331" s="1" t="inlineStr">
         <is>
-          <t>YXE</t>
+          <t>SJC</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>Saskatoon, SK, Canada</t>
+          <t>San Jose, CA, United States</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
@@ -10922,29 +10922,29 @@
       </c>
       <c r="D331" t="inlineStr">
         <is>
-          <t>Saskatoon, SK</t>
+          <t>San Jose, CA</t>
         </is>
       </c>
       <c r="E331" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F331" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="332">
       <c r="A332" s="1" t="inlineStr">
         <is>
-          <t>SEA</t>
+          <t>YXE</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>Seattle, WA, United States</t>
+          <t>Saskatoon, SK, Canada</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
@@ -10954,29 +10954,29 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>Seattle, WA</t>
+          <t>Saskatoon, SK</t>
         </is>
       </c>
       <c r="E332" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F332" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="333">
       <c r="A333" s="1" t="inlineStr">
         <is>
-          <t>FSD</t>
+          <t>SEA</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>Sioux Falls, SD, United States</t>
+          <t>Seattle, WA, United States</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
@@ -10986,7 +10986,7 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>Sioux Falls, SD</t>
+          <t>Seattle, WA</t>
         </is>
       </c>
       <c r="E333" t="inlineStr">
@@ -11003,12 +11003,12 @@
     <row r="334">
       <c r="A334" s="1" t="inlineStr">
         <is>
-          <t>STL</t>
+          <t>FSD</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>St. Louis, MO, United States</t>
+          <t>Sioux Falls, SD, United States</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
@@ -11018,7 +11018,7 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>St. Louis, MO</t>
+          <t>Sioux Falls, SD</t>
         </is>
       </c>
       <c r="E334" t="inlineStr">
@@ -11035,12 +11035,12 @@
     <row r="335">
       <c r="A335" s="1" t="inlineStr">
         <is>
-          <t>TLH</t>
+          <t>STL</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>Tallahassee, FL, United States</t>
+          <t>St. Louis, MO, United States</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
@@ -11050,7 +11050,7 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>Tallahassee, FL</t>
+          <t>St. Louis, MO</t>
         </is>
       </c>
       <c r="E335" t="inlineStr">
@@ -11067,12 +11067,12 @@
     <row r="336">
       <c r="A336" s="1" t="inlineStr">
         <is>
-          <t>TPA</t>
+          <t>TLH</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>Tampa, FL, United States</t>
+          <t>Tallahassee, FL, United States</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
@@ -11082,7 +11082,7 @@
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>Tampa, FL</t>
+          <t>Tallahassee, FL</t>
         </is>
       </c>
       <c r="E336" t="inlineStr">
@@ -11099,12 +11099,12 @@
     <row r="337">
       <c r="A337" s="1" t="inlineStr">
         <is>
-          <t>YYZ</t>
+          <t>TPA</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>Toronto, ON, Canada</t>
+          <t>Tampa, FL, United States</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
@@ -11114,29 +11114,29 @@
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>Toronto, ON</t>
+          <t>Tampa, FL</t>
         </is>
       </c>
       <c r="E337" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F337" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="338">
       <c r="A338" s="1" t="inlineStr">
         <is>
-          <t>YVR</t>
+          <t>YYZ</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>Vancouver, BC, Canada</t>
+          <t>Toronto, ON, Canada</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
@@ -11146,7 +11146,7 @@
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Toronto, ON</t>
         </is>
       </c>
       <c r="E338" t="inlineStr">
@@ -11163,12 +11163,12 @@
     <row r="339">
       <c r="A339" s="1" t="inlineStr">
         <is>
-          <t>YWG</t>
+          <t>YVR</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>Winnipeg, MB, Canada</t>
+          <t>Vancouver, BC, Canada</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
@@ -11178,7 +11178,7 @@
       </c>
       <c r="D339" t="inlineStr">
         <is>
-          <t>Winnipeg, MB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="E339" t="inlineStr">
@@ -11195,30 +11195,62 @@
     <row r="340">
       <c r="A340" s="1" t="inlineStr">
         <is>
+          <t>YWG</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>Winnipeg, MB, Canada</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>North America</t>
+        </is>
+      </c>
+      <c r="D340" t="inlineStr">
+        <is>
+          <t>Winnipeg, MB</t>
+        </is>
+      </c>
+      <c r="E340" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="F340" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" s="1" t="inlineStr">
+        <is>
           <t>CVG</t>
         </is>
       </c>
-      <c r="B340" t="inlineStr">
+      <c r="B341" t="inlineStr">
         <is>
           <t>Cincinnati, United States</t>
         </is>
       </c>
-      <c r="C340" t="inlineStr">
+      <c r="C341" t="inlineStr">
         <is>
           <t>North America</t>
         </is>
       </c>
-      <c r="D340" t="inlineStr">
+      <c r="D341" t="inlineStr">
         <is>
           <t>Cincinnati</t>
         </is>
       </c>
-      <c r="E340" t="inlineStr">
+      <c r="E341" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="F340" t="inlineStr">
+      <c r="F341" t="inlineStr">
         <is>
           <t>US</t>
         </is>

</xml_diff>

<commit_message>
update generated data Triggered by e42fc9043755c7c00dc9aa7ceb64afd1ab67614d
</commit_message>
<xml_diff>
--- a/DC-Colos.xlsx
+++ b/DC-Colos.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F341"/>
+  <dimension ref="A1:F342"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9371,44 +9371,44 @@
     <row r="283">
       <c r="A283" s="1" t="inlineStr">
         <is>
-          <t>ABQ</t>
+          <t>LHW</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>Albuquerque, NM, United States</t>
+          <t>Lanzhou, China</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>North America</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>Albuquerque, NM</t>
+          <t>Lanzhou</t>
         </is>
       </c>
       <c r="E283" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F283" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="284">
       <c r="A284" s="1" t="inlineStr">
         <is>
-          <t>ANC</t>
+          <t>ABQ</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>Anchorage, AK, United States</t>
+          <t>Albuquerque, NM, United States</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
@@ -9418,7 +9418,7 @@
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>Anchorage, AK</t>
+          <t>Albuquerque, NM</t>
         </is>
       </c>
       <c r="E284" t="inlineStr">
@@ -9435,12 +9435,12 @@
     <row r="285">
       <c r="A285" s="1" t="inlineStr">
         <is>
-          <t>IAD</t>
+          <t>ANC</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>Ashburn, VA, United States</t>
+          <t>Anchorage, AK, United States</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
@@ -9450,7 +9450,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>Ashburn, VA</t>
+          <t>Anchorage, AK</t>
         </is>
       </c>
       <c r="E285" t="inlineStr">
@@ -9467,12 +9467,12 @@
     <row r="286">
       <c r="A286" s="1" t="inlineStr">
         <is>
-          <t>ATL</t>
+          <t>IAD</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>Atlanta, GA, United States</t>
+          <t>Ashburn, VA, United States</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
@@ -9482,7 +9482,7 @@
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>Atlanta, GA</t>
+          <t>Ashburn, VA</t>
         </is>
       </c>
       <c r="E286" t="inlineStr">
@@ -9499,12 +9499,12 @@
     <row r="287">
       <c r="A287" s="1" t="inlineStr">
         <is>
-          <t>AUS</t>
+          <t>ATL</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>Austin, TX, United States</t>
+          <t>Atlanta, GA, United States</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
@@ -9514,7 +9514,7 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>Austin, TX</t>
+          <t>Atlanta, GA</t>
         </is>
       </c>
       <c r="E287" t="inlineStr">
@@ -9531,12 +9531,12 @@
     <row r="288">
       <c r="A288" s="1" t="inlineStr">
         <is>
-          <t>BGR</t>
+          <t>AUS</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>Bangor, ME, United States</t>
+          <t>Austin, TX, United States</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
@@ -9546,7 +9546,7 @@
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>Bangor, ME</t>
+          <t>Austin, TX</t>
         </is>
       </c>
       <c r="E288" t="inlineStr">
@@ -9563,12 +9563,12 @@
     <row r="289">
       <c r="A289" s="1" t="inlineStr">
         <is>
-          <t>BOS</t>
+          <t>BGR</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>Boston, MA, United States</t>
+          <t>Bangor, ME, United States</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
@@ -9578,7 +9578,7 @@
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>Boston, MA</t>
+          <t>Bangor, ME</t>
         </is>
       </c>
       <c r="E289" t="inlineStr">
@@ -9595,12 +9595,12 @@
     <row r="290">
       <c r="A290" s="1" t="inlineStr">
         <is>
-          <t>BUF</t>
+          <t>BOS</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>Buffalo, NY, United States</t>
+          <t>Boston, MA, United States</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
@@ -9610,7 +9610,7 @@
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>Buffalo, NY</t>
+          <t>Boston, MA</t>
         </is>
       </c>
       <c r="E290" t="inlineStr">
@@ -9627,12 +9627,12 @@
     <row r="291">
       <c r="A291" s="1" t="inlineStr">
         <is>
-          <t>YYC</t>
+          <t>BUF</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>Calgary, AB, Canada</t>
+          <t>Buffalo, NY, United States</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
@@ -9642,29 +9642,29 @@
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Buffalo, NY</t>
         </is>
       </c>
       <c r="E291" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F291" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="292">
       <c r="A292" s="1" t="inlineStr">
         <is>
-          <t>CLT</t>
+          <t>YYC</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>Charlotte, NC, United States</t>
+          <t>Calgary, AB, Canada</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
@@ -9674,29 +9674,29 @@
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>Charlotte, NC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="E292" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F292" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="293">
       <c r="A293" s="1" t="inlineStr">
         <is>
-          <t>ORD</t>
+          <t>CLT</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>Chicago, IL, United States</t>
+          <t>Charlotte, NC, United States</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
@@ -9706,7 +9706,7 @@
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>Chicago, IL</t>
+          <t>Charlotte, NC</t>
         </is>
       </c>
       <c r="E293" t="inlineStr">
@@ -9723,12 +9723,12 @@
     <row r="294">
       <c r="A294" s="1" t="inlineStr">
         <is>
-          <t>CLE</t>
+          <t>ORD</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>Cleveland, OH, United States</t>
+          <t>Chicago, IL, United States</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
@@ -9738,7 +9738,7 @@
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>Cleveland, OH</t>
+          <t>Chicago, IL</t>
         </is>
       </c>
       <c r="E294" t="inlineStr">
@@ -9755,12 +9755,12 @@
     <row r="295">
       <c r="A295" s="1" t="inlineStr">
         <is>
-          <t>CMH</t>
+          <t>CLE</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>Columbus, OH, United States</t>
+          <t>Cleveland, OH, United States</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -9770,7 +9770,7 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>Columbus, OH</t>
+          <t>Cleveland, OH</t>
         </is>
       </c>
       <c r="E295" t="inlineStr">
@@ -9787,12 +9787,12 @@
     <row r="296">
       <c r="A296" s="1" t="inlineStr">
         <is>
-          <t>DFW</t>
+          <t>CMH</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>Dallas, TX, United States</t>
+          <t>Columbus, OH, United States</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -9802,7 +9802,7 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>Dallas, TX</t>
+          <t>Columbus, OH</t>
         </is>
       </c>
       <c r="E296" t="inlineStr">
@@ -9819,12 +9819,12 @@
     <row r="297">
       <c r="A297" s="1" t="inlineStr">
         <is>
-          <t>DEN</t>
+          <t>DFW</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>Denver, CO, United States</t>
+          <t>Dallas, TX, United States</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
@@ -9834,7 +9834,7 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>Denver, CO</t>
+          <t>Dallas, TX</t>
         </is>
       </c>
       <c r="E297" t="inlineStr">
@@ -9851,12 +9851,12 @@
     <row r="298">
       <c r="A298" s="1" t="inlineStr">
         <is>
-          <t>DTW</t>
+          <t>DEN</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>Detroit, MI, United States</t>
+          <t>Denver, CO, United States</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
@@ -9866,7 +9866,7 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>Detroit, MI</t>
+          <t>Denver, CO</t>
         </is>
       </c>
       <c r="E298" t="inlineStr">
@@ -9883,12 +9883,12 @@
     <row r="299">
       <c r="A299" s="1" t="inlineStr">
         <is>
-          <t>RDU</t>
+          <t>DTW</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>Durham, NC, United States</t>
+          <t>Detroit, MI, United States</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
@@ -9898,7 +9898,7 @@
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>Durham, NC</t>
+          <t>Detroit, MI</t>
         </is>
       </c>
       <c r="E299" t="inlineStr">
@@ -9915,12 +9915,12 @@
     <row r="300">
       <c r="A300" s="1" t="inlineStr">
         <is>
-          <t>GDL</t>
+          <t>RDU</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>Guadalajara, Mexico</t>
+          <t>Durham, NC, United States</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
@@ -9930,29 +9930,29 @@
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>Guadalajara</t>
+          <t>Durham, NC</t>
         </is>
       </c>
       <c r="E300" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F300" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="301">
       <c r="A301" s="1" t="inlineStr">
         <is>
-          <t>YHZ</t>
+          <t>GDL</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>Halifax, Canada</t>
+          <t>Guadalajara, Mexico</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
@@ -9962,29 +9962,29 @@
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>Halifax</t>
+          <t>Guadalajara</t>
         </is>
       </c>
       <c r="E301" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F301" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>MX</t>
         </is>
       </c>
     </row>
     <row r="302">
       <c r="A302" s="1" t="inlineStr">
         <is>
-          <t>HNL</t>
+          <t>YHZ</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>Honolulu, HI, United States</t>
+          <t>Halifax, Canada</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
@@ -9994,29 +9994,29 @@
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>Honolulu, HI</t>
+          <t>Halifax</t>
         </is>
       </c>
       <c r="E302" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F302" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="303">
       <c r="A303" s="1" t="inlineStr">
         <is>
-          <t>IAH</t>
+          <t>HNL</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>Houston, TX, United States</t>
+          <t>Honolulu, HI, United States</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
@@ -10026,7 +10026,7 @@
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>Houston, TX</t>
+          <t>Honolulu, HI</t>
         </is>
       </c>
       <c r="E303" t="inlineStr">
@@ -10043,12 +10043,12 @@
     <row r="304">
       <c r="A304" s="1" t="inlineStr">
         <is>
-          <t>IND</t>
+          <t>IAH</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>Indianapolis, IN, United States</t>
+          <t>Houston, TX, United States</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
@@ -10058,7 +10058,7 @@
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>Indianapolis, IN</t>
+          <t>Houston, TX</t>
         </is>
       </c>
       <c r="E304" t="inlineStr">
@@ -10075,12 +10075,12 @@
     <row r="305">
       <c r="A305" s="1" t="inlineStr">
         <is>
-          <t>JAX</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>Jacksonville, FL, United States</t>
+          <t>Indianapolis, IN, United States</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
@@ -10090,7 +10090,7 @@
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>Jacksonville, FL</t>
+          <t>Indianapolis, IN</t>
         </is>
       </c>
       <c r="E305" t="inlineStr">
@@ -10107,12 +10107,12 @@
     <row r="306">
       <c r="A306" s="1" t="inlineStr">
         <is>
-          <t>MCI</t>
+          <t>JAX</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>Kansas City, MO, United States</t>
+          <t>Jacksonville, FL, United States</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
@@ -10122,7 +10122,7 @@
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t>Kansas City, MO</t>
+          <t>Jacksonville, FL</t>
         </is>
       </c>
       <c r="E306" t="inlineStr">
@@ -10139,12 +10139,12 @@
     <row r="307">
       <c r="A307" s="1" t="inlineStr">
         <is>
-          <t>KIN</t>
+          <t>MCI</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>Kingston, Jamaica</t>
+          <t>Kansas City, MO, United States</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
@@ -10154,29 +10154,29 @@
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>Kingston</t>
+          <t>Kansas City, MO</t>
         </is>
       </c>
       <c r="E307" t="inlineStr">
         <is>
-          <t>Jamaica</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F307" t="inlineStr">
         <is>
-          <t>JM</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="308">
       <c r="A308" s="1" t="inlineStr">
         <is>
-          <t>LAS</t>
+          <t>KIN</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>Las Vegas, NV, United States</t>
+          <t>Kingston, Jamaica</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
@@ -10186,29 +10186,29 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>Las Vegas, NV</t>
+          <t>Kingston</t>
         </is>
       </c>
       <c r="E308" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Jamaica</t>
         </is>
       </c>
       <c r="F308" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>JM</t>
         </is>
       </c>
     </row>
     <row r="309">
       <c r="A309" s="1" t="inlineStr">
         <is>
-          <t>LAX</t>
+          <t>LAS</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>Los Angeles, CA, United States</t>
+          <t>Las Vegas, NV, United States</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
@@ -10218,7 +10218,7 @@
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>Los Angeles, CA</t>
+          <t>Las Vegas, NV</t>
         </is>
       </c>
       <c r="E309" t="inlineStr">
@@ -10235,12 +10235,12 @@
     <row r="310">
       <c r="A310" s="1" t="inlineStr">
         <is>
-          <t>MEM</t>
+          <t>LAX</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>Memphis, TN, United States</t>
+          <t>Los Angeles, CA, United States</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
@@ -10250,7 +10250,7 @@
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>Memphis, TN</t>
+          <t>Los Angeles, CA</t>
         </is>
       </c>
       <c r="E310" t="inlineStr">
@@ -10267,12 +10267,12 @@
     <row r="311">
       <c r="A311" s="1" t="inlineStr">
         <is>
-          <t>MEX</t>
+          <t>MEM</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Mexico City, Mexico</t>
+          <t>Memphis, TN, United States</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
@@ -10282,29 +10282,29 @@
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>Mexico City</t>
+          <t>Memphis, TN</t>
         </is>
       </c>
       <c r="E311" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F311" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="312">
       <c r="A312" s="1" t="inlineStr">
         <is>
-          <t>MIA</t>
+          <t>MEX</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>Miami, FL, United States</t>
+          <t>Mexico City, Mexico</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
@@ -10314,29 +10314,29 @@
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>Miami, FL</t>
+          <t>Mexico City</t>
         </is>
       </c>
       <c r="E312" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F312" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
     </row>
     <row r="313">
       <c r="A313" s="1" t="inlineStr">
         <is>
-          <t>MSP</t>
+          <t>MIA</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Minneapolis, MN, United States</t>
+          <t>Miami, FL, United States</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
@@ -10346,7 +10346,7 @@
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>Minneapolis, MN</t>
+          <t>Miami, FL</t>
         </is>
       </c>
       <c r="E313" t="inlineStr">
@@ -10363,12 +10363,12 @@
     <row r="314">
       <c r="A314" s="1" t="inlineStr">
         <is>
-          <t>YUL</t>
+          <t>MSP</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Montréal, QC, Canada</t>
+          <t>Minneapolis, MN, United States</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -10378,29 +10378,29 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>Montréal, QC</t>
+          <t>Minneapolis, MN</t>
         </is>
       </c>
       <c r="E314" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F314" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="315">
       <c r="A315" s="1" t="inlineStr">
         <is>
-          <t>BNA</t>
+          <t>YUL</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>Nashville, United States</t>
+          <t>Montréal, QC, Canada</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
@@ -10410,29 +10410,29 @@
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>Nashville</t>
+          <t>Montréal, QC</t>
         </is>
       </c>
       <c r="E315" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F315" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="316">
       <c r="A316" s="1" t="inlineStr">
         <is>
-          <t>EWR</t>
+          <t>BNA</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Newark, NJ, United States</t>
+          <t>Nashville, United States</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
@@ -10442,7 +10442,7 @@
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>Newark, NJ</t>
+          <t>Nashville</t>
         </is>
       </c>
       <c r="E316" t="inlineStr">
@@ -10459,12 +10459,12 @@
     <row r="317">
       <c r="A317" s="1" t="inlineStr">
         <is>
-          <t>ORF</t>
+          <t>EWR</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Norfolk, VA, United States</t>
+          <t>Newark, NJ, United States</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -10474,7 +10474,7 @@
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t>Norfolk, VA</t>
+          <t>Newark, NJ</t>
         </is>
       </c>
       <c r="E317" t="inlineStr">
@@ -10491,12 +10491,12 @@
     <row r="318">
       <c r="A318" s="1" t="inlineStr">
         <is>
-          <t>OKC</t>
+          <t>ORF</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>Oklahoma City, OK, United States</t>
+          <t>Norfolk, VA, United States</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
@@ -10506,7 +10506,7 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>Oklahoma City, OK</t>
+          <t>Norfolk, VA</t>
         </is>
       </c>
       <c r="E318" t="inlineStr">
@@ -10523,12 +10523,12 @@
     <row r="319">
       <c r="A319" s="1" t="inlineStr">
         <is>
-          <t>OMA</t>
+          <t>OKC</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Omaha, NE, United States</t>
+          <t>Oklahoma City, OK, United States</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
@@ -10538,7 +10538,7 @@
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>Omaha, NE</t>
+          <t>Oklahoma City, OK</t>
         </is>
       </c>
       <c r="E319" t="inlineStr">
@@ -10555,12 +10555,12 @@
     <row r="320">
       <c r="A320" s="1" t="inlineStr">
         <is>
-          <t>PHL</t>
+          <t>OMA</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Philadelphia, United States</t>
+          <t>Omaha, NE, United States</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -10570,7 +10570,7 @@
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t>Philadelphia</t>
+          <t>Omaha, NE</t>
         </is>
       </c>
       <c r="E320" t="inlineStr">
@@ -10587,12 +10587,12 @@
     <row r="321">
       <c r="A321" s="1" t="inlineStr">
         <is>
-          <t>PHX</t>
+          <t>PHL</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>Phoenix, AZ, United States</t>
+          <t>Philadelphia, United States</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
@@ -10602,7 +10602,7 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>Phoenix, AZ</t>
+          <t>Philadelphia</t>
         </is>
       </c>
       <c r="E321" t="inlineStr">
@@ -10619,12 +10619,12 @@
     <row r="322">
       <c r="A322" s="1" t="inlineStr">
         <is>
-          <t>PIT</t>
+          <t>PHX</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>Pittsburgh, PA, United States</t>
+          <t>Phoenix, AZ, United States</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
@@ -10634,7 +10634,7 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>Pittsburgh, PA</t>
+          <t>Phoenix, AZ</t>
         </is>
       </c>
       <c r="E322" t="inlineStr">
@@ -10651,12 +10651,12 @@
     <row r="323">
       <c r="A323" s="1" t="inlineStr">
         <is>
-          <t>PDX</t>
+          <t>PIT</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>Portland, OR, United States</t>
+          <t>Pittsburgh, PA, United States</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -10666,7 +10666,7 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>Portland, OR</t>
+          <t>Pittsburgh, PA</t>
         </is>
       </c>
       <c r="E323" t="inlineStr">
@@ -10683,12 +10683,12 @@
     <row r="324">
       <c r="A324" s="1" t="inlineStr">
         <is>
-          <t>QRO</t>
+          <t>PDX</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>Queretaro, MX, Mexico</t>
+          <t>Portland, OR, United States</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -10698,29 +10698,29 @@
       </c>
       <c r="D324" t="inlineStr">
         <is>
-          <t>Queretaro, MX</t>
+          <t>Portland, OR</t>
         </is>
       </c>
       <c r="E324" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F324" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="325">
       <c r="A325" s="1" t="inlineStr">
         <is>
-          <t>RIC</t>
+          <t>QRO</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>Richmond, VA, United States</t>
+          <t>Queretaro, MX, Mexico</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -10730,29 +10730,29 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>Richmond, VA</t>
+          <t>Queretaro, MX</t>
         </is>
       </c>
       <c r="E325" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F325" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
     </row>
     <row r="326">
       <c r="A326" s="1" t="inlineStr">
         <is>
-          <t>SMF</t>
+          <t>RIC</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>Sacramento, CA, United States</t>
+          <t>Richmond, VA, United States</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
@@ -10762,7 +10762,7 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>Sacramento, CA</t>
+          <t>Richmond, VA</t>
         </is>
       </c>
       <c r="E326" t="inlineStr">
@@ -10779,12 +10779,12 @@
     <row r="327">
       <c r="A327" s="1" t="inlineStr">
         <is>
-          <t>SLC</t>
+          <t>SMF</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>Salt Lake City, UT, United States</t>
+          <t>Sacramento, CA, United States</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
@@ -10794,7 +10794,7 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>Salt Lake City, UT</t>
+          <t>Sacramento, CA</t>
         </is>
       </c>
       <c r="E327" t="inlineStr">
@@ -10811,12 +10811,12 @@
     <row r="328">
       <c r="A328" s="1" t="inlineStr">
         <is>
-          <t>SAT</t>
+          <t>SLC</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>San Antonio, TX, United States</t>
+          <t>Salt Lake City, UT, United States</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
@@ -10826,7 +10826,7 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>San Antonio, TX</t>
+          <t>Salt Lake City, UT</t>
         </is>
       </c>
       <c r="E328" t="inlineStr">
@@ -10843,12 +10843,12 @@
     <row r="329">
       <c r="A329" s="1" t="inlineStr">
         <is>
-          <t>SAN</t>
+          <t>SAT</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>San Diego, CA, United States</t>
+          <t>San Antonio, TX, United States</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
@@ -10858,7 +10858,7 @@
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>San Diego, CA</t>
+          <t>San Antonio, TX</t>
         </is>
       </c>
       <c r="E329" t="inlineStr">
@@ -10875,12 +10875,12 @@
     <row r="330">
       <c r="A330" s="1" t="inlineStr">
         <is>
-          <t>SFO</t>
+          <t>SAN</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>San Francisco, CA, United States</t>
+          <t>San Diego, CA, United States</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
@@ -10890,7 +10890,7 @@
       </c>
       <c r="D330" t="inlineStr">
         <is>
-          <t>San Francisco, CA</t>
+          <t>San Diego, CA</t>
         </is>
       </c>
       <c r="E330" t="inlineStr">
@@ -10907,12 +10907,12 @@
     <row r="331">
       <c r="A331" s="1" t="inlineStr">
         <is>
-          <t>SJC</t>
+          <t>SFO</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>San Jose, CA, United States</t>
+          <t>San Francisco, CA, United States</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
@@ -10922,7 +10922,7 @@
       </c>
       <c r="D331" t="inlineStr">
         <is>
-          <t>San Jose, CA</t>
+          <t>San Francisco, CA</t>
         </is>
       </c>
       <c r="E331" t="inlineStr">
@@ -10939,12 +10939,12 @@
     <row r="332">
       <c r="A332" s="1" t="inlineStr">
         <is>
-          <t>YXE</t>
+          <t>SJC</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>Saskatoon, SK, Canada</t>
+          <t>San Jose, CA, United States</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
@@ -10954,29 +10954,29 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>Saskatoon, SK</t>
+          <t>San Jose, CA</t>
         </is>
       </c>
       <c r="E332" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F332" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="333">
       <c r="A333" s="1" t="inlineStr">
         <is>
-          <t>SEA</t>
+          <t>YXE</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>Seattle, WA, United States</t>
+          <t>Saskatoon, SK, Canada</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
@@ -10986,29 +10986,29 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>Seattle, WA</t>
+          <t>Saskatoon, SK</t>
         </is>
       </c>
       <c r="E333" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F333" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="334">
       <c r="A334" s="1" t="inlineStr">
         <is>
-          <t>FSD</t>
+          <t>SEA</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>Sioux Falls, SD, United States</t>
+          <t>Seattle, WA, United States</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
@@ -11018,7 +11018,7 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>Sioux Falls, SD</t>
+          <t>Seattle, WA</t>
         </is>
       </c>
       <c r="E334" t="inlineStr">
@@ -11035,12 +11035,12 @@
     <row r="335">
       <c r="A335" s="1" t="inlineStr">
         <is>
-          <t>STL</t>
+          <t>FSD</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>St. Louis, MO, United States</t>
+          <t>Sioux Falls, SD, United States</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
@@ -11050,7 +11050,7 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>St. Louis, MO</t>
+          <t>Sioux Falls, SD</t>
         </is>
       </c>
       <c r="E335" t="inlineStr">
@@ -11067,12 +11067,12 @@
     <row r="336">
       <c r="A336" s="1" t="inlineStr">
         <is>
-          <t>TLH</t>
+          <t>STL</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>Tallahassee, FL, United States</t>
+          <t>St. Louis, MO, United States</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
@@ -11082,7 +11082,7 @@
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>Tallahassee, FL</t>
+          <t>St. Louis, MO</t>
         </is>
       </c>
       <c r="E336" t="inlineStr">
@@ -11099,12 +11099,12 @@
     <row r="337">
       <c r="A337" s="1" t="inlineStr">
         <is>
-          <t>TPA</t>
+          <t>TLH</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>Tampa, FL, United States</t>
+          <t>Tallahassee, FL, United States</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
@@ -11114,7 +11114,7 @@
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>Tampa, FL</t>
+          <t>Tallahassee, FL</t>
         </is>
       </c>
       <c r="E337" t="inlineStr">
@@ -11131,12 +11131,12 @@
     <row r="338">
       <c r="A338" s="1" t="inlineStr">
         <is>
-          <t>YYZ</t>
+          <t>TPA</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>Toronto, ON, Canada</t>
+          <t>Tampa, FL, United States</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
@@ -11146,29 +11146,29 @@
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>Toronto, ON</t>
+          <t>Tampa, FL</t>
         </is>
       </c>
       <c r="E338" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F338" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="339">
       <c r="A339" s="1" t="inlineStr">
         <is>
-          <t>YVR</t>
+          <t>YYZ</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>Vancouver, BC, Canada</t>
+          <t>Toronto, ON, Canada</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
@@ -11178,7 +11178,7 @@
       </c>
       <c r="D339" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Toronto, ON</t>
         </is>
       </c>
       <c r="E339" t="inlineStr">
@@ -11195,12 +11195,12 @@
     <row r="340">
       <c r="A340" s="1" t="inlineStr">
         <is>
-          <t>YWG</t>
+          <t>YVR</t>
         </is>
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>Winnipeg, MB, Canada</t>
+          <t>Vancouver, BC, Canada</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
@@ -11210,7 +11210,7 @@
       </c>
       <c r="D340" t="inlineStr">
         <is>
-          <t>Winnipeg, MB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="E340" t="inlineStr">
@@ -11227,30 +11227,62 @@
     <row r="341">
       <c r="A341" s="1" t="inlineStr">
         <is>
+          <t>YWG</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>Winnipeg, MB, Canada</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>North America</t>
+        </is>
+      </c>
+      <c r="D341" t="inlineStr">
+        <is>
+          <t>Winnipeg, MB</t>
+        </is>
+      </c>
+      <c r="E341" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="F341" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" s="1" t="inlineStr">
+        <is>
           <t>CVG</t>
         </is>
       </c>
-      <c r="B341" t="inlineStr">
+      <c r="B342" t="inlineStr">
         <is>
           <t>Cincinnati, United States</t>
         </is>
       </c>
-      <c r="C341" t="inlineStr">
+      <c r="C342" t="inlineStr">
         <is>
           <t>North America</t>
         </is>
       </c>
-      <c r="D341" t="inlineStr">
+      <c r="D342" t="inlineStr">
         <is>
           <t>Cincinnati</t>
         </is>
       </c>
-      <c r="E341" t="inlineStr">
+      <c r="E342" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="F341" t="inlineStr">
+      <c r="F342" t="inlineStr">
         <is>
           <t>US</t>
         </is>

</xml_diff>

<commit_message>
update generated data Triggered by 38b2f8826e7b870b1d4b3cd8d6b724faa5cb7910
</commit_message>
<xml_diff>
--- a/DC-Colos.xlsx
+++ b/DC-Colos.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F342"/>
+  <dimension ref="A1:F343"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9403,44 +9403,44 @@
     <row r="284">
       <c r="A284" s="1" t="inlineStr">
         <is>
-          <t>ABQ</t>
+          <t>DYU</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>Albuquerque, NM, United States</t>
+          <t>Dushanbe, Tajikistan</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>North America</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>Albuquerque, NM</t>
+          <t>Dushanbe</t>
         </is>
       </c>
       <c r="E284" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Tajikistan</t>
         </is>
       </c>
       <c r="F284" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>TJ</t>
         </is>
       </c>
     </row>
     <row r="285">
       <c r="A285" s="1" t="inlineStr">
         <is>
-          <t>ANC</t>
+          <t>ABQ</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>Anchorage, AK, United States</t>
+          <t>Albuquerque, NM, United States</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
@@ -9450,7 +9450,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>Anchorage, AK</t>
+          <t>Albuquerque, NM</t>
         </is>
       </c>
       <c r="E285" t="inlineStr">
@@ -9467,12 +9467,12 @@
     <row r="286">
       <c r="A286" s="1" t="inlineStr">
         <is>
-          <t>IAD</t>
+          <t>ANC</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>Ashburn, VA, United States</t>
+          <t>Anchorage, AK, United States</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
@@ -9482,7 +9482,7 @@
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>Ashburn, VA</t>
+          <t>Anchorage, AK</t>
         </is>
       </c>
       <c r="E286" t="inlineStr">
@@ -9499,12 +9499,12 @@
     <row r="287">
       <c r="A287" s="1" t="inlineStr">
         <is>
-          <t>ATL</t>
+          <t>IAD</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>Atlanta, GA, United States</t>
+          <t>Ashburn, VA, United States</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
@@ -9514,7 +9514,7 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>Atlanta, GA</t>
+          <t>Ashburn, VA</t>
         </is>
       </c>
       <c r="E287" t="inlineStr">
@@ -9531,12 +9531,12 @@
     <row r="288">
       <c r="A288" s="1" t="inlineStr">
         <is>
-          <t>AUS</t>
+          <t>ATL</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>Austin, TX, United States</t>
+          <t>Atlanta, GA, United States</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
@@ -9546,7 +9546,7 @@
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>Austin, TX</t>
+          <t>Atlanta, GA</t>
         </is>
       </c>
       <c r="E288" t="inlineStr">
@@ -9563,12 +9563,12 @@
     <row r="289">
       <c r="A289" s="1" t="inlineStr">
         <is>
-          <t>BGR</t>
+          <t>AUS</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>Bangor, ME, United States</t>
+          <t>Austin, TX, United States</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
@@ -9578,7 +9578,7 @@
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>Bangor, ME</t>
+          <t>Austin, TX</t>
         </is>
       </c>
       <c r="E289" t="inlineStr">
@@ -9595,12 +9595,12 @@
     <row r="290">
       <c r="A290" s="1" t="inlineStr">
         <is>
-          <t>BOS</t>
+          <t>BGR</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>Boston, MA, United States</t>
+          <t>Bangor, ME, United States</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
@@ -9610,7 +9610,7 @@
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>Boston, MA</t>
+          <t>Bangor, ME</t>
         </is>
       </c>
       <c r="E290" t="inlineStr">
@@ -9627,12 +9627,12 @@
     <row r="291">
       <c r="A291" s="1" t="inlineStr">
         <is>
-          <t>BUF</t>
+          <t>BOS</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>Buffalo, NY, United States</t>
+          <t>Boston, MA, United States</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
@@ -9642,7 +9642,7 @@
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>Buffalo, NY</t>
+          <t>Boston, MA</t>
         </is>
       </c>
       <c r="E291" t="inlineStr">
@@ -9659,12 +9659,12 @@
     <row r="292">
       <c r="A292" s="1" t="inlineStr">
         <is>
-          <t>YYC</t>
+          <t>BUF</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>Calgary, AB, Canada</t>
+          <t>Buffalo, NY, United States</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
@@ -9674,29 +9674,29 @@
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Buffalo, NY</t>
         </is>
       </c>
       <c r="E292" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F292" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="293">
       <c r="A293" s="1" t="inlineStr">
         <is>
-          <t>CLT</t>
+          <t>YYC</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>Charlotte, NC, United States</t>
+          <t>Calgary, AB, Canada</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
@@ -9706,29 +9706,29 @@
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>Charlotte, NC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="E293" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F293" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="294">
       <c r="A294" s="1" t="inlineStr">
         <is>
-          <t>ORD</t>
+          <t>CLT</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>Chicago, IL, United States</t>
+          <t>Charlotte, NC, United States</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
@@ -9738,7 +9738,7 @@
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>Chicago, IL</t>
+          <t>Charlotte, NC</t>
         </is>
       </c>
       <c r="E294" t="inlineStr">
@@ -9755,12 +9755,12 @@
     <row r="295">
       <c r="A295" s="1" t="inlineStr">
         <is>
-          <t>CLE</t>
+          <t>ORD</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>Cleveland, OH, United States</t>
+          <t>Chicago, IL, United States</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -9770,7 +9770,7 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>Cleveland, OH</t>
+          <t>Chicago, IL</t>
         </is>
       </c>
       <c r="E295" t="inlineStr">
@@ -9787,12 +9787,12 @@
     <row r="296">
       <c r="A296" s="1" t="inlineStr">
         <is>
-          <t>CMH</t>
+          <t>CLE</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>Columbus, OH, United States</t>
+          <t>Cleveland, OH, United States</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -9802,7 +9802,7 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>Columbus, OH</t>
+          <t>Cleveland, OH</t>
         </is>
       </c>
       <c r="E296" t="inlineStr">
@@ -9819,12 +9819,12 @@
     <row r="297">
       <c r="A297" s="1" t="inlineStr">
         <is>
-          <t>DFW</t>
+          <t>CMH</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>Dallas, TX, United States</t>
+          <t>Columbus, OH, United States</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
@@ -9834,7 +9834,7 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>Dallas, TX</t>
+          <t>Columbus, OH</t>
         </is>
       </c>
       <c r="E297" t="inlineStr">
@@ -9851,12 +9851,12 @@
     <row r="298">
       <c r="A298" s="1" t="inlineStr">
         <is>
-          <t>DEN</t>
+          <t>DFW</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>Denver, CO, United States</t>
+          <t>Dallas, TX, United States</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
@@ -9866,7 +9866,7 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>Denver, CO</t>
+          <t>Dallas, TX</t>
         </is>
       </c>
       <c r="E298" t="inlineStr">
@@ -9883,12 +9883,12 @@
     <row r="299">
       <c r="A299" s="1" t="inlineStr">
         <is>
-          <t>DTW</t>
+          <t>DEN</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>Detroit, MI, United States</t>
+          <t>Denver, CO, United States</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
@@ -9898,7 +9898,7 @@
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>Detroit, MI</t>
+          <t>Denver, CO</t>
         </is>
       </c>
       <c r="E299" t="inlineStr">
@@ -9915,12 +9915,12 @@
     <row r="300">
       <c r="A300" s="1" t="inlineStr">
         <is>
-          <t>RDU</t>
+          <t>DTW</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>Durham, NC, United States</t>
+          <t>Detroit, MI, United States</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
@@ -9930,7 +9930,7 @@
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>Durham, NC</t>
+          <t>Detroit, MI</t>
         </is>
       </c>
       <c r="E300" t="inlineStr">
@@ -9947,12 +9947,12 @@
     <row r="301">
       <c r="A301" s="1" t="inlineStr">
         <is>
-          <t>GDL</t>
+          <t>RDU</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>Guadalajara, Mexico</t>
+          <t>Durham, NC, United States</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
@@ -9962,29 +9962,29 @@
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>Guadalajara</t>
+          <t>Durham, NC</t>
         </is>
       </c>
       <c r="E301" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F301" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="302">
       <c r="A302" s="1" t="inlineStr">
         <is>
-          <t>YHZ</t>
+          <t>GDL</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>Halifax, Canada</t>
+          <t>Guadalajara, Mexico</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
@@ -9994,29 +9994,29 @@
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>Halifax</t>
+          <t>Guadalajara</t>
         </is>
       </c>
       <c r="E302" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F302" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>MX</t>
         </is>
       </c>
     </row>
     <row r="303">
       <c r="A303" s="1" t="inlineStr">
         <is>
-          <t>HNL</t>
+          <t>YHZ</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>Honolulu, HI, United States</t>
+          <t>Halifax, Canada</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
@@ -10026,29 +10026,29 @@
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>Honolulu, HI</t>
+          <t>Halifax</t>
         </is>
       </c>
       <c r="E303" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F303" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="304">
       <c r="A304" s="1" t="inlineStr">
         <is>
-          <t>IAH</t>
+          <t>HNL</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>Houston, TX, United States</t>
+          <t>Honolulu, HI, United States</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
@@ -10058,7 +10058,7 @@
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>Houston, TX</t>
+          <t>Honolulu, HI</t>
         </is>
       </c>
       <c r="E304" t="inlineStr">
@@ -10075,12 +10075,12 @@
     <row r="305">
       <c r="A305" s="1" t="inlineStr">
         <is>
-          <t>IND</t>
+          <t>IAH</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>Indianapolis, IN, United States</t>
+          <t>Houston, TX, United States</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
@@ -10090,7 +10090,7 @@
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>Indianapolis, IN</t>
+          <t>Houston, TX</t>
         </is>
       </c>
       <c r="E305" t="inlineStr">
@@ -10107,12 +10107,12 @@
     <row r="306">
       <c r="A306" s="1" t="inlineStr">
         <is>
-          <t>JAX</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>Jacksonville, FL, United States</t>
+          <t>Indianapolis, IN, United States</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
@@ -10122,7 +10122,7 @@
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t>Jacksonville, FL</t>
+          <t>Indianapolis, IN</t>
         </is>
       </c>
       <c r="E306" t="inlineStr">
@@ -10139,12 +10139,12 @@
     <row r="307">
       <c r="A307" s="1" t="inlineStr">
         <is>
-          <t>MCI</t>
+          <t>JAX</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>Kansas City, MO, United States</t>
+          <t>Jacksonville, FL, United States</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
@@ -10154,7 +10154,7 @@
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>Kansas City, MO</t>
+          <t>Jacksonville, FL</t>
         </is>
       </c>
       <c r="E307" t="inlineStr">
@@ -10171,12 +10171,12 @@
     <row r="308">
       <c r="A308" s="1" t="inlineStr">
         <is>
-          <t>KIN</t>
+          <t>MCI</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>Kingston, Jamaica</t>
+          <t>Kansas City, MO, United States</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
@@ -10186,29 +10186,29 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>Kingston</t>
+          <t>Kansas City, MO</t>
         </is>
       </c>
       <c r="E308" t="inlineStr">
         <is>
-          <t>Jamaica</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F308" t="inlineStr">
         <is>
-          <t>JM</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="309">
       <c r="A309" s="1" t="inlineStr">
         <is>
-          <t>LAS</t>
+          <t>KIN</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>Las Vegas, NV, United States</t>
+          <t>Kingston, Jamaica</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
@@ -10218,29 +10218,29 @@
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>Las Vegas, NV</t>
+          <t>Kingston</t>
         </is>
       </c>
       <c r="E309" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Jamaica</t>
         </is>
       </c>
       <c r="F309" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>JM</t>
         </is>
       </c>
     </row>
     <row r="310">
       <c r="A310" s="1" t="inlineStr">
         <is>
-          <t>LAX</t>
+          <t>LAS</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>Los Angeles, CA, United States</t>
+          <t>Las Vegas, NV, United States</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
@@ -10250,7 +10250,7 @@
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>Los Angeles, CA</t>
+          <t>Las Vegas, NV</t>
         </is>
       </c>
       <c r="E310" t="inlineStr">
@@ -10267,12 +10267,12 @@
     <row r="311">
       <c r="A311" s="1" t="inlineStr">
         <is>
-          <t>MEM</t>
+          <t>LAX</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Memphis, TN, United States</t>
+          <t>Los Angeles, CA, United States</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
@@ -10282,7 +10282,7 @@
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>Memphis, TN</t>
+          <t>Los Angeles, CA</t>
         </is>
       </c>
       <c r="E311" t="inlineStr">
@@ -10299,12 +10299,12 @@
     <row r="312">
       <c r="A312" s="1" t="inlineStr">
         <is>
-          <t>MEX</t>
+          <t>MEM</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>Mexico City, Mexico</t>
+          <t>Memphis, TN, United States</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
@@ -10314,29 +10314,29 @@
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>Mexico City</t>
+          <t>Memphis, TN</t>
         </is>
       </c>
       <c r="E312" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F312" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="313">
       <c r="A313" s="1" t="inlineStr">
         <is>
-          <t>MIA</t>
+          <t>MEX</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Miami, FL, United States</t>
+          <t>Mexico City, Mexico</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
@@ -10346,29 +10346,29 @@
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>Miami, FL</t>
+          <t>Mexico City</t>
         </is>
       </c>
       <c r="E313" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F313" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
     </row>
     <row r="314">
       <c r="A314" s="1" t="inlineStr">
         <is>
-          <t>MSP</t>
+          <t>MIA</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Minneapolis, MN, United States</t>
+          <t>Miami, FL, United States</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -10378,7 +10378,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>Minneapolis, MN</t>
+          <t>Miami, FL</t>
         </is>
       </c>
       <c r="E314" t="inlineStr">
@@ -10395,12 +10395,12 @@
     <row r="315">
       <c r="A315" s="1" t="inlineStr">
         <is>
-          <t>YUL</t>
+          <t>MSP</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>Montréal, QC, Canada</t>
+          <t>Minneapolis, MN, United States</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
@@ -10410,29 +10410,29 @@
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>Montréal, QC</t>
+          <t>Minneapolis, MN</t>
         </is>
       </c>
       <c r="E315" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F315" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="316">
       <c r="A316" s="1" t="inlineStr">
         <is>
-          <t>BNA</t>
+          <t>YUL</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Nashville, United States</t>
+          <t>Montréal, QC, Canada</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
@@ -10442,29 +10442,29 @@
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>Nashville</t>
+          <t>Montréal, QC</t>
         </is>
       </c>
       <c r="E316" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F316" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="317">
       <c r="A317" s="1" t="inlineStr">
         <is>
-          <t>EWR</t>
+          <t>BNA</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Newark, NJ, United States</t>
+          <t>Nashville, United States</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -10474,7 +10474,7 @@
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t>Newark, NJ</t>
+          <t>Nashville</t>
         </is>
       </c>
       <c r="E317" t="inlineStr">
@@ -10491,12 +10491,12 @@
     <row r="318">
       <c r="A318" s="1" t="inlineStr">
         <is>
-          <t>ORF</t>
+          <t>EWR</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>Norfolk, VA, United States</t>
+          <t>Newark, NJ, United States</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
@@ -10506,7 +10506,7 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>Norfolk, VA</t>
+          <t>Newark, NJ</t>
         </is>
       </c>
       <c r="E318" t="inlineStr">
@@ -10523,12 +10523,12 @@
     <row r="319">
       <c r="A319" s="1" t="inlineStr">
         <is>
-          <t>OKC</t>
+          <t>ORF</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Oklahoma City, OK, United States</t>
+          <t>Norfolk, VA, United States</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
@@ -10538,7 +10538,7 @@
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>Oklahoma City, OK</t>
+          <t>Norfolk, VA</t>
         </is>
       </c>
       <c r="E319" t="inlineStr">
@@ -10555,12 +10555,12 @@
     <row r="320">
       <c r="A320" s="1" t="inlineStr">
         <is>
-          <t>OMA</t>
+          <t>OKC</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Omaha, NE, United States</t>
+          <t>Oklahoma City, OK, United States</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -10570,7 +10570,7 @@
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t>Omaha, NE</t>
+          <t>Oklahoma City, OK</t>
         </is>
       </c>
       <c r="E320" t="inlineStr">
@@ -10587,12 +10587,12 @@
     <row r="321">
       <c r="A321" s="1" t="inlineStr">
         <is>
-          <t>PHL</t>
+          <t>OMA</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>Philadelphia, United States</t>
+          <t>Omaha, NE, United States</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
@@ -10602,7 +10602,7 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>Philadelphia</t>
+          <t>Omaha, NE</t>
         </is>
       </c>
       <c r="E321" t="inlineStr">
@@ -10619,12 +10619,12 @@
     <row r="322">
       <c r="A322" s="1" t="inlineStr">
         <is>
-          <t>PHX</t>
+          <t>PHL</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>Phoenix, AZ, United States</t>
+          <t>Philadelphia, United States</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
@@ -10634,7 +10634,7 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>Phoenix, AZ</t>
+          <t>Philadelphia</t>
         </is>
       </c>
       <c r="E322" t="inlineStr">
@@ -10651,12 +10651,12 @@
     <row r="323">
       <c r="A323" s="1" t="inlineStr">
         <is>
-          <t>PIT</t>
+          <t>PHX</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>Pittsburgh, PA, United States</t>
+          <t>Phoenix, AZ, United States</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -10666,7 +10666,7 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>Pittsburgh, PA</t>
+          <t>Phoenix, AZ</t>
         </is>
       </c>
       <c r="E323" t="inlineStr">
@@ -10683,12 +10683,12 @@
     <row r="324">
       <c r="A324" s="1" t="inlineStr">
         <is>
-          <t>PDX</t>
+          <t>PIT</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>Portland, OR, United States</t>
+          <t>Pittsburgh, PA, United States</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -10698,7 +10698,7 @@
       </c>
       <c r="D324" t="inlineStr">
         <is>
-          <t>Portland, OR</t>
+          <t>Pittsburgh, PA</t>
         </is>
       </c>
       <c r="E324" t="inlineStr">
@@ -10715,12 +10715,12 @@
     <row r="325">
       <c r="A325" s="1" t="inlineStr">
         <is>
-          <t>QRO</t>
+          <t>PDX</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>Queretaro, MX, Mexico</t>
+          <t>Portland, OR, United States</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -10730,29 +10730,29 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>Queretaro, MX</t>
+          <t>Portland, OR</t>
         </is>
       </c>
       <c r="E325" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F325" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="326">
       <c r="A326" s="1" t="inlineStr">
         <is>
-          <t>RIC</t>
+          <t>QRO</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>Richmond, VA, United States</t>
+          <t>Queretaro, MX, Mexico</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
@@ -10762,29 +10762,29 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>Richmond, VA</t>
+          <t>Queretaro, MX</t>
         </is>
       </c>
       <c r="E326" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F326" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
     </row>
     <row r="327">
       <c r="A327" s="1" t="inlineStr">
         <is>
-          <t>SMF</t>
+          <t>RIC</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>Sacramento, CA, United States</t>
+          <t>Richmond, VA, United States</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
@@ -10794,7 +10794,7 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>Sacramento, CA</t>
+          <t>Richmond, VA</t>
         </is>
       </c>
       <c r="E327" t="inlineStr">
@@ -10811,12 +10811,12 @@
     <row r="328">
       <c r="A328" s="1" t="inlineStr">
         <is>
-          <t>SLC</t>
+          <t>SMF</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>Salt Lake City, UT, United States</t>
+          <t>Sacramento, CA, United States</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
@@ -10826,7 +10826,7 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>Salt Lake City, UT</t>
+          <t>Sacramento, CA</t>
         </is>
       </c>
       <c r="E328" t="inlineStr">
@@ -10843,12 +10843,12 @@
     <row r="329">
       <c r="A329" s="1" t="inlineStr">
         <is>
-          <t>SAT</t>
+          <t>SLC</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>San Antonio, TX, United States</t>
+          <t>Salt Lake City, UT, United States</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
@@ -10858,7 +10858,7 @@
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>San Antonio, TX</t>
+          <t>Salt Lake City, UT</t>
         </is>
       </c>
       <c r="E329" t="inlineStr">
@@ -10875,12 +10875,12 @@
     <row r="330">
       <c r="A330" s="1" t="inlineStr">
         <is>
-          <t>SAN</t>
+          <t>SAT</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>San Diego, CA, United States</t>
+          <t>San Antonio, TX, United States</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
@@ -10890,7 +10890,7 @@
       </c>
       <c r="D330" t="inlineStr">
         <is>
-          <t>San Diego, CA</t>
+          <t>San Antonio, TX</t>
         </is>
       </c>
       <c r="E330" t="inlineStr">
@@ -10907,12 +10907,12 @@
     <row r="331">
       <c r="A331" s="1" t="inlineStr">
         <is>
-          <t>SFO</t>
+          <t>SAN</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>San Francisco, CA, United States</t>
+          <t>San Diego, CA, United States</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
@@ -10922,7 +10922,7 @@
       </c>
       <c r="D331" t="inlineStr">
         <is>
-          <t>San Francisco, CA</t>
+          <t>San Diego, CA</t>
         </is>
       </c>
       <c r="E331" t="inlineStr">
@@ -10939,12 +10939,12 @@
     <row r="332">
       <c r="A332" s="1" t="inlineStr">
         <is>
-          <t>SJC</t>
+          <t>SFO</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>San Jose, CA, United States</t>
+          <t>San Francisco, CA, United States</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
@@ -10954,7 +10954,7 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>San Jose, CA</t>
+          <t>San Francisco, CA</t>
         </is>
       </c>
       <c r="E332" t="inlineStr">
@@ -10971,12 +10971,12 @@
     <row r="333">
       <c r="A333" s="1" t="inlineStr">
         <is>
-          <t>YXE</t>
+          <t>SJC</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>Saskatoon, SK, Canada</t>
+          <t>San Jose, CA, United States</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
@@ -10986,29 +10986,29 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>Saskatoon, SK</t>
+          <t>San Jose, CA</t>
         </is>
       </c>
       <c r="E333" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F333" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="334">
       <c r="A334" s="1" t="inlineStr">
         <is>
-          <t>SEA</t>
+          <t>YXE</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>Seattle, WA, United States</t>
+          <t>Saskatoon, SK, Canada</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
@@ -11018,29 +11018,29 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>Seattle, WA</t>
+          <t>Saskatoon, SK</t>
         </is>
       </c>
       <c r="E334" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F334" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="335">
       <c r="A335" s="1" t="inlineStr">
         <is>
-          <t>FSD</t>
+          <t>SEA</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>Sioux Falls, SD, United States</t>
+          <t>Seattle, WA, United States</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
@@ -11050,7 +11050,7 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>Sioux Falls, SD</t>
+          <t>Seattle, WA</t>
         </is>
       </c>
       <c r="E335" t="inlineStr">
@@ -11067,12 +11067,12 @@
     <row r="336">
       <c r="A336" s="1" t="inlineStr">
         <is>
-          <t>STL</t>
+          <t>FSD</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>St. Louis, MO, United States</t>
+          <t>Sioux Falls, SD, United States</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
@@ -11082,7 +11082,7 @@
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>St. Louis, MO</t>
+          <t>Sioux Falls, SD</t>
         </is>
       </c>
       <c r="E336" t="inlineStr">
@@ -11099,12 +11099,12 @@
     <row r="337">
       <c r="A337" s="1" t="inlineStr">
         <is>
-          <t>TLH</t>
+          <t>STL</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>Tallahassee, FL, United States</t>
+          <t>St. Louis, MO, United States</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
@@ -11114,7 +11114,7 @@
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>Tallahassee, FL</t>
+          <t>St. Louis, MO</t>
         </is>
       </c>
       <c r="E337" t="inlineStr">
@@ -11131,12 +11131,12 @@
     <row r="338">
       <c r="A338" s="1" t="inlineStr">
         <is>
-          <t>TPA</t>
+          <t>TLH</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>Tampa, FL, United States</t>
+          <t>Tallahassee, FL, United States</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
@@ -11146,7 +11146,7 @@
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>Tampa, FL</t>
+          <t>Tallahassee, FL</t>
         </is>
       </c>
       <c r="E338" t="inlineStr">
@@ -11163,12 +11163,12 @@
     <row r="339">
       <c r="A339" s="1" t="inlineStr">
         <is>
-          <t>YYZ</t>
+          <t>TPA</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>Toronto, ON, Canada</t>
+          <t>Tampa, FL, United States</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
@@ -11178,29 +11178,29 @@
       </c>
       <c r="D339" t="inlineStr">
         <is>
-          <t>Toronto, ON</t>
+          <t>Tampa, FL</t>
         </is>
       </c>
       <c r="E339" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F339" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="340">
       <c r="A340" s="1" t="inlineStr">
         <is>
-          <t>YVR</t>
+          <t>YYZ</t>
         </is>
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>Vancouver, BC, Canada</t>
+          <t>Toronto, ON, Canada</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
@@ -11210,7 +11210,7 @@
       </c>
       <c r="D340" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Toronto, ON</t>
         </is>
       </c>
       <c r="E340" t="inlineStr">
@@ -11227,12 +11227,12 @@
     <row r="341">
       <c r="A341" s="1" t="inlineStr">
         <is>
-          <t>YWG</t>
+          <t>YVR</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>Winnipeg, MB, Canada</t>
+          <t>Vancouver, BC, Canada</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
@@ -11242,7 +11242,7 @@
       </c>
       <c r="D341" t="inlineStr">
         <is>
-          <t>Winnipeg, MB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="E341" t="inlineStr">
@@ -11259,30 +11259,62 @@
     <row r="342">
       <c r="A342" s="1" t="inlineStr">
         <is>
+          <t>YWG</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>Winnipeg, MB, Canada</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>North America</t>
+        </is>
+      </c>
+      <c r="D342" t="inlineStr">
+        <is>
+          <t>Winnipeg, MB</t>
+        </is>
+      </c>
+      <c r="E342" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="F342" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" s="1" t="inlineStr">
+        <is>
           <t>CVG</t>
         </is>
       </c>
-      <c r="B342" t="inlineStr">
+      <c r="B343" t="inlineStr">
         <is>
           <t>Cincinnati, United States</t>
         </is>
       </c>
-      <c r="C342" t="inlineStr">
+      <c r="C343" t="inlineStr">
         <is>
           <t>North America</t>
         </is>
       </c>
-      <c r="D342" t="inlineStr">
+      <c r="D343" t="inlineStr">
         <is>
           <t>Cincinnati</t>
         </is>
       </c>
-      <c r="E342" t="inlineStr">
+      <c r="E343" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="F342" t="inlineStr">
+      <c r="F343" t="inlineStr">
         <is>
           <t>US</t>
         </is>

</xml_diff>

<commit_message>
update generated data Triggered by 30842af570214579405b6f07c729bda3fb4ca825
</commit_message>
<xml_diff>
--- a/DC-Colos.xlsx
+++ b/DC-Colos.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F343"/>
+  <dimension ref="A1:F344"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9435,44 +9435,44 @@
     <row r="285">
       <c r="A285" s="1" t="inlineStr">
         <is>
-          <t>ABQ</t>
+          <t>LUH</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>Albuquerque, NM, United States</t>
+          <t>Ludhiana, India</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>North America</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>Albuquerque, NM</t>
+          <t>Ludhiana</t>
         </is>
       </c>
       <c r="E285" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F285" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="286">
       <c r="A286" s="1" t="inlineStr">
         <is>
-          <t>ANC</t>
+          <t>ABQ</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>Anchorage, AK, United States</t>
+          <t>Albuquerque, NM, United States</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
@@ -9482,7 +9482,7 @@
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>Anchorage, AK</t>
+          <t>Albuquerque, NM</t>
         </is>
       </c>
       <c r="E286" t="inlineStr">
@@ -9499,12 +9499,12 @@
     <row r="287">
       <c r="A287" s="1" t="inlineStr">
         <is>
-          <t>IAD</t>
+          <t>ANC</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>Ashburn, VA, United States</t>
+          <t>Anchorage, AK, United States</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
@@ -9514,7 +9514,7 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>Ashburn, VA</t>
+          <t>Anchorage, AK</t>
         </is>
       </c>
       <c r="E287" t="inlineStr">
@@ -9531,12 +9531,12 @@
     <row r="288">
       <c r="A288" s="1" t="inlineStr">
         <is>
-          <t>ATL</t>
+          <t>IAD</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>Atlanta, GA, United States</t>
+          <t>Ashburn, VA, United States</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
@@ -9546,7 +9546,7 @@
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>Atlanta, GA</t>
+          <t>Ashburn, VA</t>
         </is>
       </c>
       <c r="E288" t="inlineStr">
@@ -9563,12 +9563,12 @@
     <row r="289">
       <c r="A289" s="1" t="inlineStr">
         <is>
-          <t>AUS</t>
+          <t>ATL</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>Austin, TX, United States</t>
+          <t>Atlanta, GA, United States</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
@@ -9578,7 +9578,7 @@
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>Austin, TX</t>
+          <t>Atlanta, GA</t>
         </is>
       </c>
       <c r="E289" t="inlineStr">
@@ -9595,12 +9595,12 @@
     <row r="290">
       <c r="A290" s="1" t="inlineStr">
         <is>
-          <t>BGR</t>
+          <t>AUS</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>Bangor, ME, United States</t>
+          <t>Austin, TX, United States</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
@@ -9610,7 +9610,7 @@
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>Bangor, ME</t>
+          <t>Austin, TX</t>
         </is>
       </c>
       <c r="E290" t="inlineStr">
@@ -9627,12 +9627,12 @@
     <row r="291">
       <c r="A291" s="1" t="inlineStr">
         <is>
-          <t>BOS</t>
+          <t>BGR</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>Boston, MA, United States</t>
+          <t>Bangor, ME, United States</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
@@ -9642,7 +9642,7 @@
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>Boston, MA</t>
+          <t>Bangor, ME</t>
         </is>
       </c>
       <c r="E291" t="inlineStr">
@@ -9659,12 +9659,12 @@
     <row r="292">
       <c r="A292" s="1" t="inlineStr">
         <is>
-          <t>BUF</t>
+          <t>BOS</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>Buffalo, NY, United States</t>
+          <t>Boston, MA, United States</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
@@ -9674,7 +9674,7 @@
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>Buffalo, NY</t>
+          <t>Boston, MA</t>
         </is>
       </c>
       <c r="E292" t="inlineStr">
@@ -9691,12 +9691,12 @@
     <row r="293">
       <c r="A293" s="1" t="inlineStr">
         <is>
-          <t>YYC</t>
+          <t>BUF</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>Calgary, AB, Canada</t>
+          <t>Buffalo, NY, United States</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
@@ -9706,29 +9706,29 @@
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Buffalo, NY</t>
         </is>
       </c>
       <c r="E293" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F293" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="294">
       <c r="A294" s="1" t="inlineStr">
         <is>
-          <t>CLT</t>
+          <t>YYC</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>Charlotte, NC, United States</t>
+          <t>Calgary, AB, Canada</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
@@ -9738,29 +9738,29 @@
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>Charlotte, NC</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="E294" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F294" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="295">
       <c r="A295" s="1" t="inlineStr">
         <is>
-          <t>ORD</t>
+          <t>CLT</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>Chicago, IL, United States</t>
+          <t>Charlotte, NC, United States</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -9770,7 +9770,7 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>Chicago, IL</t>
+          <t>Charlotte, NC</t>
         </is>
       </c>
       <c r="E295" t="inlineStr">
@@ -9787,12 +9787,12 @@
     <row r="296">
       <c r="A296" s="1" t="inlineStr">
         <is>
-          <t>CLE</t>
+          <t>ORD</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>Cleveland, OH, United States</t>
+          <t>Chicago, IL, United States</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -9802,7 +9802,7 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>Cleveland, OH</t>
+          <t>Chicago, IL</t>
         </is>
       </c>
       <c r="E296" t="inlineStr">
@@ -9819,12 +9819,12 @@
     <row r="297">
       <c r="A297" s="1" t="inlineStr">
         <is>
-          <t>CMH</t>
+          <t>CLE</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>Columbus, OH, United States</t>
+          <t>Cleveland, OH, United States</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
@@ -9834,7 +9834,7 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>Columbus, OH</t>
+          <t>Cleveland, OH</t>
         </is>
       </c>
       <c r="E297" t="inlineStr">
@@ -9851,12 +9851,12 @@
     <row r="298">
       <c r="A298" s="1" t="inlineStr">
         <is>
-          <t>DFW</t>
+          <t>CMH</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>Dallas, TX, United States</t>
+          <t>Columbus, OH, United States</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
@@ -9866,7 +9866,7 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>Dallas, TX</t>
+          <t>Columbus, OH</t>
         </is>
       </c>
       <c r="E298" t="inlineStr">
@@ -9883,12 +9883,12 @@
     <row r="299">
       <c r="A299" s="1" t="inlineStr">
         <is>
-          <t>DEN</t>
+          <t>DFW</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>Denver, CO, United States</t>
+          <t>Dallas, TX, United States</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
@@ -9898,7 +9898,7 @@
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>Denver, CO</t>
+          <t>Dallas, TX</t>
         </is>
       </c>
       <c r="E299" t="inlineStr">
@@ -9915,12 +9915,12 @@
     <row r="300">
       <c r="A300" s="1" t="inlineStr">
         <is>
-          <t>DTW</t>
+          <t>DEN</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>Detroit, MI, United States</t>
+          <t>Denver, CO, United States</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
@@ -9930,7 +9930,7 @@
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>Detroit, MI</t>
+          <t>Denver, CO</t>
         </is>
       </c>
       <c r="E300" t="inlineStr">
@@ -9947,12 +9947,12 @@
     <row r="301">
       <c r="A301" s="1" t="inlineStr">
         <is>
-          <t>RDU</t>
+          <t>DTW</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>Durham, NC, United States</t>
+          <t>Detroit, MI, United States</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
@@ -9962,7 +9962,7 @@
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>Durham, NC</t>
+          <t>Detroit, MI</t>
         </is>
       </c>
       <c r="E301" t="inlineStr">
@@ -9979,12 +9979,12 @@
     <row r="302">
       <c r="A302" s="1" t="inlineStr">
         <is>
-          <t>GDL</t>
+          <t>RDU</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>Guadalajara, Mexico</t>
+          <t>Durham, NC, United States</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
@@ -9994,29 +9994,29 @@
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>Guadalajara</t>
+          <t>Durham, NC</t>
         </is>
       </c>
       <c r="E302" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F302" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="303">
       <c r="A303" s="1" t="inlineStr">
         <is>
-          <t>YHZ</t>
+          <t>GDL</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>Halifax, Canada</t>
+          <t>Guadalajara, Mexico</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
@@ -10026,29 +10026,29 @@
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>Halifax</t>
+          <t>Guadalajara</t>
         </is>
       </c>
       <c r="E303" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F303" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>MX</t>
         </is>
       </c>
     </row>
     <row r="304">
       <c r="A304" s="1" t="inlineStr">
         <is>
-          <t>HNL</t>
+          <t>YHZ</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>Honolulu, HI, United States</t>
+          <t>Halifax, Canada</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
@@ -10058,29 +10058,29 @@
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>Honolulu, HI</t>
+          <t>Halifax</t>
         </is>
       </c>
       <c r="E304" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F304" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="305">
       <c r="A305" s="1" t="inlineStr">
         <is>
-          <t>IAH</t>
+          <t>HNL</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>Houston, TX, United States</t>
+          <t>Honolulu, HI, United States</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
@@ -10090,7 +10090,7 @@
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>Houston, TX</t>
+          <t>Honolulu, HI</t>
         </is>
       </c>
       <c r="E305" t="inlineStr">
@@ -10107,12 +10107,12 @@
     <row r="306">
       <c r="A306" s="1" t="inlineStr">
         <is>
-          <t>IND</t>
+          <t>IAH</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>Indianapolis, IN, United States</t>
+          <t>Houston, TX, United States</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
@@ -10122,7 +10122,7 @@
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t>Indianapolis, IN</t>
+          <t>Houston, TX</t>
         </is>
       </c>
       <c r="E306" t="inlineStr">
@@ -10139,12 +10139,12 @@
     <row r="307">
       <c r="A307" s="1" t="inlineStr">
         <is>
-          <t>JAX</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>Jacksonville, FL, United States</t>
+          <t>Indianapolis, IN, United States</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
@@ -10154,7 +10154,7 @@
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>Jacksonville, FL</t>
+          <t>Indianapolis, IN</t>
         </is>
       </c>
       <c r="E307" t="inlineStr">
@@ -10171,12 +10171,12 @@
     <row r="308">
       <c r="A308" s="1" t="inlineStr">
         <is>
-          <t>MCI</t>
+          <t>JAX</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>Kansas City, MO, United States</t>
+          <t>Jacksonville, FL, United States</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
@@ -10186,7 +10186,7 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>Kansas City, MO</t>
+          <t>Jacksonville, FL</t>
         </is>
       </c>
       <c r="E308" t="inlineStr">
@@ -10203,12 +10203,12 @@
     <row r="309">
       <c r="A309" s="1" t="inlineStr">
         <is>
-          <t>KIN</t>
+          <t>MCI</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>Kingston, Jamaica</t>
+          <t>Kansas City, MO, United States</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
@@ -10218,29 +10218,29 @@
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>Kingston</t>
+          <t>Kansas City, MO</t>
         </is>
       </c>
       <c r="E309" t="inlineStr">
         <is>
-          <t>Jamaica</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F309" t="inlineStr">
         <is>
-          <t>JM</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="310">
       <c r="A310" s="1" t="inlineStr">
         <is>
-          <t>LAS</t>
+          <t>KIN</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>Las Vegas, NV, United States</t>
+          <t>Kingston, Jamaica</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
@@ -10250,29 +10250,29 @@
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>Las Vegas, NV</t>
+          <t>Kingston</t>
         </is>
       </c>
       <c r="E310" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Jamaica</t>
         </is>
       </c>
       <c r="F310" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>JM</t>
         </is>
       </c>
     </row>
     <row r="311">
       <c r="A311" s="1" t="inlineStr">
         <is>
-          <t>LAX</t>
+          <t>LAS</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Los Angeles, CA, United States</t>
+          <t>Las Vegas, NV, United States</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
@@ -10282,7 +10282,7 @@
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>Los Angeles, CA</t>
+          <t>Las Vegas, NV</t>
         </is>
       </c>
       <c r="E311" t="inlineStr">
@@ -10299,12 +10299,12 @@
     <row r="312">
       <c r="A312" s="1" t="inlineStr">
         <is>
-          <t>MEM</t>
+          <t>LAX</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>Memphis, TN, United States</t>
+          <t>Los Angeles, CA, United States</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
@@ -10314,7 +10314,7 @@
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>Memphis, TN</t>
+          <t>Los Angeles, CA</t>
         </is>
       </c>
       <c r="E312" t="inlineStr">
@@ -10331,12 +10331,12 @@
     <row r="313">
       <c r="A313" s="1" t="inlineStr">
         <is>
-          <t>MEX</t>
+          <t>MEM</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Mexico City, Mexico</t>
+          <t>Memphis, TN, United States</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
@@ -10346,29 +10346,29 @@
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>Mexico City</t>
+          <t>Memphis, TN</t>
         </is>
       </c>
       <c r="E313" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F313" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="314">
       <c r="A314" s="1" t="inlineStr">
         <is>
-          <t>MIA</t>
+          <t>MEX</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Miami, FL, United States</t>
+          <t>Mexico City, Mexico</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -10378,29 +10378,29 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>Miami, FL</t>
+          <t>Mexico City</t>
         </is>
       </c>
       <c r="E314" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F314" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
     </row>
     <row r="315">
       <c r="A315" s="1" t="inlineStr">
         <is>
-          <t>MSP</t>
+          <t>MIA</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>Minneapolis, MN, United States</t>
+          <t>Miami, FL, United States</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
@@ -10410,7 +10410,7 @@
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>Minneapolis, MN</t>
+          <t>Miami, FL</t>
         </is>
       </c>
       <c r="E315" t="inlineStr">
@@ -10427,12 +10427,12 @@
     <row r="316">
       <c r="A316" s="1" t="inlineStr">
         <is>
-          <t>YUL</t>
+          <t>MSP</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Montréal, QC, Canada</t>
+          <t>Minneapolis, MN, United States</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
@@ -10442,29 +10442,29 @@
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>Montréal, QC</t>
+          <t>Minneapolis, MN</t>
         </is>
       </c>
       <c r="E316" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F316" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="317">
       <c r="A317" s="1" t="inlineStr">
         <is>
-          <t>BNA</t>
+          <t>YUL</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Nashville, United States</t>
+          <t>Montréal, QC, Canada</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -10474,29 +10474,29 @@
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t>Nashville</t>
+          <t>Montréal, QC</t>
         </is>
       </c>
       <c r="E317" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F317" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="318">
       <c r="A318" s="1" t="inlineStr">
         <is>
-          <t>EWR</t>
+          <t>BNA</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>Newark, NJ, United States</t>
+          <t>Nashville, United States</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
@@ -10506,7 +10506,7 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>Newark, NJ</t>
+          <t>Nashville</t>
         </is>
       </c>
       <c r="E318" t="inlineStr">
@@ -10523,12 +10523,12 @@
     <row r="319">
       <c r="A319" s="1" t="inlineStr">
         <is>
-          <t>ORF</t>
+          <t>EWR</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Norfolk, VA, United States</t>
+          <t>Newark, NJ, United States</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
@@ -10538,7 +10538,7 @@
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>Norfolk, VA</t>
+          <t>Newark, NJ</t>
         </is>
       </c>
       <c r="E319" t="inlineStr">
@@ -10555,12 +10555,12 @@
     <row r="320">
       <c r="A320" s="1" t="inlineStr">
         <is>
-          <t>OKC</t>
+          <t>ORF</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Oklahoma City, OK, United States</t>
+          <t>Norfolk, VA, United States</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -10570,7 +10570,7 @@
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t>Oklahoma City, OK</t>
+          <t>Norfolk, VA</t>
         </is>
       </c>
       <c r="E320" t="inlineStr">
@@ -10587,12 +10587,12 @@
     <row r="321">
       <c r="A321" s="1" t="inlineStr">
         <is>
-          <t>OMA</t>
+          <t>OKC</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>Omaha, NE, United States</t>
+          <t>Oklahoma City, OK, United States</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
@@ -10602,7 +10602,7 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>Omaha, NE</t>
+          <t>Oklahoma City, OK</t>
         </is>
       </c>
       <c r="E321" t="inlineStr">
@@ -10619,12 +10619,12 @@
     <row r="322">
       <c r="A322" s="1" t="inlineStr">
         <is>
-          <t>PHL</t>
+          <t>OMA</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>Philadelphia, United States</t>
+          <t>Omaha, NE, United States</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
@@ -10634,7 +10634,7 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>Philadelphia</t>
+          <t>Omaha, NE</t>
         </is>
       </c>
       <c r="E322" t="inlineStr">
@@ -10651,12 +10651,12 @@
     <row r="323">
       <c r="A323" s="1" t="inlineStr">
         <is>
-          <t>PHX</t>
+          <t>PHL</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>Phoenix, AZ, United States</t>
+          <t>Philadelphia, United States</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -10666,7 +10666,7 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>Phoenix, AZ</t>
+          <t>Philadelphia</t>
         </is>
       </c>
       <c r="E323" t="inlineStr">
@@ -10683,12 +10683,12 @@
     <row r="324">
       <c r="A324" s="1" t="inlineStr">
         <is>
-          <t>PIT</t>
+          <t>PHX</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>Pittsburgh, PA, United States</t>
+          <t>Phoenix, AZ, United States</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -10698,7 +10698,7 @@
       </c>
       <c r="D324" t="inlineStr">
         <is>
-          <t>Pittsburgh, PA</t>
+          <t>Phoenix, AZ</t>
         </is>
       </c>
       <c r="E324" t="inlineStr">
@@ -10715,12 +10715,12 @@
     <row r="325">
       <c r="A325" s="1" t="inlineStr">
         <is>
-          <t>PDX</t>
+          <t>PIT</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>Portland, OR, United States</t>
+          <t>Pittsburgh, PA, United States</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -10730,7 +10730,7 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>Portland, OR</t>
+          <t>Pittsburgh, PA</t>
         </is>
       </c>
       <c r="E325" t="inlineStr">
@@ -10747,12 +10747,12 @@
     <row r="326">
       <c r="A326" s="1" t="inlineStr">
         <is>
-          <t>QRO</t>
+          <t>PDX</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>Queretaro, MX, Mexico</t>
+          <t>Portland, OR, United States</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
@@ -10762,29 +10762,29 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>Queretaro, MX</t>
+          <t>Portland, OR</t>
         </is>
       </c>
       <c r="E326" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F326" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="327">
       <c r="A327" s="1" t="inlineStr">
         <is>
-          <t>RIC</t>
+          <t>QRO</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>Richmond, VA, United States</t>
+          <t>Queretaro, MX, Mexico</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
@@ -10794,29 +10794,29 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>Richmond, VA</t>
+          <t>Queretaro, MX</t>
         </is>
       </c>
       <c r="E327" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F327" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
     </row>
     <row r="328">
       <c r="A328" s="1" t="inlineStr">
         <is>
-          <t>SMF</t>
+          <t>RIC</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>Sacramento, CA, United States</t>
+          <t>Richmond, VA, United States</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
@@ -10826,7 +10826,7 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>Sacramento, CA</t>
+          <t>Richmond, VA</t>
         </is>
       </c>
       <c r="E328" t="inlineStr">
@@ -10843,12 +10843,12 @@
     <row r="329">
       <c r="A329" s="1" t="inlineStr">
         <is>
-          <t>SLC</t>
+          <t>SMF</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>Salt Lake City, UT, United States</t>
+          <t>Sacramento, CA, United States</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
@@ -10858,7 +10858,7 @@
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>Salt Lake City, UT</t>
+          <t>Sacramento, CA</t>
         </is>
       </c>
       <c r="E329" t="inlineStr">
@@ -10875,12 +10875,12 @@
     <row r="330">
       <c r="A330" s="1" t="inlineStr">
         <is>
-          <t>SAT</t>
+          <t>SLC</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>San Antonio, TX, United States</t>
+          <t>Salt Lake City, UT, United States</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
@@ -10890,7 +10890,7 @@
       </c>
       <c r="D330" t="inlineStr">
         <is>
-          <t>San Antonio, TX</t>
+          <t>Salt Lake City, UT</t>
         </is>
       </c>
       <c r="E330" t="inlineStr">
@@ -10907,12 +10907,12 @@
     <row r="331">
       <c r="A331" s="1" t="inlineStr">
         <is>
-          <t>SAN</t>
+          <t>SAT</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>San Diego, CA, United States</t>
+          <t>San Antonio, TX, United States</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
@@ -10922,7 +10922,7 @@
       </c>
       <c r="D331" t="inlineStr">
         <is>
-          <t>San Diego, CA</t>
+          <t>San Antonio, TX</t>
         </is>
       </c>
       <c r="E331" t="inlineStr">
@@ -10939,12 +10939,12 @@
     <row r="332">
       <c r="A332" s="1" t="inlineStr">
         <is>
-          <t>SFO</t>
+          <t>SAN</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>San Francisco, CA, United States</t>
+          <t>San Diego, CA, United States</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
@@ -10954,7 +10954,7 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>San Francisco, CA</t>
+          <t>San Diego, CA</t>
         </is>
       </c>
       <c r="E332" t="inlineStr">
@@ -10971,12 +10971,12 @@
     <row r="333">
       <c r="A333" s="1" t="inlineStr">
         <is>
-          <t>SJC</t>
+          <t>SFO</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>San Jose, CA, United States</t>
+          <t>San Francisco, CA, United States</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
@@ -10986,7 +10986,7 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>San Jose, CA</t>
+          <t>San Francisco, CA</t>
         </is>
       </c>
       <c r="E333" t="inlineStr">
@@ -11003,12 +11003,12 @@
     <row r="334">
       <c r="A334" s="1" t="inlineStr">
         <is>
-          <t>YXE</t>
+          <t>SJC</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>Saskatoon, SK, Canada</t>
+          <t>San Jose, CA, United States</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
@@ -11018,29 +11018,29 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>Saskatoon, SK</t>
+          <t>San Jose, CA</t>
         </is>
       </c>
       <c r="E334" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F334" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="335">
       <c r="A335" s="1" t="inlineStr">
         <is>
-          <t>SEA</t>
+          <t>YXE</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>Seattle, WA, United States</t>
+          <t>Saskatoon, SK, Canada</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
@@ -11050,29 +11050,29 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>Seattle, WA</t>
+          <t>Saskatoon, SK</t>
         </is>
       </c>
       <c r="E335" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F335" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="336">
       <c r="A336" s="1" t="inlineStr">
         <is>
-          <t>FSD</t>
+          <t>SEA</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>Sioux Falls, SD, United States</t>
+          <t>Seattle, WA, United States</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
@@ -11082,7 +11082,7 @@
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>Sioux Falls, SD</t>
+          <t>Seattle, WA</t>
         </is>
       </c>
       <c r="E336" t="inlineStr">
@@ -11099,12 +11099,12 @@
     <row r="337">
       <c r="A337" s="1" t="inlineStr">
         <is>
-          <t>STL</t>
+          <t>FSD</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>St. Louis, MO, United States</t>
+          <t>Sioux Falls, SD, United States</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
@@ -11114,7 +11114,7 @@
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>St. Louis, MO</t>
+          <t>Sioux Falls, SD</t>
         </is>
       </c>
       <c r="E337" t="inlineStr">
@@ -11131,12 +11131,12 @@
     <row r="338">
       <c r="A338" s="1" t="inlineStr">
         <is>
-          <t>TLH</t>
+          <t>STL</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>Tallahassee, FL, United States</t>
+          <t>St. Louis, MO, United States</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
@@ -11146,7 +11146,7 @@
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>Tallahassee, FL</t>
+          <t>St. Louis, MO</t>
         </is>
       </c>
       <c r="E338" t="inlineStr">
@@ -11163,12 +11163,12 @@
     <row r="339">
       <c r="A339" s="1" t="inlineStr">
         <is>
-          <t>TPA</t>
+          <t>TLH</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>Tampa, FL, United States</t>
+          <t>Tallahassee, FL, United States</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
@@ -11178,7 +11178,7 @@
       </c>
       <c r="D339" t="inlineStr">
         <is>
-          <t>Tampa, FL</t>
+          <t>Tallahassee, FL</t>
         </is>
       </c>
       <c r="E339" t="inlineStr">
@@ -11195,12 +11195,12 @@
     <row r="340">
       <c r="A340" s="1" t="inlineStr">
         <is>
-          <t>YYZ</t>
+          <t>TPA</t>
         </is>
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>Toronto, ON, Canada</t>
+          <t>Tampa, FL, United States</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
@@ -11210,29 +11210,29 @@
       </c>
       <c r="D340" t="inlineStr">
         <is>
-          <t>Toronto, ON</t>
+          <t>Tampa, FL</t>
         </is>
       </c>
       <c r="E340" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F340" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="341">
       <c r="A341" s="1" t="inlineStr">
         <is>
-          <t>YVR</t>
+          <t>YYZ</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>Vancouver, BC, Canada</t>
+          <t>Toronto, ON, Canada</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
@@ -11242,7 +11242,7 @@
       </c>
       <c r="D341" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Toronto, ON</t>
         </is>
       </c>
       <c r="E341" t="inlineStr">
@@ -11259,12 +11259,12 @@
     <row r="342">
       <c r="A342" s="1" t="inlineStr">
         <is>
-          <t>YWG</t>
+          <t>YVR</t>
         </is>
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>Winnipeg, MB, Canada</t>
+          <t>Vancouver, BC, Canada</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
@@ -11274,7 +11274,7 @@
       </c>
       <c r="D342" t="inlineStr">
         <is>
-          <t>Winnipeg, MB</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="E342" t="inlineStr">
@@ -11291,30 +11291,62 @@
     <row r="343">
       <c r="A343" s="1" t="inlineStr">
         <is>
+          <t>YWG</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>Winnipeg, MB, Canada</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>North America</t>
+        </is>
+      </c>
+      <c r="D343" t="inlineStr">
+        <is>
+          <t>Winnipeg, MB</t>
+        </is>
+      </c>
+      <c r="E343" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="F343" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" s="1" t="inlineStr">
+        <is>
           <t>CVG</t>
         </is>
       </c>
-      <c r="B343" t="inlineStr">
+      <c r="B344" t="inlineStr">
         <is>
           <t>Cincinnati, United States</t>
         </is>
       </c>
-      <c r="C343" t="inlineStr">
+      <c r="C344" t="inlineStr">
         <is>
           <t>North America</t>
         </is>
       </c>
-      <c r="D343" t="inlineStr">
+      <c r="D344" t="inlineStr">
         <is>
           <t>Cincinnati</t>
         </is>
       </c>
-      <c r="E343" t="inlineStr">
+      <c r="E344" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="F343" t="inlineStr">
+      <c r="F344" t="inlineStr">
         <is>
           <t>US</t>
         </is>

</xml_diff>

<commit_message>
update generated data Triggered by ed208bc1c5c4e3338e143f1819e87893c076c541
</commit_message>
<xml_diff>
--- a/DC-Colos.xlsx
+++ b/DC-Colos.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F344"/>
+  <dimension ref="A1:F343"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7283,12 +7283,12 @@
     <row r="217">
       <c r="A217" s="1" t="inlineStr">
         <is>
-          <t>KJA</t>
+          <t>KUL</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>Krasnoyarsk, Russia</t>
+          <t>Kuala Lumpur, Malaysia</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
@@ -7298,29 +7298,29 @@
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>Krasnoyarsk</t>
+          <t>Kuala Lumpur</t>
         </is>
       </c>
       <c r="E217" t="inlineStr">
         <is>
-          <t>Russia</t>
+          <t>Malaysia</t>
         </is>
       </c>
       <c r="F217" t="inlineStr">
         <is>
-          <t>RU</t>
+          <t>MY</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="1" t="inlineStr">
         <is>
-          <t>KUL</t>
+          <t>PKX</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>Kuala Lumpur, Malaysia</t>
+          <t>Langfang, China</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
@@ -7330,29 +7330,29 @@
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>Kuala Lumpur</t>
+          <t>Langfang</t>
         </is>
       </c>
       <c r="E218" t="inlineStr">
         <is>
-          <t>Malaysia</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F218" t="inlineStr">
         <is>
-          <t>MY</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="1" t="inlineStr">
         <is>
-          <t>PKX</t>
+          <t>MFM</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>Langfang, China</t>
+          <t>Macau</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
@@ -7360,31 +7360,19 @@
           <t>Asia</t>
         </is>
       </c>
-      <c r="D219" t="inlineStr">
-        <is>
-          <t>Langfang</t>
-        </is>
-      </c>
-      <c r="E219" t="inlineStr">
-        <is>
-          <t>China</t>
-        </is>
-      </c>
-      <c r="F219" t="inlineStr">
-        <is>
-          <t>CN</t>
-        </is>
-      </c>
+      <c r="D219" t="inlineStr"/>
+      <c r="E219" t="inlineStr"/>
+      <c r="F219" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" s="1" t="inlineStr">
         <is>
-          <t>MFM</t>
+          <t>MLE</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>Macau</t>
+          <t>Malé, Maldives</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
@@ -7392,19 +7380,31 @@
           <t>Asia</t>
         </is>
       </c>
-      <c r="D220" t="inlineStr"/>
-      <c r="E220" t="inlineStr"/>
-      <c r="F220" t="inlineStr"/>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>Malé</t>
+        </is>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>Maldives</t>
+        </is>
+      </c>
+      <c r="F220" t="inlineStr">
+        <is>
+          <t>MV</t>
+        </is>
+      </c>
     </row>
     <row r="221">
       <c r="A221" s="1" t="inlineStr">
         <is>
-          <t>MLE</t>
+          <t>MNL</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>Malé, Maldives</t>
+          <t>Manila, Philippines</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
@@ -7414,29 +7414,29 @@
       </c>
       <c r="D221" t="inlineStr">
         <is>
-          <t>Malé</t>
+          <t>Manila</t>
         </is>
       </c>
       <c r="E221" t="inlineStr">
         <is>
-          <t>Maldives</t>
+          <t>Philippines</t>
         </is>
       </c>
       <c r="F221" t="inlineStr">
         <is>
-          <t>MV</t>
+          <t>PH</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="1" t="inlineStr">
         <is>
-          <t>MNL</t>
+          <t>BOM</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>Manila, Philippines</t>
+          <t>Mumbai, India</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
@@ -7446,29 +7446,29 @@
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t>Manila</t>
+          <t>Mumbai</t>
         </is>
       </c>
       <c r="E222" t="inlineStr">
         <is>
-          <t>Philippines</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F222" t="inlineStr">
         <is>
-          <t>PH</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="1" t="inlineStr">
         <is>
-          <t>BOM</t>
+          <t>NAG</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>Mumbai, India</t>
+          <t>Nagpur, India</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
@@ -7478,7 +7478,7 @@
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>Mumbai</t>
+          <t>Nagpur</t>
         </is>
       </c>
       <c r="E223" t="inlineStr">
@@ -7495,12 +7495,12 @@
     <row r="224">
       <c r="A224" s="1" t="inlineStr">
         <is>
-          <t>NAG</t>
+          <t>OKA</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>Nagpur, India</t>
+          <t>Naha, Japan</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
@@ -7510,29 +7510,29 @@
       </c>
       <c r="D224" t="inlineStr">
         <is>
-          <t>Nagpur</t>
+          <t>Naha</t>
         </is>
       </c>
       <c r="E224" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="F224" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>JP</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" s="1" t="inlineStr">
         <is>
-          <t>OKA</t>
+          <t>DEL</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>Naha, Japan</t>
+          <t>New Delhi, India</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
@@ -7542,29 +7542,29 @@
       </c>
       <c r="D225" t="inlineStr">
         <is>
-          <t>Naha</t>
+          <t>New Delhi</t>
         </is>
       </c>
       <c r="E225" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F225" t="inlineStr">
         <is>
-          <t>JP</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" s="1" t="inlineStr">
         <is>
-          <t>DEL</t>
+          <t>KIX</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>New Delhi, India</t>
+          <t>Osaka, Japan</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
@@ -7574,29 +7574,29 @@
       </c>
       <c r="D226" t="inlineStr">
         <is>
-          <t>New Delhi</t>
+          <t>Osaka</t>
         </is>
       </c>
       <c r="E226" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="F226" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>JP</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" s="1" t="inlineStr">
         <is>
-          <t>KIX</t>
+          <t>PAT</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>Osaka, Japan</t>
+          <t>Patna, India</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
@@ -7606,29 +7606,29 @@
       </c>
       <c r="D227" t="inlineStr">
         <is>
-          <t>Osaka</t>
+          <t>Patna</t>
         </is>
       </c>
       <c r="E227" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F227" t="inlineStr">
         <is>
-          <t>JP</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" s="1" t="inlineStr">
         <is>
-          <t>PAT</t>
+          <t>PNH</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>Patna, India</t>
+          <t>Phnom Penh, Cambodia</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
@@ -7638,29 +7638,29 @@
       </c>
       <c r="D228" t="inlineStr">
         <is>
-          <t>Patna</t>
+          <t>Phnom Penh</t>
         </is>
       </c>
       <c r="E228" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Cambodia</t>
         </is>
       </c>
       <c r="F228" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>KH</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" s="1" t="inlineStr">
         <is>
-          <t>PNH</t>
+          <t>TAO</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>Phnom Penh, Cambodia</t>
+          <t>Qingdao, China</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
@@ -7670,29 +7670,29 @@
       </c>
       <c r="D229" t="inlineStr">
         <is>
-          <t>Phnom Penh</t>
+          <t>Qingdao</t>
         </is>
       </c>
       <c r="E229" t="inlineStr">
         <is>
-          <t>Cambodia</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F229" t="inlineStr">
         <is>
-          <t>KH</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" s="1" t="inlineStr">
         <is>
-          <t>TAO</t>
+          <t>ICN</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>Qingdao, China</t>
+          <t>Seoul, South Korea</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
@@ -7702,29 +7702,29 @@
       </c>
       <c r="D230" t="inlineStr">
         <is>
-          <t>Qingdao</t>
+          <t>Seoul</t>
         </is>
       </c>
       <c r="E230" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>South Korea</t>
         </is>
       </c>
       <c r="F230" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>KR</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" s="1" t="inlineStr">
         <is>
-          <t>ICN</t>
+          <t>SHA</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>Seoul, South Korea</t>
+          <t>Shanghai, China</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
@@ -7734,29 +7734,29 @@
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>Seoul</t>
+          <t>Shanghai</t>
         </is>
       </c>
       <c r="E231" t="inlineStr">
         <is>
-          <t>South Korea</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F231" t="inlineStr">
         <is>
-          <t>KR</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" s="1" t="inlineStr">
         <is>
-          <t>SHA</t>
+          <t>SIN</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>Shanghai, China</t>
+          <t>Singapore, Singapore</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
@@ -7766,29 +7766,29 @@
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>Shanghai</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="E232" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="F232" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>SG</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" s="1" t="inlineStr">
         <is>
-          <t>SIN</t>
+          <t>URT</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>Singapore, Singapore</t>
+          <t>Surat Thani, Thailand</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
@@ -7798,29 +7798,29 @@
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Surat Thani</t>
         </is>
       </c>
       <c r="E233" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Thailand</t>
         </is>
       </c>
       <c r="F233" t="inlineStr">
         <is>
-          <t>SG</t>
+          <t>TH</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" s="1" t="inlineStr">
         <is>
-          <t>URT</t>
+          <t>TPE</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>Surat Thani, Thailand</t>
+          <t>Taipei</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
@@ -7828,31 +7828,19 @@
           <t>Asia</t>
         </is>
       </c>
-      <c r="D234" t="inlineStr">
-        <is>
-          <t>Surat Thani</t>
-        </is>
-      </c>
-      <c r="E234" t="inlineStr">
-        <is>
-          <t>Thailand</t>
-        </is>
-      </c>
-      <c r="F234" t="inlineStr">
-        <is>
-          <t>TH</t>
-        </is>
-      </c>
+      <c r="D234" t="inlineStr"/>
+      <c r="E234" t="inlineStr"/>
+      <c r="F234" t="inlineStr"/>
     </row>
     <row r="235">
       <c r="A235" s="1" t="inlineStr">
         <is>
-          <t>TPE</t>
+          <t>NRT</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>Taipei</t>
+          <t>Tokyo, Japan</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
@@ -7860,19 +7848,31 @@
           <t>Asia</t>
         </is>
       </c>
-      <c r="D235" t="inlineStr"/>
-      <c r="E235" t="inlineStr"/>
-      <c r="F235" t="inlineStr"/>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>Tokyo</t>
+        </is>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="F235" t="inlineStr">
+        <is>
+          <t>JP</t>
+        </is>
+      </c>
     </row>
     <row r="236">
       <c r="A236" s="1" t="inlineStr">
         <is>
-          <t>NRT</t>
+          <t>ULN</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>Tokyo, Japan</t>
+          <t>Ulaanbaatar, Mongolia</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
@@ -7882,29 +7882,29 @@
       </c>
       <c r="D236" t="inlineStr">
         <is>
-          <t>Tokyo</t>
+          <t>Ulaanbaatar</t>
         </is>
       </c>
       <c r="E236" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Mongolia</t>
         </is>
       </c>
       <c r="F236" t="inlineStr">
         <is>
-          <t>JP</t>
+          <t>MN</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" s="1" t="inlineStr">
         <is>
-          <t>ULN</t>
+          <t>VTE</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>Ulaanbaatar, Mongolia</t>
+          <t>Vientiane, Laos</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
@@ -7914,29 +7914,29 @@
       </c>
       <c r="D237" t="inlineStr">
         <is>
-          <t>Ulaanbaatar</t>
+          <t>Vientiane</t>
         </is>
       </c>
       <c r="E237" t="inlineStr">
         <is>
-          <t>Mongolia</t>
+          <t>Laos</t>
         </is>
       </c>
       <c r="F237" t="inlineStr">
         <is>
-          <t>MN</t>
+          <t>LA</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" s="1" t="inlineStr">
         <is>
-          <t>VTE</t>
+          <t>KHN</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>Vientiane, Laos</t>
+          <t>Xinyu, China</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
@@ -7946,29 +7946,29 @@
       </c>
       <c r="D238" t="inlineStr">
         <is>
-          <t>Vientiane</t>
+          <t>Xinyu</t>
         </is>
       </c>
       <c r="E238" t="inlineStr">
         <is>
-          <t>Laos</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F238" t="inlineStr">
         <is>
-          <t>LA</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" s="1" t="inlineStr">
         <is>
-          <t>KHN</t>
+          <t>EVN</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>Xinyu, China</t>
+          <t>Yerevan, Armenia</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
@@ -7978,29 +7978,29 @@
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>Xinyu</t>
+          <t>Yerevan</t>
         </is>
       </c>
       <c r="E239" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Armenia</t>
         </is>
       </c>
       <c r="F239" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>AM</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" s="1" t="inlineStr">
         <is>
-          <t>EVN</t>
+          <t>JOG</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>Yerevan, Armenia</t>
+          <t>Yogyakarta, Indonesia</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
@@ -8010,29 +8010,29 @@
       </c>
       <c r="D240" t="inlineStr">
         <is>
-          <t>Yerevan</t>
+          <t>Yogyakarta</t>
         </is>
       </c>
       <c r="E240" t="inlineStr">
         <is>
-          <t>Armenia</t>
+          <t>Indonesia</t>
         </is>
       </c>
       <c r="F240" t="inlineStr">
         <is>
-          <t>AM</t>
+          <t>ID</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" s="1" t="inlineStr">
         <is>
-          <t>JOG</t>
+          <t>CGY</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>Yogyakarta, Indonesia</t>
+          <t>Cagayan de Oro, Philippines</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
@@ -8042,29 +8042,29 @@
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t>Yogyakarta</t>
+          <t>Cagayan de Oro</t>
         </is>
       </c>
       <c r="E241" t="inlineStr">
         <is>
-          <t>Indonesia</t>
+          <t>Philippines</t>
         </is>
       </c>
       <c r="F241" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>PH</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" s="1" t="inlineStr">
         <is>
-          <t>CGY</t>
+          <t>COK</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>Cagayan de Oro, Philippines</t>
+          <t>Kochi, India</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
@@ -8074,29 +8074,29 @@
       </c>
       <c r="D242" t="inlineStr">
         <is>
-          <t>Cagayan de Oro</t>
+          <t>Kochi</t>
         </is>
       </c>
       <c r="E242" t="inlineStr">
         <is>
-          <t>Philippines</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F242" t="inlineStr">
         <is>
-          <t>PH</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" s="1" t="inlineStr">
         <is>
-          <t>COK</t>
+          <t>DPS</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>Kochi, India</t>
+          <t>Denpasar, Indonesia</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
@@ -8106,29 +8106,29 @@
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>Kochi</t>
+          <t>Denpasar</t>
         </is>
       </c>
       <c r="E243" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Indonesia</t>
         </is>
       </c>
       <c r="F243" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>ID</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" s="1" t="inlineStr">
         <is>
-          <t>DPS</t>
+          <t>CNN</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>Denpasar, Indonesia</t>
+          <t>Kannur, India</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
@@ -8138,29 +8138,29 @@
       </c>
       <c r="D244" t="inlineStr">
         <is>
-          <t>Denpasar</t>
+          <t>Kannur</t>
         </is>
       </c>
       <c r="E244" t="inlineStr">
         <is>
-          <t>Indonesia</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F244" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" s="1" t="inlineStr">
         <is>
-          <t>CNN</t>
+          <t>SZX</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>Kannur, India</t>
+          <t>Shenzhen, China</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
@@ -8170,29 +8170,29 @@
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>Kannur</t>
+          <t>Shenzhen</t>
         </is>
       </c>
       <c r="E245" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F245" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" s="1" t="inlineStr">
         <is>
-          <t>SZX</t>
+          <t>KWE</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>Shenzhen, China</t>
+          <t>Guiyang, China</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
@@ -8202,7 +8202,7 @@
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>Shenzhen</t>
+          <t>Guiyang</t>
         </is>
       </c>
       <c r="E246" t="inlineStr">
@@ -8219,12 +8219,12 @@
     <row r="247">
       <c r="A247" s="1" t="inlineStr">
         <is>
-          <t>KWE</t>
+          <t>HGH</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>Guiyang, China</t>
+          <t>Shaoxing, China</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
@@ -8234,7 +8234,7 @@
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>Guiyang</t>
+          <t>Shaoxing</t>
         </is>
       </c>
       <c r="E247" t="inlineStr">
@@ -8251,12 +8251,12 @@
     <row r="248">
       <c r="A248" s="1" t="inlineStr">
         <is>
-          <t>HGH</t>
+          <t>CZX</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>Shaoxing, China</t>
+          <t>Changzhou, China</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
@@ -8266,7 +8266,7 @@
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>Shaoxing</t>
+          <t>Changzhou</t>
         </is>
       </c>
       <c r="E248" t="inlineStr">
@@ -8283,12 +8283,12 @@
     <row r="249">
       <c r="A249" s="1" t="inlineStr">
         <is>
-          <t>CZX</t>
+          <t>KMG</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>Changzhou, China</t>
+          <t>Kunming, China</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
@@ -8298,7 +8298,7 @@
       </c>
       <c r="D249" t="inlineStr">
         <is>
-          <t>Changzhou</t>
+          <t>Kunming</t>
         </is>
       </c>
       <c r="E249" t="inlineStr">
@@ -8315,12 +8315,12 @@
     <row r="250">
       <c r="A250" s="1" t="inlineStr">
         <is>
-          <t>KMG</t>
+          <t>CNX</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>Kunming, China</t>
+          <t>Chiang Mai, Thailand</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
@@ -8330,29 +8330,29 @@
       </c>
       <c r="D250" t="inlineStr">
         <is>
-          <t>Kunming</t>
+          <t>Chiang Mai</t>
         </is>
       </c>
       <c r="E250" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Thailand</t>
         </is>
       </c>
       <c r="F250" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>TH</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" s="1" t="inlineStr">
         <is>
-          <t>CNX</t>
+          <t>CGO</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>Chiang Mai, Thailand</t>
+          <t>Zhengzhou, China</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
@@ -8362,29 +8362,29 @@
       </c>
       <c r="D251" t="inlineStr">
         <is>
-          <t>Chiang Mai</t>
+          <t>Zhengzhou</t>
         </is>
       </c>
       <c r="E251" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F251" t="inlineStr">
         <is>
-          <t>TH</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" s="1" t="inlineStr">
         <is>
-          <t>CGO</t>
+          <t>TYN</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>Zhengzhou, China</t>
+          <t>Yangquan, China</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
@@ -8394,7 +8394,7 @@
       </c>
       <c r="D252" t="inlineStr">
         <is>
-          <t>Zhengzhou</t>
+          <t>Yangquan</t>
         </is>
       </c>
       <c r="E252" t="inlineStr">
@@ -8411,12 +8411,12 @@
     <row r="253">
       <c r="A253" s="1" t="inlineStr">
         <is>
-          <t>TYN</t>
+          <t>CSX</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>Yangquan, China</t>
+          <t>Changsha, China</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
@@ -8426,7 +8426,7 @@
       </c>
       <c r="D253" t="inlineStr">
         <is>
-          <t>Yangquan</t>
+          <t>Changsha</t>
         </is>
       </c>
       <c r="E253" t="inlineStr">
@@ -8443,12 +8443,12 @@
     <row r="254">
       <c r="A254" s="1" t="inlineStr">
         <is>
-          <t>CSX</t>
+          <t>DLC</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>Changsha, China</t>
+          <t>Dalian, China</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
@@ -8458,7 +8458,7 @@
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t>Changsha</t>
+          <t>Dalian</t>
         </is>
       </c>
       <c r="E254" t="inlineStr">
@@ -8475,12 +8475,12 @@
     <row r="255">
       <c r="A255" s="1" t="inlineStr">
         <is>
-          <t>DLC</t>
+          <t>CKG</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>Dalian, China</t>
+          <t>Chongqing, China</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
@@ -8490,7 +8490,7 @@
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>Dalian</t>
+          <t>Chongqing</t>
         </is>
       </c>
       <c r="E255" t="inlineStr">
@@ -8507,12 +8507,12 @@
     <row r="256">
       <c r="A256" s="1" t="inlineStr">
         <is>
-          <t>CKG</t>
+          <t>XFN</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>Chongqing, China</t>
+          <t>Xiangyang, China</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
@@ -8522,7 +8522,7 @@
       </c>
       <c r="D256" t="inlineStr">
         <is>
-          <t>Chongqing</t>
+          <t>Xiangyang</t>
         </is>
       </c>
       <c r="E256" t="inlineStr">
@@ -8539,12 +8539,12 @@
     <row r="257">
       <c r="A257" s="1" t="inlineStr">
         <is>
-          <t>XFN</t>
+          <t>DAD</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>Xiangyang, China</t>
+          <t>Da Nang, Vietnam</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
@@ -8554,29 +8554,29 @@
       </c>
       <c r="D257" t="inlineStr">
         <is>
-          <t>Xiangyang</t>
+          <t>Da Nang</t>
         </is>
       </c>
       <c r="E257" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Vietnam</t>
         </is>
       </c>
       <c r="F257" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>VN</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" s="1" t="inlineStr">
         <is>
-          <t>DAD</t>
+          <t>JXG</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>Da Nang, Vietnam</t>
+          <t>Jiaxing, China</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
@@ -8586,29 +8586,29 @@
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>Da Nang</t>
+          <t>Jiaxing</t>
         </is>
       </c>
       <c r="E258" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F258" t="inlineStr">
         <is>
-          <t>VN</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" s="1" t="inlineStr">
         <is>
-          <t>JXG</t>
+          <t>CRK</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>Jiaxing, China</t>
+          <t>Tarlac City, Philippines</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
@@ -8618,29 +8618,29 @@
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>Jiaxing</t>
+          <t>Tarlac City</t>
         </is>
       </c>
       <c r="E259" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Philippines</t>
         </is>
       </c>
       <c r="F259" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>PH</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" s="1" t="inlineStr">
         <is>
-          <t>CRK</t>
+          <t>PBH</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>Tarlac City, Philippines</t>
+          <t>Thimphu, Bhutan</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
@@ -8650,29 +8650,29 @@
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>Tarlac City</t>
+          <t>Thimphu</t>
         </is>
       </c>
       <c r="E260" t="inlineStr">
         <is>
-          <t>Philippines</t>
+          <t>Bhutan</t>
         </is>
       </c>
       <c r="F260" t="inlineStr">
         <is>
-          <t>PH</t>
+          <t>BT</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" s="1" t="inlineStr">
         <is>
-          <t>PBH</t>
+          <t>XIY</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>Thimphu, Bhutan</t>
+          <t>Baoji, China</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
@@ -8682,29 +8682,29 @@
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>Thimphu</t>
+          <t>Baoji</t>
         </is>
       </c>
       <c r="E261" t="inlineStr">
         <is>
-          <t>Bhutan</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F261" t="inlineStr">
         <is>
-          <t>BT</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" s="1" t="inlineStr">
         <is>
-          <t>XIY</t>
+          <t>KCH</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>Baoji, China</t>
+          <t>Kuching, Malaysia</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
@@ -8714,29 +8714,29 @@
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t>Baoji</t>
+          <t>Kuching</t>
         </is>
       </c>
       <c r="E262" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Malaysia</t>
         </is>
       </c>
       <c r="F262" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>MY</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" s="1" t="inlineStr">
         <is>
-          <t>KCH</t>
+          <t>AKX</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>Kuching, Malaysia</t>
+          <t>Aktobe, Kazakhstan</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
@@ -8746,29 +8746,29 @@
       </c>
       <c r="D263" t="inlineStr">
         <is>
-          <t>Kuching</t>
+          <t>Aktobe</t>
         </is>
       </c>
       <c r="E263" t="inlineStr">
         <is>
-          <t>Malaysia</t>
+          <t>Kazakhstan</t>
         </is>
       </c>
       <c r="F263" t="inlineStr">
         <is>
-          <t>MY</t>
+          <t>KZ</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" s="1" t="inlineStr">
         <is>
-          <t>AKX</t>
+          <t>TEN</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>Aktobe, Kazakhstan</t>
+          <t>Tongren, China</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
@@ -8778,29 +8778,29 @@
       </c>
       <c r="D264" t="inlineStr">
         <is>
-          <t>Aktobe</t>
+          <t>Tongren</t>
         </is>
       </c>
       <c r="E264" t="inlineStr">
         <is>
-          <t>Kazakhstan</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F264" t="inlineStr">
         <is>
-          <t>KZ</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" s="1" t="inlineStr">
         <is>
-          <t>TEN</t>
+          <t>HYN</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>Tongren, China</t>
+          <t>Taizhou, China</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
@@ -8810,7 +8810,7 @@
       </c>
       <c r="D265" t="inlineStr">
         <is>
-          <t>Tongren</t>
+          <t>Taizhou</t>
         </is>
       </c>
       <c r="E265" t="inlineStr">
@@ -8827,12 +8827,12 @@
     <row r="266">
       <c r="A266" s="1" t="inlineStr">
         <is>
-          <t>HYN</t>
+          <t>FRU</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>Taizhou, China</t>
+          <t>Bishkek, Kyrgyzstan</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
@@ -8842,29 +8842,29 @@
       </c>
       <c r="D266" t="inlineStr">
         <is>
-          <t>Taizhou</t>
+          <t>Bishkek</t>
         </is>
       </c>
       <c r="E266" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Kyrgyzstan</t>
         </is>
       </c>
       <c r="F266" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>KG</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" s="1" t="inlineStr">
         <is>
-          <t>FRU</t>
+          <t>MLG</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>Bishkek, Kyrgyzstan</t>
+          <t>Malang, Indonesia</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
@@ -8874,29 +8874,29 @@
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>Bishkek</t>
+          <t>Malang</t>
         </is>
       </c>
       <c r="E267" t="inlineStr">
         <is>
-          <t>Kyrgyzstan</t>
+          <t>Indonesia</t>
         </is>
       </c>
       <c r="F267" t="inlineStr">
         <is>
-          <t>KG</t>
+          <t>ID</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" s="1" t="inlineStr">
         <is>
-          <t>MLG</t>
+          <t>LHE</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>Malang, Indonesia</t>
+          <t>Lahore, Pakistan</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
@@ -8906,29 +8906,29 @@
       </c>
       <c r="D268" t="inlineStr">
         <is>
-          <t>Malang</t>
+          <t>Lahore</t>
         </is>
       </c>
       <c r="E268" t="inlineStr">
         <is>
-          <t>Indonesia</t>
+          <t>Pakistan</t>
         </is>
       </c>
       <c r="F268" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>PK</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" s="1" t="inlineStr">
         <is>
-          <t>LHE</t>
+          <t>CTU</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>Lahore, Pakistan</t>
+          <t>Chengdu, China</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
@@ -8938,29 +8938,29 @@
       </c>
       <c r="D269" t="inlineStr">
         <is>
-          <t>Lahore</t>
+          <t>Chengdu</t>
         </is>
       </c>
       <c r="E269" t="inlineStr">
         <is>
-          <t>Pakistan</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F269" t="inlineStr">
         <is>
-          <t>PK</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" s="1" t="inlineStr">
         <is>
-          <t>CTU</t>
+          <t>AGR</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>Chengdu, China</t>
+          <t>Agra, India</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
@@ -8970,29 +8970,29 @@
       </c>
       <c r="D270" t="inlineStr">
         <is>
-          <t>Chengdu</t>
+          <t>Agra</t>
         </is>
       </c>
       <c r="E270" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F270" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" s="1" t="inlineStr">
         <is>
-          <t>AGR</t>
+          <t>CJB</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>Agra, India</t>
+          <t>Coimbatore, India</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
@@ -9002,7 +9002,7 @@
       </c>
       <c r="D271" t="inlineStr">
         <is>
-          <t>Agra</t>
+          <t>Coimbatore</t>
         </is>
       </c>
       <c r="E271" t="inlineStr">
@@ -9019,12 +9019,12 @@
     <row r="272">
       <c r="A272" s="1" t="inlineStr">
         <is>
-          <t>CJB</t>
+          <t>ACX</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>Coimbatore, India</t>
+          <t>Xingyi, China</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
@@ -9034,29 +9034,29 @@
       </c>
       <c r="D272" t="inlineStr">
         <is>
-          <t>Coimbatore</t>
+          <t>Xingyi</t>
         </is>
       </c>
       <c r="E272" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F272" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="273">
       <c r="A273" s="1" t="inlineStr">
         <is>
-          <t>ACX</t>
+          <t>BBI</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>Xingyi, China</t>
+          <t>Bhubaneswar, India</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
@@ -9066,29 +9066,29 @@
       </c>
       <c r="D273" t="inlineStr">
         <is>
-          <t>Xingyi</t>
+          <t>Bhubaneswar</t>
         </is>
       </c>
       <c r="E273" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F273" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="274">
       <c r="A274" s="1" t="inlineStr">
         <is>
-          <t>BBI</t>
+          <t>LYA</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>Bhubaneswar, India</t>
+          <t>Luoyang, China</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
@@ -9098,29 +9098,29 @@
       </c>
       <c r="D274" t="inlineStr">
         <is>
-          <t>Bhubaneswar</t>
+          <t>Luoyang</t>
         </is>
       </c>
       <c r="E274" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F274" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="275">
       <c r="A275" s="1" t="inlineStr">
         <is>
-          <t>LYA</t>
+          <t>PNQ</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>Luoyang, China</t>
+          <t>Pune, India</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
@@ -9130,29 +9130,29 @@
       </c>
       <c r="D275" t="inlineStr">
         <is>
-          <t>Luoyang</t>
+          <t>Pune</t>
         </is>
       </c>
       <c r="E275" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F275" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="276">
       <c r="A276" s="1" t="inlineStr">
         <is>
-          <t>PNQ</t>
+          <t>JRG</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>Pune, India</t>
+          <t>Sambalpur, India</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
@@ -9162,7 +9162,7 @@
       </c>
       <c r="D276" t="inlineStr">
         <is>
-          <t>Pune</t>
+          <t>Sambalpur</t>
         </is>
       </c>
       <c r="E276" t="inlineStr">
@@ -9179,12 +9179,12 @@
     <row r="277">
       <c r="A277" s="1" t="inlineStr">
         <is>
-          <t>JRG</t>
+          <t>AVA</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>Sambalpur, India</t>
+          <t>Anshun, China</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
@@ -9194,29 +9194,29 @@
       </c>
       <c r="D277" t="inlineStr">
         <is>
-          <t>Sambalpur</t>
+          <t>Anshun</t>
         </is>
       </c>
       <c r="E277" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F277" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="278">
       <c r="A278" s="1" t="inlineStr">
         <is>
-          <t>AVA</t>
+          <t>NQZ</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>Anshun, China</t>
+          <t>Astana, Kazakhstan</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
@@ -9226,29 +9226,29 @@
       </c>
       <c r="D278" t="inlineStr">
         <is>
-          <t>Anshun</t>
+          <t>Astana</t>
         </is>
       </c>
       <c r="E278" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Kazakhstan</t>
         </is>
       </c>
       <c r="F278" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>KZ</t>
         </is>
       </c>
     </row>
     <row r="279">
       <c r="A279" s="1" t="inlineStr">
         <is>
-          <t>NQZ</t>
+          <t>BDQ</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>Astana, Kazakhstan</t>
+          <t>Jamnagar, India</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
@@ -9258,29 +9258,29 @@
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>Astana</t>
+          <t>Jamnagar</t>
         </is>
       </c>
       <c r="E279" t="inlineStr">
         <is>
-          <t>Kazakhstan</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F279" t="inlineStr">
         <is>
-          <t>KZ</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" s="1" t="inlineStr">
         <is>
-          <t>BDQ</t>
+          <t>UDR</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>Jamnagar, India</t>
+          <t>Udaipur, India</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
@@ -9290,7 +9290,7 @@
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>Jamnagar</t>
+          <t>Udaipur</t>
         </is>
       </c>
       <c r="E280" t="inlineStr">
@@ -9307,12 +9307,12 @@
     <row r="281">
       <c r="A281" s="1" t="inlineStr">
         <is>
-          <t>UDR</t>
+          <t>AIP</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>Udaipur, India</t>
+          <t>Jalandhar, India</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
@@ -9322,7 +9322,7 @@
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>Udaipur</t>
+          <t>Jalandhar</t>
         </is>
       </c>
       <c r="E281" t="inlineStr">
@@ -9339,12 +9339,12 @@
     <row r="282">
       <c r="A282" s="1" t="inlineStr">
         <is>
-          <t>AIP</t>
+          <t>LHW</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>Jalandhar, India</t>
+          <t>Lanzhou, China</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
@@ -9354,29 +9354,29 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>Jalandhar</t>
+          <t>Lanzhou</t>
         </is>
       </c>
       <c r="E282" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F282" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>CN</t>
         </is>
       </c>
     </row>
     <row r="283">
       <c r="A283" s="1" t="inlineStr">
         <is>
-          <t>LHW</t>
+          <t>DYU</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>Lanzhou, China</t>
+          <t>Dushanbe, Tajikistan</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
@@ -9386,29 +9386,29 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>Lanzhou</t>
+          <t>Dushanbe</t>
         </is>
       </c>
       <c r="E283" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Tajikistan</t>
         </is>
       </c>
       <c r="F283" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>TJ</t>
         </is>
       </c>
     </row>
     <row r="284">
       <c r="A284" s="1" t="inlineStr">
         <is>
-          <t>DYU</t>
+          <t>LUH</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>Dushanbe, Tajikistan</t>
+          <t>Ludhiana, India</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
@@ -9418,61 +9418,61 @@
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>Dushanbe</t>
+          <t>Ludhiana</t>
         </is>
       </c>
       <c r="E284" t="inlineStr">
         <is>
-          <t>Tajikistan</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F284" t="inlineStr">
         <is>
-          <t>TJ</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="285">
       <c r="A285" s="1" t="inlineStr">
         <is>
-          <t>LUH</t>
+          <t>ABQ</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>Ludhiana, India</t>
+          <t>Albuquerque, NM, United States</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>Asia</t>
+          <t>North America</t>
         </is>
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>Ludhiana</t>
+          <t>Albuquerque, NM</t>
         </is>
       </c>
       <c r="E285" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F285" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="286">
       <c r="A286" s="1" t="inlineStr">
         <is>
-          <t>ABQ</t>
+          <t>ANC</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>Albuquerque, NM, United States</t>
+          <t>Anchorage, AK, United States</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
@@ -9482,7 +9482,7 @@
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>Albuquerque, NM</t>
+          <t>Anchorage, AK</t>
         </is>
       </c>
       <c r="E286" t="inlineStr">
@@ -9499,12 +9499,12 @@
     <row r="287">
       <c r="A287" s="1" t="inlineStr">
         <is>
-          <t>ANC</t>
+          <t>IAD</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>Anchorage, AK, United States</t>
+          <t>Ashburn, VA, United States</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
@@ -9514,7 +9514,7 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>Anchorage, AK</t>
+          <t>Ashburn, VA</t>
         </is>
       </c>
       <c r="E287" t="inlineStr">
@@ -9531,12 +9531,12 @@
     <row r="288">
       <c r="A288" s="1" t="inlineStr">
         <is>
-          <t>IAD</t>
+          <t>ATL</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>Ashburn, VA, United States</t>
+          <t>Atlanta, GA, United States</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
@@ -9546,7 +9546,7 @@
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>Ashburn, VA</t>
+          <t>Atlanta, GA</t>
         </is>
       </c>
       <c r="E288" t="inlineStr">
@@ -9563,12 +9563,12 @@
     <row r="289">
       <c r="A289" s="1" t="inlineStr">
         <is>
-          <t>ATL</t>
+          <t>AUS</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>Atlanta, GA, United States</t>
+          <t>Austin, TX, United States</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
@@ -9578,7 +9578,7 @@
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>Atlanta, GA</t>
+          <t>Austin, TX</t>
         </is>
       </c>
       <c r="E289" t="inlineStr">
@@ -9595,12 +9595,12 @@
     <row r="290">
       <c r="A290" s="1" t="inlineStr">
         <is>
-          <t>AUS</t>
+          <t>BGR</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>Austin, TX, United States</t>
+          <t>Bangor, ME, United States</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
@@ -9610,7 +9610,7 @@
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>Austin, TX</t>
+          <t>Bangor, ME</t>
         </is>
       </c>
       <c r="E290" t="inlineStr">
@@ -9627,12 +9627,12 @@
     <row r="291">
       <c r="A291" s="1" t="inlineStr">
         <is>
-          <t>BGR</t>
+          <t>BOS</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>Bangor, ME, United States</t>
+          <t>Boston, MA, United States</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
@@ -9642,7 +9642,7 @@
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>Bangor, ME</t>
+          <t>Boston, MA</t>
         </is>
       </c>
       <c r="E291" t="inlineStr">
@@ -9659,12 +9659,12 @@
     <row r="292">
       <c r="A292" s="1" t="inlineStr">
         <is>
-          <t>BOS</t>
+          <t>BUF</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>Boston, MA, United States</t>
+          <t>Buffalo, NY, United States</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
@@ -9674,7 +9674,7 @@
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>Boston, MA</t>
+          <t>Buffalo, NY</t>
         </is>
       </c>
       <c r="E292" t="inlineStr">
@@ -9691,12 +9691,12 @@
     <row r="293">
       <c r="A293" s="1" t="inlineStr">
         <is>
-          <t>BUF</t>
+          <t>YYC</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>Buffalo, NY, United States</t>
+          <t>Calgary, AB, Canada</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
@@ -9706,29 +9706,29 @@
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>Buffalo, NY</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="E293" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F293" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="294">
       <c r="A294" s="1" t="inlineStr">
         <is>
-          <t>YYC</t>
+          <t>CLT</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>Calgary, AB, Canada</t>
+          <t>Charlotte, NC, United States</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
@@ -9738,29 +9738,29 @@
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Charlotte, NC</t>
         </is>
       </c>
       <c r="E294" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F294" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="295">
       <c r="A295" s="1" t="inlineStr">
         <is>
-          <t>CLT</t>
+          <t>ORD</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>Charlotte, NC, United States</t>
+          <t>Chicago, IL, United States</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -9770,7 +9770,7 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>Charlotte, NC</t>
+          <t>Chicago, IL</t>
         </is>
       </c>
       <c r="E295" t="inlineStr">
@@ -9787,12 +9787,12 @@
     <row r="296">
       <c r="A296" s="1" t="inlineStr">
         <is>
-          <t>ORD</t>
+          <t>CLE</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>Chicago, IL, United States</t>
+          <t>Cleveland, OH, United States</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -9802,7 +9802,7 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>Chicago, IL</t>
+          <t>Cleveland, OH</t>
         </is>
       </c>
       <c r="E296" t="inlineStr">
@@ -9819,12 +9819,12 @@
     <row r="297">
       <c r="A297" s="1" t="inlineStr">
         <is>
-          <t>CLE</t>
+          <t>CMH</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>Cleveland, OH, United States</t>
+          <t>Columbus, OH, United States</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
@@ -9834,7 +9834,7 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>Cleveland, OH</t>
+          <t>Columbus, OH</t>
         </is>
       </c>
       <c r="E297" t="inlineStr">
@@ -9851,12 +9851,12 @@
     <row r="298">
       <c r="A298" s="1" t="inlineStr">
         <is>
-          <t>CMH</t>
+          <t>DFW</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>Columbus, OH, United States</t>
+          <t>Dallas, TX, United States</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
@@ -9866,7 +9866,7 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>Columbus, OH</t>
+          <t>Dallas, TX</t>
         </is>
       </c>
       <c r="E298" t="inlineStr">
@@ -9883,12 +9883,12 @@
     <row r="299">
       <c r="A299" s="1" t="inlineStr">
         <is>
-          <t>DFW</t>
+          <t>DEN</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>Dallas, TX, United States</t>
+          <t>Denver, CO, United States</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
@@ -9898,7 +9898,7 @@
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>Dallas, TX</t>
+          <t>Denver, CO</t>
         </is>
       </c>
       <c r="E299" t="inlineStr">
@@ -9915,12 +9915,12 @@
     <row r="300">
       <c r="A300" s="1" t="inlineStr">
         <is>
-          <t>DEN</t>
+          <t>DTW</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>Denver, CO, United States</t>
+          <t>Detroit, MI, United States</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
@@ -9930,7 +9930,7 @@
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>Denver, CO</t>
+          <t>Detroit, MI</t>
         </is>
       </c>
       <c r="E300" t="inlineStr">
@@ -9947,12 +9947,12 @@
     <row r="301">
       <c r="A301" s="1" t="inlineStr">
         <is>
-          <t>DTW</t>
+          <t>RDU</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>Detroit, MI, United States</t>
+          <t>Durham, NC, United States</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
@@ -9962,7 +9962,7 @@
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>Detroit, MI</t>
+          <t>Durham, NC</t>
         </is>
       </c>
       <c r="E301" t="inlineStr">
@@ -9979,12 +9979,12 @@
     <row r="302">
       <c r="A302" s="1" t="inlineStr">
         <is>
-          <t>RDU</t>
+          <t>GDL</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>Durham, NC, United States</t>
+          <t>Guadalajara, Mexico</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
@@ -9994,29 +9994,29 @@
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>Durham, NC</t>
+          <t>Guadalajara</t>
         </is>
       </c>
       <c r="E302" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F302" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
     </row>
     <row r="303">
       <c r="A303" s="1" t="inlineStr">
         <is>
-          <t>GDL</t>
+          <t>YHZ</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>Guadalajara, Mexico</t>
+          <t>Halifax, Canada</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
@@ -10026,29 +10026,29 @@
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>Guadalajara</t>
+          <t>Halifax</t>
         </is>
       </c>
       <c r="E303" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F303" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="304">
       <c r="A304" s="1" t="inlineStr">
         <is>
-          <t>YHZ</t>
+          <t>HNL</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>Halifax, Canada</t>
+          <t>Honolulu, HI, United States</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
@@ -10058,29 +10058,29 @@
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>Halifax</t>
+          <t>Honolulu, HI</t>
         </is>
       </c>
       <c r="E304" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F304" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="305">
       <c r="A305" s="1" t="inlineStr">
         <is>
-          <t>HNL</t>
+          <t>IAH</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>Honolulu, HI, United States</t>
+          <t>Houston, TX, United States</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
@@ -10090,7 +10090,7 @@
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>Honolulu, HI</t>
+          <t>Houston, TX</t>
         </is>
       </c>
       <c r="E305" t="inlineStr">
@@ -10107,12 +10107,12 @@
     <row r="306">
       <c r="A306" s="1" t="inlineStr">
         <is>
-          <t>IAH</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>Houston, TX, United States</t>
+          <t>Indianapolis, IN, United States</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
@@ -10122,7 +10122,7 @@
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t>Houston, TX</t>
+          <t>Indianapolis, IN</t>
         </is>
       </c>
       <c r="E306" t="inlineStr">
@@ -10139,12 +10139,12 @@
     <row r="307">
       <c r="A307" s="1" t="inlineStr">
         <is>
-          <t>IND</t>
+          <t>JAX</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>Indianapolis, IN, United States</t>
+          <t>Jacksonville, FL, United States</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
@@ -10154,7 +10154,7 @@
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>Indianapolis, IN</t>
+          <t>Jacksonville, FL</t>
         </is>
       </c>
       <c r="E307" t="inlineStr">
@@ -10171,12 +10171,12 @@
     <row r="308">
       <c r="A308" s="1" t="inlineStr">
         <is>
-          <t>JAX</t>
+          <t>MCI</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>Jacksonville, FL, United States</t>
+          <t>Kansas City, MO, United States</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
@@ -10186,7 +10186,7 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>Jacksonville, FL</t>
+          <t>Kansas City, MO</t>
         </is>
       </c>
       <c r="E308" t="inlineStr">
@@ -10203,12 +10203,12 @@
     <row r="309">
       <c r="A309" s="1" t="inlineStr">
         <is>
-          <t>MCI</t>
+          <t>KIN</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>Kansas City, MO, United States</t>
+          <t>Kingston, Jamaica</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
@@ -10218,29 +10218,29 @@
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>Kansas City, MO</t>
+          <t>Kingston</t>
         </is>
       </c>
       <c r="E309" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Jamaica</t>
         </is>
       </c>
       <c r="F309" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>JM</t>
         </is>
       </c>
     </row>
     <row r="310">
       <c r="A310" s="1" t="inlineStr">
         <is>
-          <t>KIN</t>
+          <t>LAS</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>Kingston, Jamaica</t>
+          <t>Las Vegas, NV, United States</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
@@ -10250,29 +10250,29 @@
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>Kingston</t>
+          <t>Las Vegas, NV</t>
         </is>
       </c>
       <c r="E310" t="inlineStr">
         <is>
-          <t>Jamaica</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F310" t="inlineStr">
         <is>
-          <t>JM</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="311">
       <c r="A311" s="1" t="inlineStr">
         <is>
-          <t>LAS</t>
+          <t>LAX</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Las Vegas, NV, United States</t>
+          <t>Los Angeles, CA, United States</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
@@ -10282,7 +10282,7 @@
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>Las Vegas, NV</t>
+          <t>Los Angeles, CA</t>
         </is>
       </c>
       <c r="E311" t="inlineStr">
@@ -10299,12 +10299,12 @@
     <row r="312">
       <c r="A312" s="1" t="inlineStr">
         <is>
-          <t>LAX</t>
+          <t>MEM</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>Los Angeles, CA, United States</t>
+          <t>Memphis, TN, United States</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
@@ -10314,7 +10314,7 @@
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>Los Angeles, CA</t>
+          <t>Memphis, TN</t>
         </is>
       </c>
       <c r="E312" t="inlineStr">
@@ -10331,12 +10331,12 @@
     <row r="313">
       <c r="A313" s="1" t="inlineStr">
         <is>
-          <t>MEM</t>
+          <t>MEX</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Memphis, TN, United States</t>
+          <t>Mexico City, Mexico</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
@@ -10346,29 +10346,29 @@
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>Memphis, TN</t>
+          <t>Mexico City</t>
         </is>
       </c>
       <c r="E313" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F313" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
     </row>
     <row r="314">
       <c r="A314" s="1" t="inlineStr">
         <is>
-          <t>MEX</t>
+          <t>MIA</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Mexico City, Mexico</t>
+          <t>Miami, FL, United States</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -10378,29 +10378,29 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>Mexico City</t>
+          <t>Miami, FL</t>
         </is>
       </c>
       <c r="E314" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F314" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="315">
       <c r="A315" s="1" t="inlineStr">
         <is>
-          <t>MIA</t>
+          <t>MSP</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>Miami, FL, United States</t>
+          <t>Minneapolis, MN, United States</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
@@ -10410,7 +10410,7 @@
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>Miami, FL</t>
+          <t>Minneapolis, MN</t>
         </is>
       </c>
       <c r="E315" t="inlineStr">
@@ -10427,12 +10427,12 @@
     <row r="316">
       <c r="A316" s="1" t="inlineStr">
         <is>
-          <t>MSP</t>
+          <t>YUL</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Minneapolis, MN, United States</t>
+          <t>Montréal, QC, Canada</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
@@ -10442,29 +10442,29 @@
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>Minneapolis, MN</t>
+          <t>Montréal, QC</t>
         </is>
       </c>
       <c r="E316" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F316" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="317">
       <c r="A317" s="1" t="inlineStr">
         <is>
-          <t>YUL</t>
+          <t>BNA</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Montréal, QC, Canada</t>
+          <t>Nashville, United States</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -10474,29 +10474,29 @@
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t>Montréal, QC</t>
+          <t>Nashville</t>
         </is>
       </c>
       <c r="E317" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F317" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="318">
       <c r="A318" s="1" t="inlineStr">
         <is>
-          <t>BNA</t>
+          <t>EWR</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>Nashville, United States</t>
+          <t>Newark, NJ, United States</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
@@ -10506,7 +10506,7 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>Nashville</t>
+          <t>Newark, NJ</t>
         </is>
       </c>
       <c r="E318" t="inlineStr">
@@ -10523,12 +10523,12 @@
     <row r="319">
       <c r="A319" s="1" t="inlineStr">
         <is>
-          <t>EWR</t>
+          <t>ORF</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Newark, NJ, United States</t>
+          <t>Norfolk, VA, United States</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
@@ -10538,7 +10538,7 @@
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>Newark, NJ</t>
+          <t>Norfolk, VA</t>
         </is>
       </c>
       <c r="E319" t="inlineStr">
@@ -10555,12 +10555,12 @@
     <row r="320">
       <c r="A320" s="1" t="inlineStr">
         <is>
-          <t>ORF</t>
+          <t>OKC</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Norfolk, VA, United States</t>
+          <t>Oklahoma City, OK, United States</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -10570,7 +10570,7 @@
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t>Norfolk, VA</t>
+          <t>Oklahoma City, OK</t>
         </is>
       </c>
       <c r="E320" t="inlineStr">
@@ -10587,12 +10587,12 @@
     <row r="321">
       <c r="A321" s="1" t="inlineStr">
         <is>
-          <t>OKC</t>
+          <t>OMA</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>Oklahoma City, OK, United States</t>
+          <t>Omaha, NE, United States</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
@@ -10602,7 +10602,7 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>Oklahoma City, OK</t>
+          <t>Omaha, NE</t>
         </is>
       </c>
       <c r="E321" t="inlineStr">
@@ -10619,12 +10619,12 @@
     <row r="322">
       <c r="A322" s="1" t="inlineStr">
         <is>
-          <t>OMA</t>
+          <t>PHL</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>Omaha, NE, United States</t>
+          <t>Philadelphia, United States</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
@@ -10634,7 +10634,7 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>Omaha, NE</t>
+          <t>Philadelphia</t>
         </is>
       </c>
       <c r="E322" t="inlineStr">
@@ -10651,12 +10651,12 @@
     <row r="323">
       <c r="A323" s="1" t="inlineStr">
         <is>
-          <t>PHL</t>
+          <t>PHX</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>Philadelphia, United States</t>
+          <t>Phoenix, AZ, United States</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -10666,7 +10666,7 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>Philadelphia</t>
+          <t>Phoenix, AZ</t>
         </is>
       </c>
       <c r="E323" t="inlineStr">
@@ -10683,12 +10683,12 @@
     <row r="324">
       <c r="A324" s="1" t="inlineStr">
         <is>
-          <t>PHX</t>
+          <t>PIT</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>Phoenix, AZ, United States</t>
+          <t>Pittsburgh, PA, United States</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -10698,7 +10698,7 @@
       </c>
       <c r="D324" t="inlineStr">
         <is>
-          <t>Phoenix, AZ</t>
+          <t>Pittsburgh, PA</t>
         </is>
       </c>
       <c r="E324" t="inlineStr">
@@ -10715,12 +10715,12 @@
     <row r="325">
       <c r="A325" s="1" t="inlineStr">
         <is>
-          <t>PIT</t>
+          <t>PDX</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>Pittsburgh, PA, United States</t>
+          <t>Portland, OR, United States</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -10730,7 +10730,7 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>Pittsburgh, PA</t>
+          <t>Portland, OR</t>
         </is>
       </c>
       <c r="E325" t="inlineStr">
@@ -10747,12 +10747,12 @@
     <row r="326">
       <c r="A326" s="1" t="inlineStr">
         <is>
-          <t>PDX</t>
+          <t>QRO</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>Portland, OR, United States</t>
+          <t>Queretaro, MX, Mexico</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
@@ -10762,29 +10762,29 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>Portland, OR</t>
+          <t>Queretaro, MX</t>
         </is>
       </c>
       <c r="E326" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F326" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
     </row>
     <row r="327">
       <c r="A327" s="1" t="inlineStr">
         <is>
-          <t>QRO</t>
+          <t>RIC</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>Queretaro, MX, Mexico</t>
+          <t>Richmond, VA, United States</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
@@ -10794,29 +10794,29 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>Queretaro, MX</t>
+          <t>Richmond, VA</t>
         </is>
       </c>
       <c r="E327" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F327" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="328">
       <c r="A328" s="1" t="inlineStr">
         <is>
-          <t>RIC</t>
+          <t>SMF</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>Richmond, VA, United States</t>
+          <t>Sacramento, CA, United States</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
@@ -10826,7 +10826,7 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>Richmond, VA</t>
+          <t>Sacramento, CA</t>
         </is>
       </c>
       <c r="E328" t="inlineStr">
@@ -10843,12 +10843,12 @@
     <row r="329">
       <c r="A329" s="1" t="inlineStr">
         <is>
-          <t>SMF</t>
+          <t>SLC</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>Sacramento, CA, United States</t>
+          <t>Salt Lake City, UT, United States</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
@@ -10858,7 +10858,7 @@
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>Sacramento, CA</t>
+          <t>Salt Lake City, UT</t>
         </is>
       </c>
       <c r="E329" t="inlineStr">
@@ -10875,12 +10875,12 @@
     <row r="330">
       <c r="A330" s="1" t="inlineStr">
         <is>
-          <t>SLC</t>
+          <t>SAT</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>Salt Lake City, UT, United States</t>
+          <t>San Antonio, TX, United States</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
@@ -10890,7 +10890,7 @@
       </c>
       <c r="D330" t="inlineStr">
         <is>
-          <t>Salt Lake City, UT</t>
+          <t>San Antonio, TX</t>
         </is>
       </c>
       <c r="E330" t="inlineStr">
@@ -10907,12 +10907,12 @@
     <row r="331">
       <c r="A331" s="1" t="inlineStr">
         <is>
-          <t>SAT</t>
+          <t>SAN</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>San Antonio, TX, United States</t>
+          <t>San Diego, CA, United States</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
@@ -10922,7 +10922,7 @@
       </c>
       <c r="D331" t="inlineStr">
         <is>
-          <t>San Antonio, TX</t>
+          <t>San Diego, CA</t>
         </is>
       </c>
       <c r="E331" t="inlineStr">
@@ -10939,12 +10939,12 @@
     <row r="332">
       <c r="A332" s="1" t="inlineStr">
         <is>
-          <t>SAN</t>
+          <t>SFO</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>San Diego, CA, United States</t>
+          <t>San Francisco, CA, United States</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
@@ -10954,7 +10954,7 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>San Diego, CA</t>
+          <t>San Francisco, CA</t>
         </is>
       </c>
       <c r="E332" t="inlineStr">
@@ -10971,12 +10971,12 @@
     <row r="333">
       <c r="A333" s="1" t="inlineStr">
         <is>
-          <t>SFO</t>
+          <t>SJC</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>San Francisco, CA, United States</t>
+          <t>San Jose, CA, United States</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
@@ -10986,7 +10986,7 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>San Francisco, CA</t>
+          <t>San Jose, CA</t>
         </is>
       </c>
       <c r="E333" t="inlineStr">
@@ -11003,12 +11003,12 @@
     <row r="334">
       <c r="A334" s="1" t="inlineStr">
         <is>
-          <t>SJC</t>
+          <t>YXE</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>San Jose, CA, United States</t>
+          <t>Saskatoon, SK, Canada</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
@@ -11018,29 +11018,29 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>San Jose, CA</t>
+          <t>Saskatoon, SK</t>
         </is>
       </c>
       <c r="E334" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F334" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="335">
       <c r="A335" s="1" t="inlineStr">
         <is>
-          <t>YXE</t>
+          <t>SEA</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>Saskatoon, SK, Canada</t>
+          <t>Seattle, WA, United States</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
@@ -11050,29 +11050,29 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>Saskatoon, SK</t>
+          <t>Seattle, WA</t>
         </is>
       </c>
       <c r="E335" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F335" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="336">
       <c r="A336" s="1" t="inlineStr">
         <is>
-          <t>SEA</t>
+          <t>FSD</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>Seattle, WA, United States</t>
+          <t>Sioux Falls, SD, United States</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
@@ -11082,7 +11082,7 @@
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>Seattle, WA</t>
+          <t>Sioux Falls, SD</t>
         </is>
       </c>
       <c r="E336" t="inlineStr">
@@ -11099,12 +11099,12 @@
     <row r="337">
       <c r="A337" s="1" t="inlineStr">
         <is>
-          <t>FSD</t>
+          <t>STL</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>Sioux Falls, SD, United States</t>
+          <t>St. Louis, MO, United States</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
@@ -11114,7 +11114,7 @@
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>Sioux Falls, SD</t>
+          <t>St. Louis, MO</t>
         </is>
       </c>
       <c r="E337" t="inlineStr">
@@ -11131,12 +11131,12 @@
     <row r="338">
       <c r="A338" s="1" t="inlineStr">
         <is>
-          <t>STL</t>
+          <t>TLH</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>St. Louis, MO, United States</t>
+          <t>Tallahassee, FL, United States</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
@@ -11146,7 +11146,7 @@
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>St. Louis, MO</t>
+          <t>Tallahassee, FL</t>
         </is>
       </c>
       <c r="E338" t="inlineStr">
@@ -11163,12 +11163,12 @@
     <row r="339">
       <c r="A339" s="1" t="inlineStr">
         <is>
-          <t>TLH</t>
+          <t>TPA</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>Tallahassee, FL, United States</t>
+          <t>Tampa, FL, United States</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
@@ -11178,7 +11178,7 @@
       </c>
       <c r="D339" t="inlineStr">
         <is>
-          <t>Tallahassee, FL</t>
+          <t>Tampa, FL</t>
         </is>
       </c>
       <c r="E339" t="inlineStr">
@@ -11195,12 +11195,12 @@
     <row r="340">
       <c r="A340" s="1" t="inlineStr">
         <is>
-          <t>TPA</t>
+          <t>YYZ</t>
         </is>
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>Tampa, FL, United States</t>
+          <t>Toronto, ON, Canada</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
@@ -11210,29 +11210,29 @@
       </c>
       <c r="D340" t="inlineStr">
         <is>
-          <t>Tampa, FL</t>
+          <t>Toronto, ON</t>
         </is>
       </c>
       <c r="E340" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F340" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="341">
       <c r="A341" s="1" t="inlineStr">
         <is>
-          <t>YYZ</t>
+          <t>YVR</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>Toronto, ON, Canada</t>
+          <t>Vancouver, BC, Canada</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
@@ -11242,7 +11242,7 @@
       </c>
       <c r="D341" t="inlineStr">
         <is>
-          <t>Toronto, ON</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="E341" t="inlineStr">
@@ -11259,12 +11259,12 @@
     <row r="342">
       <c r="A342" s="1" t="inlineStr">
         <is>
-          <t>YVR</t>
+          <t>YWG</t>
         </is>
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>Vancouver, BC, Canada</t>
+          <t>Winnipeg, MB, Canada</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
@@ -11274,7 +11274,7 @@
       </c>
       <c r="D342" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Winnipeg, MB</t>
         </is>
       </c>
       <c r="E342" t="inlineStr">
@@ -11291,12 +11291,12 @@
     <row r="343">
       <c r="A343" s="1" t="inlineStr">
         <is>
-          <t>YWG</t>
+          <t>CVG</t>
         </is>
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>Winnipeg, MB, Canada</t>
+          <t>Cincinnati, United States</t>
         </is>
       </c>
       <c r="C343" t="inlineStr">
@@ -11306,47 +11306,15 @@
       </c>
       <c r="D343" t="inlineStr">
         <is>
-          <t>Winnipeg, MB</t>
+          <t>Cincinnati</t>
         </is>
       </c>
       <c r="E343" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F343" t="inlineStr">
-        <is>
-          <t>CA</t>
-        </is>
-      </c>
-    </row>
-    <row r="344">
-      <c r="A344" s="1" t="inlineStr">
-        <is>
-          <t>CVG</t>
-        </is>
-      </c>
-      <c r="B344" t="inlineStr">
-        <is>
-          <t>Cincinnati, United States</t>
-        </is>
-      </c>
-      <c r="C344" t="inlineStr">
-        <is>
-          <t>North America</t>
-        </is>
-      </c>
-      <c r="D344" t="inlineStr">
-        <is>
-          <t>Cincinnati</t>
-        </is>
-      </c>
-      <c r="E344" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="F344" t="inlineStr">
         <is>
           <t>US</t>
         </is>

</xml_diff>

<commit_message>
update generated data Triggered by 5a9ffa35f3cce90a20537dd3267813f0ea3376fc
</commit_message>
<xml_diff>
--- a/DC-Colos.xlsx
+++ b/DC-Colos.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F343"/>
+  <dimension ref="A1:F342"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9659,12 +9659,12 @@
     <row r="292">
       <c r="A292" s="1" t="inlineStr">
         <is>
-          <t>BUF</t>
+          <t>YYC</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>Buffalo, NY, United States</t>
+          <t>Calgary, AB, Canada</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
@@ -9674,29 +9674,29 @@
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>Buffalo, NY</t>
+          <t>Calgary, AB</t>
         </is>
       </c>
       <c r="E292" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F292" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="293">
       <c r="A293" s="1" t="inlineStr">
         <is>
-          <t>YYC</t>
+          <t>CLT</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>Calgary, AB, Canada</t>
+          <t>Charlotte, NC, United States</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
@@ -9706,29 +9706,29 @@
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>Calgary, AB</t>
+          <t>Charlotte, NC</t>
         </is>
       </c>
       <c r="E293" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F293" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="294">
       <c r="A294" s="1" t="inlineStr">
         <is>
-          <t>CLT</t>
+          <t>ORD</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>Charlotte, NC, United States</t>
+          <t>Chicago, IL, United States</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
@@ -9738,7 +9738,7 @@
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>Charlotte, NC</t>
+          <t>Chicago, IL</t>
         </is>
       </c>
       <c r="E294" t="inlineStr">
@@ -9755,12 +9755,12 @@
     <row r="295">
       <c r="A295" s="1" t="inlineStr">
         <is>
-          <t>ORD</t>
+          <t>CLE</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>Chicago, IL, United States</t>
+          <t>Cleveland, OH, United States</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -9770,7 +9770,7 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>Chicago, IL</t>
+          <t>Cleveland, OH</t>
         </is>
       </c>
       <c r="E295" t="inlineStr">
@@ -9787,12 +9787,12 @@
     <row r="296">
       <c r="A296" s="1" t="inlineStr">
         <is>
-          <t>CLE</t>
+          <t>CMH</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>Cleveland, OH, United States</t>
+          <t>Columbus, OH, United States</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -9802,7 +9802,7 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>Cleveland, OH</t>
+          <t>Columbus, OH</t>
         </is>
       </c>
       <c r="E296" t="inlineStr">
@@ -9819,12 +9819,12 @@
     <row r="297">
       <c r="A297" s="1" t="inlineStr">
         <is>
-          <t>CMH</t>
+          <t>DFW</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>Columbus, OH, United States</t>
+          <t>Dallas, TX, United States</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
@@ -9834,7 +9834,7 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>Columbus, OH</t>
+          <t>Dallas, TX</t>
         </is>
       </c>
       <c r="E297" t="inlineStr">
@@ -9851,12 +9851,12 @@
     <row r="298">
       <c r="A298" s="1" t="inlineStr">
         <is>
-          <t>DFW</t>
+          <t>DEN</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>Dallas, TX, United States</t>
+          <t>Denver, CO, United States</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
@@ -9866,7 +9866,7 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>Dallas, TX</t>
+          <t>Denver, CO</t>
         </is>
       </c>
       <c r="E298" t="inlineStr">
@@ -9883,12 +9883,12 @@
     <row r="299">
       <c r="A299" s="1" t="inlineStr">
         <is>
-          <t>DEN</t>
+          <t>DTW</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>Denver, CO, United States</t>
+          <t>Detroit, MI, United States</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
@@ -9898,7 +9898,7 @@
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>Denver, CO</t>
+          <t>Detroit, MI</t>
         </is>
       </c>
       <c r="E299" t="inlineStr">
@@ -9915,12 +9915,12 @@
     <row r="300">
       <c r="A300" s="1" t="inlineStr">
         <is>
-          <t>DTW</t>
+          <t>RDU</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>Detroit, MI, United States</t>
+          <t>Durham, NC, United States</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
@@ -9930,7 +9930,7 @@
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>Detroit, MI</t>
+          <t>Durham, NC</t>
         </is>
       </c>
       <c r="E300" t="inlineStr">
@@ -9947,12 +9947,12 @@
     <row r="301">
       <c r="A301" s="1" t="inlineStr">
         <is>
-          <t>RDU</t>
+          <t>GDL</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>Durham, NC, United States</t>
+          <t>Guadalajara, Mexico</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
@@ -9962,29 +9962,29 @@
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>Durham, NC</t>
+          <t>Guadalajara</t>
         </is>
       </c>
       <c r="E301" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F301" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
     </row>
     <row r="302">
       <c r="A302" s="1" t="inlineStr">
         <is>
-          <t>GDL</t>
+          <t>YHZ</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>Guadalajara, Mexico</t>
+          <t>Halifax, Canada</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
@@ -9994,29 +9994,29 @@
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>Guadalajara</t>
+          <t>Halifax</t>
         </is>
       </c>
       <c r="E302" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F302" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="303">
       <c r="A303" s="1" t="inlineStr">
         <is>
-          <t>YHZ</t>
+          <t>HNL</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>Halifax, Canada</t>
+          <t>Honolulu, HI, United States</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
@@ -10026,29 +10026,29 @@
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>Halifax</t>
+          <t>Honolulu, HI</t>
         </is>
       </c>
       <c r="E303" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F303" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="304">
       <c r="A304" s="1" t="inlineStr">
         <is>
-          <t>HNL</t>
+          <t>IAH</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>Honolulu, HI, United States</t>
+          <t>Houston, TX, United States</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
@@ -10058,7 +10058,7 @@
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>Honolulu, HI</t>
+          <t>Houston, TX</t>
         </is>
       </c>
       <c r="E304" t="inlineStr">
@@ -10075,12 +10075,12 @@
     <row r="305">
       <c r="A305" s="1" t="inlineStr">
         <is>
-          <t>IAH</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>Houston, TX, United States</t>
+          <t>Indianapolis, IN, United States</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
@@ -10090,7 +10090,7 @@
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>Houston, TX</t>
+          <t>Indianapolis, IN</t>
         </is>
       </c>
       <c r="E305" t="inlineStr">
@@ -10107,12 +10107,12 @@
     <row r="306">
       <c r="A306" s="1" t="inlineStr">
         <is>
-          <t>IND</t>
+          <t>JAX</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>Indianapolis, IN, United States</t>
+          <t>Jacksonville, FL, United States</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
@@ -10122,7 +10122,7 @@
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t>Indianapolis, IN</t>
+          <t>Jacksonville, FL</t>
         </is>
       </c>
       <c r="E306" t="inlineStr">
@@ -10139,12 +10139,12 @@
     <row r="307">
       <c r="A307" s="1" t="inlineStr">
         <is>
-          <t>JAX</t>
+          <t>MCI</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>Jacksonville, FL, United States</t>
+          <t>Kansas City, MO, United States</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
@@ -10154,7 +10154,7 @@
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>Jacksonville, FL</t>
+          <t>Kansas City, MO</t>
         </is>
       </c>
       <c r="E307" t="inlineStr">
@@ -10171,12 +10171,12 @@
     <row r="308">
       <c r="A308" s="1" t="inlineStr">
         <is>
-          <t>MCI</t>
+          <t>KIN</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>Kansas City, MO, United States</t>
+          <t>Kingston, Jamaica</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
@@ -10186,29 +10186,29 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>Kansas City, MO</t>
+          <t>Kingston</t>
         </is>
       </c>
       <c r="E308" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Jamaica</t>
         </is>
       </c>
       <c r="F308" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>JM</t>
         </is>
       </c>
     </row>
     <row r="309">
       <c r="A309" s="1" t="inlineStr">
         <is>
-          <t>KIN</t>
+          <t>LAS</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>Kingston, Jamaica</t>
+          <t>Las Vegas, NV, United States</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
@@ -10218,29 +10218,29 @@
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>Kingston</t>
+          <t>Las Vegas, NV</t>
         </is>
       </c>
       <c r="E309" t="inlineStr">
         <is>
-          <t>Jamaica</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F309" t="inlineStr">
         <is>
-          <t>JM</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="310">
       <c r="A310" s="1" t="inlineStr">
         <is>
-          <t>LAS</t>
+          <t>LAX</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>Las Vegas, NV, United States</t>
+          <t>Los Angeles, CA, United States</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
@@ -10250,7 +10250,7 @@
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>Las Vegas, NV</t>
+          <t>Los Angeles, CA</t>
         </is>
       </c>
       <c r="E310" t="inlineStr">
@@ -10267,12 +10267,12 @@
     <row r="311">
       <c r="A311" s="1" t="inlineStr">
         <is>
-          <t>LAX</t>
+          <t>MEM</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Los Angeles, CA, United States</t>
+          <t>Memphis, TN, United States</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
@@ -10282,7 +10282,7 @@
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>Los Angeles, CA</t>
+          <t>Memphis, TN</t>
         </is>
       </c>
       <c r="E311" t="inlineStr">
@@ -10299,12 +10299,12 @@
     <row r="312">
       <c r="A312" s="1" t="inlineStr">
         <is>
-          <t>MEM</t>
+          <t>MEX</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>Memphis, TN, United States</t>
+          <t>Mexico City, Mexico</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
@@ -10314,29 +10314,29 @@
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>Memphis, TN</t>
+          <t>Mexico City</t>
         </is>
       </c>
       <c r="E312" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F312" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
     </row>
     <row r="313">
       <c r="A313" s="1" t="inlineStr">
         <is>
-          <t>MEX</t>
+          <t>MIA</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Mexico City, Mexico</t>
+          <t>Miami, FL, United States</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
@@ -10346,29 +10346,29 @@
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>Mexico City</t>
+          <t>Miami, FL</t>
         </is>
       </c>
       <c r="E313" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F313" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="314">
       <c r="A314" s="1" t="inlineStr">
         <is>
-          <t>MIA</t>
+          <t>MSP</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Miami, FL, United States</t>
+          <t>Minneapolis, MN, United States</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -10378,7 +10378,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>Miami, FL</t>
+          <t>Minneapolis, MN</t>
         </is>
       </c>
       <c r="E314" t="inlineStr">
@@ -10395,12 +10395,12 @@
     <row r="315">
       <c r="A315" s="1" t="inlineStr">
         <is>
-          <t>MSP</t>
+          <t>YUL</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>Minneapolis, MN, United States</t>
+          <t>Montréal, QC, Canada</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
@@ -10410,29 +10410,29 @@
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>Minneapolis, MN</t>
+          <t>Montréal, QC</t>
         </is>
       </c>
       <c r="E315" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F315" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="316">
       <c r="A316" s="1" t="inlineStr">
         <is>
-          <t>YUL</t>
+          <t>BNA</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Montréal, QC, Canada</t>
+          <t>Nashville, United States</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
@@ -10442,29 +10442,29 @@
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>Montréal, QC</t>
+          <t>Nashville</t>
         </is>
       </c>
       <c r="E316" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F316" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="317">
       <c r="A317" s="1" t="inlineStr">
         <is>
-          <t>BNA</t>
+          <t>EWR</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Nashville, United States</t>
+          <t>Newark, NJ, United States</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -10474,7 +10474,7 @@
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t>Nashville</t>
+          <t>Newark, NJ</t>
         </is>
       </c>
       <c r="E317" t="inlineStr">
@@ -10491,12 +10491,12 @@
     <row r="318">
       <c r="A318" s="1" t="inlineStr">
         <is>
-          <t>EWR</t>
+          <t>ORF</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>Newark, NJ, United States</t>
+          <t>Norfolk, VA, United States</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
@@ -10506,7 +10506,7 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>Newark, NJ</t>
+          <t>Norfolk, VA</t>
         </is>
       </c>
       <c r="E318" t="inlineStr">
@@ -10523,12 +10523,12 @@
     <row r="319">
       <c r="A319" s="1" t="inlineStr">
         <is>
-          <t>ORF</t>
+          <t>OKC</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Norfolk, VA, United States</t>
+          <t>Oklahoma City, OK, United States</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
@@ -10538,7 +10538,7 @@
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>Norfolk, VA</t>
+          <t>Oklahoma City, OK</t>
         </is>
       </c>
       <c r="E319" t="inlineStr">
@@ -10555,12 +10555,12 @@
     <row r="320">
       <c r="A320" s="1" t="inlineStr">
         <is>
-          <t>OKC</t>
+          <t>OMA</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Oklahoma City, OK, United States</t>
+          <t>Omaha, NE, United States</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -10570,7 +10570,7 @@
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t>Oklahoma City, OK</t>
+          <t>Omaha, NE</t>
         </is>
       </c>
       <c r="E320" t="inlineStr">
@@ -10587,12 +10587,12 @@
     <row r="321">
       <c r="A321" s="1" t="inlineStr">
         <is>
-          <t>OMA</t>
+          <t>PHL</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>Omaha, NE, United States</t>
+          <t>Philadelphia, United States</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
@@ -10602,7 +10602,7 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>Omaha, NE</t>
+          <t>Philadelphia</t>
         </is>
       </c>
       <c r="E321" t="inlineStr">
@@ -10619,12 +10619,12 @@
     <row r="322">
       <c r="A322" s="1" t="inlineStr">
         <is>
-          <t>PHL</t>
+          <t>PHX</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>Philadelphia, United States</t>
+          <t>Phoenix, AZ, United States</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
@@ -10634,7 +10634,7 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>Philadelphia</t>
+          <t>Phoenix, AZ</t>
         </is>
       </c>
       <c r="E322" t="inlineStr">
@@ -10651,12 +10651,12 @@
     <row r="323">
       <c r="A323" s="1" t="inlineStr">
         <is>
-          <t>PHX</t>
+          <t>PIT</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>Phoenix, AZ, United States</t>
+          <t>Pittsburgh, PA, United States</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -10666,7 +10666,7 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>Phoenix, AZ</t>
+          <t>Pittsburgh, PA</t>
         </is>
       </c>
       <c r="E323" t="inlineStr">
@@ -10683,12 +10683,12 @@
     <row r="324">
       <c r="A324" s="1" t="inlineStr">
         <is>
-          <t>PIT</t>
+          <t>PDX</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>Pittsburgh, PA, United States</t>
+          <t>Portland, OR, United States</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -10698,7 +10698,7 @@
       </c>
       <c r="D324" t="inlineStr">
         <is>
-          <t>Pittsburgh, PA</t>
+          <t>Portland, OR</t>
         </is>
       </c>
       <c r="E324" t="inlineStr">
@@ -10715,12 +10715,12 @@
     <row r="325">
       <c r="A325" s="1" t="inlineStr">
         <is>
-          <t>PDX</t>
+          <t>QRO</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>Portland, OR, United States</t>
+          <t>Queretaro, MX, Mexico</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -10730,29 +10730,29 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>Portland, OR</t>
+          <t>Queretaro, MX</t>
         </is>
       </c>
       <c r="E325" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F325" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
     </row>
     <row r="326">
       <c r="A326" s="1" t="inlineStr">
         <is>
-          <t>QRO</t>
+          <t>RIC</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>Queretaro, MX, Mexico</t>
+          <t>Richmond, VA, United States</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
@@ -10762,29 +10762,29 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>Queretaro, MX</t>
+          <t>Richmond, VA</t>
         </is>
       </c>
       <c r="E326" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F326" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="327">
       <c r="A327" s="1" t="inlineStr">
         <is>
-          <t>RIC</t>
+          <t>SMF</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>Richmond, VA, United States</t>
+          <t>Sacramento, CA, United States</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
@@ -10794,7 +10794,7 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>Richmond, VA</t>
+          <t>Sacramento, CA</t>
         </is>
       </c>
       <c r="E327" t="inlineStr">
@@ -10811,12 +10811,12 @@
     <row r="328">
       <c r="A328" s="1" t="inlineStr">
         <is>
-          <t>SMF</t>
+          <t>SLC</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>Sacramento, CA, United States</t>
+          <t>Salt Lake City, UT, United States</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
@@ -10826,7 +10826,7 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>Sacramento, CA</t>
+          <t>Salt Lake City, UT</t>
         </is>
       </c>
       <c r="E328" t="inlineStr">
@@ -10843,12 +10843,12 @@
     <row r="329">
       <c r="A329" s="1" t="inlineStr">
         <is>
-          <t>SLC</t>
+          <t>SAT</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>Salt Lake City, UT, United States</t>
+          <t>San Antonio, TX, United States</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
@@ -10858,7 +10858,7 @@
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>Salt Lake City, UT</t>
+          <t>San Antonio, TX</t>
         </is>
       </c>
       <c r="E329" t="inlineStr">
@@ -10875,12 +10875,12 @@
     <row r="330">
       <c r="A330" s="1" t="inlineStr">
         <is>
-          <t>SAT</t>
+          <t>SAN</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>San Antonio, TX, United States</t>
+          <t>San Diego, CA, United States</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
@@ -10890,7 +10890,7 @@
       </c>
       <c r="D330" t="inlineStr">
         <is>
-          <t>San Antonio, TX</t>
+          <t>San Diego, CA</t>
         </is>
       </c>
       <c r="E330" t="inlineStr">
@@ -10907,12 +10907,12 @@
     <row r="331">
       <c r="A331" s="1" t="inlineStr">
         <is>
-          <t>SAN</t>
+          <t>SFO</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>San Diego, CA, United States</t>
+          <t>San Francisco, CA, United States</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
@@ -10922,7 +10922,7 @@
       </c>
       <c r="D331" t="inlineStr">
         <is>
-          <t>San Diego, CA</t>
+          <t>San Francisco, CA</t>
         </is>
       </c>
       <c r="E331" t="inlineStr">
@@ -10939,12 +10939,12 @@
     <row r="332">
       <c r="A332" s="1" t="inlineStr">
         <is>
-          <t>SFO</t>
+          <t>SJC</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>San Francisco, CA, United States</t>
+          <t>San Jose, CA, United States</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
@@ -10954,7 +10954,7 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>San Francisco, CA</t>
+          <t>San Jose, CA</t>
         </is>
       </c>
       <c r="E332" t="inlineStr">
@@ -10971,12 +10971,12 @@
     <row r="333">
       <c r="A333" s="1" t="inlineStr">
         <is>
-          <t>SJC</t>
+          <t>YXE</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>San Jose, CA, United States</t>
+          <t>Saskatoon, SK, Canada</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
@@ -10986,29 +10986,29 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>San Jose, CA</t>
+          <t>Saskatoon, SK</t>
         </is>
       </c>
       <c r="E333" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F333" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="334">
       <c r="A334" s="1" t="inlineStr">
         <is>
-          <t>YXE</t>
+          <t>SEA</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>Saskatoon, SK, Canada</t>
+          <t>Seattle, WA, United States</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
@@ -11018,29 +11018,29 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>Saskatoon, SK</t>
+          <t>Seattle, WA</t>
         </is>
       </c>
       <c r="E334" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F334" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="335">
       <c r="A335" s="1" t="inlineStr">
         <is>
-          <t>SEA</t>
+          <t>FSD</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>Seattle, WA, United States</t>
+          <t>Sioux Falls, SD, United States</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
@@ -11050,7 +11050,7 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>Seattle, WA</t>
+          <t>Sioux Falls, SD</t>
         </is>
       </c>
       <c r="E335" t="inlineStr">
@@ -11067,12 +11067,12 @@
     <row r="336">
       <c r="A336" s="1" t="inlineStr">
         <is>
-          <t>FSD</t>
+          <t>STL</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>Sioux Falls, SD, United States</t>
+          <t>St. Louis, MO, United States</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
@@ -11082,7 +11082,7 @@
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>Sioux Falls, SD</t>
+          <t>St. Louis, MO</t>
         </is>
       </c>
       <c r="E336" t="inlineStr">
@@ -11099,12 +11099,12 @@
     <row r="337">
       <c r="A337" s="1" t="inlineStr">
         <is>
-          <t>STL</t>
+          <t>TLH</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>St. Louis, MO, United States</t>
+          <t>Tallahassee, FL, United States</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
@@ -11114,7 +11114,7 @@
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>St. Louis, MO</t>
+          <t>Tallahassee, FL</t>
         </is>
       </c>
       <c r="E337" t="inlineStr">
@@ -11131,12 +11131,12 @@
     <row r="338">
       <c r="A338" s="1" t="inlineStr">
         <is>
-          <t>TLH</t>
+          <t>TPA</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>Tallahassee, FL, United States</t>
+          <t>Tampa, FL, United States</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
@@ -11146,7 +11146,7 @@
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>Tallahassee, FL</t>
+          <t>Tampa, FL</t>
         </is>
       </c>
       <c r="E338" t="inlineStr">
@@ -11163,12 +11163,12 @@
     <row r="339">
       <c r="A339" s="1" t="inlineStr">
         <is>
-          <t>TPA</t>
+          <t>YYZ</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>Tampa, FL, United States</t>
+          <t>Toronto, ON, Canada</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
@@ -11178,29 +11178,29 @@
       </c>
       <c r="D339" t="inlineStr">
         <is>
-          <t>Tampa, FL</t>
+          <t>Toronto, ON</t>
         </is>
       </c>
       <c r="E339" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F339" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="340">
       <c r="A340" s="1" t="inlineStr">
         <is>
-          <t>YYZ</t>
+          <t>YVR</t>
         </is>
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>Toronto, ON, Canada</t>
+          <t>Vancouver, BC, Canada</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
@@ -11210,7 +11210,7 @@
       </c>
       <c r="D340" t="inlineStr">
         <is>
-          <t>Toronto, ON</t>
+          <t>Vancouver, BC</t>
         </is>
       </c>
       <c r="E340" t="inlineStr">
@@ -11227,12 +11227,12 @@
     <row r="341">
       <c r="A341" s="1" t="inlineStr">
         <is>
-          <t>YVR</t>
+          <t>YWG</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>Vancouver, BC, Canada</t>
+          <t>Winnipeg, MB, Canada</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
@@ -11242,7 +11242,7 @@
       </c>
       <c r="D341" t="inlineStr">
         <is>
-          <t>Vancouver, BC</t>
+          <t>Winnipeg, MB</t>
         </is>
       </c>
       <c r="E341" t="inlineStr">
@@ -11259,12 +11259,12 @@
     <row r="342">
       <c r="A342" s="1" t="inlineStr">
         <is>
-          <t>YWG</t>
+          <t>CVG</t>
         </is>
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>Winnipeg, MB, Canada</t>
+          <t>Cincinnati, United States</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
@@ -11274,47 +11274,15 @@
       </c>
       <c r="D342" t="inlineStr">
         <is>
-          <t>Winnipeg, MB</t>
+          <t>Cincinnati</t>
         </is>
       </c>
       <c r="E342" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F342" t="inlineStr">
-        <is>
-          <t>CA</t>
-        </is>
-      </c>
-    </row>
-    <row r="343">
-      <c r="A343" s="1" t="inlineStr">
-        <is>
-          <t>CVG</t>
-        </is>
-      </c>
-      <c r="B343" t="inlineStr">
-        <is>
-          <t>Cincinnati, United States</t>
-        </is>
-      </c>
-      <c r="C343" t="inlineStr">
-        <is>
-          <t>North America</t>
-        </is>
-      </c>
-      <c r="D343" t="inlineStr">
-        <is>
-          <t>Cincinnati</t>
-        </is>
-      </c>
-      <c r="E343" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="F343" t="inlineStr">
         <is>
           <t>US</t>
         </is>

</xml_diff>

<commit_message>
update generated data Triggered by b3896aec12d7871e80bcabe71900d9f8167fd6dc
</commit_message>
<xml_diff>
--- a/DC-Colos.xlsx
+++ b/DC-Colos.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F342"/>
+  <dimension ref="A1:F343"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9279,44 +9279,44 @@
     <row r="280">
       <c r="A280" s="1" t="inlineStr">
         <is>
-          <t>ABQ</t>
+          <t>JAI</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>Albuquerque, United States</t>
+          <t>“Jaipur”, India</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>North America</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>Albuquerque</t>
+          <t>“Jaipur”</t>
         </is>
       </c>
       <c r="E280" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F280" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
     <row r="281">
       <c r="A281" s="1" t="inlineStr">
         <is>
-          <t>ANC</t>
+          <t>ABQ</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>Anchorage, United States</t>
+          <t>Albuquerque, United States</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
@@ -9326,7 +9326,7 @@
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>Anchorage</t>
+          <t>Albuquerque</t>
         </is>
       </c>
       <c r="E281" t="inlineStr">
@@ -9343,12 +9343,12 @@
     <row r="282">
       <c r="A282" s="1" t="inlineStr">
         <is>
-          <t>IAD</t>
+          <t>ANC</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>Ashburn, United States</t>
+          <t>Anchorage, United States</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
@@ -9358,7 +9358,7 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>Ashburn</t>
+          <t>Anchorage</t>
         </is>
       </c>
       <c r="E282" t="inlineStr">
@@ -9375,12 +9375,12 @@
     <row r="283">
       <c r="A283" s="1" t="inlineStr">
         <is>
-          <t>ATL</t>
+          <t>IAD</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>Atlanta, United States</t>
+          <t>Ashburn, United States</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
@@ -9390,7 +9390,7 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>Atlanta</t>
+          <t>Ashburn</t>
         </is>
       </c>
       <c r="E283" t="inlineStr">
@@ -9407,12 +9407,12 @@
     <row r="284">
       <c r="A284" s="1" t="inlineStr">
         <is>
-          <t>AUS</t>
+          <t>ATL</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>Austin, United States</t>
+          <t>Atlanta, United States</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
@@ -9422,7 +9422,7 @@
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>Austin</t>
+          <t>Atlanta</t>
         </is>
       </c>
       <c r="E284" t="inlineStr">
@@ -9439,12 +9439,12 @@
     <row r="285">
       <c r="A285" s="1" t="inlineStr">
         <is>
-          <t>BGR</t>
+          <t>AUS</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>Bangor, United States</t>
+          <t>Austin, United States</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
@@ -9454,7 +9454,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>Bangor</t>
+          <t>Austin</t>
         </is>
       </c>
       <c r="E285" t="inlineStr">
@@ -9471,12 +9471,12 @@
     <row r="286">
       <c r="A286" s="1" t="inlineStr">
         <is>
-          <t>BOS</t>
+          <t>BGR</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>Boston, United States</t>
+          <t>Bangor, United States</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
@@ -9486,7 +9486,7 @@
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>Boston</t>
+          <t>Bangor</t>
         </is>
       </c>
       <c r="E286" t="inlineStr">
@@ -9503,12 +9503,12 @@
     <row r="287">
       <c r="A287" s="1" t="inlineStr">
         <is>
-          <t>YYC</t>
+          <t>BOS</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>Calgary, Canada</t>
+          <t>Boston, United States</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
@@ -9518,29 +9518,29 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>Calgary</t>
+          <t>Boston</t>
         </is>
       </c>
       <c r="E287" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F287" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="288">
       <c r="A288" s="1" t="inlineStr">
         <is>
-          <t>CLT</t>
+          <t>YYC</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>Charlotte, United States</t>
+          <t>Calgary, Canada</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
@@ -9550,29 +9550,29 @@
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>Charlotte</t>
+          <t>Calgary</t>
         </is>
       </c>
       <c r="E288" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F288" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="289">
       <c r="A289" s="1" t="inlineStr">
         <is>
-          <t>ORD</t>
+          <t>CLT</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>Chicago, United States</t>
+          <t>Charlotte, United States</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
@@ -9582,7 +9582,7 @@
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Charlotte</t>
         </is>
       </c>
       <c r="E289" t="inlineStr">
@@ -9599,12 +9599,12 @@
     <row r="290">
       <c r="A290" s="1" t="inlineStr">
         <is>
-          <t>CLE</t>
+          <t>ORD</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>Cleveland, United States</t>
+          <t>Chicago, United States</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
@@ -9614,7 +9614,7 @@
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>Cleveland</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="E290" t="inlineStr">
@@ -9631,12 +9631,12 @@
     <row r="291">
       <c r="A291" s="1" t="inlineStr">
         <is>
-          <t>CMH</t>
+          <t>CLE</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>Columbus, United States</t>
+          <t>Cleveland, United States</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
@@ -9646,7 +9646,7 @@
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>Columbus</t>
+          <t>Cleveland</t>
         </is>
       </c>
       <c r="E291" t="inlineStr">
@@ -9663,12 +9663,12 @@
     <row r="292">
       <c r="A292" s="1" t="inlineStr">
         <is>
-          <t>DFW</t>
+          <t>CMH</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>Dallas, United States</t>
+          <t>Columbus, United States</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
@@ -9678,7 +9678,7 @@
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>Dallas</t>
+          <t>Columbus</t>
         </is>
       </c>
       <c r="E292" t="inlineStr">
@@ -9695,12 +9695,12 @@
     <row r="293">
       <c r="A293" s="1" t="inlineStr">
         <is>
-          <t>DEN</t>
+          <t>DFW</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>Denver, United States</t>
+          <t>Dallas, United States</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
@@ -9710,7 +9710,7 @@
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>Denver</t>
+          <t>Dallas</t>
         </is>
       </c>
       <c r="E293" t="inlineStr">
@@ -9727,12 +9727,12 @@
     <row r="294">
       <c r="A294" s="1" t="inlineStr">
         <is>
-          <t>DTW</t>
+          <t>DEN</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>Detroit, United States</t>
+          <t>Denver, United States</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
@@ -9742,7 +9742,7 @@
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>Detroit</t>
+          <t>Denver</t>
         </is>
       </c>
       <c r="E294" t="inlineStr">
@@ -9759,12 +9759,12 @@
     <row r="295">
       <c r="A295" s="1" t="inlineStr">
         <is>
-          <t>RDU</t>
+          <t>DTW</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>Durham, United States</t>
+          <t>Detroit, United States</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -9774,7 +9774,7 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>Durham</t>
+          <t>Detroit</t>
         </is>
       </c>
       <c r="E295" t="inlineStr">
@@ -9791,12 +9791,12 @@
     <row r="296">
       <c r="A296" s="1" t="inlineStr">
         <is>
-          <t>GDL</t>
+          <t>RDU</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>Guadalajara, Mexico</t>
+          <t>Durham, United States</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -9806,29 +9806,29 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>Guadalajara</t>
+          <t>Durham</t>
         </is>
       </c>
       <c r="E296" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F296" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="297">
       <c r="A297" s="1" t="inlineStr">
         <is>
-          <t>YHZ</t>
+          <t>GDL</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>Halifax, Canada</t>
+          <t>Guadalajara, Mexico</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
@@ -9838,29 +9838,29 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>Halifax</t>
+          <t>Guadalajara</t>
         </is>
       </c>
       <c r="E297" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F297" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>MX</t>
         </is>
       </c>
     </row>
     <row r="298">
       <c r="A298" s="1" t="inlineStr">
         <is>
-          <t>GUA</t>
+          <t>YHZ</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>Guatemala City, Guatemala</t>
+          <t>Halifax, Canada</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
@@ -9870,29 +9870,29 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>Guatemala City</t>
+          <t>Halifax</t>
         </is>
       </c>
       <c r="E298" t="inlineStr">
         <is>
-          <t>Guatemala</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F298" t="inlineStr">
         <is>
-          <t>GT</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="299">
       <c r="A299" s="1" t="inlineStr">
         <is>
-          <t>HNL</t>
+          <t>GUA</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>Honolulu, United States</t>
+          <t>Guatemala City, Guatemala</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
@@ -9902,29 +9902,29 @@
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>Honolulu</t>
+          <t>Guatemala City</t>
         </is>
       </c>
       <c r="E299" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Guatemala</t>
         </is>
       </c>
       <c r="F299" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>GT</t>
         </is>
       </c>
     </row>
     <row r="300">
       <c r="A300" s="1" t="inlineStr">
         <is>
-          <t>IAH</t>
+          <t>HNL</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>Houston, United States</t>
+          <t>Honolulu, United States</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
@@ -9934,7 +9934,7 @@
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Honolulu</t>
         </is>
       </c>
       <c r="E300" t="inlineStr">
@@ -9951,12 +9951,12 @@
     <row r="301">
       <c r="A301" s="1" t="inlineStr">
         <is>
-          <t>IND</t>
+          <t>IAH</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>Indianapolis, United States</t>
+          <t>Houston, United States</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
@@ -9966,7 +9966,7 @@
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>Indianapolis</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="E301" t="inlineStr">
@@ -9983,12 +9983,12 @@
     <row r="302">
       <c r="A302" s="1" t="inlineStr">
         <is>
-          <t>JAX</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>Jacksonville, United States</t>
+          <t>Indianapolis, United States</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
@@ -9998,7 +9998,7 @@
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>Jacksonville</t>
+          <t>Indianapolis</t>
         </is>
       </c>
       <c r="E302" t="inlineStr">
@@ -10015,12 +10015,12 @@
     <row r="303">
       <c r="A303" s="1" t="inlineStr">
         <is>
-          <t>MCI</t>
+          <t>JAX</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>Kansas City, United States</t>
+          <t>Jacksonville, United States</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
@@ -10030,7 +10030,7 @@
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>Kansas City</t>
+          <t>Jacksonville</t>
         </is>
       </c>
       <c r="E303" t="inlineStr">
@@ -10047,12 +10047,12 @@
     <row r="304">
       <c r="A304" s="1" t="inlineStr">
         <is>
-          <t>KIN</t>
+          <t>MCI</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>Kingston, Jamaica</t>
+          <t>Kansas City, United States</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
@@ -10062,29 +10062,29 @@
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>Kingston</t>
+          <t>Kansas City</t>
         </is>
       </c>
       <c r="E304" t="inlineStr">
         <is>
-          <t>Jamaica</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F304" t="inlineStr">
         <is>
-          <t>JM</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="305">
       <c r="A305" s="1" t="inlineStr">
         <is>
-          <t>LAS</t>
+          <t>KIN</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>Las Vegas, United States</t>
+          <t>Kingston, Jamaica</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
@@ -10094,29 +10094,29 @@
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>Las Vegas</t>
+          <t>Kingston</t>
         </is>
       </c>
       <c r="E305" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Jamaica</t>
         </is>
       </c>
       <c r="F305" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>JM</t>
         </is>
       </c>
     </row>
     <row r="306">
       <c r="A306" s="1" t="inlineStr">
         <is>
-          <t>LAX</t>
+          <t>LAS</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>Los Angeles, United States</t>
+          <t>Las Vegas, United States</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
@@ -10126,7 +10126,7 @@
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t>Los Angeles</t>
+          <t>Las Vegas</t>
         </is>
       </c>
       <c r="E306" t="inlineStr">
@@ -10143,12 +10143,12 @@
     <row r="307">
       <c r="A307" s="1" t="inlineStr">
         <is>
-          <t>MEM</t>
+          <t>LAX</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>Memphis, United States</t>
+          <t>Los Angeles, United States</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
@@ -10158,7 +10158,7 @@
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>Memphis</t>
+          <t>Los Angeles</t>
         </is>
       </c>
       <c r="E307" t="inlineStr">
@@ -10175,12 +10175,12 @@
     <row r="308">
       <c r="A308" s="1" t="inlineStr">
         <is>
-          <t>MEX</t>
+          <t>MEM</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>Mexico City, Mexico</t>
+          <t>Memphis, United States</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
@@ -10190,29 +10190,29 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>Mexico City</t>
+          <t>Memphis</t>
         </is>
       </c>
       <c r="E308" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F308" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="309">
       <c r="A309" s="1" t="inlineStr">
         <is>
-          <t>MIA</t>
+          <t>MEX</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>Miami, United States</t>
+          <t>Mexico City, Mexico</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
@@ -10222,29 +10222,29 @@
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>Miami</t>
+          <t>Mexico City</t>
         </is>
       </c>
       <c r="E309" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F309" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
     </row>
     <row r="310">
       <c r="A310" s="1" t="inlineStr">
         <is>
-          <t>MSP</t>
+          <t>MIA</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>Minneapolis, United States</t>
+          <t>Miami, United States</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
@@ -10254,7 +10254,7 @@
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>Minneapolis</t>
+          <t>Miami</t>
         </is>
       </c>
       <c r="E310" t="inlineStr">
@@ -10271,12 +10271,12 @@
     <row r="311">
       <c r="A311" s="1" t="inlineStr">
         <is>
-          <t>YUL</t>
+          <t>MSP</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Montréal, Canada</t>
+          <t>Minneapolis, United States</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
@@ -10286,29 +10286,29 @@
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>Montréal</t>
+          <t>Minneapolis</t>
         </is>
       </c>
       <c r="E311" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F311" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="312">
       <c r="A312" s="1" t="inlineStr">
         <is>
-          <t>BNA</t>
+          <t>YUL</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>Nashville, United States</t>
+          <t>Montréal, Canada</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
@@ -10318,29 +10318,29 @@
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>Nashville</t>
+          <t>Montréal</t>
         </is>
       </c>
       <c r="E312" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F312" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="313">
       <c r="A313" s="1" t="inlineStr">
         <is>
-          <t>EWR</t>
+          <t>BNA</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Newark, United States</t>
+          <t>Nashville, United States</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
@@ -10350,7 +10350,7 @@
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>Newark</t>
+          <t>Nashville</t>
         </is>
       </c>
       <c r="E313" t="inlineStr">
@@ -10367,12 +10367,12 @@
     <row r="314">
       <c r="A314" s="1" t="inlineStr">
         <is>
-          <t>ORF</t>
+          <t>EWR</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Norfolk, United States</t>
+          <t>Newark, United States</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -10382,7 +10382,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>Norfolk</t>
+          <t>Newark</t>
         </is>
       </c>
       <c r="E314" t="inlineStr">
@@ -10399,12 +10399,12 @@
     <row r="315">
       <c r="A315" s="1" t="inlineStr">
         <is>
-          <t>OKC</t>
+          <t>ORF</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>Oklahoma City, United States</t>
+          <t>Norfolk, United States</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
@@ -10414,7 +10414,7 @@
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>Oklahoma City</t>
+          <t>Norfolk</t>
         </is>
       </c>
       <c r="E315" t="inlineStr">
@@ -10431,12 +10431,12 @@
     <row r="316">
       <c r="A316" s="1" t="inlineStr">
         <is>
-          <t>OMA</t>
+          <t>OKC</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Omaha, United States</t>
+          <t>Oklahoma City, United States</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
@@ -10446,7 +10446,7 @@
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>Omaha</t>
+          <t>Oklahoma City</t>
         </is>
       </c>
       <c r="E316" t="inlineStr">
@@ -10463,12 +10463,12 @@
     <row r="317">
       <c r="A317" s="1" t="inlineStr">
         <is>
-          <t>PHL</t>
+          <t>OMA</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Philadelphia, United States</t>
+          <t>Omaha, United States</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -10478,7 +10478,7 @@
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t>Philadelphia</t>
+          <t>Omaha</t>
         </is>
       </c>
       <c r="E317" t="inlineStr">
@@ -10495,12 +10495,12 @@
     <row r="318">
       <c r="A318" s="1" t="inlineStr">
         <is>
-          <t>PHX</t>
+          <t>PHL</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>Phoenix, United States</t>
+          <t>Philadelphia, United States</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
@@ -10510,7 +10510,7 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>Phoenix</t>
+          <t>Philadelphia</t>
         </is>
       </c>
       <c r="E318" t="inlineStr">
@@ -10527,12 +10527,12 @@
     <row r="319">
       <c r="A319" s="1" t="inlineStr">
         <is>
-          <t>SDQ</t>
+          <t>PHX</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Santo Domingo, Dominican Republic</t>
+          <t>Phoenix, United States</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
@@ -10542,29 +10542,29 @@
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>Santo Domingo</t>
+          <t>Phoenix</t>
         </is>
       </c>
       <c r="E319" t="inlineStr">
         <is>
-          <t>Dominican Republic</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F319" t="inlineStr">
         <is>
-          <t>DO</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="320">
       <c r="A320" s="1" t="inlineStr">
         <is>
-          <t>PIT</t>
+          <t>SDQ</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Pittsburgh, United States</t>
+          <t>Santo Domingo, Dominican Republic</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -10574,29 +10574,29 @@
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t>Pittsburgh</t>
+          <t>Santo Domingo</t>
         </is>
       </c>
       <c r="E320" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Dominican Republic</t>
         </is>
       </c>
       <c r="F320" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>DO</t>
         </is>
       </c>
     </row>
     <row r="321">
       <c r="A321" s="1" t="inlineStr">
         <is>
-          <t>PDX</t>
+          <t>PIT</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>Portland, United States</t>
+          <t>Pittsburgh, United States</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
@@ -10606,7 +10606,7 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>Portland</t>
+          <t>Pittsburgh</t>
         </is>
       </c>
       <c r="E321" t="inlineStr">
@@ -10623,12 +10623,12 @@
     <row r="322">
       <c r="A322" s="1" t="inlineStr">
         <is>
-          <t>QRO</t>
+          <t>PDX</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>Queretaro, Mexico</t>
+          <t>Portland, United States</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
@@ -10638,29 +10638,29 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>Queretaro</t>
+          <t>Portland</t>
         </is>
       </c>
       <c r="E322" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F322" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="323">
       <c r="A323" s="1" t="inlineStr">
         <is>
-          <t>RIC</t>
+          <t>QRO</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>Richmond, United States</t>
+          <t>Queretaro, Mexico</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -10670,29 +10670,29 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>Richmond</t>
+          <t>Queretaro</t>
         </is>
       </c>
       <c r="E323" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F323" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
     </row>
     <row r="324">
       <c r="A324" s="1" t="inlineStr">
         <is>
-          <t>SMF</t>
+          <t>RIC</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>Sacramento, United States</t>
+          <t>Richmond, United States</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -10702,7 +10702,7 @@
       </c>
       <c r="D324" t="inlineStr">
         <is>
-          <t>Sacramento</t>
+          <t>Richmond</t>
         </is>
       </c>
       <c r="E324" t="inlineStr">
@@ -10719,12 +10719,12 @@
     <row r="325">
       <c r="A325" s="1" t="inlineStr">
         <is>
-          <t>SLC</t>
+          <t>SMF</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>Salt Lake City, United States</t>
+          <t>Sacramento, United States</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -10734,7 +10734,7 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>Salt Lake City</t>
+          <t>Sacramento</t>
         </is>
       </c>
       <c r="E325" t="inlineStr">
@@ -10751,12 +10751,12 @@
     <row r="326">
       <c r="A326" s="1" t="inlineStr">
         <is>
-          <t>SAT</t>
+          <t>SLC</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>San Antonio, United States</t>
+          <t>Salt Lake City, United States</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
@@ -10766,7 +10766,7 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>San Antonio</t>
+          <t>Salt Lake City</t>
         </is>
       </c>
       <c r="E326" t="inlineStr">
@@ -10783,12 +10783,12 @@
     <row r="327">
       <c r="A327" s="1" t="inlineStr">
         <is>
-          <t>SAN</t>
+          <t>SAT</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>San Diego, United States</t>
+          <t>San Antonio, United States</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
@@ -10798,7 +10798,7 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>San Diego</t>
+          <t>San Antonio</t>
         </is>
       </c>
       <c r="E327" t="inlineStr">
@@ -10815,12 +10815,12 @@
     <row r="328">
       <c r="A328" s="1" t="inlineStr">
         <is>
-          <t>SFO</t>
+          <t>SAN</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>San Francisco, United States</t>
+          <t>San Diego, United States</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
@@ -10830,7 +10830,7 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>San Francisco</t>
+          <t>San Diego</t>
         </is>
       </c>
       <c r="E328" t="inlineStr">
@@ -10847,12 +10847,12 @@
     <row r="329">
       <c r="A329" s="1" t="inlineStr">
         <is>
-          <t>SJC</t>
+          <t>SFO</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>San Jose, United States</t>
+          <t>San Francisco, United States</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
@@ -10862,7 +10862,7 @@
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>San Jose</t>
+          <t>San Francisco</t>
         </is>
       </c>
       <c r="E329" t="inlineStr">
@@ -10879,12 +10879,12 @@
     <row r="330">
       <c r="A330" s="1" t="inlineStr">
         <is>
-          <t>YXE</t>
+          <t>SJC</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>Saskatoon, Canada</t>
+          <t>San Jose, United States</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
@@ -10894,29 +10894,29 @@
       </c>
       <c r="D330" t="inlineStr">
         <is>
-          <t>Saskatoon</t>
+          <t>San Jose</t>
         </is>
       </c>
       <c r="E330" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F330" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="331">
       <c r="A331" s="1" t="inlineStr">
         <is>
-          <t>SEA</t>
+          <t>YXE</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>Seattle, United States</t>
+          <t>Saskatoon, Canada</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
@@ -10926,29 +10926,29 @@
       </c>
       <c r="D331" t="inlineStr">
         <is>
-          <t>Seattle</t>
+          <t>Saskatoon</t>
         </is>
       </c>
       <c r="E331" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F331" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="332">
       <c r="A332" s="1" t="inlineStr">
         <is>
-          <t>FSD</t>
+          <t>SEA</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>Sioux Falls, United States</t>
+          <t>Seattle, United States</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
@@ -10958,7 +10958,7 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>Sioux Falls</t>
+          <t>Seattle</t>
         </is>
       </c>
       <c r="E332" t="inlineStr">
@@ -10975,12 +10975,12 @@
     <row r="333">
       <c r="A333" s="1" t="inlineStr">
         <is>
-          <t>BGI</t>
+          <t>FSD</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>Bridgetown, Barbados</t>
+          <t>Sioux Falls, United States</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
@@ -10990,29 +10990,29 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>Bridgetown</t>
+          <t>Sioux Falls</t>
         </is>
       </c>
       <c r="E333" t="inlineStr">
         <is>
-          <t>Barbados</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F333" t="inlineStr">
         <is>
-          <t>BB</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="334">
       <c r="A334" s="1" t="inlineStr">
         <is>
-          <t>STL</t>
+          <t>BGI</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>St. Louis, United States</t>
+          <t>Bridgetown, Barbados</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
@@ -11022,29 +11022,29 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>St. Louis</t>
+          <t>Bridgetown</t>
         </is>
       </c>
       <c r="E334" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Barbados</t>
         </is>
       </c>
       <c r="F334" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>BB</t>
         </is>
       </c>
     </row>
     <row r="335">
       <c r="A335" s="1" t="inlineStr">
         <is>
-          <t>TLH</t>
+          <t>STL</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>Tallahassee, United States</t>
+          <t>St. Louis, United States</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
@@ -11054,7 +11054,7 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>Tallahassee</t>
+          <t>St. Louis</t>
         </is>
       </c>
       <c r="E335" t="inlineStr">
@@ -11071,12 +11071,12 @@
     <row r="336">
       <c r="A336" s="1" t="inlineStr">
         <is>
-          <t>STI</t>
+          <t>TLH</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>Santiago de los Caballeros, Dominican Republic</t>
+          <t>Tallahassee, United States</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
@@ -11086,29 +11086,29 @@
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>Santiago de los Caballeros</t>
+          <t>Tallahassee</t>
         </is>
       </c>
       <c r="E336" t="inlineStr">
         <is>
-          <t>Dominican Republic</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F336" t="inlineStr">
         <is>
-          <t>DO</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="337">
       <c r="A337" s="1" t="inlineStr">
         <is>
-          <t>TPA</t>
+          <t>STI</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>Tampa, United States</t>
+          <t>Santiago de los Caballeros, Dominican Republic</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
@@ -11118,29 +11118,29 @@
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>Tampa</t>
+          <t>Santiago de los Caballeros</t>
         </is>
       </c>
       <c r="E337" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Dominican Republic</t>
         </is>
       </c>
       <c r="F337" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>DO</t>
         </is>
       </c>
     </row>
     <row r="338">
       <c r="A338" s="1" t="inlineStr">
         <is>
-          <t>YYZ</t>
+          <t>TPA</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>Toronto, Canada</t>
+          <t>Tampa, United States</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
@@ -11150,29 +11150,29 @@
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>Toronto</t>
+          <t>Tampa</t>
         </is>
       </c>
       <c r="E338" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F338" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="339">
       <c r="A339" s="1" t="inlineStr">
         <is>
-          <t>YVR</t>
+          <t>YYZ</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>Vancouver, Canada</t>
+          <t>Toronto, Canada</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
@@ -11182,7 +11182,7 @@
       </c>
       <c r="D339" t="inlineStr">
         <is>
-          <t>Vancouver</t>
+          <t>Toronto</t>
         </is>
       </c>
       <c r="E339" t="inlineStr">
@@ -11199,12 +11199,12 @@
     <row r="340">
       <c r="A340" s="1" t="inlineStr">
         <is>
-          <t>SJU</t>
+          <t>YVR</t>
         </is>
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>San Juan, Puerto Rico</t>
+          <t>Vancouver, Canada</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
@@ -11214,29 +11214,29 @@
       </c>
       <c r="D340" t="inlineStr">
         <is>
-          <t>San Juan</t>
+          <t>Vancouver</t>
         </is>
       </c>
       <c r="E340" t="inlineStr">
         <is>
-          <t>Puerto Rico</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F340" t="inlineStr">
         <is>
-          <t>PR</t>
+          <t>CA</t>
         </is>
       </c>
     </row>
     <row r="341">
       <c r="A341" s="1" t="inlineStr">
         <is>
-          <t>YWG</t>
+          <t>SJU</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>Winnipeg, Canada</t>
+          <t>San Juan, Puerto Rico</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
@@ -11246,47 +11246,79 @@
       </c>
       <c r="D341" t="inlineStr">
         <is>
-          <t>Winnipeg</t>
+          <t>San Juan</t>
         </is>
       </c>
       <c r="E341" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Puerto Rico</t>
         </is>
       </c>
       <c r="F341" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>PR</t>
         </is>
       </c>
     </row>
     <row r="342">
       <c r="A342" s="1" t="inlineStr">
         <is>
+          <t>YWG</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>Winnipeg, Canada</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>North America</t>
+        </is>
+      </c>
+      <c r="D342" t="inlineStr">
+        <is>
+          <t>Winnipeg</t>
+        </is>
+      </c>
+      <c r="E342" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="F342" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" s="1" t="inlineStr">
+        <is>
           <t>CVG</t>
         </is>
       </c>
-      <c r="B342" t="inlineStr">
+      <c r="B343" t="inlineStr">
         <is>
           <t>Cincinnati, United States</t>
         </is>
       </c>
-      <c r="C342" t="inlineStr">
+      <c r="C343" t="inlineStr">
         <is>
           <t>North America</t>
         </is>
       </c>
-      <c r="D342" t="inlineStr">
+      <c r="D343" t="inlineStr">
         <is>
           <t>Cincinnati</t>
         </is>
       </c>
-      <c r="E342" t="inlineStr">
+      <c r="E343" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="F342" t="inlineStr">
+      <c r="F343" t="inlineStr">
         <is>
           <t>US</t>
         </is>

</xml_diff>